<commit_message>
auto: snapshot 2026-07-16 13:01:00
</commit_message>
<xml_diff>
--- a/clan_3815.xlsx
+++ b/clan_3815.xlsx
@@ -8,6 +8,7 @@
   </bookViews>
   <sheets>
     <sheet name="2026-07-15" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="2026-07-16" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -935,4 +936,508 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C33"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="25" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Clan: Mans Best Friend (3815)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Timestamp: 2026-07-16 13:01:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>Total Reps</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>Daily Reps (+1d)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>Nobodys Son</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="n">
+        <v>21308</v>
+      </c>
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>-12700</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>Create Character III</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="n">
+        <v>22920</v>
+      </c>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>+2078</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>Create Character IV</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="n">
+        <v>22831</v>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>+2055</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>Create Character V</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="n">
+        <v>22674</v>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>+2073</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>Anti-Hero</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="n">
+        <v>23948</v>
+      </c>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>Vigilante Shit</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="n">
+        <v>18454</v>
+      </c>
+      <c r="C9" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>Sweet Nothing</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="n">
+        <v>18834</v>
+      </c>
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>The Great War</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="n">
+        <v>18204</v>
+      </c>
+      <c r="C11" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">We Almost Broke Up </t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="n">
+        <v>24371</v>
+      </c>
+      <c r="C12" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="4" t="inlineStr">
+        <is>
+          <t>When Did You Get Hot</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="n">
+        <v>18854</v>
+      </c>
+      <c r="C13" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="4" t="inlineStr">
+        <is>
+          <t>Dont Worry Ill Make</t>
+        </is>
+      </c>
+      <c r="B14" s="5" t="n">
+        <v>19078</v>
+      </c>
+      <c r="C14" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="4" t="inlineStr">
+        <is>
+          <t>Goodbye</t>
+        </is>
+      </c>
+      <c r="B15" s="5" t="n">
+        <v>16849</v>
+      </c>
+      <c r="C15" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="4" t="inlineStr">
+        <is>
+          <t>Mans Best Friend</t>
+        </is>
+      </c>
+      <c r="B16" s="5" t="n">
+        <v>16410</v>
+      </c>
+      <c r="C16" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="4" t="inlineStr">
+        <is>
+          <t>Lavender Haze</t>
+        </is>
+      </c>
+      <c r="B17" s="5" t="n">
+        <v>15683</v>
+      </c>
+      <c r="C17" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="4" t="inlineStr">
+        <is>
+          <t>Never Getting Laid</t>
+        </is>
+      </c>
+      <c r="B18" s="5" t="n">
+        <v>24593</v>
+      </c>
+      <c r="C18" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="4" t="inlineStr">
+        <is>
+          <t>My Man on Willpower</t>
+        </is>
+      </c>
+      <c r="B19" s="5" t="n">
+        <v>18584</v>
+      </c>
+      <c r="C19" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="4" t="inlineStr">
+        <is>
+          <t>Manchild</t>
+        </is>
+      </c>
+      <c r="B20" s="5" t="n">
+        <v>19619</v>
+      </c>
+      <c r="C20" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="4" t="inlineStr">
+        <is>
+          <t>Sugar Talking</t>
+        </is>
+      </c>
+      <c r="B21" s="5" t="n">
+        <v>18618</v>
+      </c>
+      <c r="C21" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="4" t="inlineStr">
+        <is>
+          <t>Midnight Rain</t>
+        </is>
+      </c>
+      <c r="B22" s="5" t="n">
+        <v>16228</v>
+      </c>
+      <c r="C22" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="4" t="inlineStr">
+        <is>
+          <t>Nobodys Son</t>
+        </is>
+      </c>
+      <c r="B23" s="5" t="n">
+        <v>34008</v>
+      </c>
+      <c r="C23" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="4" t="inlineStr">
+        <is>
+          <t>House Tour</t>
+        </is>
+      </c>
+      <c r="B24" s="5" t="n">
+        <v>19332</v>
+      </c>
+      <c r="C24" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="4" t="inlineStr">
+        <is>
+          <t>Hanabi  Î±Î·Ð²Ï…</t>
+        </is>
+      </c>
+      <c r="B25" s="5" t="n">
+        <v>3550</v>
+      </c>
+      <c r="C25" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="4" t="inlineStr">
+        <is>
+          <t>Dummy</t>
+        </is>
+      </c>
+      <c r="B26" s="5" t="n">
+        <v>3500</v>
+      </c>
+      <c r="C26" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="4" t="inlineStr">
+        <is>
+          <t>DarkFire</t>
+        </is>
+      </c>
+      <c r="B27" s="5" t="n">
+        <v>8471</v>
+      </c>
+      <c r="C27" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="4" t="inlineStr">
+        <is>
+          <t>DarkSunny</t>
+        </is>
+      </c>
+      <c r="B28" s="5" t="n">
+        <v>8524</v>
+      </c>
+      <c r="C28" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="4" t="inlineStr">
+        <is>
+          <t>Dairen Uchiha</t>
+        </is>
+      </c>
+      <c r="B29" s="5" t="n">
+        <v>8364</v>
+      </c>
+      <c r="C29" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="4" t="inlineStr">
+        <is>
+          <t>LILI ZENIN®</t>
+        </is>
+      </c>
+      <c r="B30" s="5" t="n">
+        <v>7672</v>
+      </c>
+      <c r="C30" s="5" t="inlineStr">
+        <is>
+          <t>+1291</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="4" t="inlineStr">
+        <is>
+          <t>linda ZENIN ®</t>
+        </is>
+      </c>
+      <c r="B31" s="5" t="n">
+        <v>7572</v>
+      </c>
+      <c r="C31" s="5" t="inlineStr">
+        <is>
+          <t>+1241</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="4" t="inlineStr">
+        <is>
+          <t>SHINRAIN ZENIN®</t>
+        </is>
+      </c>
+      <c r="B32" s="5" t="n">
+        <v>7528</v>
+      </c>
+      <c r="C32" s="5" t="inlineStr">
+        <is>
+          <t>+1232</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="4" t="inlineStr">
+        <is>
+          <t>Go Go Juice</t>
+        </is>
+      </c>
+      <c r="B33" s="5" t="n">
+        <v>19512</v>
+      </c>
+      <c r="C33" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A2:C2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
auto: snapshot 2026-07-16 13:31:00
</commit_message>
<xml_diff>
--- a/clan_3815.xlsx
+++ b/clan_3815.xlsx
@@ -962,7 +962,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Timestamp: 2026-07-16 13:01:00</t>
+          <t>Timestamp: 2026-07-16 13:31:00</t>
         </is>
       </c>
     </row>
@@ -1005,11 +1005,11 @@
         </is>
       </c>
       <c r="B5" s="5" t="n">
-        <v>22920</v>
+        <v>22970</v>
       </c>
       <c r="C5" s="5" t="inlineStr">
         <is>
-          <t>+2078</t>
+          <t>+2128</t>
         </is>
       </c>
     </row>
@@ -1020,11 +1020,11 @@
         </is>
       </c>
       <c r="B6" s="5" t="n">
-        <v>22831</v>
+        <v>22881</v>
       </c>
       <c r="C6" s="5" t="inlineStr">
         <is>
-          <t>+2055</t>
+          <t>+2105</t>
         </is>
       </c>
     </row>
@@ -1035,11 +1035,11 @@
         </is>
       </c>
       <c r="B7" s="5" t="n">
-        <v>22674</v>
+        <v>22724</v>
       </c>
       <c r="C7" s="5" t="inlineStr">
         <is>
-          <t>+2073</t>
+          <t>+2123</t>
         </is>
       </c>
     </row>
@@ -1380,11 +1380,11 @@
         </is>
       </c>
       <c r="B30" s="5" t="n">
-        <v>7672</v>
+        <v>7722</v>
       </c>
       <c r="C30" s="5" t="inlineStr">
         <is>
-          <t>+1291</t>
+          <t>+1341</t>
         </is>
       </c>
     </row>
@@ -1395,11 +1395,11 @@
         </is>
       </c>
       <c r="B31" s="5" t="n">
-        <v>7572</v>
+        <v>7622</v>
       </c>
       <c r="C31" s="5" t="inlineStr">
         <is>
-          <t>+1241</t>
+          <t>+1291</t>
         </is>
       </c>
     </row>
@@ -1410,11 +1410,11 @@
         </is>
       </c>
       <c r="B32" s="5" t="n">
-        <v>7528</v>
+        <v>7578</v>
       </c>
       <c r="C32" s="5" t="inlineStr">
         <is>
-          <t>+1232</t>
+          <t>+1282</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: snapshot 2026-07-17 13:01:00
</commit_message>
<xml_diff>
--- a/clan_3815.xlsx
+++ b/clan_3815.xlsx
@@ -9,6 +9,7 @@
   <sheets>
     <sheet name="2026-07-15" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="2026-07-16" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="2026-07-17" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -1440,4 +1441,508 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C33"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="25" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Clan: Mans Best Friend (3815)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Timestamp: 2026-07-17 13:01:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>Total Reps</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>Daily Reps (+1d)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>Nobodys Son</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="n">
+        <v>21308</v>
+      </c>
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>-12700</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>Create Character III</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="n">
+        <v>24307</v>
+      </c>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>+1337</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>Create Character IV</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="n">
+        <v>24281</v>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>+1400</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>Create Character V</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="n">
+        <v>24106</v>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>+1382</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>Anti-Hero</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="n">
+        <v>23948</v>
+      </c>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>Vigilante Shit</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="n">
+        <v>18454</v>
+      </c>
+      <c r="C9" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>Sweet Nothing</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="n">
+        <v>18834</v>
+      </c>
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>The Great War</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="n">
+        <v>18204</v>
+      </c>
+      <c r="C11" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">We Almost Broke Up </t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="n">
+        <v>24371</v>
+      </c>
+      <c r="C12" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="4" t="inlineStr">
+        <is>
+          <t>When Did You Get Hot</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="n">
+        <v>18854</v>
+      </c>
+      <c r="C13" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="4" t="inlineStr">
+        <is>
+          <t>Dont Worry Ill Make</t>
+        </is>
+      </c>
+      <c r="B14" s="5" t="n">
+        <v>19078</v>
+      </c>
+      <c r="C14" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="4" t="inlineStr">
+        <is>
+          <t>Goodbye</t>
+        </is>
+      </c>
+      <c r="B15" s="5" t="n">
+        <v>16849</v>
+      </c>
+      <c r="C15" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="4" t="inlineStr">
+        <is>
+          <t>Mans Best Friend</t>
+        </is>
+      </c>
+      <c r="B16" s="5" t="n">
+        <v>16410</v>
+      </c>
+      <c r="C16" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="4" t="inlineStr">
+        <is>
+          <t>Lavender Haze</t>
+        </is>
+      </c>
+      <c r="B17" s="5" t="n">
+        <v>15683</v>
+      </c>
+      <c r="C17" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="4" t="inlineStr">
+        <is>
+          <t>Never Getting Laid</t>
+        </is>
+      </c>
+      <c r="B18" s="5" t="n">
+        <v>24593</v>
+      </c>
+      <c r="C18" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="4" t="inlineStr">
+        <is>
+          <t>My Man on Willpower</t>
+        </is>
+      </c>
+      <c r="B19" s="5" t="n">
+        <v>18584</v>
+      </c>
+      <c r="C19" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="4" t="inlineStr">
+        <is>
+          <t>Manchild</t>
+        </is>
+      </c>
+      <c r="B20" s="5" t="n">
+        <v>19619</v>
+      </c>
+      <c r="C20" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="4" t="inlineStr">
+        <is>
+          <t>Sugar Talking</t>
+        </is>
+      </c>
+      <c r="B21" s="5" t="n">
+        <v>18618</v>
+      </c>
+      <c r="C21" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="4" t="inlineStr">
+        <is>
+          <t>Midnight Rain</t>
+        </is>
+      </c>
+      <c r="B22" s="5" t="n">
+        <v>16228</v>
+      </c>
+      <c r="C22" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="4" t="inlineStr">
+        <is>
+          <t>Nobodys Son</t>
+        </is>
+      </c>
+      <c r="B23" s="5" t="n">
+        <v>34008</v>
+      </c>
+      <c r="C23" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="4" t="inlineStr">
+        <is>
+          <t>House Tour</t>
+        </is>
+      </c>
+      <c r="B24" s="5" t="n">
+        <v>19332</v>
+      </c>
+      <c r="C24" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="4" t="inlineStr">
+        <is>
+          <t>Hanabi  Î±Î·Ð²Ï…</t>
+        </is>
+      </c>
+      <c r="B25" s="5" t="n">
+        <v>3550</v>
+      </c>
+      <c r="C25" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="4" t="inlineStr">
+        <is>
+          <t>Dummy</t>
+        </is>
+      </c>
+      <c r="B26" s="5" t="n">
+        <v>3500</v>
+      </c>
+      <c r="C26" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="4" t="inlineStr">
+        <is>
+          <t>DarkFire</t>
+        </is>
+      </c>
+      <c r="B27" s="5" t="n">
+        <v>8471</v>
+      </c>
+      <c r="C27" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="4" t="inlineStr">
+        <is>
+          <t>DarkSunny</t>
+        </is>
+      </c>
+      <c r="B28" s="5" t="n">
+        <v>8524</v>
+      </c>
+      <c r="C28" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="4" t="inlineStr">
+        <is>
+          <t>Dairen Uchiha</t>
+        </is>
+      </c>
+      <c r="B29" s="5" t="n">
+        <v>8364</v>
+      </c>
+      <c r="C29" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="4" t="inlineStr">
+        <is>
+          <t>LILI ZENIN®</t>
+        </is>
+      </c>
+      <c r="B30" s="5" t="n">
+        <v>9045</v>
+      </c>
+      <c r="C30" s="5" t="inlineStr">
+        <is>
+          <t>+1323</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="4" t="inlineStr">
+        <is>
+          <t>linda ZENIN ®</t>
+        </is>
+      </c>
+      <c r="B31" s="5" t="n">
+        <v>8909</v>
+      </c>
+      <c r="C31" s="5" t="inlineStr">
+        <is>
+          <t>+1287</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="4" t="inlineStr">
+        <is>
+          <t>SHINRAIN ZENIN®</t>
+        </is>
+      </c>
+      <c r="B32" s="5" t="n">
+        <v>8892</v>
+      </c>
+      <c r="C32" s="5" t="inlineStr">
+        <is>
+          <t>+1314</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="4" t="inlineStr">
+        <is>
+          <t>Go Go Juice</t>
+        </is>
+      </c>
+      <c r="B33" s="5" t="n">
+        <v>19512</v>
+      </c>
+      <c r="C33" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A2:C2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
auto: snapshot 2026-07-17 13:31:00
</commit_message>
<xml_diff>
--- a/clan_3815.xlsx
+++ b/clan_3815.xlsx
@@ -1467,7 +1467,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Timestamp: 2026-07-17 13:01:00</t>
+          <t>Timestamp: 2026-07-17 13:31:00</t>
         </is>
       </c>
     </row>
@@ -1510,11 +1510,11 @@
         </is>
       </c>
       <c r="B5" s="5" t="n">
-        <v>24307</v>
+        <v>24357</v>
       </c>
       <c r="C5" s="5" t="inlineStr">
         <is>
-          <t>+1337</t>
+          <t>+1387</t>
         </is>
       </c>
     </row>
@@ -1525,11 +1525,11 @@
         </is>
       </c>
       <c r="B6" s="5" t="n">
-        <v>24281</v>
+        <v>24331</v>
       </c>
       <c r="C6" s="5" t="inlineStr">
         <is>
-          <t>+1400</t>
+          <t>+1450</t>
         </is>
       </c>
     </row>
@@ -1540,11 +1540,11 @@
         </is>
       </c>
       <c r="B7" s="5" t="n">
-        <v>24106</v>
+        <v>24156</v>
       </c>
       <c r="C7" s="5" t="inlineStr">
         <is>
-          <t>+1382</t>
+          <t>+1432</t>
         </is>
       </c>
     </row>
@@ -1885,11 +1885,11 @@
         </is>
       </c>
       <c r="B30" s="5" t="n">
-        <v>9045</v>
+        <v>9095</v>
       </c>
       <c r="C30" s="5" t="inlineStr">
         <is>
-          <t>+1323</t>
+          <t>+1373</t>
         </is>
       </c>
     </row>
@@ -1900,11 +1900,11 @@
         </is>
       </c>
       <c r="B31" s="5" t="n">
-        <v>8909</v>
+        <v>8959</v>
       </c>
       <c r="C31" s="5" t="inlineStr">
         <is>
-          <t>+1287</t>
+          <t>+1337</t>
         </is>
       </c>
     </row>
@@ -1915,11 +1915,11 @@
         </is>
       </c>
       <c r="B32" s="5" t="n">
-        <v>8892</v>
+        <v>8942</v>
       </c>
       <c r="C32" s="5" t="inlineStr">
         <is>
-          <t>+1314</t>
+          <t>+1364</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: snapshot 2026-07-18 13:01:00
</commit_message>
<xml_diff>
--- a/clan_3815.xlsx
+++ b/clan_3815.xlsx
@@ -10,6 +10,7 @@
     <sheet name="2026-07-15" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="2026-07-16" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="2026-07-17" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="2026-07-18" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -1945,4 +1946,508 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C33"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="25" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Clan: Mans Best Friend (3815)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Timestamp: 2026-07-18 13:01:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>Total Reps</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>Daily Reps (+1d)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>Nobodys Son</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="n">
+        <v>21458</v>
+      </c>
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>-12550</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>Create Character III</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="n">
+        <v>26057</v>
+      </c>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>+1700</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>Create Character IV</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="n">
+        <v>26022</v>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>+1691</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>Create Character V</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="n">
+        <v>25856</v>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>+1700</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>Anti-Hero</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="n">
+        <v>24098</v>
+      </c>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>+150</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>Vigilante Shit</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="n">
+        <v>18604</v>
+      </c>
+      <c r="C9" s="5" t="inlineStr">
+        <is>
+          <t>+150</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>Sweet Nothing</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="n">
+        <v>18984</v>
+      </c>
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>+150</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>The Great War</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="n">
+        <v>18354</v>
+      </c>
+      <c r="C11" s="5" t="inlineStr">
+        <is>
+          <t>+150</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">We Almost Broke Up </t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="n">
+        <v>24521</v>
+      </c>
+      <c r="C12" s="5" t="inlineStr">
+        <is>
+          <t>+150</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="4" t="inlineStr">
+        <is>
+          <t>When Did You Get Hot</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="n">
+        <v>19004</v>
+      </c>
+      <c r="C13" s="5" t="inlineStr">
+        <is>
+          <t>+150</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="4" t="inlineStr">
+        <is>
+          <t>Dont Worry Ill Make</t>
+        </is>
+      </c>
+      <c r="B14" s="5" t="n">
+        <v>19228</v>
+      </c>
+      <c r="C14" s="5" t="inlineStr">
+        <is>
+          <t>+150</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="4" t="inlineStr">
+        <is>
+          <t>Goodbye</t>
+        </is>
+      </c>
+      <c r="B15" s="5" t="n">
+        <v>16999</v>
+      </c>
+      <c r="C15" s="5" t="inlineStr">
+        <is>
+          <t>+150</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="4" t="inlineStr">
+        <is>
+          <t>Mans Best Friend</t>
+        </is>
+      </c>
+      <c r="B16" s="5" t="n">
+        <v>16560</v>
+      </c>
+      <c r="C16" s="5" t="inlineStr">
+        <is>
+          <t>+150</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="4" t="inlineStr">
+        <is>
+          <t>Lavender Haze</t>
+        </is>
+      </c>
+      <c r="B17" s="5" t="n">
+        <v>15833</v>
+      </c>
+      <c r="C17" s="5" t="inlineStr">
+        <is>
+          <t>+150</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="4" t="inlineStr">
+        <is>
+          <t>Never Getting Laid</t>
+        </is>
+      </c>
+      <c r="B18" s="5" t="n">
+        <v>24743</v>
+      </c>
+      <c r="C18" s="5" t="inlineStr">
+        <is>
+          <t>+150</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="4" t="inlineStr">
+        <is>
+          <t>My Man on Willpower</t>
+        </is>
+      </c>
+      <c r="B19" s="5" t="n">
+        <v>18684</v>
+      </c>
+      <c r="C19" s="5" t="inlineStr">
+        <is>
+          <t>+100</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="4" t="inlineStr">
+        <is>
+          <t>Manchild</t>
+        </is>
+      </c>
+      <c r="B20" s="5" t="n">
+        <v>19769</v>
+      </c>
+      <c r="C20" s="5" t="inlineStr">
+        <is>
+          <t>+150</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="4" t="inlineStr">
+        <is>
+          <t>Sugar Talking</t>
+        </is>
+      </c>
+      <c r="B21" s="5" t="n">
+        <v>18768</v>
+      </c>
+      <c r="C21" s="5" t="inlineStr">
+        <is>
+          <t>+150</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="4" t="inlineStr">
+        <is>
+          <t>Midnight Rain</t>
+        </is>
+      </c>
+      <c r="B22" s="5" t="n">
+        <v>16378</v>
+      </c>
+      <c r="C22" s="5" t="inlineStr">
+        <is>
+          <t>+150</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="4" t="inlineStr">
+        <is>
+          <t>Nobodys Son</t>
+        </is>
+      </c>
+      <c r="B23" s="5" t="n">
+        <v>34158</v>
+      </c>
+      <c r="C23" s="5" t="inlineStr">
+        <is>
+          <t>+150</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="4" t="inlineStr">
+        <is>
+          <t>House Tour</t>
+        </is>
+      </c>
+      <c r="B24" s="5" t="n">
+        <v>19482</v>
+      </c>
+      <c r="C24" s="5" t="inlineStr">
+        <is>
+          <t>+150</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="4" t="inlineStr">
+        <is>
+          <t>Hanabi  Î±Î·Ð²Ï…</t>
+        </is>
+      </c>
+      <c r="B25" s="5" t="n">
+        <v>3550</v>
+      </c>
+      <c r="C25" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="4" t="inlineStr">
+        <is>
+          <t>Dummy</t>
+        </is>
+      </c>
+      <c r="B26" s="5" t="n">
+        <v>3500</v>
+      </c>
+      <c r="C26" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="4" t="inlineStr">
+        <is>
+          <t>DarkFire</t>
+        </is>
+      </c>
+      <c r="B27" s="5" t="n">
+        <v>8471</v>
+      </c>
+      <c r="C27" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="4" t="inlineStr">
+        <is>
+          <t>DarkSunny</t>
+        </is>
+      </c>
+      <c r="B28" s="5" t="n">
+        <v>8524</v>
+      </c>
+      <c r="C28" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="4" t="inlineStr">
+        <is>
+          <t>Dairen Uchiha</t>
+        </is>
+      </c>
+      <c r="B29" s="5" t="n">
+        <v>8364</v>
+      </c>
+      <c r="C29" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="4" t="inlineStr">
+        <is>
+          <t>LILI ZENIN®</t>
+        </is>
+      </c>
+      <c r="B30" s="5" t="n">
+        <v>9650</v>
+      </c>
+      <c r="C30" s="5" t="inlineStr">
+        <is>
+          <t>+555</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="4" t="inlineStr">
+        <is>
+          <t>linda ZENIN ®</t>
+        </is>
+      </c>
+      <c r="B31" s="5" t="n">
+        <v>9328</v>
+      </c>
+      <c r="C31" s="5" t="inlineStr">
+        <is>
+          <t>+369</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="4" t="inlineStr">
+        <is>
+          <t>SHINRAIN ZENIN®</t>
+        </is>
+      </c>
+      <c r="B32" s="5" t="n">
+        <v>9392</v>
+      </c>
+      <c r="C32" s="5" t="inlineStr">
+        <is>
+          <t>+450</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="4" t="inlineStr">
+        <is>
+          <t>Go Go Juice</t>
+        </is>
+      </c>
+      <c r="B33" s="5" t="n">
+        <v>19662</v>
+      </c>
+      <c r="C33" s="5" t="inlineStr">
+        <is>
+          <t>+150</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A2:C2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
auto: snapshot 2026-07-18 13:31:00
</commit_message>
<xml_diff>
--- a/clan_3815.xlsx
+++ b/clan_3815.xlsx
@@ -1972,7 +1972,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Timestamp: 2026-07-18 13:01:00</t>
+          <t>Timestamp: 2026-07-18 13:31:00</t>
         </is>
       </c>
     </row>
@@ -2000,11 +2000,11 @@
         </is>
       </c>
       <c r="B4" s="5" t="n">
-        <v>21458</v>
+        <v>21558</v>
       </c>
       <c r="C4" s="5" t="inlineStr">
         <is>
-          <t>-12550</t>
+          <t>-12450</t>
         </is>
       </c>
     </row>
@@ -2120,11 +2120,11 @@
         </is>
       </c>
       <c r="B12" s="5" t="n">
-        <v>24521</v>
+        <v>24621</v>
       </c>
       <c r="C12" s="5" t="inlineStr">
         <is>
-          <t>+150</t>
+          <t>+250</t>
         </is>
       </c>
     </row>
@@ -2135,11 +2135,11 @@
         </is>
       </c>
       <c r="B13" s="5" t="n">
-        <v>19004</v>
+        <v>19104</v>
       </c>
       <c r="C13" s="5" t="inlineStr">
         <is>
-          <t>+150</t>
+          <t>+250</t>
         </is>
       </c>
     </row>
@@ -2150,11 +2150,11 @@
         </is>
       </c>
       <c r="B14" s="5" t="n">
-        <v>19228</v>
+        <v>19328</v>
       </c>
       <c r="C14" s="5" t="inlineStr">
         <is>
-          <t>+150</t>
+          <t>+250</t>
         </is>
       </c>
     </row>
@@ -2165,11 +2165,11 @@
         </is>
       </c>
       <c r="B15" s="5" t="n">
-        <v>16999</v>
+        <v>17099</v>
       </c>
       <c r="C15" s="5" t="inlineStr">
         <is>
-          <t>+150</t>
+          <t>+250</t>
         </is>
       </c>
     </row>
@@ -2180,11 +2180,11 @@
         </is>
       </c>
       <c r="B16" s="5" t="n">
-        <v>16560</v>
+        <v>16660</v>
       </c>
       <c r="C16" s="5" t="inlineStr">
         <is>
-          <t>+150</t>
+          <t>+250</t>
         </is>
       </c>
     </row>
@@ -2195,11 +2195,11 @@
         </is>
       </c>
       <c r="B17" s="5" t="n">
-        <v>15833</v>
+        <v>15933</v>
       </c>
       <c r="C17" s="5" t="inlineStr">
         <is>
-          <t>+150</t>
+          <t>+250</t>
         </is>
       </c>
     </row>
@@ -2210,11 +2210,11 @@
         </is>
       </c>
       <c r="B18" s="5" t="n">
-        <v>24743</v>
+        <v>24843</v>
       </c>
       <c r="C18" s="5" t="inlineStr">
         <is>
-          <t>+150</t>
+          <t>+250</t>
         </is>
       </c>
     </row>
@@ -2225,11 +2225,11 @@
         </is>
       </c>
       <c r="B19" s="5" t="n">
-        <v>18684</v>
+        <v>18784</v>
       </c>
       <c r="C19" s="5" t="inlineStr">
         <is>
-          <t>+100</t>
+          <t>+200</t>
         </is>
       </c>
     </row>
@@ -2240,11 +2240,11 @@
         </is>
       </c>
       <c r="B20" s="5" t="n">
-        <v>19769</v>
+        <v>19869</v>
       </c>
       <c r="C20" s="5" t="inlineStr">
         <is>
-          <t>+150</t>
+          <t>+250</t>
         </is>
       </c>
     </row>
@@ -2255,11 +2255,11 @@
         </is>
       </c>
       <c r="B21" s="5" t="n">
-        <v>18768</v>
+        <v>18868</v>
       </c>
       <c r="C21" s="5" t="inlineStr">
         <is>
-          <t>+150</t>
+          <t>+250</t>
         </is>
       </c>
     </row>
@@ -2270,11 +2270,11 @@
         </is>
       </c>
       <c r="B22" s="5" t="n">
-        <v>16378</v>
+        <v>16478</v>
       </c>
       <c r="C22" s="5" t="inlineStr">
         <is>
-          <t>+150</t>
+          <t>+250</t>
         </is>
       </c>
     </row>
@@ -2285,11 +2285,11 @@
         </is>
       </c>
       <c r="B23" s="5" t="n">
-        <v>34158</v>
+        <v>34258</v>
       </c>
       <c r="C23" s="5" t="inlineStr">
         <is>
-          <t>+150</t>
+          <t>+250</t>
         </is>
       </c>
     </row>
@@ -2300,11 +2300,11 @@
         </is>
       </c>
       <c r="B24" s="5" t="n">
-        <v>19482</v>
+        <v>19582</v>
       </c>
       <c r="C24" s="5" t="inlineStr">
         <is>
-          <t>+150</t>
+          <t>+250</t>
         </is>
       </c>
     </row>
@@ -2435,11 +2435,11 @@
         </is>
       </c>
       <c r="B33" s="5" t="n">
-        <v>19662</v>
+        <v>19762</v>
       </c>
       <c r="C33" s="5" t="inlineStr">
         <is>
-          <t>+150</t>
+          <t>+250</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: snapshot 2026-07-19 13:01:00
</commit_message>
<xml_diff>
--- a/clan_3815.xlsx
+++ b/clan_3815.xlsx
@@ -11,6 +11,7 @@
     <sheet name="2026-07-16" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="2026-07-17" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="2026-07-18" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="2026-07-19" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -2450,4 +2451,508 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C33"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="25" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Clan: Mans Best Friend (3815)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Timestamp: 2026-07-19 13:01:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>Total Reps</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>Daily Reps (+1d)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>Nobodys Son</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="n">
+        <v>23665</v>
+      </c>
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>-10593</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>Create Character III</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="n">
+        <v>26057</v>
+      </c>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>Create Character IV</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="n">
+        <v>26022</v>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>Create Character V</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="n">
+        <v>25856</v>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>Anti-Hero</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="n">
+        <v>37874</v>
+      </c>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>+13776</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>Vigilante Shit</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="n">
+        <v>23767</v>
+      </c>
+      <c r="C9" s="5" t="inlineStr">
+        <is>
+          <t>+5163</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>Sweet Nothing</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="n">
+        <v>19584</v>
+      </c>
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>+600</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>The Great War</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="n">
+        <v>18954</v>
+      </c>
+      <c r="C11" s="5" t="inlineStr">
+        <is>
+          <t>+600</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">We Almost Broke Up </t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="n">
+        <v>38821</v>
+      </c>
+      <c r="C12" s="5" t="inlineStr">
+        <is>
+          <t>+14200</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="4" t="inlineStr">
+        <is>
+          <t>When Did You Get Hot</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="n">
+        <v>24666</v>
+      </c>
+      <c r="C13" s="5" t="inlineStr">
+        <is>
+          <t>+5562</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="4" t="inlineStr">
+        <is>
+          <t>Dont Worry Ill Make</t>
+        </is>
+      </c>
+      <c r="B14" s="5" t="n">
+        <v>20333</v>
+      </c>
+      <c r="C14" s="5" t="inlineStr">
+        <is>
+          <t>+1005</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="4" t="inlineStr">
+        <is>
+          <t>Goodbye</t>
+        </is>
+      </c>
+      <c r="B15" s="5" t="n">
+        <v>19339</v>
+      </c>
+      <c r="C15" s="5" t="inlineStr">
+        <is>
+          <t>+2240</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="4" t="inlineStr">
+        <is>
+          <t>Mans Best Friend</t>
+        </is>
+      </c>
+      <c r="B16" s="5" t="n">
+        <v>18900</v>
+      </c>
+      <c r="C16" s="5" t="inlineStr">
+        <is>
+          <t>+2240</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="4" t="inlineStr">
+        <is>
+          <t>Lavender Haze</t>
+        </is>
+      </c>
+      <c r="B17" s="5" t="n">
+        <v>18092</v>
+      </c>
+      <c r="C17" s="5" t="inlineStr">
+        <is>
+          <t>+2159</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="4" t="inlineStr">
+        <is>
+          <t>Never Getting Laid</t>
+        </is>
+      </c>
+      <c r="B18" s="5" t="n">
+        <v>30086</v>
+      </c>
+      <c r="C18" s="5" t="inlineStr">
+        <is>
+          <t>+5243</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="4" t="inlineStr">
+        <is>
+          <t>My Man on Willpower</t>
+        </is>
+      </c>
+      <c r="B19" s="5" t="n">
+        <v>32772</v>
+      </c>
+      <c r="C19" s="5" t="inlineStr">
+        <is>
+          <t>+13988</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="4" t="inlineStr">
+        <is>
+          <t>Manchild</t>
+        </is>
+      </c>
+      <c r="B20" s="5" t="n">
+        <v>20774</v>
+      </c>
+      <c r="C20" s="5" t="inlineStr">
+        <is>
+          <t>+905</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="4" t="inlineStr">
+        <is>
+          <t>Sugar Talking</t>
+        </is>
+      </c>
+      <c r="B21" s="5" t="n">
+        <v>19948</v>
+      </c>
+      <c r="C21" s="5" t="inlineStr">
+        <is>
+          <t>+1080</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="4" t="inlineStr">
+        <is>
+          <t>Midnight Rain</t>
+        </is>
+      </c>
+      <c r="B22" s="5" t="n">
+        <v>18565</v>
+      </c>
+      <c r="C22" s="5" t="inlineStr">
+        <is>
+          <t>+2087</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="4" t="inlineStr">
+        <is>
+          <t>Nobodys Son</t>
+        </is>
+      </c>
+      <c r="B23" s="5" t="n">
+        <v>36383</v>
+      </c>
+      <c r="C23" s="5" t="inlineStr">
+        <is>
+          <t>+2125</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="4" t="inlineStr">
+        <is>
+          <t>House Tour</t>
+        </is>
+      </c>
+      <c r="B24" s="5" t="n">
+        <v>20606</v>
+      </c>
+      <c r="C24" s="5" t="inlineStr">
+        <is>
+          <t>+1024</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="4" t="inlineStr">
+        <is>
+          <t>Hanabi  Î±Î·Ð²Ï…</t>
+        </is>
+      </c>
+      <c r="B25" s="5" t="n">
+        <v>3550</v>
+      </c>
+      <c r="C25" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="4" t="inlineStr">
+        <is>
+          <t>Dummy</t>
+        </is>
+      </c>
+      <c r="B26" s="5" t="n">
+        <v>3500</v>
+      </c>
+      <c r="C26" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="4" t="inlineStr">
+        <is>
+          <t>DarkFire</t>
+        </is>
+      </c>
+      <c r="B27" s="5" t="n">
+        <v>8471</v>
+      </c>
+      <c r="C27" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="4" t="inlineStr">
+        <is>
+          <t>DarkSunny</t>
+        </is>
+      </c>
+      <c r="B28" s="5" t="n">
+        <v>8524</v>
+      </c>
+      <c r="C28" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="4" t="inlineStr">
+        <is>
+          <t>Dairen Uchiha</t>
+        </is>
+      </c>
+      <c r="B29" s="5" t="n">
+        <v>8364</v>
+      </c>
+      <c r="C29" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="4" t="inlineStr">
+        <is>
+          <t>LILI ZENIN®</t>
+        </is>
+      </c>
+      <c r="B30" s="5" t="n">
+        <v>9650</v>
+      </c>
+      <c r="C30" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="4" t="inlineStr">
+        <is>
+          <t>linda ZENIN ®</t>
+        </is>
+      </c>
+      <c r="B31" s="5" t="n">
+        <v>9328</v>
+      </c>
+      <c r="C31" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="4" t="inlineStr">
+        <is>
+          <t>SHINRAIN ZENIN®</t>
+        </is>
+      </c>
+      <c r="B32" s="5" t="n">
+        <v>9392</v>
+      </c>
+      <c r="C32" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="4" t="inlineStr">
+        <is>
+          <t>Go Go Juice</t>
+        </is>
+      </c>
+      <c r="B33" s="5" t="n">
+        <v>20762</v>
+      </c>
+      <c r="C33" s="5" t="inlineStr">
+        <is>
+          <t>+1000</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A2:C2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
auto: snapshot 2026-07-19 13:31:00
</commit_message>
<xml_diff>
--- a/clan_3815.xlsx
+++ b/clan_3815.xlsx
@@ -2477,7 +2477,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Timestamp: 2026-07-19 13:01:00</t>
+          <t>Timestamp: 2026-07-19 13:31:00</t>
         </is>
       </c>
     </row>
@@ -2505,11 +2505,11 @@
         </is>
       </c>
       <c r="B4" s="5" t="n">
-        <v>23665</v>
+        <v>0</v>
       </c>
       <c r="C4" s="5" t="inlineStr">
         <is>
-          <t>-10593</t>
+          <t>-34258</t>
         </is>
       </c>
     </row>
@@ -2520,11 +2520,11 @@
         </is>
       </c>
       <c r="B5" s="5" t="n">
-        <v>26057</v>
+        <v>0</v>
       </c>
       <c r="C5" s="5" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>-26057</t>
         </is>
       </c>
     </row>
@@ -2535,11 +2535,11 @@
         </is>
       </c>
       <c r="B6" s="5" t="n">
-        <v>26022</v>
+        <v>0</v>
       </c>
       <c r="C6" s="5" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>-26022</t>
         </is>
       </c>
     </row>
@@ -2550,11 +2550,11 @@
         </is>
       </c>
       <c r="B7" s="5" t="n">
-        <v>25856</v>
+        <v>0</v>
       </c>
       <c r="C7" s="5" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>-25856</t>
         </is>
       </c>
     </row>
@@ -2565,11 +2565,11 @@
         </is>
       </c>
       <c r="B8" s="5" t="n">
-        <v>37874</v>
+        <v>0</v>
       </c>
       <c r="C8" s="5" t="inlineStr">
         <is>
-          <t>+13776</t>
+          <t>-24098</t>
         </is>
       </c>
     </row>
@@ -2580,11 +2580,11 @@
         </is>
       </c>
       <c r="B9" s="5" t="n">
-        <v>23767</v>
+        <v>0</v>
       </c>
       <c r="C9" s="5" t="inlineStr">
         <is>
-          <t>+5163</t>
+          <t>-18604</t>
         </is>
       </c>
     </row>
@@ -2595,11 +2595,11 @@
         </is>
       </c>
       <c r="B10" s="5" t="n">
-        <v>19584</v>
+        <v>0</v>
       </c>
       <c r="C10" s="5" t="inlineStr">
         <is>
-          <t>+600</t>
+          <t>-18984</t>
         </is>
       </c>
     </row>
@@ -2610,11 +2610,11 @@
         </is>
       </c>
       <c r="B11" s="5" t="n">
-        <v>18954</v>
+        <v>0</v>
       </c>
       <c r="C11" s="5" t="inlineStr">
         <is>
-          <t>+600</t>
+          <t>-18354</t>
         </is>
       </c>
     </row>
@@ -2625,11 +2625,11 @@
         </is>
       </c>
       <c r="B12" s="5" t="n">
-        <v>38821</v>
+        <v>0</v>
       </c>
       <c r="C12" s="5" t="inlineStr">
         <is>
-          <t>+14200</t>
+          <t>-24621</t>
         </is>
       </c>
     </row>
@@ -2640,11 +2640,11 @@
         </is>
       </c>
       <c r="B13" s="5" t="n">
-        <v>24666</v>
+        <v>0</v>
       </c>
       <c r="C13" s="5" t="inlineStr">
         <is>
-          <t>+5562</t>
+          <t>-19104</t>
         </is>
       </c>
     </row>
@@ -2655,11 +2655,11 @@
         </is>
       </c>
       <c r="B14" s="5" t="n">
-        <v>20333</v>
+        <v>0</v>
       </c>
       <c r="C14" s="5" t="inlineStr">
         <is>
-          <t>+1005</t>
+          <t>-19328</t>
         </is>
       </c>
     </row>
@@ -2670,11 +2670,11 @@
         </is>
       </c>
       <c r="B15" s="5" t="n">
-        <v>19339</v>
+        <v>0</v>
       </c>
       <c r="C15" s="5" t="inlineStr">
         <is>
-          <t>+2240</t>
+          <t>-17099</t>
         </is>
       </c>
     </row>
@@ -2685,11 +2685,11 @@
         </is>
       </c>
       <c r="B16" s="5" t="n">
-        <v>18900</v>
+        <v>0</v>
       </c>
       <c r="C16" s="5" t="inlineStr">
         <is>
-          <t>+2240</t>
+          <t>-16660</t>
         </is>
       </c>
     </row>
@@ -2700,11 +2700,11 @@
         </is>
       </c>
       <c r="B17" s="5" t="n">
-        <v>18092</v>
+        <v>0</v>
       </c>
       <c r="C17" s="5" t="inlineStr">
         <is>
-          <t>+2159</t>
+          <t>-15933</t>
         </is>
       </c>
     </row>
@@ -2715,11 +2715,11 @@
         </is>
       </c>
       <c r="B18" s="5" t="n">
-        <v>30086</v>
+        <v>0</v>
       </c>
       <c r="C18" s="5" t="inlineStr">
         <is>
-          <t>+5243</t>
+          <t>-24843</t>
         </is>
       </c>
     </row>
@@ -2730,11 +2730,11 @@
         </is>
       </c>
       <c r="B19" s="5" t="n">
-        <v>32772</v>
+        <v>0</v>
       </c>
       <c r="C19" s="5" t="inlineStr">
         <is>
-          <t>+13988</t>
+          <t>-18784</t>
         </is>
       </c>
     </row>
@@ -2745,11 +2745,11 @@
         </is>
       </c>
       <c r="B20" s="5" t="n">
-        <v>20774</v>
+        <v>0</v>
       </c>
       <c r="C20" s="5" t="inlineStr">
         <is>
-          <t>+905</t>
+          <t>-19869</t>
         </is>
       </c>
     </row>
@@ -2760,11 +2760,11 @@
         </is>
       </c>
       <c r="B21" s="5" t="n">
-        <v>19948</v>
+        <v>0</v>
       </c>
       <c r="C21" s="5" t="inlineStr">
         <is>
-          <t>+1080</t>
+          <t>-18868</t>
         </is>
       </c>
     </row>
@@ -2775,11 +2775,11 @@
         </is>
       </c>
       <c r="B22" s="5" t="n">
-        <v>18565</v>
+        <v>0</v>
       </c>
       <c r="C22" s="5" t="inlineStr">
         <is>
-          <t>+2087</t>
+          <t>-16478</t>
         </is>
       </c>
     </row>
@@ -2790,11 +2790,11 @@
         </is>
       </c>
       <c r="B23" s="5" t="n">
-        <v>36383</v>
+        <v>0</v>
       </c>
       <c r="C23" s="5" t="inlineStr">
         <is>
-          <t>+2125</t>
+          <t>-34258</t>
         </is>
       </c>
     </row>
@@ -2805,11 +2805,11 @@
         </is>
       </c>
       <c r="B24" s="5" t="n">
-        <v>20606</v>
+        <v>0</v>
       </c>
       <c r="C24" s="5" t="inlineStr">
         <is>
-          <t>+1024</t>
+          <t>-19582</t>
         </is>
       </c>
     </row>
@@ -2820,11 +2820,11 @@
         </is>
       </c>
       <c r="B25" s="5" t="n">
-        <v>3550</v>
+        <v>0</v>
       </c>
       <c r="C25" s="5" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>-3550</t>
         </is>
       </c>
     </row>
@@ -2835,11 +2835,11 @@
         </is>
       </c>
       <c r="B26" s="5" t="n">
-        <v>3500</v>
+        <v>0</v>
       </c>
       <c r="C26" s="5" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>-3500</t>
         </is>
       </c>
     </row>
@@ -2850,11 +2850,11 @@
         </is>
       </c>
       <c r="B27" s="5" t="n">
-        <v>8471</v>
+        <v>0</v>
       </c>
       <c r="C27" s="5" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>-8471</t>
         </is>
       </c>
     </row>
@@ -2865,11 +2865,11 @@
         </is>
       </c>
       <c r="B28" s="5" t="n">
-        <v>8524</v>
+        <v>0</v>
       </c>
       <c r="C28" s="5" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>-8524</t>
         </is>
       </c>
     </row>
@@ -2880,11 +2880,11 @@
         </is>
       </c>
       <c r="B29" s="5" t="n">
-        <v>8364</v>
+        <v>0</v>
       </c>
       <c r="C29" s="5" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>-8364</t>
         </is>
       </c>
     </row>
@@ -2895,11 +2895,11 @@
         </is>
       </c>
       <c r="B30" s="5" t="n">
-        <v>9650</v>
+        <v>0</v>
       </c>
       <c r="C30" s="5" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>-9650</t>
         </is>
       </c>
     </row>
@@ -2910,11 +2910,11 @@
         </is>
       </c>
       <c r="B31" s="5" t="n">
-        <v>9328</v>
+        <v>0</v>
       </c>
       <c r="C31" s="5" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>-9328</t>
         </is>
       </c>
     </row>
@@ -2925,11 +2925,11 @@
         </is>
       </c>
       <c r="B32" s="5" t="n">
-        <v>9392</v>
+        <v>0</v>
       </c>
       <c r="C32" s="5" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>-9392</t>
         </is>
       </c>
     </row>
@@ -2940,11 +2940,11 @@
         </is>
       </c>
       <c r="B33" s="5" t="n">
-        <v>20762</v>
+        <v>0</v>
       </c>
       <c r="C33" s="5" t="inlineStr">
         <is>
-          <t>+1000</t>
+          <t>-19762</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: snapshot 2026-07-20 13:01:00
</commit_message>
<xml_diff>
--- a/clan_3815.xlsx
+++ b/clan_3815.xlsx
@@ -12,6 +12,7 @@
     <sheet name="2026-07-17" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="2026-07-18" sheetId="4" state="visible" r:id="rId4"/>
     <sheet name="2026-07-19" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="2026-07-20" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -2955,4 +2956,688 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C45"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="29" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Clan: Mans Best Friend (3815)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Timestamp: 2026-07-20 13:01:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>Total Reps</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>Daily Reps (+1d)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>Nobodys Son</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="n">
+        <v>1428</v>
+      </c>
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>+1428</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>Create Character III</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="n">
+        <v>1422</v>
+      </c>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>+1422</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>Create Character IV</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="n">
+        <v>2288</v>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>+2288</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>Create Character V</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="n">
+        <v>2198</v>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>+2198</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>Tears</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="n">
+        <v>300</v>
+      </c>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>Sugar Talking</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="n">
+        <v>258</v>
+      </c>
+      <c r="C9" s="5" t="inlineStr">
+        <is>
+          <t>+258</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="n">
+        <v>300</v>
+      </c>
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>Anti-Hero</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="n">
+        <v>1100</v>
+      </c>
+      <c r="C11" s="5" t="inlineStr">
+        <is>
+          <t>+1100</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t>Vigilante Shit</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="n">
+        <v>1100</v>
+      </c>
+      <c r="C12" s="5" t="inlineStr">
+        <is>
+          <t>+1100</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="4" t="inlineStr">
+        <is>
+          <t>Sweet Nothing</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="n">
+        <v>1064</v>
+      </c>
+      <c r="C13" s="5" t="inlineStr">
+        <is>
+          <t>+1064</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="4" t="inlineStr">
+        <is>
+          <t>The Great War</t>
+        </is>
+      </c>
+      <c r="B14" s="5" t="n">
+        <v>860</v>
+      </c>
+      <c r="C14" s="5" t="inlineStr">
+        <is>
+          <t>+860</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">We Almost Broke Up </t>
+        </is>
+      </c>
+      <c r="B15" s="5" t="n">
+        <v>1631</v>
+      </c>
+      <c r="C15" s="5" t="inlineStr">
+        <is>
+          <t>+1631</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="4" t="inlineStr">
+        <is>
+          <t>When Did You Get Hot</t>
+        </is>
+      </c>
+      <c r="B16" s="5" t="n">
+        <v>1480</v>
+      </c>
+      <c r="C16" s="5" t="inlineStr">
+        <is>
+          <t>+1480</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="4" t="inlineStr">
+        <is>
+          <t>Dont Worry Ill Make</t>
+        </is>
+      </c>
+      <c r="B17" s="5" t="n">
+        <v>1330</v>
+      </c>
+      <c r="C17" s="5" t="inlineStr">
+        <is>
+          <t>+1330</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="4" t="inlineStr">
+        <is>
+          <t>Goodbye</t>
+        </is>
+      </c>
+      <c r="B18" s="5" t="n">
+        <v>1420</v>
+      </c>
+      <c r="C18" s="5" t="inlineStr">
+        <is>
+          <t>+1420</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="4" t="inlineStr">
+        <is>
+          <t>Mans Best Friend</t>
+        </is>
+      </c>
+      <c r="B19" s="5" t="n">
+        <v>1350</v>
+      </c>
+      <c r="C19" s="5" t="inlineStr">
+        <is>
+          <t>+1350</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="4" t="inlineStr">
+        <is>
+          <t>Lavender Haze</t>
+        </is>
+      </c>
+      <c r="B20" s="5" t="n">
+        <v>1322</v>
+      </c>
+      <c r="C20" s="5" t="inlineStr">
+        <is>
+          <t>+1322</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="4" t="inlineStr">
+        <is>
+          <t>Never Getting Laid</t>
+        </is>
+      </c>
+      <c r="B21" s="5" t="n">
+        <v>1635</v>
+      </c>
+      <c r="C21" s="5" t="inlineStr">
+        <is>
+          <t>+1635</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="4" t="inlineStr">
+        <is>
+          <t>My Man on Willpower</t>
+        </is>
+      </c>
+      <c r="B22" s="5" t="n">
+        <v>1321</v>
+      </c>
+      <c r="C22" s="5" t="inlineStr">
+        <is>
+          <t>+1321</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="4" t="inlineStr">
+        <is>
+          <t>Manchild</t>
+        </is>
+      </c>
+      <c r="B23" s="5" t="n">
+        <v>1701</v>
+      </c>
+      <c r="C23" s="5" t="inlineStr">
+        <is>
+          <t>+1701</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="4" t="inlineStr">
+        <is>
+          <t>Sugar Talking</t>
+        </is>
+      </c>
+      <c r="B24" s="5" t="n">
+        <v>1148</v>
+      </c>
+      <c r="C24" s="5" t="inlineStr">
+        <is>
+          <t>+1148</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="4" t="inlineStr">
+        <is>
+          <t>My Man on Willpower</t>
+        </is>
+      </c>
+      <c r="B25" s="5" t="n">
+        <v>229</v>
+      </c>
+      <c r="C25" s="5" t="inlineStr">
+        <is>
+          <t>+229</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="4" t="inlineStr">
+        <is>
+          <t>Midnight Rain</t>
+        </is>
+      </c>
+      <c r="B26" s="5" t="n">
+        <v>1164</v>
+      </c>
+      <c r="C26" s="5" t="inlineStr">
+        <is>
+          <t>+1164</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="4" t="inlineStr">
+        <is>
+          <t>Nobodys Son</t>
+        </is>
+      </c>
+      <c r="B27" s="5" t="n">
+        <v>1920</v>
+      </c>
+      <c r="C27" s="5" t="inlineStr">
+        <is>
+          <t>+1920</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="4" t="inlineStr">
+        <is>
+          <t>House Tour</t>
+        </is>
+      </c>
+      <c r="B28" s="5" t="n">
+        <v>1090</v>
+      </c>
+      <c r="C28" s="5" t="inlineStr">
+        <is>
+          <t>+1090</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="4" t="inlineStr">
+        <is>
+          <t>Hanabi  Î±Î·Ð²Ï…</t>
+        </is>
+      </c>
+      <c r="B29" s="5" t="n">
+        <v>2250</v>
+      </c>
+      <c r="C29" s="5" t="inlineStr">
+        <is>
+          <t>+2250</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="4" t="inlineStr">
+        <is>
+          <t>Dummy</t>
+        </is>
+      </c>
+      <c r="B30" s="5" t="n">
+        <v>2003</v>
+      </c>
+      <c r="C30" s="5" t="inlineStr">
+        <is>
+          <t>+2003</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="4" t="inlineStr">
+        <is>
+          <t>Besos Mojados</t>
+        </is>
+      </c>
+      <c r="B31" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C31" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="4" t="inlineStr">
+        <is>
+          <t>DarkFire</t>
+        </is>
+      </c>
+      <c r="B32" s="5" t="n">
+        <v>2203</v>
+      </c>
+      <c r="C32" s="5" t="inlineStr">
+        <is>
+          <t>+2203</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="4" t="inlineStr">
+        <is>
+          <t>DarkSunny</t>
+        </is>
+      </c>
+      <c r="B33" s="5" t="n">
+        <v>2327</v>
+      </c>
+      <c r="C33" s="5" t="inlineStr">
+        <is>
+          <t>+2327</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="4" t="inlineStr">
+        <is>
+          <t>Dairen Uchiha</t>
+        </is>
+      </c>
+      <c r="B34" s="5" t="n">
+        <v>2863</v>
+      </c>
+      <c r="C34" s="5" t="inlineStr">
+        <is>
+          <t>+2863</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="4" t="inlineStr">
+        <is>
+          <t>LILI ZENIN®</t>
+        </is>
+      </c>
+      <c r="B35" s="5" t="n">
+        <v>1729</v>
+      </c>
+      <c r="C35" s="5" t="inlineStr">
+        <is>
+          <t>+1729</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="4" t="inlineStr">
+        <is>
+          <t>linda ZENIN ®</t>
+        </is>
+      </c>
+      <c r="B36" s="5" t="n">
+        <v>2120</v>
+      </c>
+      <c r="C36" s="5" t="inlineStr">
+        <is>
+          <t>+2120</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="4" t="inlineStr">
+        <is>
+          <t>SHINRAIN ZENIN®</t>
+        </is>
+      </c>
+      <c r="B37" s="5" t="n">
+        <v>1948</v>
+      </c>
+      <c r="C37" s="5" t="inlineStr">
+        <is>
+          <t>+1948</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="4" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B38" s="5" t="n">
+        <v>1761</v>
+      </c>
+      <c r="C38" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="4" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B39" s="5" t="n">
+        <v>1940</v>
+      </c>
+      <c r="C39" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="4" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="B40" s="5" t="n">
+        <v>1812</v>
+      </c>
+      <c r="C40" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="4" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="B41" s="5" t="n">
+        <v>1905</v>
+      </c>
+      <c r="C41" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="4" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="B42" s="5" t="n">
+        <v>1845</v>
+      </c>
+      <c r="C42" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="4" t="inlineStr">
+        <is>
+          <t>Go Go Juice</t>
+        </is>
+      </c>
+      <c r="B43" s="5" t="n">
+        <v>1520</v>
+      </c>
+      <c r="C43" s="5" t="inlineStr">
+        <is>
+          <t>+1520</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="4" t="inlineStr">
+        <is>
+          <t>Jhayco - Imaginaste</t>
+        </is>
+      </c>
+      <c r="B44" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C44" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="4" t="inlineStr">
+        <is>
+          <t>PuNch</t>
+        </is>
+      </c>
+      <c r="B45" s="5" t="n">
+        <v>350</v>
+      </c>
+      <c r="C45" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A2:C2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
auto: snapshot 2026-07-20 13:31:00
</commit_message>
<xml_diff>
--- a/clan_3815.xlsx
+++ b/clan_3815.xlsx
@@ -2982,7 +2982,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Timestamp: 2026-07-20 13:01:00</t>
+          <t>Timestamp: 2026-07-20 13:31:00</t>
         </is>
       </c>
     </row>
@@ -3010,11 +3010,11 @@
         </is>
       </c>
       <c r="B4" s="5" t="n">
-        <v>1428</v>
+        <v>1443</v>
       </c>
       <c r="C4" s="5" t="inlineStr">
         <is>
-          <t>+1428</t>
+          <t>+1443</t>
         </is>
       </c>
     </row>
@@ -3025,11 +3025,11 @@
         </is>
       </c>
       <c r="B5" s="5" t="n">
-        <v>1422</v>
+        <v>1447</v>
       </c>
       <c r="C5" s="5" t="inlineStr">
         <is>
-          <t>+1422</t>
+          <t>+1447</t>
         </is>
       </c>
     </row>
@@ -3040,11 +3040,11 @@
         </is>
       </c>
       <c r="B6" s="5" t="n">
-        <v>2288</v>
+        <v>2303</v>
       </c>
       <c r="C6" s="5" t="inlineStr">
         <is>
-          <t>+2288</t>
+          <t>+2303</t>
         </is>
       </c>
     </row>
@@ -3055,11 +3055,11 @@
         </is>
       </c>
       <c r="B7" s="5" t="n">
-        <v>2198</v>
+        <v>2213</v>
       </c>
       <c r="C7" s="5" t="inlineStr">
         <is>
-          <t>+2198</t>
+          <t>+2213</t>
         </is>
       </c>
     </row>
@@ -3070,7 +3070,7 @@
         </is>
       </c>
       <c r="B8" s="5" t="n">
-        <v>300</v>
+        <v>317</v>
       </c>
       <c r="C8" s="5" t="inlineStr">
         <is>
@@ -3085,11 +3085,11 @@
         </is>
       </c>
       <c r="B9" s="5" t="n">
-        <v>258</v>
+        <v>283</v>
       </c>
       <c r="C9" s="5" t="inlineStr">
         <is>
-          <t>+258</t>
+          <t>+283</t>
         </is>
       </c>
     </row>
@@ -3160,11 +3160,11 @@
         </is>
       </c>
       <c r="B14" s="5" t="n">
-        <v>860</v>
+        <v>890</v>
       </c>
       <c r="C14" s="5" t="inlineStr">
         <is>
-          <t>+860</t>
+          <t>+890</t>
         </is>
       </c>
     </row>
@@ -3175,11 +3175,11 @@
         </is>
       </c>
       <c r="B15" s="5" t="n">
-        <v>1631</v>
+        <v>1646</v>
       </c>
       <c r="C15" s="5" t="inlineStr">
         <is>
-          <t>+1631</t>
+          <t>+1646</t>
         </is>
       </c>
     </row>
@@ -3190,11 +3190,11 @@
         </is>
       </c>
       <c r="B16" s="5" t="n">
-        <v>1480</v>
+        <v>1530</v>
       </c>
       <c r="C16" s="5" t="inlineStr">
         <is>
-          <t>+1480</t>
+          <t>+1530</t>
         </is>
       </c>
     </row>
@@ -3205,11 +3205,11 @@
         </is>
       </c>
       <c r="B17" s="5" t="n">
-        <v>1330</v>
+        <v>1380</v>
       </c>
       <c r="C17" s="5" t="inlineStr">
         <is>
-          <t>+1330</t>
+          <t>+1380</t>
         </is>
       </c>
     </row>
@@ -3220,11 +3220,11 @@
         </is>
       </c>
       <c r="B18" s="5" t="n">
-        <v>1420</v>
+        <v>1435</v>
       </c>
       <c r="C18" s="5" t="inlineStr">
         <is>
-          <t>+1420</t>
+          <t>+1435</t>
         </is>
       </c>
     </row>
@@ -3235,11 +3235,11 @@
         </is>
       </c>
       <c r="B19" s="5" t="n">
-        <v>1350</v>
+        <v>1365</v>
       </c>
       <c r="C19" s="5" t="inlineStr">
         <is>
-          <t>+1350</t>
+          <t>+1365</t>
         </is>
       </c>
     </row>
@@ -3250,11 +3250,11 @@
         </is>
       </c>
       <c r="B20" s="5" t="n">
-        <v>1322</v>
+        <v>1337</v>
       </c>
       <c r="C20" s="5" t="inlineStr">
         <is>
-          <t>+1322</t>
+          <t>+1337</t>
         </is>
       </c>
     </row>
@@ -3265,11 +3265,11 @@
         </is>
       </c>
       <c r="B21" s="5" t="n">
-        <v>1635</v>
+        <v>1660</v>
       </c>
       <c r="C21" s="5" t="inlineStr">
         <is>
-          <t>+1635</t>
+          <t>+1660</t>
         </is>
       </c>
     </row>
@@ -3280,11 +3280,11 @@
         </is>
       </c>
       <c r="B22" s="5" t="n">
-        <v>1321</v>
+        <v>1340</v>
       </c>
       <c r="C22" s="5" t="inlineStr">
         <is>
-          <t>+1321</t>
+          <t>+1340</t>
         </is>
       </c>
     </row>
@@ -3295,11 +3295,11 @@
         </is>
       </c>
       <c r="B23" s="5" t="n">
-        <v>1701</v>
+        <v>1716</v>
       </c>
       <c r="C23" s="5" t="inlineStr">
         <is>
-          <t>+1701</t>
+          <t>+1716</t>
         </is>
       </c>
     </row>
@@ -3310,11 +3310,11 @@
         </is>
       </c>
       <c r="B24" s="5" t="n">
-        <v>1148</v>
+        <v>1198</v>
       </c>
       <c r="C24" s="5" t="inlineStr">
         <is>
-          <t>+1148</t>
+          <t>+1198</t>
         </is>
       </c>
     </row>
@@ -3325,11 +3325,11 @@
         </is>
       </c>
       <c r="B25" s="5" t="n">
-        <v>229</v>
+        <v>254</v>
       </c>
       <c r="C25" s="5" t="inlineStr">
         <is>
-          <t>+229</t>
+          <t>+254</t>
         </is>
       </c>
     </row>
@@ -3340,11 +3340,11 @@
         </is>
       </c>
       <c r="B26" s="5" t="n">
-        <v>1164</v>
+        <v>1169</v>
       </c>
       <c r="C26" s="5" t="inlineStr">
         <is>
-          <t>+1164</t>
+          <t>+1169</t>
         </is>
       </c>
     </row>
@@ -3355,11 +3355,11 @@
         </is>
       </c>
       <c r="B27" s="5" t="n">
-        <v>1920</v>
+        <v>1945</v>
       </c>
       <c r="C27" s="5" t="inlineStr">
         <is>
-          <t>+1920</t>
+          <t>+1945</t>
         </is>
       </c>
     </row>
@@ -3370,11 +3370,11 @@
         </is>
       </c>
       <c r="B28" s="5" t="n">
-        <v>1090</v>
+        <v>1115</v>
       </c>
       <c r="C28" s="5" t="inlineStr">
         <is>
-          <t>+1090</t>
+          <t>+1115</t>
         </is>
       </c>
     </row>
@@ -3385,11 +3385,11 @@
         </is>
       </c>
       <c r="B29" s="5" t="n">
-        <v>2250</v>
+        <v>2271</v>
       </c>
       <c r="C29" s="5" t="inlineStr">
         <is>
-          <t>+2250</t>
+          <t>+2271</t>
         </is>
       </c>
     </row>
@@ -3400,11 +3400,11 @@
         </is>
       </c>
       <c r="B30" s="5" t="n">
-        <v>2003</v>
+        <v>2045</v>
       </c>
       <c r="C30" s="5" t="inlineStr">
         <is>
-          <t>+2003</t>
+          <t>+2045</t>
         </is>
       </c>
     </row>
@@ -3430,11 +3430,11 @@
         </is>
       </c>
       <c r="B32" s="5" t="n">
-        <v>2203</v>
+        <v>2228</v>
       </c>
       <c r="C32" s="5" t="inlineStr">
         <is>
-          <t>+2203</t>
+          <t>+2228</t>
         </is>
       </c>
     </row>
@@ -3445,11 +3445,11 @@
         </is>
       </c>
       <c r="B33" s="5" t="n">
-        <v>2327</v>
+        <v>2346</v>
       </c>
       <c r="C33" s="5" t="inlineStr">
         <is>
-          <t>+2327</t>
+          <t>+2346</t>
         </is>
       </c>
     </row>
@@ -3460,11 +3460,11 @@
         </is>
       </c>
       <c r="B34" s="5" t="n">
-        <v>2863</v>
+        <v>2878</v>
       </c>
       <c r="C34" s="5" t="inlineStr">
         <is>
-          <t>+2863</t>
+          <t>+2878</t>
         </is>
       </c>
     </row>
@@ -3475,11 +3475,11 @@
         </is>
       </c>
       <c r="B35" s="5" t="n">
-        <v>1729</v>
+        <v>1754</v>
       </c>
       <c r="C35" s="5" t="inlineStr">
         <is>
-          <t>+1729</t>
+          <t>+1754</t>
         </is>
       </c>
     </row>
@@ -3490,11 +3490,11 @@
         </is>
       </c>
       <c r="B36" s="5" t="n">
-        <v>2120</v>
+        <v>2145</v>
       </c>
       <c r="C36" s="5" t="inlineStr">
         <is>
-          <t>+2120</t>
+          <t>+2145</t>
         </is>
       </c>
     </row>
@@ -3505,11 +3505,11 @@
         </is>
       </c>
       <c r="B37" s="5" t="n">
-        <v>1948</v>
+        <v>1973</v>
       </c>
       <c r="C37" s="5" t="inlineStr">
         <is>
-          <t>+1948</t>
+          <t>+1973</t>
         </is>
       </c>
     </row>
@@ -3580,7 +3580,7 @@
         </is>
       </c>
       <c r="B42" s="5" t="n">
-        <v>1845</v>
+        <v>1895</v>
       </c>
       <c r="C42" s="5" t="inlineStr">
         <is>
@@ -3595,11 +3595,11 @@
         </is>
       </c>
       <c r="B43" s="5" t="n">
-        <v>1520</v>
+        <v>1535</v>
       </c>
       <c r="C43" s="5" t="inlineStr">
         <is>
-          <t>+1520</t>
+          <t>+1535</t>
         </is>
       </c>
     </row>
@@ -3625,7 +3625,7 @@
         </is>
       </c>
       <c r="B45" s="5" t="n">
-        <v>350</v>
+        <v>369</v>
       </c>
       <c r="C45" s="5" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
auto: snapshot 2026-07-21 13:01:00
</commit_message>
<xml_diff>
--- a/clan_3815.xlsx
+++ b/clan_3815.xlsx
@@ -13,6 +13,7 @@
     <sheet name="2026-07-18" sheetId="4" state="visible" r:id="rId4"/>
     <sheet name="2026-07-19" sheetId="5" state="visible" r:id="rId5"/>
     <sheet name="2026-07-20" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="2026-07-21" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -3640,4 +3641,688 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C45"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="29" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Clan: Mans Best Friend (3815)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Timestamp: 2026-07-21 13:01:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>Total Reps</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>Daily Reps (+1d)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>Nobodys Son</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="n">
+        <v>1948</v>
+      </c>
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>+3</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>Create Character III</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="n">
+        <v>1765</v>
+      </c>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>+318</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>Create Character IV</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="n">
+        <v>2593</v>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>+290</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>Create Character V</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="n">
+        <v>2493</v>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>+280</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>Tears</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="n">
+        <v>744</v>
+      </c>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>+427</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>Sugar Talking</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="n">
+        <v>796</v>
+      </c>
+      <c r="C9" s="5" t="inlineStr">
+        <is>
+          <t>-402</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="n">
+        <v>695</v>
+      </c>
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>-1066</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>Anti-Hero</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="n">
+        <v>1484</v>
+      </c>
+      <c r="C11" s="5" t="inlineStr">
+        <is>
+          <t>+384</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t>Vigilante Shit</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="n">
+        <v>1454</v>
+      </c>
+      <c r="C12" s="5" t="inlineStr">
+        <is>
+          <t>+354</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="4" t="inlineStr">
+        <is>
+          <t>Sweet Nothing</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="n">
+        <v>1410</v>
+      </c>
+      <c r="C13" s="5" t="inlineStr">
+        <is>
+          <t>+346</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="4" t="inlineStr">
+        <is>
+          <t>The Great War</t>
+        </is>
+      </c>
+      <c r="B14" s="5" t="n">
+        <v>1218</v>
+      </c>
+      <c r="C14" s="5" t="inlineStr">
+        <is>
+          <t>+328</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">We Almost Broke Up </t>
+        </is>
+      </c>
+      <c r="B15" s="5" t="n">
+        <v>2185</v>
+      </c>
+      <c r="C15" s="5" t="inlineStr">
+        <is>
+          <t>+539</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="4" t="inlineStr">
+        <is>
+          <t>When Did You Get Hot</t>
+        </is>
+      </c>
+      <c r="B16" s="5" t="n">
+        <v>1998</v>
+      </c>
+      <c r="C16" s="5" t="inlineStr">
+        <is>
+          <t>+468</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="4" t="inlineStr">
+        <is>
+          <t>Dont Worry Ill Make</t>
+        </is>
+      </c>
+      <c r="B17" s="5" t="n">
+        <v>1837</v>
+      </c>
+      <c r="C17" s="5" t="inlineStr">
+        <is>
+          <t>+457</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="4" t="inlineStr">
+        <is>
+          <t>Goodbye</t>
+        </is>
+      </c>
+      <c r="B18" s="5" t="n">
+        <v>1940</v>
+      </c>
+      <c r="C18" s="5" t="inlineStr">
+        <is>
+          <t>+505</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="4" t="inlineStr">
+        <is>
+          <t>Mans Best Friend</t>
+        </is>
+      </c>
+      <c r="B19" s="5" t="n">
+        <v>1819</v>
+      </c>
+      <c r="C19" s="5" t="inlineStr">
+        <is>
+          <t>+454</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="4" t="inlineStr">
+        <is>
+          <t>Lavender Haze</t>
+        </is>
+      </c>
+      <c r="B20" s="5" t="n">
+        <v>1756</v>
+      </c>
+      <c r="C20" s="5" t="inlineStr">
+        <is>
+          <t>+419</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="4" t="inlineStr">
+        <is>
+          <t>Never Getting Laid</t>
+        </is>
+      </c>
+      <c r="B21" s="5" t="n">
+        <v>2067</v>
+      </c>
+      <c r="C21" s="5" t="inlineStr">
+        <is>
+          <t>+407</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="4" t="inlineStr">
+        <is>
+          <t>My Man on Willpower</t>
+        </is>
+      </c>
+      <c r="B22" s="5" t="n">
+        <v>1669</v>
+      </c>
+      <c r="C22" s="5" t="inlineStr">
+        <is>
+          <t>+1415</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="4" t="inlineStr">
+        <is>
+          <t>Manchild</t>
+        </is>
+      </c>
+      <c r="B23" s="5" t="n">
+        <v>2091</v>
+      </c>
+      <c r="C23" s="5" t="inlineStr">
+        <is>
+          <t>+375</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="4" t="inlineStr">
+        <is>
+          <t>Sugar Talking</t>
+        </is>
+      </c>
+      <c r="B24" s="5" t="n">
+        <v>1625</v>
+      </c>
+      <c r="C24" s="5" t="inlineStr">
+        <is>
+          <t>+427</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="4" t="inlineStr">
+        <is>
+          <t>My Man on Willpower</t>
+        </is>
+      </c>
+      <c r="B25" s="5" t="n">
+        <v>762</v>
+      </c>
+      <c r="C25" s="5" t="inlineStr">
+        <is>
+          <t>+508</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="4" t="inlineStr">
+        <is>
+          <t>Midnight Rain</t>
+        </is>
+      </c>
+      <c r="B26" s="5" t="n">
+        <v>1605</v>
+      </c>
+      <c r="C26" s="5" t="inlineStr">
+        <is>
+          <t>+436</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="4" t="inlineStr">
+        <is>
+          <t>Nobodys Son</t>
+        </is>
+      </c>
+      <c r="B27" s="5" t="n">
+        <v>2426</v>
+      </c>
+      <c r="C27" s="5" t="inlineStr">
+        <is>
+          <t>+481</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="4" t="inlineStr">
+        <is>
+          <t>House Tour</t>
+        </is>
+      </c>
+      <c r="B28" s="5" t="n">
+        <v>1536</v>
+      </c>
+      <c r="C28" s="5" t="inlineStr">
+        <is>
+          <t>+421</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="4" t="inlineStr">
+        <is>
+          <t>Hanabi  Î±Î·Ð²Ï…</t>
+        </is>
+      </c>
+      <c r="B29" s="5" t="n">
+        <v>2612</v>
+      </c>
+      <c r="C29" s="5" t="inlineStr">
+        <is>
+          <t>+341</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="4" t="inlineStr">
+        <is>
+          <t>Dummy</t>
+        </is>
+      </c>
+      <c r="B30" s="5" t="n">
+        <v>2368</v>
+      </c>
+      <c r="C30" s="5" t="inlineStr">
+        <is>
+          <t>+323</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="4" t="inlineStr">
+        <is>
+          <t>Besos Mojados</t>
+        </is>
+      </c>
+      <c r="B31" s="5" t="n">
+        <v>302</v>
+      </c>
+      <c r="C31" s="5" t="inlineStr">
+        <is>
+          <t>+302</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="4" t="inlineStr">
+        <is>
+          <t>DarkFire</t>
+        </is>
+      </c>
+      <c r="B32" s="5" t="n">
+        <v>2503</v>
+      </c>
+      <c r="C32" s="5" t="inlineStr">
+        <is>
+          <t>+275</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="4" t="inlineStr">
+        <is>
+          <t>DarkSunny</t>
+        </is>
+      </c>
+      <c r="B33" s="5" t="n">
+        <v>2627</v>
+      </c>
+      <c r="C33" s="5" t="inlineStr">
+        <is>
+          <t>+281</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="4" t="inlineStr">
+        <is>
+          <t>Dairen Uchiha</t>
+        </is>
+      </c>
+      <c r="B34" s="5" t="n">
+        <v>3173</v>
+      </c>
+      <c r="C34" s="5" t="inlineStr">
+        <is>
+          <t>+295</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="4" t="inlineStr">
+        <is>
+          <t>LILI ZENIN®</t>
+        </is>
+      </c>
+      <c r="B35" s="5" t="n">
+        <v>2106</v>
+      </c>
+      <c r="C35" s="5" t="inlineStr">
+        <is>
+          <t>+352</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="4" t="inlineStr">
+        <is>
+          <t>linda ZENIN ®</t>
+        </is>
+      </c>
+      <c r="B36" s="5" t="n">
+        <v>2491</v>
+      </c>
+      <c r="C36" s="5" t="inlineStr">
+        <is>
+          <t>+346</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="4" t="inlineStr">
+        <is>
+          <t>SHINRAIN ZENIN®</t>
+        </is>
+      </c>
+      <c r="B37" s="5" t="n">
+        <v>2307</v>
+      </c>
+      <c r="C37" s="5" t="inlineStr">
+        <is>
+          <t>+334</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="4" t="inlineStr">
+        <is>
+          <t>Jhayco - Mokai</t>
+        </is>
+      </c>
+      <c r="B38" s="5" t="n">
+        <v>2301</v>
+      </c>
+      <c r="C38" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="4" t="inlineStr">
+        <is>
+          <t>Jhayco - Joe</t>
+        </is>
+      </c>
+      <c r="B39" s="5" t="n">
+        <v>2489</v>
+      </c>
+      <c r="C39" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="4" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="B40" s="5" t="n">
+        <v>2306</v>
+      </c>
+      <c r="C40" s="5" t="inlineStr">
+        <is>
+          <t>+494</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="4" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="B41" s="5" t="n">
+        <v>2394</v>
+      </c>
+      <c r="C41" s="5" t="inlineStr">
+        <is>
+          <t>+489</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="4" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="B42" s="5" t="n">
+        <v>2362</v>
+      </c>
+      <c r="C42" s="5" t="inlineStr">
+        <is>
+          <t>+467</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="4" t="inlineStr">
+        <is>
+          <t>Go Go Juice</t>
+        </is>
+      </c>
+      <c r="B43" s="5" t="n">
+        <v>1895</v>
+      </c>
+      <c r="C43" s="5" t="inlineStr">
+        <is>
+          <t>+360</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="4" t="inlineStr">
+        <is>
+          <t>Jhayco - Imaginaste</t>
+        </is>
+      </c>
+      <c r="B44" s="5" t="n">
+        <v>302</v>
+      </c>
+      <c r="C44" s="5" t="inlineStr">
+        <is>
+          <t>+302</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="4" t="inlineStr">
+        <is>
+          <t>PuNch</t>
+        </is>
+      </c>
+      <c r="B45" s="5" t="n">
+        <v>665</v>
+      </c>
+      <c r="C45" s="5" t="inlineStr">
+        <is>
+          <t>+296</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A2:C2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
auto: snapshot 2026-07-21 13:31:00
</commit_message>
<xml_diff>
--- a/clan_3815.xlsx
+++ b/clan_3815.xlsx
@@ -3667,7 +3667,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Timestamp: 2026-07-21 13:01:00</t>
+          <t>Timestamp: 2026-07-21 13:31:00</t>
         </is>
       </c>
     </row>
@@ -3755,11 +3755,11 @@
         </is>
       </c>
       <c r="B8" s="5" t="n">
-        <v>744</v>
+        <v>769</v>
       </c>
       <c r="C8" s="5" t="inlineStr">
         <is>
-          <t>+427</t>
+          <t>+452</t>
         </is>
       </c>
     </row>
@@ -3770,11 +3770,11 @@
         </is>
       </c>
       <c r="B9" s="5" t="n">
-        <v>796</v>
+        <v>821</v>
       </c>
       <c r="C9" s="5" t="inlineStr">
         <is>
-          <t>-402</t>
+          <t>-377</t>
         </is>
       </c>
     </row>
@@ -3890,11 +3890,11 @@
         </is>
       </c>
       <c r="B17" s="5" t="n">
-        <v>1837</v>
+        <v>1855</v>
       </c>
       <c r="C17" s="5" t="inlineStr">
         <is>
-          <t>+457</t>
+          <t>+475</t>
         </is>
       </c>
     </row>
@@ -3935,11 +3935,11 @@
         </is>
       </c>
       <c r="B20" s="5" t="n">
-        <v>1756</v>
+        <v>1806</v>
       </c>
       <c r="C20" s="5" t="inlineStr">
         <is>
-          <t>+419</t>
+          <t>+469</t>
         </is>
       </c>
     </row>
@@ -3950,11 +3950,11 @@
         </is>
       </c>
       <c r="B21" s="5" t="n">
-        <v>2067</v>
+        <v>2092</v>
       </c>
       <c r="C21" s="5" t="inlineStr">
         <is>
-          <t>+407</t>
+          <t>+432</t>
         </is>
       </c>
     </row>
@@ -3965,11 +3965,11 @@
         </is>
       </c>
       <c r="B22" s="5" t="n">
-        <v>1669</v>
+        <v>1694</v>
       </c>
       <c r="C22" s="5" t="inlineStr">
         <is>
-          <t>+1415</t>
+          <t>+1440</t>
         </is>
       </c>
     </row>
@@ -3980,11 +3980,11 @@
         </is>
       </c>
       <c r="B23" s="5" t="n">
-        <v>2091</v>
+        <v>2116</v>
       </c>
       <c r="C23" s="5" t="inlineStr">
         <is>
-          <t>+375</t>
+          <t>+400</t>
         </is>
       </c>
     </row>
@@ -3995,11 +3995,11 @@
         </is>
       </c>
       <c r="B24" s="5" t="n">
-        <v>1625</v>
+        <v>1651</v>
       </c>
       <c r="C24" s="5" t="inlineStr">
         <is>
-          <t>+427</t>
+          <t>+453</t>
         </is>
       </c>
     </row>
@@ -4010,11 +4010,11 @@
         </is>
       </c>
       <c r="B25" s="5" t="n">
-        <v>762</v>
+        <v>787</v>
       </c>
       <c r="C25" s="5" t="inlineStr">
         <is>
-          <t>+508</t>
+          <t>+533</t>
         </is>
       </c>
     </row>
@@ -4025,11 +4025,11 @@
         </is>
       </c>
       <c r="B26" s="5" t="n">
-        <v>1605</v>
+        <v>1655</v>
       </c>
       <c r="C26" s="5" t="inlineStr">
         <is>
-          <t>+436</t>
+          <t>+486</t>
         </is>
       </c>
     </row>
@@ -4040,11 +4040,11 @@
         </is>
       </c>
       <c r="B27" s="5" t="n">
-        <v>2426</v>
+        <v>2451</v>
       </c>
       <c r="C27" s="5" t="inlineStr">
         <is>
-          <t>+481</t>
+          <t>+506</t>
         </is>
       </c>
     </row>
@@ -4055,11 +4055,11 @@
         </is>
       </c>
       <c r="B28" s="5" t="n">
-        <v>1536</v>
+        <v>1586</v>
       </c>
       <c r="C28" s="5" t="inlineStr">
         <is>
-          <t>+421</t>
+          <t>+471</t>
         </is>
       </c>
     </row>
@@ -4265,11 +4265,11 @@
         </is>
       </c>
       <c r="B42" s="5" t="n">
-        <v>2362</v>
+        <v>2372</v>
       </c>
       <c r="C42" s="5" t="inlineStr">
         <is>
-          <t>+467</t>
+          <t>+477</t>
         </is>
       </c>
     </row>
@@ -4280,11 +4280,11 @@
         </is>
       </c>
       <c r="B43" s="5" t="n">
-        <v>1895</v>
+        <v>1920</v>
       </c>
       <c r="C43" s="5" t="inlineStr">
         <is>
-          <t>+360</t>
+          <t>+385</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: snapshot 2026-07-22 13:01:00
</commit_message>
<xml_diff>
--- a/clan_3815.xlsx
+++ b/clan_3815.xlsx
@@ -14,6 +14,7 @@
     <sheet name="2026-07-19" sheetId="5" state="visible" r:id="rId5"/>
     <sheet name="2026-07-20" sheetId="6" state="visible" r:id="rId6"/>
     <sheet name="2026-07-21" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="2026-07-22" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -4325,4 +4326,688 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C45"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="29" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Clan: Mans Best Friend (3815)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Timestamp: 2026-07-22 13:01:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>Total Reps</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>Daily Reps (+1d)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>Nobodys Son</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="n">
+        <v>2373</v>
+      </c>
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>-78</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>Create Character III</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="n">
+        <v>1765</v>
+      </c>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>Create Character IV</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="n">
+        <v>2593</v>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>Create Character V</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="n">
+        <v>2493</v>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>Tears</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="n">
+        <v>1117</v>
+      </c>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>+348</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>Sugar Talking</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="n">
+        <v>1055</v>
+      </c>
+      <c r="C9" s="5" t="inlineStr">
+        <is>
+          <t>-596</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="n">
+        <v>695</v>
+      </c>
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>Anti-Hero</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="n">
+        <v>1484</v>
+      </c>
+      <c r="C11" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t>Vigilante Shit</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="n">
+        <v>1454</v>
+      </c>
+      <c r="C12" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="4" t="inlineStr">
+        <is>
+          <t>Sweet Nothing</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="n">
+        <v>1410</v>
+      </c>
+      <c r="C13" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="4" t="inlineStr">
+        <is>
+          <t>The Great War</t>
+        </is>
+      </c>
+      <c r="B14" s="5" t="n">
+        <v>1218</v>
+      </c>
+      <c r="C14" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">We Almost Broke Up </t>
+        </is>
+      </c>
+      <c r="B15" s="5" t="n">
+        <v>2574</v>
+      </c>
+      <c r="C15" s="5" t="inlineStr">
+        <is>
+          <t>+389</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="4" t="inlineStr">
+        <is>
+          <t>When Did You Get Hot</t>
+        </is>
+      </c>
+      <c r="B16" s="5" t="n">
+        <v>2398</v>
+      </c>
+      <c r="C16" s="5" t="inlineStr">
+        <is>
+          <t>+400</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="4" t="inlineStr">
+        <is>
+          <t>Dont Worry Ill Make</t>
+        </is>
+      </c>
+      <c r="B17" s="5" t="n">
+        <v>2235</v>
+      </c>
+      <c r="C17" s="5" t="inlineStr">
+        <is>
+          <t>+380</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="4" t="inlineStr">
+        <is>
+          <t>Goodbye</t>
+        </is>
+      </c>
+      <c r="B18" s="5" t="n">
+        <v>2365</v>
+      </c>
+      <c r="C18" s="5" t="inlineStr">
+        <is>
+          <t>+425</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="4" t="inlineStr">
+        <is>
+          <t>Mans Best Friend</t>
+        </is>
+      </c>
+      <c r="B19" s="5" t="n">
+        <v>2219</v>
+      </c>
+      <c r="C19" s="5" t="inlineStr">
+        <is>
+          <t>+400</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="4" t="inlineStr">
+        <is>
+          <t>Lavender Haze</t>
+        </is>
+      </c>
+      <c r="B20" s="5" t="n">
+        <v>2166</v>
+      </c>
+      <c r="C20" s="5" t="inlineStr">
+        <is>
+          <t>+360</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="4" t="inlineStr">
+        <is>
+          <t>Never Getting Laid</t>
+        </is>
+      </c>
+      <c r="B21" s="5" t="n">
+        <v>2456</v>
+      </c>
+      <c r="C21" s="5" t="inlineStr">
+        <is>
+          <t>+364</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="4" t="inlineStr">
+        <is>
+          <t>My Man on Willpower</t>
+        </is>
+      </c>
+      <c r="B22" s="5" t="n">
+        <v>2066</v>
+      </c>
+      <c r="C22" s="5" t="inlineStr">
+        <is>
+          <t>+1279</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="4" t="inlineStr">
+        <is>
+          <t>Manchild</t>
+        </is>
+      </c>
+      <c r="B23" s="5" t="n">
+        <v>2436</v>
+      </c>
+      <c r="C23" s="5" t="inlineStr">
+        <is>
+          <t>+320</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="4" t="inlineStr">
+        <is>
+          <t>Sugar Talking</t>
+        </is>
+      </c>
+      <c r="B24" s="5" t="n">
+        <v>2011</v>
+      </c>
+      <c r="C24" s="5" t="inlineStr">
+        <is>
+          <t>+360</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="4" t="inlineStr">
+        <is>
+          <t>My Man on Willpower</t>
+        </is>
+      </c>
+      <c r="B25" s="5" t="n">
+        <v>1012</v>
+      </c>
+      <c r="C25" s="5" t="inlineStr">
+        <is>
+          <t>+225</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="4" t="inlineStr">
+        <is>
+          <t>Midnight Rain</t>
+        </is>
+      </c>
+      <c r="B26" s="5" t="n">
+        <v>1999</v>
+      </c>
+      <c r="C26" s="5" t="inlineStr">
+        <is>
+          <t>+344</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="4" t="inlineStr">
+        <is>
+          <t>Nobodys Son</t>
+        </is>
+      </c>
+      <c r="B27" s="5" t="n">
+        <v>2668</v>
+      </c>
+      <c r="C27" s="5" t="inlineStr">
+        <is>
+          <t>+217</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="4" t="inlineStr">
+        <is>
+          <t>House Tour</t>
+        </is>
+      </c>
+      <c r="B28" s="5" t="n">
+        <v>1970</v>
+      </c>
+      <c r="C28" s="5" t="inlineStr">
+        <is>
+          <t>+384</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="4" t="inlineStr">
+        <is>
+          <t>Hanabi  Î±Î·Ð²Ï…</t>
+        </is>
+      </c>
+      <c r="B29" s="5" t="n">
+        <v>2612</v>
+      </c>
+      <c r="C29" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="4" t="inlineStr">
+        <is>
+          <t>Dummy</t>
+        </is>
+      </c>
+      <c r="B30" s="5" t="n">
+        <v>2368</v>
+      </c>
+      <c r="C30" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="4" t="inlineStr">
+        <is>
+          <t>Besos Mojados</t>
+        </is>
+      </c>
+      <c r="B31" s="5" t="n">
+        <v>302</v>
+      </c>
+      <c r="C31" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="4" t="inlineStr">
+        <is>
+          <t>DarkFire</t>
+        </is>
+      </c>
+      <c r="B32" s="5" t="n">
+        <v>2503</v>
+      </c>
+      <c r="C32" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="4" t="inlineStr">
+        <is>
+          <t>DarkSunny</t>
+        </is>
+      </c>
+      <c r="B33" s="5" t="n">
+        <v>2627</v>
+      </c>
+      <c r="C33" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="4" t="inlineStr">
+        <is>
+          <t>Dairen Uchiha</t>
+        </is>
+      </c>
+      <c r="B34" s="5" t="n">
+        <v>3173</v>
+      </c>
+      <c r="C34" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="4" t="inlineStr">
+        <is>
+          <t>LILI ZENIN®</t>
+        </is>
+      </c>
+      <c r="B35" s="5" t="n">
+        <v>2106</v>
+      </c>
+      <c r="C35" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="4" t="inlineStr">
+        <is>
+          <t>linda ZENIN ®</t>
+        </is>
+      </c>
+      <c r="B36" s="5" t="n">
+        <v>2491</v>
+      </c>
+      <c r="C36" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="4" t="inlineStr">
+        <is>
+          <t>SHINRAIN ZENIN®</t>
+        </is>
+      </c>
+      <c r="B37" s="5" t="n">
+        <v>2307</v>
+      </c>
+      <c r="C37" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="4" t="inlineStr">
+        <is>
+          <t>Jhayco - Mokai</t>
+        </is>
+      </c>
+      <c r="B38" s="5" t="n">
+        <v>2706</v>
+      </c>
+      <c r="C38" s="5" t="inlineStr">
+        <is>
+          <t>+405</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="4" t="inlineStr">
+        <is>
+          <t>Jhayco - Joe</t>
+        </is>
+      </c>
+      <c r="B39" s="5" t="n">
+        <v>2862</v>
+      </c>
+      <c r="C39" s="5" t="inlineStr">
+        <is>
+          <t>+373</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="4" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="B40" s="5" t="n">
+        <v>2731</v>
+      </c>
+      <c r="C40" s="5" t="inlineStr">
+        <is>
+          <t>+425</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="4" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="B41" s="5" t="n">
+        <v>2774</v>
+      </c>
+      <c r="C41" s="5" t="inlineStr">
+        <is>
+          <t>+380</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="4" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="B42" s="5" t="n">
+        <v>2728</v>
+      </c>
+      <c r="C42" s="5" t="inlineStr">
+        <is>
+          <t>+356</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="4" t="inlineStr">
+        <is>
+          <t>Go Go Juice</t>
+        </is>
+      </c>
+      <c r="B43" s="5" t="n">
+        <v>2284</v>
+      </c>
+      <c r="C43" s="5" t="inlineStr">
+        <is>
+          <t>+364</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="4" t="inlineStr">
+        <is>
+          <t>Jhayco - Imaginaste</t>
+        </is>
+      </c>
+      <c r="B44" s="5" t="n">
+        <v>302</v>
+      </c>
+      <c r="C44" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="4" t="inlineStr">
+        <is>
+          <t>PuNch</t>
+        </is>
+      </c>
+      <c r="B45" s="5" t="n">
+        <v>665</v>
+      </c>
+      <c r="C45" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A2:C2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
auto: snapshot 2026-07-23 13:01:01
</commit_message>
<xml_diff>
--- a/clan_3815.xlsx
+++ b/clan_3815.xlsx
@@ -15,6 +15,7 @@
     <sheet name="2026-07-20" sheetId="6" state="visible" r:id="rId6"/>
     <sheet name="2026-07-21" sheetId="7" state="visible" r:id="rId7"/>
     <sheet name="2026-07-22" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="2026-07-23" sheetId="9" state="visible" r:id="rId9"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -5010,4 +5011,688 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C45"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="29" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Clan: Mans Best Friend (3815)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Timestamp: 2026-07-23 13:01:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>Total Reps</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>Daily Reps (+1d)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>Nobodys Son</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="n">
+        <v>2373</v>
+      </c>
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>-295</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>Create Character III</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="n">
+        <v>1765</v>
+      </c>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>Create Character IV</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="n">
+        <v>2593</v>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>Create Character V</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="n">
+        <v>2493</v>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>Tears</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="n">
+        <v>1117</v>
+      </c>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>Sugar Talking</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="n">
+        <v>1055</v>
+      </c>
+      <c r="C9" s="5" t="inlineStr">
+        <is>
+          <t>-956</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="n">
+        <v>695</v>
+      </c>
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>Anti-Hero</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="n">
+        <v>1484</v>
+      </c>
+      <c r="C11" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t>Vigilante Shit</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="n">
+        <v>1454</v>
+      </c>
+      <c r="C12" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="4" t="inlineStr">
+        <is>
+          <t>Sweet Nothing</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="n">
+        <v>1410</v>
+      </c>
+      <c r="C13" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="4" t="inlineStr">
+        <is>
+          <t>The Great War</t>
+        </is>
+      </c>
+      <c r="B14" s="5" t="n">
+        <v>1218</v>
+      </c>
+      <c r="C14" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">We Almost Broke Up </t>
+        </is>
+      </c>
+      <c r="B15" s="5" t="n">
+        <v>2574</v>
+      </c>
+      <c r="C15" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="4" t="inlineStr">
+        <is>
+          <t>When Did You Get Hot</t>
+        </is>
+      </c>
+      <c r="B16" s="5" t="n">
+        <v>2398</v>
+      </c>
+      <c r="C16" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="4" t="inlineStr">
+        <is>
+          <t>Dont Worry Ill Make</t>
+        </is>
+      </c>
+      <c r="B17" s="5" t="n">
+        <v>2235</v>
+      </c>
+      <c r="C17" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="4" t="inlineStr">
+        <is>
+          <t>Goodbye</t>
+        </is>
+      </c>
+      <c r="B18" s="5" t="n">
+        <v>2365</v>
+      </c>
+      <c r="C18" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="4" t="inlineStr">
+        <is>
+          <t>Mans Best Friend</t>
+        </is>
+      </c>
+      <c r="B19" s="5" t="n">
+        <v>2219</v>
+      </c>
+      <c r="C19" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="4" t="inlineStr">
+        <is>
+          <t>Lavender Haze</t>
+        </is>
+      </c>
+      <c r="B20" s="5" t="n">
+        <v>2166</v>
+      </c>
+      <c r="C20" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="4" t="inlineStr">
+        <is>
+          <t>Never Getting Laid</t>
+        </is>
+      </c>
+      <c r="B21" s="5" t="n">
+        <v>2456</v>
+      </c>
+      <c r="C21" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="4" t="inlineStr">
+        <is>
+          <t>My Man on Willpower</t>
+        </is>
+      </c>
+      <c r="B22" s="5" t="n">
+        <v>2066</v>
+      </c>
+      <c r="C22" s="5" t="inlineStr">
+        <is>
+          <t>+1054</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="4" t="inlineStr">
+        <is>
+          <t>Manchild</t>
+        </is>
+      </c>
+      <c r="B23" s="5" t="n">
+        <v>2436</v>
+      </c>
+      <c r="C23" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="4" t="inlineStr">
+        <is>
+          <t>Sugar Talking</t>
+        </is>
+      </c>
+      <c r="B24" s="5" t="n">
+        <v>2011</v>
+      </c>
+      <c r="C24" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="4" t="inlineStr">
+        <is>
+          <t>My Man on Willpower</t>
+        </is>
+      </c>
+      <c r="B25" s="5" t="n">
+        <v>1012</v>
+      </c>
+      <c r="C25" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="4" t="inlineStr">
+        <is>
+          <t>Midnight Rain</t>
+        </is>
+      </c>
+      <c r="B26" s="5" t="n">
+        <v>1999</v>
+      </c>
+      <c r="C26" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="4" t="inlineStr">
+        <is>
+          <t>Nobodys Son</t>
+        </is>
+      </c>
+      <c r="B27" s="5" t="n">
+        <v>2668</v>
+      </c>
+      <c r="C27" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="4" t="inlineStr">
+        <is>
+          <t>House Tour</t>
+        </is>
+      </c>
+      <c r="B28" s="5" t="n">
+        <v>1970</v>
+      </c>
+      <c r="C28" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="4" t="inlineStr">
+        <is>
+          <t>Hanabi  Î±Î·Ð²Ï…</t>
+        </is>
+      </c>
+      <c r="B29" s="5" t="n">
+        <v>2612</v>
+      </c>
+      <c r="C29" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="4" t="inlineStr">
+        <is>
+          <t>Dummy</t>
+        </is>
+      </c>
+      <c r="B30" s="5" t="n">
+        <v>2368</v>
+      </c>
+      <c r="C30" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="4" t="inlineStr">
+        <is>
+          <t>Besos Mojados</t>
+        </is>
+      </c>
+      <c r="B31" s="5" t="n">
+        <v>512</v>
+      </c>
+      <c r="C31" s="5" t="inlineStr">
+        <is>
+          <t>+210</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="4" t="inlineStr">
+        <is>
+          <t>DarkFire</t>
+        </is>
+      </c>
+      <c r="B32" s="5" t="n">
+        <v>2503</v>
+      </c>
+      <c r="C32" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="4" t="inlineStr">
+        <is>
+          <t>DarkSunny</t>
+        </is>
+      </c>
+      <c r="B33" s="5" t="n">
+        <v>2627</v>
+      </c>
+      <c r="C33" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="4" t="inlineStr">
+        <is>
+          <t>Dairen Uchiha</t>
+        </is>
+      </c>
+      <c r="B34" s="5" t="n">
+        <v>3173</v>
+      </c>
+      <c r="C34" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="4" t="inlineStr">
+        <is>
+          <t>LILI ZENIN®</t>
+        </is>
+      </c>
+      <c r="B35" s="5" t="n">
+        <v>2106</v>
+      </c>
+      <c r="C35" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="4" t="inlineStr">
+        <is>
+          <t>linda ZENIN ®</t>
+        </is>
+      </c>
+      <c r="B36" s="5" t="n">
+        <v>2491</v>
+      </c>
+      <c r="C36" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="4" t="inlineStr">
+        <is>
+          <t>SHINRAIN ZENIN®</t>
+        </is>
+      </c>
+      <c r="B37" s="5" t="n">
+        <v>2307</v>
+      </c>
+      <c r="C37" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="4" t="inlineStr">
+        <is>
+          <t>Jhayco - Mokai</t>
+        </is>
+      </c>
+      <c r="B38" s="5" t="n">
+        <v>2706</v>
+      </c>
+      <c r="C38" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="4" t="inlineStr">
+        <is>
+          <t>Jhayco - Joe</t>
+        </is>
+      </c>
+      <c r="B39" s="5" t="n">
+        <v>2862</v>
+      </c>
+      <c r="C39" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="4" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="B40" s="5" t="n">
+        <v>2731</v>
+      </c>
+      <c r="C40" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="4" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="B41" s="5" t="n">
+        <v>2774</v>
+      </c>
+      <c r="C41" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="4" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="B42" s="5" t="n">
+        <v>2728</v>
+      </c>
+      <c r="C42" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="4" t="inlineStr">
+        <is>
+          <t>Go Go Juice</t>
+        </is>
+      </c>
+      <c r="B43" s="5" t="n">
+        <v>2284</v>
+      </c>
+      <c r="C43" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="4" t="inlineStr">
+        <is>
+          <t>Jhayco - Imaginaste</t>
+        </is>
+      </c>
+      <c r="B44" s="5" t="n">
+        <v>512</v>
+      </c>
+      <c r="C44" s="5" t="inlineStr">
+        <is>
+          <t>+210</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="4" t="inlineStr">
+        <is>
+          <t>PuNch</t>
+        </is>
+      </c>
+      <c r="B45" s="5" t="n">
+        <v>665</v>
+      </c>
+      <c r="C45" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A2:C2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
auto: snapshot 2026-07-24 13:01:00
</commit_message>
<xml_diff>
--- a/clan_3815.xlsx
+++ b/clan_3815.xlsx
@@ -16,6 +16,7 @@
     <sheet name="2026-07-21" sheetId="7" state="visible" r:id="rId7"/>
     <sheet name="2026-07-22" sheetId="8" state="visible" r:id="rId8"/>
     <sheet name="2026-07-23" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="2026-07-24" sheetId="10" state="visible" r:id="rId10"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -945,6 +946,750 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C49"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="29" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Clan: Mans Best Friend (3815)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Timestamp: 2026-07-24 13:01:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>Total Reps</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>Daily Reps (+1d)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>Nobodys Son</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="n">
+        <v>2653</v>
+      </c>
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>-15</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>X y L O T A</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="n">
+        <v>1504</v>
+      </c>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>AbdiHyde ID 13496</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="n">
+        <v>420</v>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>Create Character III</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="n">
+        <v>2185</v>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>+420</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>Create Character IV</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="n">
+        <v>3013</v>
+      </c>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>+420</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>Create Character V</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="n">
+        <v>2913</v>
+      </c>
+      <c r="C9" s="5" t="inlineStr">
+        <is>
+          <t>+420</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>Tears</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="n">
+        <v>1537</v>
+      </c>
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>+420</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>Sugar Talking</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="n">
+        <v>1428</v>
+      </c>
+      <c r="C11" s="5" t="inlineStr">
+        <is>
+          <t>-583</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="n">
+        <v>1115</v>
+      </c>
+      <c r="C12" s="5" t="inlineStr">
+        <is>
+          <t>+420</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="4" t="inlineStr">
+        <is>
+          <t>Anti-Hero</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="n">
+        <v>1904</v>
+      </c>
+      <c r="C13" s="5" t="inlineStr">
+        <is>
+          <t>+420</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="4" t="inlineStr">
+        <is>
+          <t>Vigilante Shit</t>
+        </is>
+      </c>
+      <c r="B14" s="5" t="n">
+        <v>1874</v>
+      </c>
+      <c r="C14" s="5" t="inlineStr">
+        <is>
+          <t>+420</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="4" t="inlineStr">
+        <is>
+          <t>Sweet Nothing</t>
+        </is>
+      </c>
+      <c r="B15" s="5" t="n">
+        <v>1778</v>
+      </c>
+      <c r="C15" s="5" t="inlineStr">
+        <is>
+          <t>+368</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="4" t="inlineStr">
+        <is>
+          <t>The Great War</t>
+        </is>
+      </c>
+      <c r="B16" s="5" t="n">
+        <v>1568</v>
+      </c>
+      <c r="C16" s="5" t="inlineStr">
+        <is>
+          <t>+350</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">We Almost Broke Up </t>
+        </is>
+      </c>
+      <c r="B17" s="5" t="n">
+        <v>2994</v>
+      </c>
+      <c r="C17" s="5" t="inlineStr">
+        <is>
+          <t>+420</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="4" t="inlineStr">
+        <is>
+          <t>When Did You Get Hot</t>
+        </is>
+      </c>
+      <c r="B18" s="5" t="n">
+        <v>2818</v>
+      </c>
+      <c r="C18" s="5" t="inlineStr">
+        <is>
+          <t>+420</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="4" t="inlineStr">
+        <is>
+          <t>Dont Worry Ill Make</t>
+        </is>
+      </c>
+      <c r="B19" s="5" t="n">
+        <v>2590</v>
+      </c>
+      <c r="C19" s="5" t="inlineStr">
+        <is>
+          <t>+355</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="4" t="inlineStr">
+        <is>
+          <t>Goodbye</t>
+        </is>
+      </c>
+      <c r="B20" s="5" t="n">
+        <v>2632</v>
+      </c>
+      <c r="C20" s="5" t="inlineStr">
+        <is>
+          <t>+267</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="4" t="inlineStr">
+        <is>
+          <t>Mans Best Friend</t>
+        </is>
+      </c>
+      <c r="B21" s="5" t="n">
+        <v>2499</v>
+      </c>
+      <c r="C21" s="5" t="inlineStr">
+        <is>
+          <t>+280</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="4" t="inlineStr">
+        <is>
+          <t>Lavender Haze</t>
+        </is>
+      </c>
+      <c r="B22" s="5" t="n">
+        <v>2446</v>
+      </c>
+      <c r="C22" s="5" t="inlineStr">
+        <is>
+          <t>+280</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="4" t="inlineStr">
+        <is>
+          <t>Never Getting Laid</t>
+        </is>
+      </c>
+      <c r="B23" s="5" t="n">
+        <v>2837</v>
+      </c>
+      <c r="C23" s="5" t="inlineStr">
+        <is>
+          <t>+381</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="4" t="inlineStr">
+        <is>
+          <t>My Man on Willpower</t>
+        </is>
+      </c>
+      <c r="B24" s="5" t="n">
+        <v>2416</v>
+      </c>
+      <c r="C24" s="5" t="inlineStr">
+        <is>
+          <t>+1404</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="4" t="inlineStr">
+        <is>
+          <t>Manchild</t>
+        </is>
+      </c>
+      <c r="B25" s="5" t="n">
+        <v>2856</v>
+      </c>
+      <c r="C25" s="5" t="inlineStr">
+        <is>
+          <t>+420</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="4" t="inlineStr">
+        <is>
+          <t>Sugar Talking</t>
+        </is>
+      </c>
+      <c r="B26" s="5" t="n">
+        <v>2431</v>
+      </c>
+      <c r="C26" s="5" t="inlineStr">
+        <is>
+          <t>+420</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="4" t="inlineStr">
+        <is>
+          <t>My Man on Willpower</t>
+        </is>
+      </c>
+      <c r="B27" s="5" t="n">
+        <v>1310</v>
+      </c>
+      <c r="C27" s="5" t="inlineStr">
+        <is>
+          <t>+298</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="4" t="inlineStr">
+        <is>
+          <t>Midnight Rain</t>
+        </is>
+      </c>
+      <c r="B28" s="5" t="n">
+        <v>2209</v>
+      </c>
+      <c r="C28" s="5" t="inlineStr">
+        <is>
+          <t>+210</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="4" t="inlineStr">
+        <is>
+          <t>Nobodys Son</t>
+        </is>
+      </c>
+      <c r="B29" s="5" t="n">
+        <v>3018</v>
+      </c>
+      <c r="C29" s="5" t="inlineStr">
+        <is>
+          <t>+350</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="4" t="inlineStr">
+        <is>
+          <t>House Tour</t>
+        </is>
+      </c>
+      <c r="B30" s="5" t="n">
+        <v>2325</v>
+      </c>
+      <c r="C30" s="5" t="inlineStr">
+        <is>
+          <t>+355</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="4" t="inlineStr">
+        <is>
+          <t>Hanabi  Î±Î·Ð²Ï…</t>
+        </is>
+      </c>
+      <c r="B31" s="5" t="n">
+        <v>2612</v>
+      </c>
+      <c r="C31" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="4" t="inlineStr">
+        <is>
+          <t>Dummy</t>
+        </is>
+      </c>
+      <c r="B32" s="5" t="n">
+        <v>2368</v>
+      </c>
+      <c r="C32" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="4" t="inlineStr">
+        <is>
+          <t>Besos Mojados</t>
+        </is>
+      </c>
+      <c r="B33" s="5" t="n">
+        <v>670</v>
+      </c>
+      <c r="C33" s="5" t="inlineStr">
+        <is>
+          <t>+158</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="4" t="inlineStr">
+        <is>
+          <t>DarkFire</t>
+        </is>
+      </c>
+      <c r="B34" s="5" t="n">
+        <v>3751</v>
+      </c>
+      <c r="C34" s="5" t="inlineStr">
+        <is>
+          <t>+1248</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="4" t="inlineStr">
+        <is>
+          <t>DarkSunny</t>
+        </is>
+      </c>
+      <c r="B35" s="5" t="n">
+        <v>3979</v>
+      </c>
+      <c r="C35" s="5" t="inlineStr">
+        <is>
+          <t>+1352</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="4" t="inlineStr">
+        <is>
+          <t>Dairen Uchiha</t>
+        </is>
+      </c>
+      <c r="B36" s="5" t="n">
+        <v>4593</v>
+      </c>
+      <c r="C36" s="5" t="inlineStr">
+        <is>
+          <t>+1420</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="4" t="inlineStr">
+        <is>
+          <t>LILI ZENIN®</t>
+        </is>
+      </c>
+      <c r="B37" s="5" t="n">
+        <v>3546</v>
+      </c>
+      <c r="C37" s="5" t="inlineStr">
+        <is>
+          <t>+1440</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="4" t="inlineStr">
+        <is>
+          <t>linda ZENIN ®</t>
+        </is>
+      </c>
+      <c r="B38" s="5" t="n">
+        <v>3711</v>
+      </c>
+      <c r="C38" s="5" t="inlineStr">
+        <is>
+          <t>+1220</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="4" t="inlineStr">
+        <is>
+          <t>SHINRAIN ZENIN®</t>
+        </is>
+      </c>
+      <c r="B39" s="5" t="n">
+        <v>3546</v>
+      </c>
+      <c r="C39" s="5" t="inlineStr">
+        <is>
+          <t>+1239</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="4" t="inlineStr">
+        <is>
+          <t>PlyRed-</t>
+        </is>
+      </c>
+      <c r="B40" s="5" t="n">
+        <v>350</v>
+      </c>
+      <c r="C40" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="4" t="inlineStr">
+        <is>
+          <t>equin0x</t>
+        </is>
+      </c>
+      <c r="B41" s="5" t="n">
+        <v>1500</v>
+      </c>
+      <c r="C41" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="4" t="inlineStr">
+        <is>
+          <t>Jhayco - Mokai</t>
+        </is>
+      </c>
+      <c r="B42" s="5" t="n">
+        <v>4476</v>
+      </c>
+      <c r="C42" s="5" t="inlineStr">
+        <is>
+          <t>+1770</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="4" t="inlineStr">
+        <is>
+          <t>Jhayco - Joe</t>
+        </is>
+      </c>
+      <c r="B43" s="5" t="n">
+        <v>4554</v>
+      </c>
+      <c r="C43" s="5" t="inlineStr">
+        <is>
+          <t>+1692</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="4" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="B44" s="5" t="n">
+        <v>4351</v>
+      </c>
+      <c r="C44" s="5" t="inlineStr">
+        <is>
+          <t>+1620</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="4" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="B45" s="5" t="n">
+        <v>4564</v>
+      </c>
+      <c r="C45" s="5" t="inlineStr">
+        <is>
+          <t>+1790</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="4" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="B46" s="5" t="n">
+        <v>4426</v>
+      </c>
+      <c r="C46" s="5" t="inlineStr">
+        <is>
+          <t>+1698</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="4" t="inlineStr">
+        <is>
+          <t>Go Go Juice</t>
+        </is>
+      </c>
+      <c r="B47" s="5" t="n">
+        <v>2652</v>
+      </c>
+      <c r="C47" s="5" t="inlineStr">
+        <is>
+          <t>+368</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="4" t="inlineStr">
+        <is>
+          <t>Jhayco - Imaginaste</t>
+        </is>
+      </c>
+      <c r="B48" s="5" t="n">
+        <v>722</v>
+      </c>
+      <c r="C48" s="5" t="inlineStr">
+        <is>
+          <t>+210</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="4" t="inlineStr">
+        <is>
+          <t>PuNch</t>
+        </is>
+      </c>
+      <c r="B49" s="5" t="n">
+        <v>2435</v>
+      </c>
+      <c r="C49" s="5" t="inlineStr">
+        <is>
+          <t>+1770</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A2:C2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
auto: snapshot 2026-07-24 13:31:00
</commit_message>
<xml_diff>
--- a/clan_3815.xlsx
+++ b/clan_3815.xlsx
@@ -970,7 +970,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Timestamp: 2026-07-24 13:01:00</t>
+          <t>Timestamp: 2026-07-24 13:31:00</t>
         </is>
       </c>
     </row>
@@ -1013,7 +1013,7 @@
         </is>
       </c>
       <c r="B5" s="5" t="n">
-        <v>1504</v>
+        <v>1574</v>
       </c>
       <c r="C5" s="5" t="inlineStr">
         <is>
@@ -1028,7 +1028,7 @@
         </is>
       </c>
       <c r="B6" s="5" t="n">
-        <v>420</v>
+        <v>490</v>
       </c>
       <c r="C6" s="5" t="inlineStr">
         <is>
@@ -1043,11 +1043,11 @@
         </is>
       </c>
       <c r="B7" s="5" t="n">
-        <v>2185</v>
+        <v>2255</v>
       </c>
       <c r="C7" s="5" t="inlineStr">
         <is>
-          <t>+420</t>
+          <t>+490</t>
         </is>
       </c>
     </row>
@@ -1058,11 +1058,11 @@
         </is>
       </c>
       <c r="B8" s="5" t="n">
-        <v>3013</v>
+        <v>3083</v>
       </c>
       <c r="C8" s="5" t="inlineStr">
         <is>
-          <t>+420</t>
+          <t>+490</t>
         </is>
       </c>
     </row>
@@ -1073,11 +1073,11 @@
         </is>
       </c>
       <c r="B9" s="5" t="n">
-        <v>2913</v>
+        <v>2983</v>
       </c>
       <c r="C9" s="5" t="inlineStr">
         <is>
-          <t>+420</t>
+          <t>+490</t>
         </is>
       </c>
     </row>
@@ -1088,11 +1088,11 @@
         </is>
       </c>
       <c r="B10" s="5" t="n">
-        <v>1537</v>
+        <v>1607</v>
       </c>
       <c r="C10" s="5" t="inlineStr">
         <is>
-          <t>+420</t>
+          <t>+490</t>
         </is>
       </c>
     </row>
@@ -1118,11 +1118,11 @@
         </is>
       </c>
       <c r="B12" s="5" t="n">
-        <v>1115</v>
+        <v>1185</v>
       </c>
       <c r="C12" s="5" t="inlineStr">
         <is>
-          <t>+420</t>
+          <t>+490</t>
         </is>
       </c>
     </row>
@@ -1133,11 +1133,11 @@
         </is>
       </c>
       <c r="B13" s="5" t="n">
-        <v>1904</v>
+        <v>1974</v>
       </c>
       <c r="C13" s="5" t="inlineStr">
         <is>
-          <t>+420</t>
+          <t>+490</t>
         </is>
       </c>
     </row>
@@ -1148,11 +1148,11 @@
         </is>
       </c>
       <c r="B14" s="5" t="n">
-        <v>1874</v>
+        <v>1944</v>
       </c>
       <c r="C14" s="5" t="inlineStr">
         <is>
-          <t>+420</t>
+          <t>+490</t>
         </is>
       </c>
     </row>
@@ -1163,11 +1163,11 @@
         </is>
       </c>
       <c r="B15" s="5" t="n">
-        <v>1778</v>
+        <v>1848</v>
       </c>
       <c r="C15" s="5" t="inlineStr">
         <is>
-          <t>+368</t>
+          <t>+438</t>
         </is>
       </c>
     </row>
@@ -1178,11 +1178,11 @@
         </is>
       </c>
       <c r="B16" s="5" t="n">
-        <v>1568</v>
+        <v>1638</v>
       </c>
       <c r="C16" s="5" t="inlineStr">
         <is>
-          <t>+350</t>
+          <t>+420</t>
         </is>
       </c>
     </row>
@@ -1193,11 +1193,11 @@
         </is>
       </c>
       <c r="B17" s="5" t="n">
-        <v>2994</v>
+        <v>3064</v>
       </c>
       <c r="C17" s="5" t="inlineStr">
         <is>
-          <t>+420</t>
+          <t>+490</t>
         </is>
       </c>
     </row>
@@ -1208,11 +1208,11 @@
         </is>
       </c>
       <c r="B18" s="5" t="n">
-        <v>2818</v>
+        <v>2888</v>
       </c>
       <c r="C18" s="5" t="inlineStr">
         <is>
-          <t>+420</t>
+          <t>+490</t>
         </is>
       </c>
     </row>
@@ -1223,11 +1223,11 @@
         </is>
       </c>
       <c r="B19" s="5" t="n">
-        <v>2590</v>
+        <v>2660</v>
       </c>
       <c r="C19" s="5" t="inlineStr">
         <is>
-          <t>+355</t>
+          <t>+425</t>
         </is>
       </c>
     </row>
@@ -1283,11 +1283,11 @@
         </is>
       </c>
       <c r="B23" s="5" t="n">
-        <v>2837</v>
+        <v>2907</v>
       </c>
       <c r="C23" s="5" t="inlineStr">
         <is>
-          <t>+381</t>
+          <t>+451</t>
         </is>
       </c>
     </row>
@@ -1298,11 +1298,11 @@
         </is>
       </c>
       <c r="B24" s="5" t="n">
-        <v>2416</v>
+        <v>2486</v>
       </c>
       <c r="C24" s="5" t="inlineStr">
         <is>
-          <t>+1404</t>
+          <t>+1474</t>
         </is>
       </c>
     </row>
@@ -1313,11 +1313,11 @@
         </is>
       </c>
       <c r="B25" s="5" t="n">
-        <v>2856</v>
+        <v>2926</v>
       </c>
       <c r="C25" s="5" t="inlineStr">
         <is>
-          <t>+420</t>
+          <t>+490</t>
         </is>
       </c>
     </row>
@@ -1328,11 +1328,11 @@
         </is>
       </c>
       <c r="B26" s="5" t="n">
-        <v>2431</v>
+        <v>2501</v>
       </c>
       <c r="C26" s="5" t="inlineStr">
         <is>
-          <t>+420</t>
+          <t>+490</t>
         </is>
       </c>
     </row>
@@ -1343,11 +1343,11 @@
         </is>
       </c>
       <c r="B27" s="5" t="n">
-        <v>1310</v>
+        <v>1411</v>
       </c>
       <c r="C27" s="5" t="inlineStr">
         <is>
-          <t>+298</t>
+          <t>+399</t>
         </is>
       </c>
     </row>
@@ -1373,11 +1373,11 @@
         </is>
       </c>
       <c r="B29" s="5" t="n">
-        <v>3018</v>
+        <v>3158</v>
       </c>
       <c r="C29" s="5" t="inlineStr">
         <is>
-          <t>+350</t>
+          <t>+490</t>
         </is>
       </c>
     </row>
@@ -1388,11 +1388,11 @@
         </is>
       </c>
       <c r="B30" s="5" t="n">
-        <v>2325</v>
+        <v>2395</v>
       </c>
       <c r="C30" s="5" t="inlineStr">
         <is>
-          <t>+355</t>
+          <t>+425</t>
         </is>
       </c>
     </row>
@@ -1448,11 +1448,11 @@
         </is>
       </c>
       <c r="B34" s="5" t="n">
-        <v>3751</v>
+        <v>3852</v>
       </c>
       <c r="C34" s="5" t="inlineStr">
         <is>
-          <t>+1248</t>
+          <t>+1349</t>
         </is>
       </c>
     </row>
@@ -1538,7 +1538,7 @@
         </is>
       </c>
       <c r="B40" s="5" t="n">
-        <v>350</v>
+        <v>420</v>
       </c>
       <c r="C40" s="5" t="inlineStr">
         <is>
@@ -1553,7 +1553,7 @@
         </is>
       </c>
       <c r="B41" s="5" t="n">
-        <v>1500</v>
+        <v>1570</v>
       </c>
       <c r="C41" s="5" t="inlineStr">
         <is>
@@ -1568,11 +1568,11 @@
         </is>
       </c>
       <c r="B42" s="5" t="n">
-        <v>4476</v>
+        <v>4546</v>
       </c>
       <c r="C42" s="5" t="inlineStr">
         <is>
-          <t>+1770</t>
+          <t>+1840</t>
         </is>
       </c>
     </row>
@@ -1583,11 +1583,11 @@
         </is>
       </c>
       <c r="B43" s="5" t="n">
-        <v>4554</v>
+        <v>4624</v>
       </c>
       <c r="C43" s="5" t="inlineStr">
         <is>
-          <t>+1692</t>
+          <t>+1762</t>
         </is>
       </c>
     </row>
@@ -1598,11 +1598,11 @@
         </is>
       </c>
       <c r="B44" s="5" t="n">
-        <v>4351</v>
+        <v>4421</v>
       </c>
       <c r="C44" s="5" t="inlineStr">
         <is>
-          <t>+1620</t>
+          <t>+1690</t>
         </is>
       </c>
     </row>
@@ -1613,11 +1613,11 @@
         </is>
       </c>
       <c r="B45" s="5" t="n">
-        <v>4564</v>
+        <v>4634</v>
       </c>
       <c r="C45" s="5" t="inlineStr">
         <is>
-          <t>+1790</t>
+          <t>+1860</t>
         </is>
       </c>
     </row>
@@ -1628,11 +1628,11 @@
         </is>
       </c>
       <c r="B46" s="5" t="n">
-        <v>4426</v>
+        <v>4496</v>
       </c>
       <c r="C46" s="5" t="inlineStr">
         <is>
-          <t>+1698</t>
+          <t>+1768</t>
         </is>
       </c>
     </row>
@@ -1643,11 +1643,11 @@
         </is>
       </c>
       <c r="B47" s="5" t="n">
-        <v>2652</v>
+        <v>2722</v>
       </c>
       <c r="C47" s="5" t="inlineStr">
         <is>
-          <t>+368</t>
+          <t>+438</t>
         </is>
       </c>
     </row>
@@ -1673,11 +1673,11 @@
         </is>
       </c>
       <c r="B49" s="5" t="n">
-        <v>2435</v>
+        <v>2505</v>
       </c>
       <c r="C49" s="5" t="inlineStr">
         <is>
-          <t>+1770</t>
+          <t>+1840</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: snapshot 2026-07-25 13:01:00
</commit_message>
<xml_diff>
--- a/clan_3815.xlsx
+++ b/clan_3815.xlsx
@@ -17,6 +17,7 @@
     <sheet name="2026-07-22" sheetId="8" state="visible" r:id="rId8"/>
     <sheet name="2026-07-23" sheetId="9" state="visible" r:id="rId9"/>
     <sheet name="2026-07-24" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="2026-07-25" sheetId="11" state="visible" r:id="rId11"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -1690,6 +1691,750 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C49"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="29" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Clan: Mans Best Friend (3815)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Timestamp: 2026-07-25 13:01:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>Total Reps</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>Daily Reps (+1d)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>Nobodys Son</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="n">
+        <v>2803</v>
+      </c>
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>-355</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>X y L O T A</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="n">
+        <v>2174</v>
+      </c>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>+600</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>AbdiHyde ID 13496</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="n">
+        <v>2137</v>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>+1647</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>Create Character III</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="n">
+        <v>3917</v>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>+1662</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>Create Character IV</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="n">
+        <v>4739</v>
+      </c>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>+1656</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>Create Character V</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="n">
+        <v>4641</v>
+      </c>
+      <c r="C9" s="5" t="inlineStr">
+        <is>
+          <t>+1658</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>Tears</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="n">
+        <v>3672</v>
+      </c>
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>+2065</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>Sugar Talking</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="n">
+        <v>2688</v>
+      </c>
+      <c r="C11" s="5" t="inlineStr">
+        <is>
+          <t>+187</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="n">
+        <v>1932</v>
+      </c>
+      <c r="C12" s="5" t="inlineStr">
+        <is>
+          <t>+747</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="4" t="inlineStr">
+        <is>
+          <t>Anti-Hero</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="n">
+        <v>2687</v>
+      </c>
+      <c r="C13" s="5" t="inlineStr">
+        <is>
+          <t>+713</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="4" t="inlineStr">
+        <is>
+          <t>Vigilante Shit</t>
+        </is>
+      </c>
+      <c r="B14" s="5" t="n">
+        <v>2684</v>
+      </c>
+      <c r="C14" s="5" t="inlineStr">
+        <is>
+          <t>+740</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="4" t="inlineStr">
+        <is>
+          <t>Sweet Nothing</t>
+        </is>
+      </c>
+      <c r="B15" s="5" t="n">
+        <v>2588</v>
+      </c>
+      <c r="C15" s="5" t="inlineStr">
+        <is>
+          <t>+740</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="4" t="inlineStr">
+        <is>
+          <t>The Great War</t>
+        </is>
+      </c>
+      <c r="B16" s="5" t="n">
+        <v>2352</v>
+      </c>
+      <c r="C16" s="5" t="inlineStr">
+        <is>
+          <t>+714</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">We Almost Broke Up </t>
+        </is>
+      </c>
+      <c r="B17" s="5" t="n">
+        <v>3424</v>
+      </c>
+      <c r="C17" s="5" t="inlineStr">
+        <is>
+          <t>+360</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="4" t="inlineStr">
+        <is>
+          <t>When Did You Get Hot</t>
+        </is>
+      </c>
+      <c r="B18" s="5" t="n">
+        <v>3248</v>
+      </c>
+      <c r="C18" s="5" t="inlineStr">
+        <is>
+          <t>+360</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="4" t="inlineStr">
+        <is>
+          <t>Dont Worry Ill Make</t>
+        </is>
+      </c>
+      <c r="B19" s="5" t="n">
+        <v>3020</v>
+      </c>
+      <c r="C19" s="5" t="inlineStr">
+        <is>
+          <t>+360</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="4" t="inlineStr">
+        <is>
+          <t>Goodbye</t>
+        </is>
+      </c>
+      <c r="B20" s="5" t="n">
+        <v>2782</v>
+      </c>
+      <c r="C20" s="5" t="inlineStr">
+        <is>
+          <t>+150</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="4" t="inlineStr">
+        <is>
+          <t>Mans Best Friend</t>
+        </is>
+      </c>
+      <c r="B21" s="5" t="n">
+        <v>2649</v>
+      </c>
+      <c r="C21" s="5" t="inlineStr">
+        <is>
+          <t>+150</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="4" t="inlineStr">
+        <is>
+          <t>Lavender Haze</t>
+        </is>
+      </c>
+      <c r="B22" s="5" t="n">
+        <v>2596</v>
+      </c>
+      <c r="C22" s="5" t="inlineStr">
+        <is>
+          <t>+150</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="4" t="inlineStr">
+        <is>
+          <t>Never Getting Laid</t>
+        </is>
+      </c>
+      <c r="B23" s="5" t="n">
+        <v>4918</v>
+      </c>
+      <c r="C23" s="5" t="inlineStr">
+        <is>
+          <t>+2011</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="4" t="inlineStr">
+        <is>
+          <t>My Man on Willpower</t>
+        </is>
+      </c>
+      <c r="B24" s="5" t="n">
+        <v>4420</v>
+      </c>
+      <c r="C24" s="5" t="inlineStr">
+        <is>
+          <t>+3009</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="4" t="inlineStr">
+        <is>
+          <t>Manchild</t>
+        </is>
+      </c>
+      <c r="B25" s="5" t="n">
+        <v>5000</v>
+      </c>
+      <c r="C25" s="5" t="inlineStr">
+        <is>
+          <t>+2074</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="4" t="inlineStr">
+        <is>
+          <t>Sugar Talking</t>
+        </is>
+      </c>
+      <c r="B26" s="5" t="n">
+        <v>2861</v>
+      </c>
+      <c r="C26" s="5" t="inlineStr">
+        <is>
+          <t>+360</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="4" t="inlineStr">
+        <is>
+          <t>My Man on Willpower</t>
+        </is>
+      </c>
+      <c r="B27" s="5" t="n">
+        <v>2671</v>
+      </c>
+      <c r="C27" s="5" t="inlineStr">
+        <is>
+          <t>+1260</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="4" t="inlineStr">
+        <is>
+          <t>Midnight Rain</t>
+        </is>
+      </c>
+      <c r="B28" s="5" t="n">
+        <v>2359</v>
+      </c>
+      <c r="C28" s="5" t="inlineStr">
+        <is>
+          <t>+150</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="4" t="inlineStr">
+        <is>
+          <t>Nobodys Son</t>
+        </is>
+      </c>
+      <c r="B29" s="5" t="n">
+        <v>4323</v>
+      </c>
+      <c r="C29" s="5" t="inlineStr">
+        <is>
+          <t>+1165</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="4" t="inlineStr">
+        <is>
+          <t>House Tour</t>
+        </is>
+      </c>
+      <c r="B30" s="5" t="n">
+        <v>2685</v>
+      </c>
+      <c r="C30" s="5" t="inlineStr">
+        <is>
+          <t>+290</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="4" t="inlineStr">
+        <is>
+          <t>Hanabi  Î±Î·Ð²Ï…</t>
+        </is>
+      </c>
+      <c r="B31" s="5" t="n">
+        <v>2612</v>
+      </c>
+      <c r="C31" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="4" t="inlineStr">
+        <is>
+          <t>Dummy</t>
+        </is>
+      </c>
+      <c r="B32" s="5" t="n">
+        <v>2368</v>
+      </c>
+      <c r="C32" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="4" t="inlineStr">
+        <is>
+          <t>Besos Mojados</t>
+        </is>
+      </c>
+      <c r="B33" s="5" t="n">
+        <v>820</v>
+      </c>
+      <c r="C33" s="5" t="inlineStr">
+        <is>
+          <t>+150</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="4" t="inlineStr">
+        <is>
+          <t>DarkFire</t>
+        </is>
+      </c>
+      <c r="B34" s="5" t="n">
+        <v>5042</v>
+      </c>
+      <c r="C34" s="5" t="inlineStr">
+        <is>
+          <t>+1190</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="4" t="inlineStr">
+        <is>
+          <t>DarkSunny</t>
+        </is>
+      </c>
+      <c r="B35" s="5" t="n">
+        <v>5237</v>
+      </c>
+      <c r="C35" s="5" t="inlineStr">
+        <is>
+          <t>+1258</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="4" t="inlineStr">
+        <is>
+          <t>Dairen Uchiha</t>
+        </is>
+      </c>
+      <c r="B36" s="5" t="n">
+        <v>5897</v>
+      </c>
+      <c r="C36" s="5" t="inlineStr">
+        <is>
+          <t>+1304</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="4" t="inlineStr">
+        <is>
+          <t>LILI ZENIN®</t>
+        </is>
+      </c>
+      <c r="B37" s="5" t="n">
+        <v>3546</v>
+      </c>
+      <c r="C37" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="4" t="inlineStr">
+        <is>
+          <t>linda ZENIN ®</t>
+        </is>
+      </c>
+      <c r="B38" s="5" t="n">
+        <v>3711</v>
+      </c>
+      <c r="C38" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="4" t="inlineStr">
+        <is>
+          <t>SHINRAIN ZENIN®</t>
+        </is>
+      </c>
+      <c r="B39" s="5" t="n">
+        <v>3546</v>
+      </c>
+      <c r="C39" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="4" t="inlineStr">
+        <is>
+          <t>PlyRed-</t>
+        </is>
+      </c>
+      <c r="B40" s="5" t="n">
+        <v>1725</v>
+      </c>
+      <c r="C40" s="5" t="inlineStr">
+        <is>
+          <t>+1305</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="4" t="inlineStr">
+        <is>
+          <t>equin0x</t>
+        </is>
+      </c>
+      <c r="B41" s="5" t="n">
+        <v>3349</v>
+      </c>
+      <c r="C41" s="5" t="inlineStr">
+        <is>
+          <t>+1779</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="4" t="inlineStr">
+        <is>
+          <t>Jhayco - Mokai</t>
+        </is>
+      </c>
+      <c r="B42" s="5" t="n">
+        <v>6267</v>
+      </c>
+      <c r="C42" s="5" t="inlineStr">
+        <is>
+          <t>+1721</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="4" t="inlineStr">
+        <is>
+          <t>Jhayco - Joe</t>
+        </is>
+      </c>
+      <c r="B43" s="5" t="n">
+        <v>6424</v>
+      </c>
+      <c r="C43" s="5" t="inlineStr">
+        <is>
+          <t>+1800</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="4" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="B44" s="5" t="n">
+        <v>6295</v>
+      </c>
+      <c r="C44" s="5" t="inlineStr">
+        <is>
+          <t>+1874</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="4" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="B45" s="5" t="n">
+        <v>6526</v>
+      </c>
+      <c r="C45" s="5" t="inlineStr">
+        <is>
+          <t>+1892</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="4" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="B46" s="5" t="n">
+        <v>6315</v>
+      </c>
+      <c r="C46" s="5" t="inlineStr">
+        <is>
+          <t>+1819</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="4" t="inlineStr">
+        <is>
+          <t>Go Go Juice</t>
+        </is>
+      </c>
+      <c r="B47" s="5" t="n">
+        <v>4805</v>
+      </c>
+      <c r="C47" s="5" t="inlineStr">
+        <is>
+          <t>+2083</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="4" t="inlineStr">
+        <is>
+          <t>Jhayco - Imaginaste</t>
+        </is>
+      </c>
+      <c r="B48" s="5" t="n">
+        <v>872</v>
+      </c>
+      <c r="C48" s="5" t="inlineStr">
+        <is>
+          <t>+150</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="4" t="inlineStr">
+        <is>
+          <t>PuNch</t>
+        </is>
+      </c>
+      <c r="B49" s="5" t="n">
+        <v>4465</v>
+      </c>
+      <c r="C49" s="5" t="inlineStr">
+        <is>
+          <t>+1960</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A2:C2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
auto: snapshot 2026-07-25 13:31:00
</commit_message>
<xml_diff>
--- a/clan_3815.xlsx
+++ b/clan_3815.xlsx
@@ -1715,7 +1715,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Timestamp: 2026-07-25 13:01:00</t>
+          <t>Timestamp: 2026-07-25 13:31:00</t>
         </is>
       </c>
     </row>
@@ -1743,11 +1743,11 @@
         </is>
       </c>
       <c r="B4" s="5" t="n">
-        <v>2803</v>
+        <v>2903</v>
       </c>
       <c r="C4" s="5" t="inlineStr">
         <is>
-          <t>-355</t>
+          <t>-255</t>
         </is>
       </c>
     </row>
@@ -1833,11 +1833,11 @@
         </is>
       </c>
       <c r="B10" s="5" t="n">
-        <v>3672</v>
+        <v>3677</v>
       </c>
       <c r="C10" s="5" t="inlineStr">
         <is>
-          <t>+2065</t>
+          <t>+2070</t>
         </is>
       </c>
     </row>
@@ -1848,11 +1848,11 @@
         </is>
       </c>
       <c r="B11" s="5" t="n">
-        <v>2688</v>
+        <v>2788</v>
       </c>
       <c r="C11" s="5" t="inlineStr">
         <is>
-          <t>+187</t>
+          <t>+287</t>
         </is>
       </c>
     </row>
@@ -1863,11 +1863,11 @@
         </is>
       </c>
       <c r="B12" s="5" t="n">
-        <v>1932</v>
+        <v>1937</v>
       </c>
       <c r="C12" s="5" t="inlineStr">
         <is>
-          <t>+747</t>
+          <t>+752</t>
         </is>
       </c>
     </row>
@@ -1878,11 +1878,11 @@
         </is>
       </c>
       <c r="B13" s="5" t="n">
-        <v>2687</v>
+        <v>2787</v>
       </c>
       <c r="C13" s="5" t="inlineStr">
         <is>
-          <t>+713</t>
+          <t>+813</t>
         </is>
       </c>
     </row>
@@ -1893,11 +1893,11 @@
         </is>
       </c>
       <c r="B14" s="5" t="n">
-        <v>2684</v>
+        <v>2784</v>
       </c>
       <c r="C14" s="5" t="inlineStr">
         <is>
-          <t>+740</t>
+          <t>+840</t>
         </is>
       </c>
     </row>
@@ -1908,11 +1908,11 @@
         </is>
       </c>
       <c r="B15" s="5" t="n">
-        <v>2588</v>
+        <v>2688</v>
       </c>
       <c r="C15" s="5" t="inlineStr">
         <is>
-          <t>+740</t>
+          <t>+840</t>
         </is>
       </c>
     </row>
@@ -1923,11 +1923,11 @@
         </is>
       </c>
       <c r="B16" s="5" t="n">
-        <v>2352</v>
+        <v>2452</v>
       </c>
       <c r="C16" s="5" t="inlineStr">
         <is>
-          <t>+714</t>
+          <t>+814</t>
         </is>
       </c>
     </row>
@@ -1938,11 +1938,11 @@
         </is>
       </c>
       <c r="B17" s="5" t="n">
-        <v>3424</v>
+        <v>3524</v>
       </c>
       <c r="C17" s="5" t="inlineStr">
         <is>
-          <t>+360</t>
+          <t>+460</t>
         </is>
       </c>
     </row>
@@ -1953,11 +1953,11 @@
         </is>
       </c>
       <c r="B18" s="5" t="n">
-        <v>3248</v>
+        <v>3348</v>
       </c>
       <c r="C18" s="5" t="inlineStr">
         <is>
-          <t>+360</t>
+          <t>+460</t>
         </is>
       </c>
     </row>
@@ -1968,11 +1968,11 @@
         </is>
       </c>
       <c r="B19" s="5" t="n">
-        <v>3020</v>
+        <v>3120</v>
       </c>
       <c r="C19" s="5" t="inlineStr">
         <is>
-          <t>+360</t>
+          <t>+460</t>
         </is>
       </c>
     </row>
@@ -1983,11 +1983,11 @@
         </is>
       </c>
       <c r="B20" s="5" t="n">
-        <v>2782</v>
+        <v>2882</v>
       </c>
       <c r="C20" s="5" t="inlineStr">
         <is>
-          <t>+150</t>
+          <t>+250</t>
         </is>
       </c>
     </row>
@@ -1998,11 +1998,11 @@
         </is>
       </c>
       <c r="B21" s="5" t="n">
-        <v>2649</v>
+        <v>2749</v>
       </c>
       <c r="C21" s="5" t="inlineStr">
         <is>
-          <t>+150</t>
+          <t>+250</t>
         </is>
       </c>
     </row>
@@ -2013,11 +2013,11 @@
         </is>
       </c>
       <c r="B22" s="5" t="n">
-        <v>2596</v>
+        <v>2696</v>
       </c>
       <c r="C22" s="5" t="inlineStr">
         <is>
-          <t>+150</t>
+          <t>+250</t>
         </is>
       </c>
     </row>
@@ -2028,11 +2028,11 @@
         </is>
       </c>
       <c r="B23" s="5" t="n">
-        <v>4918</v>
+        <v>4961</v>
       </c>
       <c r="C23" s="5" t="inlineStr">
         <is>
-          <t>+2011</t>
+          <t>+2054</t>
         </is>
       </c>
     </row>
@@ -2043,11 +2043,11 @@
         </is>
       </c>
       <c r="B24" s="5" t="n">
-        <v>4420</v>
+        <v>4520</v>
       </c>
       <c r="C24" s="5" t="inlineStr">
         <is>
-          <t>+3009</t>
+          <t>+3109</t>
         </is>
       </c>
     </row>
@@ -2058,11 +2058,11 @@
         </is>
       </c>
       <c r="B25" s="5" t="n">
-        <v>5000</v>
+        <v>5100</v>
       </c>
       <c r="C25" s="5" t="inlineStr">
         <is>
-          <t>+2074</t>
+          <t>+2174</t>
         </is>
       </c>
     </row>
@@ -2073,11 +2073,11 @@
         </is>
       </c>
       <c r="B26" s="5" t="n">
-        <v>2861</v>
+        <v>2961</v>
       </c>
       <c r="C26" s="5" t="inlineStr">
         <is>
-          <t>+360</t>
+          <t>+460</t>
         </is>
       </c>
     </row>
@@ -2088,11 +2088,11 @@
         </is>
       </c>
       <c r="B27" s="5" t="n">
-        <v>2671</v>
+        <v>2771</v>
       </c>
       <c r="C27" s="5" t="inlineStr">
         <is>
-          <t>+1260</t>
+          <t>+1360</t>
         </is>
       </c>
     </row>
@@ -2103,11 +2103,11 @@
         </is>
       </c>
       <c r="B28" s="5" t="n">
-        <v>2359</v>
+        <v>2459</v>
       </c>
       <c r="C28" s="5" t="inlineStr">
         <is>
-          <t>+150</t>
+          <t>+250</t>
         </is>
       </c>
     </row>
@@ -2118,11 +2118,11 @@
         </is>
       </c>
       <c r="B29" s="5" t="n">
-        <v>4323</v>
+        <v>4423</v>
       </c>
       <c r="C29" s="5" t="inlineStr">
         <is>
-          <t>+1165</t>
+          <t>+1265</t>
         </is>
       </c>
     </row>
@@ -2133,11 +2133,11 @@
         </is>
       </c>
       <c r="B30" s="5" t="n">
-        <v>2685</v>
+        <v>2785</v>
       </c>
       <c r="C30" s="5" t="inlineStr">
         <is>
-          <t>+290</t>
+          <t>+390</t>
         </is>
       </c>
     </row>
@@ -2178,11 +2178,11 @@
         </is>
       </c>
       <c r="B33" s="5" t="n">
-        <v>820</v>
+        <v>920</v>
       </c>
       <c r="C33" s="5" t="inlineStr">
         <is>
-          <t>+150</t>
+          <t>+250</t>
         </is>
       </c>
     </row>
@@ -2388,11 +2388,11 @@
         </is>
       </c>
       <c r="B47" s="5" t="n">
-        <v>4805</v>
+        <v>4905</v>
       </c>
       <c r="C47" s="5" t="inlineStr">
         <is>
-          <t>+2083</t>
+          <t>+2183</t>
         </is>
       </c>
     </row>
@@ -2403,11 +2403,11 @@
         </is>
       </c>
       <c r="B48" s="5" t="n">
-        <v>872</v>
+        <v>972</v>
       </c>
       <c r="C48" s="5" t="inlineStr">
         <is>
-          <t>+150</t>
+          <t>+250</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: snapshot 2026-07-26 13:01:00
</commit_message>
<xml_diff>
--- a/clan_3815.xlsx
+++ b/clan_3815.xlsx
@@ -18,6 +18,7 @@
     <sheet name="2026-07-23" sheetId="9" state="visible" r:id="rId9"/>
     <sheet name="2026-07-24" sheetId="10" state="visible" r:id="rId10"/>
     <sheet name="2026-07-25" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet name="2026-07-26" sheetId="12" state="visible" r:id="rId12"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -2435,6 +2436,885 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C58"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="29" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Clan: Mans Best Friend (3815)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Timestamp: 2026-07-26 13:01:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>Total Reps</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>Daily Reps (+1d)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>Nobodys Son</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="n">
+        <v>5526</v>
+      </c>
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>+1103</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>Player</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="n">
+        <v>900</v>
+      </c>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>Player</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="n">
+        <v>850</v>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>X y L O T A</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="n">
+        <v>3074</v>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>+900</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>AbdiHyde ID 13496</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="n">
+        <v>3647</v>
+      </c>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>+1510</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>Create Character III</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="n">
+        <v>5417</v>
+      </c>
+      <c r="C9" s="5" t="inlineStr">
+        <is>
+          <t>+1500</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>Create Character IV</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="n">
+        <v>6058</v>
+      </c>
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>+1319</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>Create Character V</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="n">
+        <v>5978</v>
+      </c>
+      <c r="C11" s="5" t="inlineStr">
+        <is>
+          <t>+1337</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t>Player</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="n">
+        <v>850</v>
+      </c>
+      <c r="C12" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="4" t="inlineStr">
+        <is>
+          <t>Player</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="n">
+        <v>850</v>
+      </c>
+      <c r="C13" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="4" t="inlineStr">
+        <is>
+          <t>hunry</t>
+        </is>
+      </c>
+      <c r="B14" s="5" t="n">
+        <v>823</v>
+      </c>
+      <c r="C14" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="4" t="inlineStr">
+        <is>
+          <t>Tears</t>
+        </is>
+      </c>
+      <c r="B15" s="5" t="n">
+        <v>5327</v>
+      </c>
+      <c r="C15" s="5" t="inlineStr">
+        <is>
+          <t>+1650</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="4" t="inlineStr">
+        <is>
+          <t>Sugar Talking</t>
+        </is>
+      </c>
+      <c r="B16" s="5" t="n">
+        <v>5762</v>
+      </c>
+      <c r="C16" s="5" t="inlineStr">
+        <is>
+          <t>+2801</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="4" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B17" s="5" t="n">
+        <v>5023</v>
+      </c>
+      <c r="C17" s="5" t="inlineStr">
+        <is>
+          <t>+3086</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="4" t="inlineStr">
+        <is>
+          <t>Anti-Hero</t>
+        </is>
+      </c>
+      <c r="B18" s="5" t="n">
+        <v>5769</v>
+      </c>
+      <c r="C18" s="5" t="inlineStr">
+        <is>
+          <t>+2982</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="4" t="inlineStr">
+        <is>
+          <t>Vigilante Shit</t>
+        </is>
+      </c>
+      <c r="B19" s="5" t="n">
+        <v>5784</v>
+      </c>
+      <c r="C19" s="5" t="inlineStr">
+        <is>
+          <t>+3000</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="4" t="inlineStr">
+        <is>
+          <t>Sweet Nothing</t>
+        </is>
+      </c>
+      <c r="B20" s="5" t="n">
+        <v>5819</v>
+      </c>
+      <c r="C20" s="5" t="inlineStr">
+        <is>
+          <t>+3131</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="4" t="inlineStr">
+        <is>
+          <t>The Great War</t>
+        </is>
+      </c>
+      <c r="B21" s="5" t="n">
+        <v>5602</v>
+      </c>
+      <c r="C21" s="5" t="inlineStr">
+        <is>
+          <t>+3150</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">We Almost Broke Up </t>
+        </is>
+      </c>
+      <c r="B22" s="5" t="n">
+        <v>6102</v>
+      </c>
+      <c r="C22" s="5" t="inlineStr">
+        <is>
+          <t>+2578</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="4" t="inlineStr">
+        <is>
+          <t>When Did You Get Hot</t>
+        </is>
+      </c>
+      <c r="B23" s="5" t="n">
+        <v>5998</v>
+      </c>
+      <c r="C23" s="5" t="inlineStr">
+        <is>
+          <t>+2650</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="4" t="inlineStr">
+        <is>
+          <t>Dont Worry Ill Make</t>
+        </is>
+      </c>
+      <c r="B24" s="5" t="n">
+        <v>5454</v>
+      </c>
+      <c r="C24" s="5" t="inlineStr">
+        <is>
+          <t>+2334</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="4" t="inlineStr">
+        <is>
+          <t>Goodbye</t>
+        </is>
+      </c>
+      <c r="B25" s="5" t="n">
+        <v>5258</v>
+      </c>
+      <c r="C25" s="5" t="inlineStr">
+        <is>
+          <t>+2376</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="4" t="inlineStr">
+        <is>
+          <t>Mans Best Friend</t>
+        </is>
+      </c>
+      <c r="B26" s="5" t="n">
+        <v>5178</v>
+      </c>
+      <c r="C26" s="5" t="inlineStr">
+        <is>
+          <t>+2429</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="4" t="inlineStr">
+        <is>
+          <t>Lavender Haze</t>
+        </is>
+      </c>
+      <c r="B27" s="5" t="n">
+        <v>5220</v>
+      </c>
+      <c r="C27" s="5" t="inlineStr">
+        <is>
+          <t>+2524</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="4" t="inlineStr">
+        <is>
+          <t>Never Getting Laid</t>
+        </is>
+      </c>
+      <c r="B28" s="5" t="n">
+        <v>6593</v>
+      </c>
+      <c r="C28" s="5" t="inlineStr">
+        <is>
+          <t>+1632</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="4" t="inlineStr">
+        <is>
+          <t>My Man on Willpower</t>
+        </is>
+      </c>
+      <c r="B29" s="5" t="n">
+        <v>5907</v>
+      </c>
+      <c r="C29" s="5" t="inlineStr">
+        <is>
+          <t>+3136</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="4" t="inlineStr">
+        <is>
+          <t>Manchild</t>
+        </is>
+      </c>
+      <c r="B30" s="5" t="n">
+        <v>6650</v>
+      </c>
+      <c r="C30" s="5" t="inlineStr">
+        <is>
+          <t>+1550</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="4" t="inlineStr">
+        <is>
+          <t>Sugar Talking</t>
+        </is>
+      </c>
+      <c r="B31" s="5" t="n">
+        <v>5428</v>
+      </c>
+      <c r="C31" s="5" t="inlineStr">
+        <is>
+          <t>+2467</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="4" t="inlineStr">
+        <is>
+          <t>My Man on Willpower</t>
+        </is>
+      </c>
+      <c r="B32" s="5" t="n">
+        <v>5821</v>
+      </c>
+      <c r="C32" s="5" t="inlineStr">
+        <is>
+          <t>+3050</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="4" t="inlineStr">
+        <is>
+          <t>Midnight Rain</t>
+        </is>
+      </c>
+      <c r="B33" s="5" t="n">
+        <v>5050</v>
+      </c>
+      <c r="C33" s="5" t="inlineStr">
+        <is>
+          <t>+2591</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="4" t="inlineStr">
+        <is>
+          <t>Nobodys Son</t>
+        </is>
+      </c>
+      <c r="B34" s="5" t="n">
+        <v>7264</v>
+      </c>
+      <c r="C34" s="5" t="inlineStr">
+        <is>
+          <t>+2841</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="4" t="inlineStr">
+        <is>
+          <t>House Tour</t>
+        </is>
+      </c>
+      <c r="B35" s="5" t="n">
+        <v>5252</v>
+      </c>
+      <c r="C35" s="5" t="inlineStr">
+        <is>
+          <t>+2467</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="4" t="inlineStr">
+        <is>
+          <t>Hanabi  Î±Î·Ð²Ï…</t>
+        </is>
+      </c>
+      <c r="B36" s="5" t="n">
+        <v>3312</v>
+      </c>
+      <c r="C36" s="5" t="inlineStr">
+        <is>
+          <t>+700</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="4" t="inlineStr">
+        <is>
+          <t>Saiyajin anbuâ„¢</t>
+        </is>
+      </c>
+      <c r="B37" s="5" t="n">
+        <v>505</v>
+      </c>
+      <c r="C37" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="4" t="inlineStr">
+        <is>
+          <t>Dummy</t>
+        </is>
+      </c>
+      <c r="B38" s="5" t="n">
+        <v>2968</v>
+      </c>
+      <c r="C38" s="5" t="inlineStr">
+        <is>
+          <t>+600</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="4" t="inlineStr">
+        <is>
+          <t>Cazador anbu â„¢</t>
+        </is>
+      </c>
+      <c r="B39" s="5" t="n">
+        <v>500</v>
+      </c>
+      <c r="C39" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="4" t="inlineStr">
+        <is>
+          <t>Besos Mojados</t>
+        </is>
+      </c>
+      <c r="B40" s="5" t="n">
+        <v>2575</v>
+      </c>
+      <c r="C40" s="5" t="inlineStr">
+        <is>
+          <t>+1655</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="4" t="inlineStr">
+        <is>
+          <t>DarkFire</t>
+        </is>
+      </c>
+      <c r="B41" s="5" t="n">
+        <v>6542</v>
+      </c>
+      <c r="C41" s="5" t="inlineStr">
+        <is>
+          <t>+1500</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="4" t="inlineStr">
+        <is>
+          <t>DarkSunny</t>
+        </is>
+      </c>
+      <c r="B42" s="5" t="n">
+        <v>6737</v>
+      </c>
+      <c r="C42" s="5" t="inlineStr">
+        <is>
+          <t>+1500</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="4" t="inlineStr">
+        <is>
+          <t>Dairen Uchiha</t>
+        </is>
+      </c>
+      <c r="B43" s="5" t="n">
+        <v>7379</v>
+      </c>
+      <c r="C43" s="5" t="inlineStr">
+        <is>
+          <t>+1482</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="4" t="inlineStr">
+        <is>
+          <t>LILI ZENIN®</t>
+        </is>
+      </c>
+      <c r="B44" s="5" t="n">
+        <v>4713</v>
+      </c>
+      <c r="C44" s="5" t="inlineStr">
+        <is>
+          <t>+1167</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="4" t="inlineStr">
+        <is>
+          <t>ryumichel ZENIN ®</t>
+        </is>
+      </c>
+      <c r="B45" s="5" t="n">
+        <v>936</v>
+      </c>
+      <c r="C45" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="4" t="inlineStr">
+        <is>
+          <t>margot ZENIN ®</t>
+        </is>
+      </c>
+      <c r="B46" s="5" t="n">
+        <v>1000</v>
+      </c>
+      <c r="C46" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="4" t="inlineStr">
+        <is>
+          <t>linda ZENIN ®</t>
+        </is>
+      </c>
+      <c r="B47" s="5" t="n">
+        <v>4911</v>
+      </c>
+      <c r="C47" s="5" t="inlineStr">
+        <is>
+          <t>+1200</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="4" t="inlineStr">
+        <is>
+          <t>SHINRAIN ZENIN®</t>
+        </is>
+      </c>
+      <c r="B48" s="5" t="n">
+        <v>4746</v>
+      </c>
+      <c r="C48" s="5" t="inlineStr">
+        <is>
+          <t>+1200</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="4" t="inlineStr">
+        <is>
+          <t>PlyRed-</t>
+        </is>
+      </c>
+      <c r="B49" s="5" t="n">
+        <v>2425</v>
+      </c>
+      <c r="C49" s="5" t="inlineStr">
+        <is>
+          <t>+700</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="4" t="inlineStr">
+        <is>
+          <t>equin0x</t>
+        </is>
+      </c>
+      <c r="B50" s="5" t="n">
+        <v>4919</v>
+      </c>
+      <c r="C50" s="5" t="inlineStr">
+        <is>
+          <t>+1570</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="4" t="inlineStr">
+        <is>
+          <t>Jhayco - Mokai</t>
+        </is>
+      </c>
+      <c r="B51" s="5" t="n">
+        <v>7467</v>
+      </c>
+      <c r="C51" s="5" t="inlineStr">
+        <is>
+          <t>+1200</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="4" t="inlineStr">
+        <is>
+          <t>Jhayco - Joe</t>
+        </is>
+      </c>
+      <c r="B52" s="5" t="n">
+        <v>7570</v>
+      </c>
+      <c r="C52" s="5" t="inlineStr">
+        <is>
+          <t>+1146</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="4" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="B53" s="5" t="n">
+        <v>7495</v>
+      </c>
+      <c r="C53" s="5" t="inlineStr">
+        <is>
+          <t>+1200</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="4" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="B54" s="5" t="n">
+        <v>7726</v>
+      </c>
+      <c r="C54" s="5" t="inlineStr">
+        <is>
+          <t>+1200</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="4" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="B55" s="5" t="n">
+        <v>7465</v>
+      </c>
+      <c r="C55" s="5" t="inlineStr">
+        <is>
+          <t>+1150</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="4" t="inlineStr">
+        <is>
+          <t>Go Go Juice</t>
+        </is>
+      </c>
+      <c r="B56" s="5" t="n">
+        <v>6280</v>
+      </c>
+      <c r="C56" s="5" t="inlineStr">
+        <is>
+          <t>+1375</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="4" t="inlineStr">
+        <is>
+          <t>Jhayco - Imaginaste</t>
+        </is>
+      </c>
+      <c r="B57" s="5" t="n">
+        <v>2427</v>
+      </c>
+      <c r="C57" s="5" t="inlineStr">
+        <is>
+          <t>+1455</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="4" t="inlineStr">
+        <is>
+          <t>PuNch</t>
+        </is>
+      </c>
+      <c r="B58" s="5" t="n">
+        <v>4965</v>
+      </c>
+      <c r="C58" s="5" t="inlineStr">
+        <is>
+          <t>+500</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A2:C2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
auto: snapshot 2026-07-27 13:01:00
</commit_message>
<xml_diff>
--- a/clan_3815.xlsx
+++ b/clan_3815.xlsx
@@ -19,6 +19,7 @@
     <sheet name="2026-07-24" sheetId="10" state="visible" r:id="rId10"/>
     <sheet name="2026-07-25" sheetId="11" state="visible" r:id="rId11"/>
     <sheet name="2026-07-26" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet name="2026-07-27" sheetId="13" state="visible" r:id="rId13"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -3315,6 +3316,885 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C58"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="29" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Clan: Mans Best Friend (3815)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Timestamp: 2026-07-27 13:01:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>Total Reps</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>Daily Reps (+1d)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>Nobodys Son</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="n">
+        <v>6126</v>
+      </c>
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>-1138</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>Player</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="n">
+        <v>3214</v>
+      </c>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>+2364</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>Player</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="n">
+        <v>3190</v>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>+2340</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>X y L O T A</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="n">
+        <v>3224</v>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>+150</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>AbdiHyde ID 13496</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="n">
+        <v>4327</v>
+      </c>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>+680</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>Create Character III</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="n">
+        <v>6097</v>
+      </c>
+      <c r="C9" s="5" t="inlineStr">
+        <is>
+          <t>+680</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>Create Character IV</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="n">
+        <v>6758</v>
+      </c>
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>+700</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>Create Character V</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="n">
+        <v>6610</v>
+      </c>
+      <c r="C11" s="5" t="inlineStr">
+        <is>
+          <t>+632</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t>Player</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="n">
+        <v>3128</v>
+      </c>
+      <c r="C12" s="5" t="inlineStr">
+        <is>
+          <t>+2278</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="4" t="inlineStr">
+        <is>
+          <t>Player</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="n">
+        <v>3155</v>
+      </c>
+      <c r="C13" s="5" t="inlineStr">
+        <is>
+          <t>+2305</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="4" t="inlineStr">
+        <is>
+          <t>hunry</t>
+        </is>
+      </c>
+      <c r="B14" s="5" t="n">
+        <v>3163</v>
+      </c>
+      <c r="C14" s="5" t="inlineStr">
+        <is>
+          <t>+2340</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="4" t="inlineStr">
+        <is>
+          <t>Tears</t>
+        </is>
+      </c>
+      <c r="B15" s="5" t="n">
+        <v>6127</v>
+      </c>
+      <c r="C15" s="5" t="inlineStr">
+        <is>
+          <t>+800</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="4" t="inlineStr">
+        <is>
+          <t>Sugar Talking</t>
+        </is>
+      </c>
+      <c r="B16" s="5" t="n">
+        <v>7162</v>
+      </c>
+      <c r="C16" s="5" t="inlineStr">
+        <is>
+          <t>+1734</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="4" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B17" s="5" t="n">
+        <v>6323</v>
+      </c>
+      <c r="C17" s="5" t="inlineStr">
+        <is>
+          <t>+1300</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="4" t="inlineStr">
+        <is>
+          <t>Anti-Hero</t>
+        </is>
+      </c>
+      <c r="B18" s="5" t="n">
+        <v>7069</v>
+      </c>
+      <c r="C18" s="5" t="inlineStr">
+        <is>
+          <t>+1300</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="4" t="inlineStr">
+        <is>
+          <t>Vigilante Shit</t>
+        </is>
+      </c>
+      <c r="B19" s="5" t="n">
+        <v>7084</v>
+      </c>
+      <c r="C19" s="5" t="inlineStr">
+        <is>
+          <t>+1300</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="4" t="inlineStr">
+        <is>
+          <t>Sweet Nothing</t>
+        </is>
+      </c>
+      <c r="B20" s="5" t="n">
+        <v>7119</v>
+      </c>
+      <c r="C20" s="5" t="inlineStr">
+        <is>
+          <t>+1300</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="4" t="inlineStr">
+        <is>
+          <t>The Great War</t>
+        </is>
+      </c>
+      <c r="B21" s="5" t="n">
+        <v>6839</v>
+      </c>
+      <c r="C21" s="5" t="inlineStr">
+        <is>
+          <t>+1237</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">We Almost Broke Up </t>
+        </is>
+      </c>
+      <c r="B22" s="5" t="n">
+        <v>7493</v>
+      </c>
+      <c r="C22" s="5" t="inlineStr">
+        <is>
+          <t>+1391</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="4" t="inlineStr">
+        <is>
+          <t>When Did You Get Hot</t>
+        </is>
+      </c>
+      <c r="B23" s="5" t="n">
+        <v>7348</v>
+      </c>
+      <c r="C23" s="5" t="inlineStr">
+        <is>
+          <t>+1350</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="4" t="inlineStr">
+        <is>
+          <t>Dont Worry Ill Make</t>
+        </is>
+      </c>
+      <c r="B24" s="5" t="n">
+        <v>6804</v>
+      </c>
+      <c r="C24" s="5" t="inlineStr">
+        <is>
+          <t>+1350</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="4" t="inlineStr">
+        <is>
+          <t>Goodbye</t>
+        </is>
+      </c>
+      <c r="B25" s="5" t="n">
+        <v>5808</v>
+      </c>
+      <c r="C25" s="5" t="inlineStr">
+        <is>
+          <t>+550</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="4" t="inlineStr">
+        <is>
+          <t>Mans Best Friend</t>
+        </is>
+      </c>
+      <c r="B26" s="5" t="n">
+        <v>5728</v>
+      </c>
+      <c r="C26" s="5" t="inlineStr">
+        <is>
+          <t>+550</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="4" t="inlineStr">
+        <is>
+          <t>Lavender Haze</t>
+        </is>
+      </c>
+      <c r="B27" s="5" t="n">
+        <v>5743</v>
+      </c>
+      <c r="C27" s="5" t="inlineStr">
+        <is>
+          <t>+523</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="4" t="inlineStr">
+        <is>
+          <t>Never Getting Laid</t>
+        </is>
+      </c>
+      <c r="B28" s="5" t="n">
+        <v>7393</v>
+      </c>
+      <c r="C28" s="5" t="inlineStr">
+        <is>
+          <t>+800</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="4" t="inlineStr">
+        <is>
+          <t>My Man on Willpower</t>
+        </is>
+      </c>
+      <c r="B29" s="5" t="n">
+        <v>6607</v>
+      </c>
+      <c r="C29" s="5" t="inlineStr">
+        <is>
+          <t>+786</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="4" t="inlineStr">
+        <is>
+          <t>Manchild</t>
+        </is>
+      </c>
+      <c r="B30" s="5" t="n">
+        <v>7405</v>
+      </c>
+      <c r="C30" s="5" t="inlineStr">
+        <is>
+          <t>+755</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="4" t="inlineStr">
+        <is>
+          <t>Sugar Talking</t>
+        </is>
+      </c>
+      <c r="B31" s="5" t="n">
+        <v>6778</v>
+      </c>
+      <c r="C31" s="5" t="inlineStr">
+        <is>
+          <t>+1350</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="4" t="inlineStr">
+        <is>
+          <t>My Man on Willpower</t>
+        </is>
+      </c>
+      <c r="B32" s="5" t="n">
+        <v>7086</v>
+      </c>
+      <c r="C32" s="5" t="inlineStr">
+        <is>
+          <t>+1265</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="4" t="inlineStr">
+        <is>
+          <t>Midnight Rain</t>
+        </is>
+      </c>
+      <c r="B33" s="5" t="n">
+        <v>5500</v>
+      </c>
+      <c r="C33" s="5" t="inlineStr">
+        <is>
+          <t>+450</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="4" t="inlineStr">
+        <is>
+          <t>Nobodys Son</t>
+        </is>
+      </c>
+      <c r="B34" s="5" t="n">
+        <v>8574</v>
+      </c>
+      <c r="C34" s="5" t="inlineStr">
+        <is>
+          <t>+1310</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="4" t="inlineStr">
+        <is>
+          <t>House Tour</t>
+        </is>
+      </c>
+      <c r="B35" s="5" t="n">
+        <v>6566</v>
+      </c>
+      <c r="C35" s="5" t="inlineStr">
+        <is>
+          <t>+1314</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="4" t="inlineStr">
+        <is>
+          <t>Hanabi  Î±Î·Ð²Ï…</t>
+        </is>
+      </c>
+      <c r="B36" s="5" t="n">
+        <v>5612</v>
+      </c>
+      <c r="C36" s="5" t="inlineStr">
+        <is>
+          <t>+2300</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="4" t="inlineStr">
+        <is>
+          <t>Saiyajin anbuâ„¢</t>
+        </is>
+      </c>
+      <c r="B37" s="5" t="n">
+        <v>2787</v>
+      </c>
+      <c r="C37" s="5" t="inlineStr">
+        <is>
+          <t>+2282</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="4" t="inlineStr">
+        <is>
+          <t>Dummy</t>
+        </is>
+      </c>
+      <c r="B38" s="5" t="n">
+        <v>5205</v>
+      </c>
+      <c r="C38" s="5" t="inlineStr">
+        <is>
+          <t>+2237</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="4" t="inlineStr">
+        <is>
+          <t>Cazador anbu â„¢</t>
+        </is>
+      </c>
+      <c r="B39" s="5" t="n">
+        <v>2764</v>
+      </c>
+      <c r="C39" s="5" t="inlineStr">
+        <is>
+          <t>+2264</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="4" t="inlineStr">
+        <is>
+          <t>Besos Mojados</t>
+        </is>
+      </c>
+      <c r="B40" s="5" t="n">
+        <v>3925</v>
+      </c>
+      <c r="C40" s="5" t="inlineStr">
+        <is>
+          <t>+1350</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="4" t="inlineStr">
+        <is>
+          <t>DarkFire</t>
+        </is>
+      </c>
+      <c r="B41" s="5" t="n">
+        <v>8861</v>
+      </c>
+      <c r="C41" s="5" t="inlineStr">
+        <is>
+          <t>+2319</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="4" t="inlineStr">
+        <is>
+          <t>DarkSunny</t>
+        </is>
+      </c>
+      <c r="B42" s="5" t="n">
+        <v>9119</v>
+      </c>
+      <c r="C42" s="5" t="inlineStr">
+        <is>
+          <t>+2382</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="4" t="inlineStr">
+        <is>
+          <t>Dairen Uchiha</t>
+        </is>
+      </c>
+      <c r="B43" s="5" t="n">
+        <v>9652</v>
+      </c>
+      <c r="C43" s="5" t="inlineStr">
+        <is>
+          <t>+2273</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="4" t="inlineStr">
+        <is>
+          <t>LILI ZENIN®</t>
+        </is>
+      </c>
+      <c r="B44" s="5" t="n">
+        <v>5413</v>
+      </c>
+      <c r="C44" s="5" t="inlineStr">
+        <is>
+          <t>+700</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="4" t="inlineStr">
+        <is>
+          <t>ryumichel ZENIN ®</t>
+        </is>
+      </c>
+      <c r="B45" s="5" t="n">
+        <v>1636</v>
+      </c>
+      <c r="C45" s="5" t="inlineStr">
+        <is>
+          <t>+700</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="4" t="inlineStr">
+        <is>
+          <t>margot ZENIN ®</t>
+        </is>
+      </c>
+      <c r="B46" s="5" t="n">
+        <v>1700</v>
+      </c>
+      <c r="C46" s="5" t="inlineStr">
+        <is>
+          <t>+700</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="4" t="inlineStr">
+        <is>
+          <t>linda ZENIN ®</t>
+        </is>
+      </c>
+      <c r="B47" s="5" t="n">
+        <v>5561</v>
+      </c>
+      <c r="C47" s="5" t="inlineStr">
+        <is>
+          <t>+650</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="4" t="inlineStr">
+        <is>
+          <t>SHINRAIN ZENIN®</t>
+        </is>
+      </c>
+      <c r="B48" s="5" t="n">
+        <v>5396</v>
+      </c>
+      <c r="C48" s="5" t="inlineStr">
+        <is>
+          <t>+650</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="4" t="inlineStr">
+        <is>
+          <t>PlyRed-</t>
+        </is>
+      </c>
+      <c r="B49" s="5" t="n">
+        <v>4707</v>
+      </c>
+      <c r="C49" s="5" t="inlineStr">
+        <is>
+          <t>+2282</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="4" t="inlineStr">
+        <is>
+          <t>equin0x</t>
+        </is>
+      </c>
+      <c r="B50" s="5" t="n">
+        <v>7210</v>
+      </c>
+      <c r="C50" s="5" t="inlineStr">
+        <is>
+          <t>+2291</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="4" t="inlineStr">
+        <is>
+          <t>Jhayco - Mokai</t>
+        </is>
+      </c>
+      <c r="B51" s="5" t="n">
+        <v>8677</v>
+      </c>
+      <c r="C51" s="5" t="inlineStr">
+        <is>
+          <t>+1210</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="4" t="inlineStr">
+        <is>
+          <t>Jhayco - Joe</t>
+        </is>
+      </c>
+      <c r="B52" s="5" t="n">
+        <v>8861</v>
+      </c>
+      <c r="C52" s="5" t="inlineStr">
+        <is>
+          <t>+1291</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="4" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="B53" s="5" t="n">
+        <v>8732</v>
+      </c>
+      <c r="C53" s="5" t="inlineStr">
+        <is>
+          <t>+1237</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="4" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="B54" s="5" t="n">
+        <v>9026</v>
+      </c>
+      <c r="C54" s="5" t="inlineStr">
+        <is>
+          <t>+1300</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="4" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="B55" s="5" t="n">
+        <v>8765</v>
+      </c>
+      <c r="C55" s="5" t="inlineStr">
+        <is>
+          <t>+1300</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="4" t="inlineStr">
+        <is>
+          <t>Go Go Juice</t>
+        </is>
+      </c>
+      <c r="B56" s="5" t="n">
+        <v>7030</v>
+      </c>
+      <c r="C56" s="5" t="inlineStr">
+        <is>
+          <t>+750</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="4" t="inlineStr">
+        <is>
+          <t>Jhayco - Imaginaste</t>
+        </is>
+      </c>
+      <c r="B57" s="5" t="n">
+        <v>3777</v>
+      </c>
+      <c r="C57" s="5" t="inlineStr">
+        <is>
+          <t>+1350</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="4" t="inlineStr">
+        <is>
+          <t>PuNch</t>
+        </is>
+      </c>
+      <c r="B58" s="5" t="n">
+        <v>5365</v>
+      </c>
+      <c r="C58" s="5" t="inlineStr">
+        <is>
+          <t>+400</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A2:C2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
auto: snapshot 2026-07-27 13:31:00
</commit_message>
<xml_diff>
--- a/clan_3815.xlsx
+++ b/clan_3815.xlsx
@@ -3340,7 +3340,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Timestamp: 2026-07-27 13:01:00</t>
+          <t>Timestamp: 2026-07-27 13:31:00</t>
         </is>
       </c>
     </row>
@@ -3383,11 +3383,11 @@
         </is>
       </c>
       <c r="B5" s="5" t="n">
-        <v>3214</v>
+        <v>3239</v>
       </c>
       <c r="C5" s="5" t="inlineStr">
         <is>
-          <t>+2364</t>
+          <t>+2389</t>
         </is>
       </c>
     </row>
@@ -3398,11 +3398,11 @@
         </is>
       </c>
       <c r="B6" s="5" t="n">
-        <v>3190</v>
+        <v>3200</v>
       </c>
       <c r="C6" s="5" t="inlineStr">
         <is>
-          <t>+2340</t>
+          <t>+2350</t>
         </is>
       </c>
     </row>
@@ -3488,11 +3488,11 @@
         </is>
       </c>
       <c r="B12" s="5" t="n">
-        <v>3128</v>
+        <v>3129</v>
       </c>
       <c r="C12" s="5" t="inlineStr">
         <is>
-          <t>+2278</t>
+          <t>+2279</t>
         </is>
       </c>
     </row>
@@ -3848,11 +3848,11 @@
         </is>
       </c>
       <c r="B36" s="5" t="n">
-        <v>5612</v>
+        <v>5637</v>
       </c>
       <c r="C36" s="5" t="inlineStr">
         <is>
-          <t>+2300</t>
+          <t>+2325</t>
         </is>
       </c>
     </row>
@@ -3863,11 +3863,11 @@
         </is>
       </c>
       <c r="B37" s="5" t="n">
-        <v>2787</v>
+        <v>2812</v>
       </c>
       <c r="C37" s="5" t="inlineStr">
         <is>
-          <t>+2282</t>
+          <t>+2307</t>
         </is>
       </c>
     </row>
@@ -3878,11 +3878,11 @@
         </is>
       </c>
       <c r="B38" s="5" t="n">
-        <v>5205</v>
+        <v>5230</v>
       </c>
       <c r="C38" s="5" t="inlineStr">
         <is>
-          <t>+2237</t>
+          <t>+2262</t>
         </is>
       </c>
     </row>
@@ -3893,11 +3893,11 @@
         </is>
       </c>
       <c r="B39" s="5" t="n">
-        <v>2764</v>
+        <v>2786</v>
       </c>
       <c r="C39" s="5" t="inlineStr">
         <is>
-          <t>+2264</t>
+          <t>+2286</t>
         </is>
       </c>
     </row>
@@ -3923,11 +3923,11 @@
         </is>
       </c>
       <c r="B41" s="5" t="n">
-        <v>8861</v>
+        <v>8886</v>
       </c>
       <c r="C41" s="5" t="inlineStr">
         <is>
-          <t>+2319</t>
+          <t>+2344</t>
         </is>
       </c>
     </row>
@@ -3938,11 +3938,11 @@
         </is>
       </c>
       <c r="B42" s="5" t="n">
-        <v>9119</v>
+        <v>9144</v>
       </c>
       <c r="C42" s="5" t="inlineStr">
         <is>
-          <t>+2382</t>
+          <t>+2407</t>
         </is>
       </c>
     </row>
@@ -3953,11 +3953,11 @@
         </is>
       </c>
       <c r="B43" s="5" t="n">
-        <v>9652</v>
+        <v>9677</v>
       </c>
       <c r="C43" s="5" t="inlineStr">
         <is>
-          <t>+2273</t>
+          <t>+2298</t>
         </is>
       </c>
     </row>
@@ -4043,11 +4043,11 @@
         </is>
       </c>
       <c r="B49" s="5" t="n">
-        <v>4707</v>
+        <v>4732</v>
       </c>
       <c r="C49" s="5" t="inlineStr">
         <is>
-          <t>+2282</t>
+          <t>+2307</t>
         </is>
       </c>
     </row>
@@ -4058,11 +4058,11 @@
         </is>
       </c>
       <c r="B50" s="5" t="n">
-        <v>7210</v>
+        <v>7235</v>
       </c>
       <c r="C50" s="5" t="inlineStr">
         <is>
-          <t>+2291</t>
+          <t>+2316</t>
         </is>
       </c>
     </row>
@@ -4073,11 +4073,11 @@
         </is>
       </c>
       <c r="B51" s="5" t="n">
-        <v>8677</v>
+        <v>8702</v>
       </c>
       <c r="C51" s="5" t="inlineStr">
         <is>
-          <t>+1210</t>
+          <t>+1235</t>
         </is>
       </c>
     </row>
@@ -4088,11 +4088,11 @@
         </is>
       </c>
       <c r="B52" s="5" t="n">
-        <v>8861</v>
+        <v>8886</v>
       </c>
       <c r="C52" s="5" t="inlineStr">
         <is>
-          <t>+1291</t>
+          <t>+1316</t>
         </is>
       </c>
     </row>
@@ -4103,11 +4103,11 @@
         </is>
       </c>
       <c r="B53" s="5" t="n">
-        <v>8732</v>
+        <v>8757</v>
       </c>
       <c r="C53" s="5" t="inlineStr">
         <is>
-          <t>+1237</t>
+          <t>+1262</t>
         </is>
       </c>
     </row>
@@ -4118,11 +4118,11 @@
         </is>
       </c>
       <c r="B54" s="5" t="n">
-        <v>9026</v>
+        <v>9051</v>
       </c>
       <c r="C54" s="5" t="inlineStr">
         <is>
-          <t>+1300</t>
+          <t>+1325</t>
         </is>
       </c>
     </row>
@@ -4133,11 +4133,11 @@
         </is>
       </c>
       <c r="B55" s="5" t="n">
-        <v>8765</v>
+        <v>8790</v>
       </c>
       <c r="C55" s="5" t="inlineStr">
         <is>
-          <t>+1300</t>
+          <t>+1325</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: snapshot 2026-07-28 13:01:00
</commit_message>
<xml_diff>
--- a/clan_3815.xlsx
+++ b/clan_3815.xlsx
@@ -20,6 +20,7 @@
     <sheet name="2026-07-25" sheetId="11" state="visible" r:id="rId11"/>
     <sheet name="2026-07-26" sheetId="12" state="visible" r:id="rId12"/>
     <sheet name="2026-07-27" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet name="2026-07-28" sheetId="14" state="visible" r:id="rId14"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -4195,6 +4196,885 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C58"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="29" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Clan: Mans Best Friend (3815)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Timestamp: 2026-07-28 13:01:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>Total Reps</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>Daily Reps (+1d)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>Nobodys Son</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="n">
+        <v>6126</v>
+      </c>
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>-2448</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>Player</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="n">
+        <v>3414</v>
+      </c>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>+259</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>Player</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="n">
+        <v>3350</v>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>+195</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>X y L O T A</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="n">
+        <v>3224</v>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>AbdiHyde ID 13496</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="n">
+        <v>4327</v>
+      </c>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>Create Character III</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="n">
+        <v>6097</v>
+      </c>
+      <c r="C9" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>Create Character IV</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="n">
+        <v>6758</v>
+      </c>
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>Create Character V</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="n">
+        <v>6610</v>
+      </c>
+      <c r="C11" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t>Player</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="n">
+        <v>3324</v>
+      </c>
+      <c r="C12" s="5" t="inlineStr">
+        <is>
+          <t>+169</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="4" t="inlineStr">
+        <is>
+          <t>Player</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="n">
+        <v>3355</v>
+      </c>
+      <c r="C13" s="5" t="inlineStr">
+        <is>
+          <t>+200</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="4" t="inlineStr">
+        <is>
+          <t>hunry</t>
+        </is>
+      </c>
+      <c r="B14" s="5" t="n">
+        <v>3363</v>
+      </c>
+      <c r="C14" s="5" t="inlineStr">
+        <is>
+          <t>+200</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="4" t="inlineStr">
+        <is>
+          <t>Tears</t>
+        </is>
+      </c>
+      <c r="B15" s="5" t="n">
+        <v>6127</v>
+      </c>
+      <c r="C15" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="4" t="inlineStr">
+        <is>
+          <t>Sugar Talking</t>
+        </is>
+      </c>
+      <c r="B16" s="5" t="n">
+        <v>7162</v>
+      </c>
+      <c r="C16" s="5" t="inlineStr">
+        <is>
+          <t>+384</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="4" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B17" s="5" t="n">
+        <v>6323</v>
+      </c>
+      <c r="C17" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="4" t="inlineStr">
+        <is>
+          <t>Anti-Hero</t>
+        </is>
+      </c>
+      <c r="B18" s="5" t="n">
+        <v>7069</v>
+      </c>
+      <c r="C18" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="4" t="inlineStr">
+        <is>
+          <t>Vigilante Shit</t>
+        </is>
+      </c>
+      <c r="B19" s="5" t="n">
+        <v>7084</v>
+      </c>
+      <c r="C19" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="4" t="inlineStr">
+        <is>
+          <t>Sweet Nothing</t>
+        </is>
+      </c>
+      <c r="B20" s="5" t="n">
+        <v>7119</v>
+      </c>
+      <c r="C20" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="4" t="inlineStr">
+        <is>
+          <t>The Great War</t>
+        </is>
+      </c>
+      <c r="B21" s="5" t="n">
+        <v>6839</v>
+      </c>
+      <c r="C21" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">We Almost Broke Up </t>
+        </is>
+      </c>
+      <c r="B22" s="5" t="n">
+        <v>7493</v>
+      </c>
+      <c r="C22" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="4" t="inlineStr">
+        <is>
+          <t>When Did You Get Hot</t>
+        </is>
+      </c>
+      <c r="B23" s="5" t="n">
+        <v>7348</v>
+      </c>
+      <c r="C23" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="4" t="inlineStr">
+        <is>
+          <t>Dont Worry Ill Make</t>
+        </is>
+      </c>
+      <c r="B24" s="5" t="n">
+        <v>6804</v>
+      </c>
+      <c r="C24" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="4" t="inlineStr">
+        <is>
+          <t>Goodbye</t>
+        </is>
+      </c>
+      <c r="B25" s="5" t="n">
+        <v>5808</v>
+      </c>
+      <c r="C25" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="4" t="inlineStr">
+        <is>
+          <t>Mans Best Friend</t>
+        </is>
+      </c>
+      <c r="B26" s="5" t="n">
+        <v>5728</v>
+      </c>
+      <c r="C26" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="4" t="inlineStr">
+        <is>
+          <t>Lavender Haze</t>
+        </is>
+      </c>
+      <c r="B27" s="5" t="n">
+        <v>5743</v>
+      </c>
+      <c r="C27" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="4" t="inlineStr">
+        <is>
+          <t>Never Getting Laid</t>
+        </is>
+      </c>
+      <c r="B28" s="5" t="n">
+        <v>7393</v>
+      </c>
+      <c r="C28" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="4" t="inlineStr">
+        <is>
+          <t>My Man on Willpower</t>
+        </is>
+      </c>
+      <c r="B29" s="5" t="n">
+        <v>6607</v>
+      </c>
+      <c r="C29" s="5" t="inlineStr">
+        <is>
+          <t>-479</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="4" t="inlineStr">
+        <is>
+          <t>Manchild</t>
+        </is>
+      </c>
+      <c r="B30" s="5" t="n">
+        <v>7405</v>
+      </c>
+      <c r="C30" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="4" t="inlineStr">
+        <is>
+          <t>Sugar Talking</t>
+        </is>
+      </c>
+      <c r="B31" s="5" t="n">
+        <v>6778</v>
+      </c>
+      <c r="C31" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="4" t="inlineStr">
+        <is>
+          <t>My Man on Willpower</t>
+        </is>
+      </c>
+      <c r="B32" s="5" t="n">
+        <v>7086</v>
+      </c>
+      <c r="C32" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="4" t="inlineStr">
+        <is>
+          <t>Midnight Rain</t>
+        </is>
+      </c>
+      <c r="B33" s="5" t="n">
+        <v>5500</v>
+      </c>
+      <c r="C33" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="4" t="inlineStr">
+        <is>
+          <t>Nobodys Son</t>
+        </is>
+      </c>
+      <c r="B34" s="5" t="n">
+        <v>8574</v>
+      </c>
+      <c r="C34" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="4" t="inlineStr">
+        <is>
+          <t>House Tour</t>
+        </is>
+      </c>
+      <c r="B35" s="5" t="n">
+        <v>6566</v>
+      </c>
+      <c r="C35" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="4" t="inlineStr">
+        <is>
+          <t>Hanabi  Î±Î·Ð²Ï…</t>
+        </is>
+      </c>
+      <c r="B36" s="5" t="n">
+        <v>5912</v>
+      </c>
+      <c r="C36" s="5" t="inlineStr">
+        <is>
+          <t>+275</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="4" t="inlineStr">
+        <is>
+          <t>Saiyajin anbuâ„¢</t>
+        </is>
+      </c>
+      <c r="B37" s="5" t="n">
+        <v>3063</v>
+      </c>
+      <c r="C37" s="5" t="inlineStr">
+        <is>
+          <t>+251</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="4" t="inlineStr">
+        <is>
+          <t>Dummy</t>
+        </is>
+      </c>
+      <c r="B38" s="5" t="n">
+        <v>5485</v>
+      </c>
+      <c r="C38" s="5" t="inlineStr">
+        <is>
+          <t>+255</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="4" t="inlineStr">
+        <is>
+          <t>Cazador anbu â„¢</t>
+        </is>
+      </c>
+      <c r="B39" s="5" t="n">
+        <v>3036</v>
+      </c>
+      <c r="C39" s="5" t="inlineStr">
+        <is>
+          <t>+250</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="4" t="inlineStr">
+        <is>
+          <t>Besos Mojados</t>
+        </is>
+      </c>
+      <c r="B40" s="5" t="n">
+        <v>3925</v>
+      </c>
+      <c r="C40" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="4" t="inlineStr">
+        <is>
+          <t>DarkFire</t>
+        </is>
+      </c>
+      <c r="B41" s="5" t="n">
+        <v>9111</v>
+      </c>
+      <c r="C41" s="5" t="inlineStr">
+        <is>
+          <t>+225</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="4" t="inlineStr">
+        <is>
+          <t>DarkSunny</t>
+        </is>
+      </c>
+      <c r="B42" s="5" t="n">
+        <v>9369</v>
+      </c>
+      <c r="C42" s="5" t="inlineStr">
+        <is>
+          <t>+225</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="4" t="inlineStr">
+        <is>
+          <t>Dairen Uchiha</t>
+        </is>
+      </c>
+      <c r="B43" s="5" t="n">
+        <v>9902</v>
+      </c>
+      <c r="C43" s="5" t="inlineStr">
+        <is>
+          <t>+225</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="4" t="inlineStr">
+        <is>
+          <t>LILI ZENIN®</t>
+        </is>
+      </c>
+      <c r="B44" s="5" t="n">
+        <v>5413</v>
+      </c>
+      <c r="C44" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="4" t="inlineStr">
+        <is>
+          <t>ryumichel ZENIN ®</t>
+        </is>
+      </c>
+      <c r="B45" s="5" t="n">
+        <v>1636</v>
+      </c>
+      <c r="C45" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="4" t="inlineStr">
+        <is>
+          <t>margot ZENIN ®</t>
+        </is>
+      </c>
+      <c r="B46" s="5" t="n">
+        <v>1700</v>
+      </c>
+      <c r="C46" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="4" t="inlineStr">
+        <is>
+          <t>linda ZENIN ®</t>
+        </is>
+      </c>
+      <c r="B47" s="5" t="n">
+        <v>5561</v>
+      </c>
+      <c r="C47" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="4" t="inlineStr">
+        <is>
+          <t>SHINRAIN ZENIN®</t>
+        </is>
+      </c>
+      <c r="B48" s="5" t="n">
+        <v>5396</v>
+      </c>
+      <c r="C48" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="4" t="inlineStr">
+        <is>
+          <t>PlyRed-</t>
+        </is>
+      </c>
+      <c r="B49" s="5" t="n">
+        <v>5007</v>
+      </c>
+      <c r="C49" s="5" t="inlineStr">
+        <is>
+          <t>+275</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="4" t="inlineStr">
+        <is>
+          <t>equin0x</t>
+        </is>
+      </c>
+      <c r="B50" s="5" t="n">
+        <v>7510</v>
+      </c>
+      <c r="C50" s="5" t="inlineStr">
+        <is>
+          <t>+275</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="4" t="inlineStr">
+        <is>
+          <t>Jhayco - Mokai</t>
+        </is>
+      </c>
+      <c r="B51" s="5" t="n">
+        <v>8965</v>
+      </c>
+      <c r="C51" s="5" t="inlineStr">
+        <is>
+          <t>+263</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="4" t="inlineStr">
+        <is>
+          <t>Jhayco - Joe</t>
+        </is>
+      </c>
+      <c r="B52" s="5" t="n">
+        <v>9161</v>
+      </c>
+      <c r="C52" s="5" t="inlineStr">
+        <is>
+          <t>+275</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="4" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="B53" s="5" t="n">
+        <v>9032</v>
+      </c>
+      <c r="C53" s="5" t="inlineStr">
+        <is>
+          <t>+275</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="4" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="B54" s="5" t="n">
+        <v>9326</v>
+      </c>
+      <c r="C54" s="5" t="inlineStr">
+        <is>
+          <t>+275</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="4" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="B55" s="5" t="n">
+        <v>9065</v>
+      </c>
+      <c r="C55" s="5" t="inlineStr">
+        <is>
+          <t>+275</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="4" t="inlineStr">
+        <is>
+          <t>Go Go Juice</t>
+        </is>
+      </c>
+      <c r="B56" s="5" t="n">
+        <v>7030</v>
+      </c>
+      <c r="C56" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="4" t="inlineStr">
+        <is>
+          <t>Jhayco - Imaginaste</t>
+        </is>
+      </c>
+      <c r="B57" s="5" t="n">
+        <v>3777</v>
+      </c>
+      <c r="C57" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="4" t="inlineStr">
+        <is>
+          <t>PuNch</t>
+        </is>
+      </c>
+      <c r="B58" s="5" t="n">
+        <v>5365</v>
+      </c>
+      <c r="C58" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A2:C2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
auto: snapshot 2026-07-29 13:01:00
</commit_message>
<xml_diff>
--- a/clan_3815.xlsx
+++ b/clan_3815.xlsx
@@ -21,6 +21,7 @@
     <sheet name="2026-07-26" sheetId="12" state="visible" r:id="rId12"/>
     <sheet name="2026-07-27" sheetId="13" state="visible" r:id="rId13"/>
     <sheet name="2026-07-28" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet name="2026-07-29" sheetId="15" state="visible" r:id="rId15"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -5075,6 +5076,885 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C58"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="29" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Clan: Mans Best Friend (3815)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Timestamp: 2026-07-29 13:01:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>Total Reps</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>Daily Reps (+1d)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>Nobodys Son</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="n">
+        <v>6126</v>
+      </c>
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>-2448</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>Player</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="n">
+        <v>3414</v>
+      </c>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>+59</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>Player</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="n">
+        <v>3350</v>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>-5</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>X y L O T A</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="n">
+        <v>3224</v>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>AbdiHyde ID 13496</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="n">
+        <v>4327</v>
+      </c>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>Create Character III</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="n">
+        <v>6097</v>
+      </c>
+      <c r="C9" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>Create Character IV</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="n">
+        <v>6758</v>
+      </c>
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>Create Character V</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="n">
+        <v>6610</v>
+      </c>
+      <c r="C11" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t>Player</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="n">
+        <v>3324</v>
+      </c>
+      <c r="C12" s="5" t="inlineStr">
+        <is>
+          <t>-31</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="4" t="inlineStr">
+        <is>
+          <t>Player</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="n">
+        <v>3355</v>
+      </c>
+      <c r="C13" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="4" t="inlineStr">
+        <is>
+          <t>hunry</t>
+        </is>
+      </c>
+      <c r="B14" s="5" t="n">
+        <v>3363</v>
+      </c>
+      <c r="C14" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="4" t="inlineStr">
+        <is>
+          <t>Tears</t>
+        </is>
+      </c>
+      <c r="B15" s="5" t="n">
+        <v>6127</v>
+      </c>
+      <c r="C15" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="4" t="inlineStr">
+        <is>
+          <t>Sugar Talking</t>
+        </is>
+      </c>
+      <c r="B16" s="5" t="n">
+        <v>7162</v>
+      </c>
+      <c r="C16" s="5" t="inlineStr">
+        <is>
+          <t>+384</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="4" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B17" s="5" t="n">
+        <v>6323</v>
+      </c>
+      <c r="C17" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="4" t="inlineStr">
+        <is>
+          <t>Anti-Hero</t>
+        </is>
+      </c>
+      <c r="B18" s="5" t="n">
+        <v>7069</v>
+      </c>
+      <c r="C18" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="4" t="inlineStr">
+        <is>
+          <t>Vigilante Shit</t>
+        </is>
+      </c>
+      <c r="B19" s="5" t="n">
+        <v>7084</v>
+      </c>
+      <c r="C19" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="4" t="inlineStr">
+        <is>
+          <t>Sweet Nothing</t>
+        </is>
+      </c>
+      <c r="B20" s="5" t="n">
+        <v>7119</v>
+      </c>
+      <c r="C20" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="4" t="inlineStr">
+        <is>
+          <t>The Great War</t>
+        </is>
+      </c>
+      <c r="B21" s="5" t="n">
+        <v>6839</v>
+      </c>
+      <c r="C21" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">We Almost Broke Up </t>
+        </is>
+      </c>
+      <c r="B22" s="5" t="n">
+        <v>7493</v>
+      </c>
+      <c r="C22" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="4" t="inlineStr">
+        <is>
+          <t>When Did You Get Hot</t>
+        </is>
+      </c>
+      <c r="B23" s="5" t="n">
+        <v>7348</v>
+      </c>
+      <c r="C23" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="4" t="inlineStr">
+        <is>
+          <t>Dont Worry Ill Make</t>
+        </is>
+      </c>
+      <c r="B24" s="5" t="n">
+        <v>6804</v>
+      </c>
+      <c r="C24" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="4" t="inlineStr">
+        <is>
+          <t>Goodbye</t>
+        </is>
+      </c>
+      <c r="B25" s="5" t="n">
+        <v>5808</v>
+      </c>
+      <c r="C25" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="4" t="inlineStr">
+        <is>
+          <t>Mans Best Friend</t>
+        </is>
+      </c>
+      <c r="B26" s="5" t="n">
+        <v>5728</v>
+      </c>
+      <c r="C26" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="4" t="inlineStr">
+        <is>
+          <t>Lavender Haze</t>
+        </is>
+      </c>
+      <c r="B27" s="5" t="n">
+        <v>5743</v>
+      </c>
+      <c r="C27" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="4" t="inlineStr">
+        <is>
+          <t>Never Getting Laid</t>
+        </is>
+      </c>
+      <c r="B28" s="5" t="n">
+        <v>7393</v>
+      </c>
+      <c r="C28" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="4" t="inlineStr">
+        <is>
+          <t>My Man on Willpower</t>
+        </is>
+      </c>
+      <c r="B29" s="5" t="n">
+        <v>6607</v>
+      </c>
+      <c r="C29" s="5" t="inlineStr">
+        <is>
+          <t>-479</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="4" t="inlineStr">
+        <is>
+          <t>Manchild</t>
+        </is>
+      </c>
+      <c r="B30" s="5" t="n">
+        <v>7405</v>
+      </c>
+      <c r="C30" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="4" t="inlineStr">
+        <is>
+          <t>Sugar Talking</t>
+        </is>
+      </c>
+      <c r="B31" s="5" t="n">
+        <v>6778</v>
+      </c>
+      <c r="C31" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="4" t="inlineStr">
+        <is>
+          <t>My Man on Willpower</t>
+        </is>
+      </c>
+      <c r="B32" s="5" t="n">
+        <v>7086</v>
+      </c>
+      <c r="C32" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="4" t="inlineStr">
+        <is>
+          <t>Midnight Rain</t>
+        </is>
+      </c>
+      <c r="B33" s="5" t="n">
+        <v>5500</v>
+      </c>
+      <c r="C33" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="4" t="inlineStr">
+        <is>
+          <t>Nobodys Son</t>
+        </is>
+      </c>
+      <c r="B34" s="5" t="n">
+        <v>8574</v>
+      </c>
+      <c r="C34" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="4" t="inlineStr">
+        <is>
+          <t>House Tour</t>
+        </is>
+      </c>
+      <c r="B35" s="5" t="n">
+        <v>6566</v>
+      </c>
+      <c r="C35" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="4" t="inlineStr">
+        <is>
+          <t>Hanabi  Î±Î·Ð²Ï…</t>
+        </is>
+      </c>
+      <c r="B36" s="5" t="n">
+        <v>5912</v>
+      </c>
+      <c r="C36" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="4" t="inlineStr">
+        <is>
+          <t>Saiyajin anbuâ„¢</t>
+        </is>
+      </c>
+      <c r="B37" s="5" t="n">
+        <v>3063</v>
+      </c>
+      <c r="C37" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="4" t="inlineStr">
+        <is>
+          <t>Dummy</t>
+        </is>
+      </c>
+      <c r="B38" s="5" t="n">
+        <v>5485</v>
+      </c>
+      <c r="C38" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="4" t="inlineStr">
+        <is>
+          <t>Cazador anbu â„¢</t>
+        </is>
+      </c>
+      <c r="B39" s="5" t="n">
+        <v>3036</v>
+      </c>
+      <c r="C39" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="4" t="inlineStr">
+        <is>
+          <t>Besos Mojados</t>
+        </is>
+      </c>
+      <c r="B40" s="5" t="n">
+        <v>3925</v>
+      </c>
+      <c r="C40" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="4" t="inlineStr">
+        <is>
+          <t>DarkFire</t>
+        </is>
+      </c>
+      <c r="B41" s="5" t="n">
+        <v>9111</v>
+      </c>
+      <c r="C41" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="4" t="inlineStr">
+        <is>
+          <t>DarkSunny</t>
+        </is>
+      </c>
+      <c r="B42" s="5" t="n">
+        <v>9369</v>
+      </c>
+      <c r="C42" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="4" t="inlineStr">
+        <is>
+          <t>Dairen Uchiha</t>
+        </is>
+      </c>
+      <c r="B43" s="5" t="n">
+        <v>9902</v>
+      </c>
+      <c r="C43" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="4" t="inlineStr">
+        <is>
+          <t>LILI ZENIN®</t>
+        </is>
+      </c>
+      <c r="B44" s="5" t="n">
+        <v>5413</v>
+      </c>
+      <c r="C44" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="4" t="inlineStr">
+        <is>
+          <t>ryumichel ZENIN ®</t>
+        </is>
+      </c>
+      <c r="B45" s="5" t="n">
+        <v>1636</v>
+      </c>
+      <c r="C45" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="4" t="inlineStr">
+        <is>
+          <t>margot ZENIN ®</t>
+        </is>
+      </c>
+      <c r="B46" s="5" t="n">
+        <v>1700</v>
+      </c>
+      <c r="C46" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="4" t="inlineStr">
+        <is>
+          <t>linda ZENIN ®</t>
+        </is>
+      </c>
+      <c r="B47" s="5" t="n">
+        <v>5561</v>
+      </c>
+      <c r="C47" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="4" t="inlineStr">
+        <is>
+          <t>SHINRAIN ZENIN®</t>
+        </is>
+      </c>
+      <c r="B48" s="5" t="n">
+        <v>5396</v>
+      </c>
+      <c r="C48" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="4" t="inlineStr">
+        <is>
+          <t>PlyRed-</t>
+        </is>
+      </c>
+      <c r="B49" s="5" t="n">
+        <v>5007</v>
+      </c>
+      <c r="C49" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="4" t="inlineStr">
+        <is>
+          <t>equin0x</t>
+        </is>
+      </c>
+      <c r="B50" s="5" t="n">
+        <v>7510</v>
+      </c>
+      <c r="C50" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="4" t="inlineStr">
+        <is>
+          <t>Jhayco - Mokai</t>
+        </is>
+      </c>
+      <c r="B51" s="5" t="n">
+        <v>8965</v>
+      </c>
+      <c r="C51" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="4" t="inlineStr">
+        <is>
+          <t>Jhayco - Joe</t>
+        </is>
+      </c>
+      <c r="B52" s="5" t="n">
+        <v>9161</v>
+      </c>
+      <c r="C52" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="4" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="B53" s="5" t="n">
+        <v>9032</v>
+      </c>
+      <c r="C53" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="4" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="B54" s="5" t="n">
+        <v>9326</v>
+      </c>
+      <c r="C54" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="4" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="B55" s="5" t="n">
+        <v>9065</v>
+      </c>
+      <c r="C55" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="4" t="inlineStr">
+        <is>
+          <t>Go Go Juice</t>
+        </is>
+      </c>
+      <c r="B56" s="5" t="n">
+        <v>7030</v>
+      </c>
+      <c r="C56" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="4" t="inlineStr">
+        <is>
+          <t>Jhayco - Imaginaste</t>
+        </is>
+      </c>
+      <c r="B57" s="5" t="n">
+        <v>3777</v>
+      </c>
+      <c r="C57" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="4" t="inlineStr">
+        <is>
+          <t>PuNch</t>
+        </is>
+      </c>
+      <c r="B58" s="5" t="n">
+        <v>5365</v>
+      </c>
+      <c r="C58" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A2:C2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
auto: snapshot 2026-07-30 13:01:00
</commit_message>
<xml_diff>
--- a/clan_3815.xlsx
+++ b/clan_3815.xlsx
@@ -22,6 +22,7 @@
     <sheet name="2026-07-27" sheetId="13" state="visible" r:id="rId13"/>
     <sheet name="2026-07-28" sheetId="14" state="visible" r:id="rId14"/>
     <sheet name="2026-07-29" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet name="2026-07-30" sheetId="16" state="visible" r:id="rId16"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -5955,6 +5956,885 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C58"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="29" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Clan: Mans Best Friend (3815)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Timestamp: 2026-07-30 13:01:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>Total Reps</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>Daily Reps (+1d)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>Nobodys Son</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="n">
+        <v>7122</v>
+      </c>
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>-1452</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>Player</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="n">
+        <v>3964</v>
+      </c>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>+609</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>Player</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="n">
+        <v>3900</v>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>+545</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>X y L O T A</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="n">
+        <v>3748</v>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>+524</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>AbdiHyde ID 13496</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="n">
+        <v>5027</v>
+      </c>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>+700</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>Create Character III</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="n">
+        <v>6647</v>
+      </c>
+      <c r="C9" s="5" t="inlineStr">
+        <is>
+          <t>+550</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>Create Character IV</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="n">
+        <v>7308</v>
+      </c>
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>+550</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>Create Character V</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="n">
+        <v>7160</v>
+      </c>
+      <c r="C11" s="5" t="inlineStr">
+        <is>
+          <t>+550</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t>Player</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="n">
+        <v>3874</v>
+      </c>
+      <c r="C12" s="5" t="inlineStr">
+        <is>
+          <t>+519</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="4" t="inlineStr">
+        <is>
+          <t>Player</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="n">
+        <v>3815</v>
+      </c>
+      <c r="C13" s="5" t="inlineStr">
+        <is>
+          <t>+460</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="4" t="inlineStr">
+        <is>
+          <t>hunry</t>
+        </is>
+      </c>
+      <c r="B14" s="5" t="n">
+        <v>3904</v>
+      </c>
+      <c r="C14" s="5" t="inlineStr">
+        <is>
+          <t>+541</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="4" t="inlineStr">
+        <is>
+          <t>Tears</t>
+        </is>
+      </c>
+      <c r="B15" s="5" t="n">
+        <v>6927</v>
+      </c>
+      <c r="C15" s="5" t="inlineStr">
+        <is>
+          <t>+800</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="4" t="inlineStr">
+        <is>
+          <t>Sugar Talking</t>
+        </is>
+      </c>
+      <c r="B16" s="5" t="n">
+        <v>8162</v>
+      </c>
+      <c r="C16" s="5" t="inlineStr">
+        <is>
+          <t>+1384</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="4" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B17" s="5" t="n">
+        <v>7273</v>
+      </c>
+      <c r="C17" s="5" t="inlineStr">
+        <is>
+          <t>+950</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="4" t="inlineStr">
+        <is>
+          <t>Anti-Hero</t>
+        </is>
+      </c>
+      <c r="B18" s="5" t="n">
+        <v>8024</v>
+      </c>
+      <c r="C18" s="5" t="inlineStr">
+        <is>
+          <t>+955</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="4" t="inlineStr">
+        <is>
+          <t>Vigilante Shit</t>
+        </is>
+      </c>
+      <c r="B19" s="5" t="n">
+        <v>8039</v>
+      </c>
+      <c r="C19" s="5" t="inlineStr">
+        <is>
+          <t>+955</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="4" t="inlineStr">
+        <is>
+          <t>Sweet Nothing</t>
+        </is>
+      </c>
+      <c r="B20" s="5" t="n">
+        <v>8119</v>
+      </c>
+      <c r="C20" s="5" t="inlineStr">
+        <is>
+          <t>+1000</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="4" t="inlineStr">
+        <is>
+          <t>The Great War</t>
+        </is>
+      </c>
+      <c r="B21" s="5" t="n">
+        <v>7839</v>
+      </c>
+      <c r="C21" s="5" t="inlineStr">
+        <is>
+          <t>+1000</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">We Almost Broke Up </t>
+        </is>
+      </c>
+      <c r="B22" s="5" t="n">
+        <v>8043</v>
+      </c>
+      <c r="C22" s="5" t="inlineStr">
+        <is>
+          <t>+550</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="4" t="inlineStr">
+        <is>
+          <t>When Did You Get Hot</t>
+        </is>
+      </c>
+      <c r="B23" s="5" t="n">
+        <v>7912</v>
+      </c>
+      <c r="C23" s="5" t="inlineStr">
+        <is>
+          <t>+564</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="4" t="inlineStr">
+        <is>
+          <t>Dont Worry Ill Make</t>
+        </is>
+      </c>
+      <c r="B24" s="5" t="n">
+        <v>7254</v>
+      </c>
+      <c r="C24" s="5" t="inlineStr">
+        <is>
+          <t>+450</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="4" t="inlineStr">
+        <is>
+          <t>Goodbye</t>
+        </is>
+      </c>
+      <c r="B25" s="5" t="n">
+        <v>6685</v>
+      </c>
+      <c r="C25" s="5" t="inlineStr">
+        <is>
+          <t>+877</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="4" t="inlineStr">
+        <is>
+          <t>Mans Best Friend</t>
+        </is>
+      </c>
+      <c r="B26" s="5" t="n">
+        <v>6624</v>
+      </c>
+      <c r="C26" s="5" t="inlineStr">
+        <is>
+          <t>+896</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="4" t="inlineStr">
+        <is>
+          <t>Lavender Haze</t>
+        </is>
+      </c>
+      <c r="B27" s="5" t="n">
+        <v>6693</v>
+      </c>
+      <c r="C27" s="5" t="inlineStr">
+        <is>
+          <t>+950</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="4" t="inlineStr">
+        <is>
+          <t>Never Getting Laid</t>
+        </is>
+      </c>
+      <c r="B28" s="5" t="n">
+        <v>8193</v>
+      </c>
+      <c r="C28" s="5" t="inlineStr">
+        <is>
+          <t>+800</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="4" t="inlineStr">
+        <is>
+          <t>My Man on Willpower</t>
+        </is>
+      </c>
+      <c r="B29" s="5" t="n">
+        <v>7230</v>
+      </c>
+      <c r="C29" s="5" t="inlineStr">
+        <is>
+          <t>+144</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="4" t="inlineStr">
+        <is>
+          <t>Manchild</t>
+        </is>
+      </c>
+      <c r="B30" s="5" t="n">
+        <v>8055</v>
+      </c>
+      <c r="C30" s="5" t="inlineStr">
+        <is>
+          <t>+650</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="4" t="inlineStr">
+        <is>
+          <t>Sugar Talking</t>
+        </is>
+      </c>
+      <c r="B31" s="5" t="n">
+        <v>7228</v>
+      </c>
+      <c r="C31" s="5" t="inlineStr">
+        <is>
+          <t>+450</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="4" t="inlineStr">
+        <is>
+          <t>My Man on Willpower</t>
+        </is>
+      </c>
+      <c r="B32" s="5" t="n">
+        <v>7901</v>
+      </c>
+      <c r="C32" s="5" t="inlineStr">
+        <is>
+          <t>+815</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="4" t="inlineStr">
+        <is>
+          <t>Midnight Rain</t>
+        </is>
+      </c>
+      <c r="B33" s="5" t="n">
+        <v>6450</v>
+      </c>
+      <c r="C33" s="5" t="inlineStr">
+        <is>
+          <t>+950</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="4" t="inlineStr">
+        <is>
+          <t>Nobodys Son</t>
+        </is>
+      </c>
+      <c r="B34" s="5" t="n">
+        <v>9524</v>
+      </c>
+      <c r="C34" s="5" t="inlineStr">
+        <is>
+          <t>+950</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="4" t="inlineStr">
+        <is>
+          <t>House Tour</t>
+        </is>
+      </c>
+      <c r="B35" s="5" t="n">
+        <v>6916</v>
+      </c>
+      <c r="C35" s="5" t="inlineStr">
+        <is>
+          <t>+350</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="4" t="inlineStr">
+        <is>
+          <t>Hanabi  Î±Î·Ð²Ï…</t>
+        </is>
+      </c>
+      <c r="B36" s="5" t="n">
+        <v>6912</v>
+      </c>
+      <c r="C36" s="5" t="inlineStr">
+        <is>
+          <t>+1000</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="4" t="inlineStr">
+        <is>
+          <t>Saiyajin anbuâ„¢</t>
+        </is>
+      </c>
+      <c r="B37" s="5" t="n">
+        <v>4063</v>
+      </c>
+      <c r="C37" s="5" t="inlineStr">
+        <is>
+          <t>+1000</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="4" t="inlineStr">
+        <is>
+          <t>Dummy</t>
+        </is>
+      </c>
+      <c r="B38" s="5" t="n">
+        <v>6422</v>
+      </c>
+      <c r="C38" s="5" t="inlineStr">
+        <is>
+          <t>+937</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="4" t="inlineStr">
+        <is>
+          <t>Cazador anbu â„¢</t>
+        </is>
+      </c>
+      <c r="B39" s="5" t="n">
+        <v>3986</v>
+      </c>
+      <c r="C39" s="5" t="inlineStr">
+        <is>
+          <t>+950</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="4" t="inlineStr">
+        <is>
+          <t>Besos Mojados</t>
+        </is>
+      </c>
+      <c r="B40" s="5" t="n">
+        <v>4225</v>
+      </c>
+      <c r="C40" s="5" t="inlineStr">
+        <is>
+          <t>+300</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="4" t="inlineStr">
+        <is>
+          <t>DarkFire</t>
+        </is>
+      </c>
+      <c r="B41" s="5" t="n">
+        <v>10211</v>
+      </c>
+      <c r="C41" s="5" t="inlineStr">
+        <is>
+          <t>+1100</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="4" t="inlineStr">
+        <is>
+          <t>DarkSunny</t>
+        </is>
+      </c>
+      <c r="B42" s="5" t="n">
+        <v>10469</v>
+      </c>
+      <c r="C42" s="5" t="inlineStr">
+        <is>
+          <t>+1100</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="4" t="inlineStr">
+        <is>
+          <t>Dairen Uchiha</t>
+        </is>
+      </c>
+      <c r="B43" s="5" t="n">
+        <v>10957</v>
+      </c>
+      <c r="C43" s="5" t="inlineStr">
+        <is>
+          <t>+1055</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="4" t="inlineStr">
+        <is>
+          <t>LILI ZENIN®</t>
+        </is>
+      </c>
+      <c r="B44" s="5" t="n">
+        <v>6504</v>
+      </c>
+      <c r="C44" s="5" t="inlineStr">
+        <is>
+          <t>+1091</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="4" t="inlineStr">
+        <is>
+          <t>ryumichel ZENIN ®</t>
+        </is>
+      </c>
+      <c r="B45" s="5" t="n">
+        <v>2718</v>
+      </c>
+      <c r="C45" s="5" t="inlineStr">
+        <is>
+          <t>+1082</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="4" t="inlineStr">
+        <is>
+          <t>margot ZENIN ®</t>
+        </is>
+      </c>
+      <c r="B46" s="5" t="n">
+        <v>2800</v>
+      </c>
+      <c r="C46" s="5" t="inlineStr">
+        <is>
+          <t>+1100</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="4" t="inlineStr">
+        <is>
+          <t>linda ZENIN ®</t>
+        </is>
+      </c>
+      <c r="B47" s="5" t="n">
+        <v>6661</v>
+      </c>
+      <c r="C47" s="5" t="inlineStr">
+        <is>
+          <t>+1100</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="4" t="inlineStr">
+        <is>
+          <t>SHINRAIN ZENIN®</t>
+        </is>
+      </c>
+      <c r="B48" s="5" t="n">
+        <v>6442</v>
+      </c>
+      <c r="C48" s="5" t="inlineStr">
+        <is>
+          <t>+1046</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="4" t="inlineStr">
+        <is>
+          <t>PlyRed-</t>
+        </is>
+      </c>
+      <c r="B49" s="5" t="n">
+        <v>5731</v>
+      </c>
+      <c r="C49" s="5" t="inlineStr">
+        <is>
+          <t>+724</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="4" t="inlineStr">
+        <is>
+          <t>equin0x</t>
+        </is>
+      </c>
+      <c r="B50" s="5" t="n">
+        <v>8225</v>
+      </c>
+      <c r="C50" s="5" t="inlineStr">
+        <is>
+          <t>+715</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="4" t="inlineStr">
+        <is>
+          <t>Jhayco - Mokai</t>
+        </is>
+      </c>
+      <c r="B51" s="5" t="n">
+        <v>9915</v>
+      </c>
+      <c r="C51" s="5" t="inlineStr">
+        <is>
+          <t>+950</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="4" t="inlineStr">
+        <is>
+          <t>Jhayco - Joe</t>
+        </is>
+      </c>
+      <c r="B52" s="5" t="n">
+        <v>10111</v>
+      </c>
+      <c r="C52" s="5" t="inlineStr">
+        <is>
+          <t>+950</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="4" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="B53" s="5" t="n">
+        <v>9982</v>
+      </c>
+      <c r="C53" s="5" t="inlineStr">
+        <is>
+          <t>+950</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="4" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="B54" s="5" t="n">
+        <v>10276</v>
+      </c>
+      <c r="C54" s="5" t="inlineStr">
+        <is>
+          <t>+950</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="4" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="B55" s="5" t="n">
+        <v>9961</v>
+      </c>
+      <c r="C55" s="5" t="inlineStr">
+        <is>
+          <t>+896</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="4" t="inlineStr">
+        <is>
+          <t>Go Go Juice</t>
+        </is>
+      </c>
+      <c r="B56" s="5" t="n">
+        <v>7680</v>
+      </c>
+      <c r="C56" s="5" t="inlineStr">
+        <is>
+          <t>+650</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="4" t="inlineStr">
+        <is>
+          <t>Jhayco - Imaginaste</t>
+        </is>
+      </c>
+      <c r="B57" s="5" t="n">
+        <v>3927</v>
+      </c>
+      <c r="C57" s="5" t="inlineStr">
+        <is>
+          <t>+150</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="4" t="inlineStr">
+        <is>
+          <t>PuNch</t>
+        </is>
+      </c>
+      <c r="B58" s="5" t="n">
+        <v>6465</v>
+      </c>
+      <c r="C58" s="5" t="inlineStr">
+        <is>
+          <t>+1100</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A2:C2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
auto: snapshot 2026-07-30 13:31:01
</commit_message>
<xml_diff>
--- a/clan_3815.xlsx
+++ b/clan_3815.xlsx
@@ -5980,7 +5980,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Timestamp: 2026-07-30 13:01:00</t>
+          <t>Timestamp: 2026-07-30 13:31:00</t>
         </is>
       </c>
     </row>
@@ -6053,11 +6053,11 @@
         </is>
       </c>
       <c r="B7" s="5" t="n">
-        <v>3748</v>
+        <v>3798</v>
       </c>
       <c r="C7" s="5" t="inlineStr">
         <is>
-          <t>+524</t>
+          <t>+574</t>
         </is>
       </c>
     </row>
@@ -6173,11 +6173,11 @@
         </is>
       </c>
       <c r="B15" s="5" t="n">
-        <v>6927</v>
+        <v>6977</v>
       </c>
       <c r="C15" s="5" t="inlineStr">
         <is>
-          <t>+800</t>
+          <t>+850</t>
         </is>
       </c>
     </row>
@@ -6278,11 +6278,11 @@
         </is>
       </c>
       <c r="B22" s="5" t="n">
-        <v>8043</v>
+        <v>8093</v>
       </c>
       <c r="C22" s="5" t="inlineStr">
         <is>
-          <t>+550</t>
+          <t>+600</t>
         </is>
       </c>
     </row>
@@ -6293,11 +6293,11 @@
         </is>
       </c>
       <c r="B23" s="5" t="n">
-        <v>7912</v>
+        <v>7962</v>
       </c>
       <c r="C23" s="5" t="inlineStr">
         <is>
-          <t>+564</t>
+          <t>+614</t>
         </is>
       </c>
     </row>
@@ -6308,11 +6308,11 @@
         </is>
       </c>
       <c r="B24" s="5" t="n">
-        <v>7254</v>
+        <v>7304</v>
       </c>
       <c r="C24" s="5" t="inlineStr">
         <is>
-          <t>+450</t>
+          <t>+500</t>
         </is>
       </c>
     </row>
@@ -6323,11 +6323,11 @@
         </is>
       </c>
       <c r="B25" s="5" t="n">
-        <v>6685</v>
+        <v>6705</v>
       </c>
       <c r="C25" s="5" t="inlineStr">
         <is>
-          <t>+877</t>
+          <t>+897</t>
         </is>
       </c>
     </row>
@@ -6338,11 +6338,11 @@
         </is>
       </c>
       <c r="B26" s="5" t="n">
-        <v>6624</v>
+        <v>6724</v>
       </c>
       <c r="C26" s="5" t="inlineStr">
         <is>
-          <t>+896</t>
+          <t>+996</t>
         </is>
       </c>
     </row>
@@ -6353,11 +6353,11 @@
         </is>
       </c>
       <c r="B27" s="5" t="n">
-        <v>6693</v>
+        <v>6712</v>
       </c>
       <c r="C27" s="5" t="inlineStr">
         <is>
-          <t>+950</t>
+          <t>+969</t>
         </is>
       </c>
     </row>
@@ -6368,11 +6368,11 @@
         </is>
       </c>
       <c r="B28" s="5" t="n">
-        <v>8193</v>
+        <v>8243</v>
       </c>
       <c r="C28" s="5" t="inlineStr">
         <is>
-          <t>+800</t>
+          <t>+850</t>
         </is>
       </c>
     </row>
@@ -6383,11 +6383,11 @@
         </is>
       </c>
       <c r="B29" s="5" t="n">
-        <v>7230</v>
+        <v>7280</v>
       </c>
       <c r="C29" s="5" t="inlineStr">
         <is>
-          <t>+144</t>
+          <t>+194</t>
         </is>
       </c>
     </row>
@@ -6398,11 +6398,11 @@
         </is>
       </c>
       <c r="B30" s="5" t="n">
-        <v>8055</v>
+        <v>8105</v>
       </c>
       <c r="C30" s="5" t="inlineStr">
         <is>
-          <t>+650</t>
+          <t>+700</t>
         </is>
       </c>
     </row>
@@ -6413,11 +6413,11 @@
         </is>
       </c>
       <c r="B31" s="5" t="n">
-        <v>7228</v>
+        <v>7278</v>
       </c>
       <c r="C31" s="5" t="inlineStr">
         <is>
-          <t>+450</t>
+          <t>+500</t>
         </is>
       </c>
     </row>
@@ -6428,11 +6428,11 @@
         </is>
       </c>
       <c r="B32" s="5" t="n">
-        <v>7901</v>
+        <v>8001</v>
       </c>
       <c r="C32" s="5" t="inlineStr">
         <is>
-          <t>+815</t>
+          <t>+915</t>
         </is>
       </c>
     </row>
@@ -6443,11 +6443,11 @@
         </is>
       </c>
       <c r="B33" s="5" t="n">
-        <v>6450</v>
+        <v>6550</v>
       </c>
       <c r="C33" s="5" t="inlineStr">
         <is>
-          <t>+950</t>
+          <t>+1050</t>
         </is>
       </c>
     </row>
@@ -6458,11 +6458,11 @@
         </is>
       </c>
       <c r="B34" s="5" t="n">
-        <v>9524</v>
+        <v>9588</v>
       </c>
       <c r="C34" s="5" t="inlineStr">
         <is>
-          <t>+950</t>
+          <t>+1014</t>
         </is>
       </c>
     </row>
@@ -6473,11 +6473,11 @@
         </is>
       </c>
       <c r="B35" s="5" t="n">
-        <v>6916</v>
+        <v>6966</v>
       </c>
       <c r="C35" s="5" t="inlineStr">
         <is>
-          <t>+350</t>
+          <t>+400</t>
         </is>
       </c>
     </row>
@@ -6563,11 +6563,11 @@
         </is>
       </c>
       <c r="B41" s="5" t="n">
-        <v>10211</v>
+        <v>10261</v>
       </c>
       <c r="C41" s="5" t="inlineStr">
         <is>
-          <t>+1100</t>
+          <t>+1150</t>
         </is>
       </c>
     </row>
@@ -6578,11 +6578,11 @@
         </is>
       </c>
       <c r="B42" s="5" t="n">
-        <v>10469</v>
+        <v>10519</v>
       </c>
       <c r="C42" s="5" t="inlineStr">
         <is>
-          <t>+1100</t>
+          <t>+1150</t>
         </is>
       </c>
     </row>
@@ -6593,11 +6593,11 @@
         </is>
       </c>
       <c r="B43" s="5" t="n">
-        <v>10957</v>
+        <v>11007</v>
       </c>
       <c r="C43" s="5" t="inlineStr">
         <is>
-          <t>+1055</t>
+          <t>+1105</t>
         </is>
       </c>
     </row>
@@ -6608,11 +6608,11 @@
         </is>
       </c>
       <c r="B44" s="5" t="n">
-        <v>6504</v>
+        <v>6554</v>
       </c>
       <c r="C44" s="5" t="inlineStr">
         <is>
-          <t>+1091</t>
+          <t>+1141</t>
         </is>
       </c>
     </row>
@@ -6623,11 +6623,11 @@
         </is>
       </c>
       <c r="B45" s="5" t="n">
-        <v>2718</v>
+        <v>2768</v>
       </c>
       <c r="C45" s="5" t="inlineStr">
         <is>
-          <t>+1082</t>
+          <t>+1132</t>
         </is>
       </c>
     </row>
@@ -6683,11 +6683,11 @@
         </is>
       </c>
       <c r="B49" s="5" t="n">
-        <v>5731</v>
+        <v>5781</v>
       </c>
       <c r="C49" s="5" t="inlineStr">
         <is>
-          <t>+724</t>
+          <t>+774</t>
         </is>
       </c>
     </row>
@@ -6698,11 +6698,11 @@
         </is>
       </c>
       <c r="B50" s="5" t="n">
-        <v>8225</v>
+        <v>8266</v>
       </c>
       <c r="C50" s="5" t="inlineStr">
         <is>
-          <t>+715</t>
+          <t>+756</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: snapshot 2026-07-31 13:01:00
</commit_message>
<xml_diff>
--- a/clan_3815.xlsx
+++ b/clan_3815.xlsx
@@ -23,6 +23,7 @@
     <sheet name="2026-07-28" sheetId="14" state="visible" r:id="rId14"/>
     <sheet name="2026-07-29" sheetId="15" state="visible" r:id="rId15"/>
     <sheet name="2026-07-30" sheetId="16" state="visible" r:id="rId16"/>
+    <sheet name="2026-07-31" sheetId="17" state="visible" r:id="rId17"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -6835,6 +6836,885 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C58"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="29" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Clan: Mans Best Friend (3815)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Timestamp: 2026-07-31 13:01:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>Total Reps</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>Daily Reps (+1d)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>Nobodys Son</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="n">
+        <v>7372</v>
+      </c>
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>-2216</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>Player</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="n">
+        <v>4164</v>
+      </c>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>+349</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>Player</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="n">
+        <v>4100</v>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>+285</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>X y L O T A</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="n">
+        <v>4048</v>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>+250</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>AbdiHyde ID 13496</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="n">
+        <v>5227</v>
+      </c>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>+200</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>Create Character III</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="n">
+        <v>6897</v>
+      </c>
+      <c r="C9" s="5" t="inlineStr">
+        <is>
+          <t>+250</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>Create Character IV</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="n">
+        <v>7558</v>
+      </c>
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>+250</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>Create Character V</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="n">
+        <v>7410</v>
+      </c>
+      <c r="C11" s="5" t="inlineStr">
+        <is>
+          <t>+250</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t>Player</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="n">
+        <v>4074</v>
+      </c>
+      <c r="C12" s="5" t="inlineStr">
+        <is>
+          <t>+259</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="4" t="inlineStr">
+        <is>
+          <t>Player</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="n">
+        <v>4015</v>
+      </c>
+      <c r="C13" s="5" t="inlineStr">
+        <is>
+          <t>+200</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="4" t="inlineStr">
+        <is>
+          <t>hunry</t>
+        </is>
+      </c>
+      <c r="B14" s="5" t="n">
+        <v>4104</v>
+      </c>
+      <c r="C14" s="5" t="inlineStr">
+        <is>
+          <t>+200</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="4" t="inlineStr">
+        <is>
+          <t>Tears</t>
+        </is>
+      </c>
+      <c r="B15" s="5" t="n">
+        <v>7227</v>
+      </c>
+      <c r="C15" s="5" t="inlineStr">
+        <is>
+          <t>+250</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="4" t="inlineStr">
+        <is>
+          <t>Sugar Talking</t>
+        </is>
+      </c>
+      <c r="B16" s="5" t="n">
+        <v>8412</v>
+      </c>
+      <c r="C16" s="5" t="inlineStr">
+        <is>
+          <t>+1134</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="4" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B17" s="5" t="n">
+        <v>7523</v>
+      </c>
+      <c r="C17" s="5" t="inlineStr">
+        <is>
+          <t>+250</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="4" t="inlineStr">
+        <is>
+          <t>Anti-Hero</t>
+        </is>
+      </c>
+      <c r="B18" s="5" t="n">
+        <v>8274</v>
+      </c>
+      <c r="C18" s="5" t="inlineStr">
+        <is>
+          <t>+250</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="4" t="inlineStr">
+        <is>
+          <t>Vigilante Shit</t>
+        </is>
+      </c>
+      <c r="B19" s="5" t="n">
+        <v>8289</v>
+      </c>
+      <c r="C19" s="5" t="inlineStr">
+        <is>
+          <t>+250</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="4" t="inlineStr">
+        <is>
+          <t>Sweet Nothing</t>
+        </is>
+      </c>
+      <c r="B20" s="5" t="n">
+        <v>8369</v>
+      </c>
+      <c r="C20" s="5" t="inlineStr">
+        <is>
+          <t>+250</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="4" t="inlineStr">
+        <is>
+          <t>The Great War</t>
+        </is>
+      </c>
+      <c r="B21" s="5" t="n">
+        <v>8089</v>
+      </c>
+      <c r="C21" s="5" t="inlineStr">
+        <is>
+          <t>+250</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">We Almost Broke Up </t>
+        </is>
+      </c>
+      <c r="B22" s="5" t="n">
+        <v>8343</v>
+      </c>
+      <c r="C22" s="5" t="inlineStr">
+        <is>
+          <t>+250</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="4" t="inlineStr">
+        <is>
+          <t>When Did You Get Hot</t>
+        </is>
+      </c>
+      <c r="B23" s="5" t="n">
+        <v>8212</v>
+      </c>
+      <c r="C23" s="5" t="inlineStr">
+        <is>
+          <t>+250</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="4" t="inlineStr">
+        <is>
+          <t>Dont Worry Ill Make</t>
+        </is>
+      </c>
+      <c r="B24" s="5" t="n">
+        <v>7554</v>
+      </c>
+      <c r="C24" s="5" t="inlineStr">
+        <is>
+          <t>+250</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="4" t="inlineStr">
+        <is>
+          <t>Goodbye</t>
+        </is>
+      </c>
+      <c r="B25" s="5" t="n">
+        <v>6955</v>
+      </c>
+      <c r="C25" s="5" t="inlineStr">
+        <is>
+          <t>+250</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="4" t="inlineStr">
+        <is>
+          <t>Mans Best Friend</t>
+        </is>
+      </c>
+      <c r="B26" s="5" t="n">
+        <v>6974</v>
+      </c>
+      <c r="C26" s="5" t="inlineStr">
+        <is>
+          <t>+250</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="4" t="inlineStr">
+        <is>
+          <t>Lavender Haze</t>
+        </is>
+      </c>
+      <c r="B27" s="5" t="n">
+        <v>6962</v>
+      </c>
+      <c r="C27" s="5" t="inlineStr">
+        <is>
+          <t>+250</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="4" t="inlineStr">
+        <is>
+          <t>Never Getting Laid</t>
+        </is>
+      </c>
+      <c r="B28" s="5" t="n">
+        <v>8493</v>
+      </c>
+      <c r="C28" s="5" t="inlineStr">
+        <is>
+          <t>+250</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="4" t="inlineStr">
+        <is>
+          <t>My Man on Willpower</t>
+        </is>
+      </c>
+      <c r="B29" s="5" t="n">
+        <v>7480</v>
+      </c>
+      <c r="C29" s="5" t="inlineStr">
+        <is>
+          <t>-521</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="4" t="inlineStr">
+        <is>
+          <t>Manchild</t>
+        </is>
+      </c>
+      <c r="B30" s="5" t="n">
+        <v>8355</v>
+      </c>
+      <c r="C30" s="5" t="inlineStr">
+        <is>
+          <t>+250</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="4" t="inlineStr">
+        <is>
+          <t>Sugar Talking</t>
+        </is>
+      </c>
+      <c r="B31" s="5" t="n">
+        <v>7528</v>
+      </c>
+      <c r="C31" s="5" t="inlineStr">
+        <is>
+          <t>+250</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="4" t="inlineStr">
+        <is>
+          <t>My Man on Willpower</t>
+        </is>
+      </c>
+      <c r="B32" s="5" t="n">
+        <v>8251</v>
+      </c>
+      <c r="C32" s="5" t="inlineStr">
+        <is>
+          <t>+250</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="4" t="inlineStr">
+        <is>
+          <t>Midnight Rain</t>
+        </is>
+      </c>
+      <c r="B33" s="5" t="n">
+        <v>6800</v>
+      </c>
+      <c r="C33" s="5" t="inlineStr">
+        <is>
+          <t>+250</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="4" t="inlineStr">
+        <is>
+          <t>Nobodys Son</t>
+        </is>
+      </c>
+      <c r="B34" s="5" t="n">
+        <v>9838</v>
+      </c>
+      <c r="C34" s="5" t="inlineStr">
+        <is>
+          <t>+250</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="4" t="inlineStr">
+        <is>
+          <t>House Tour</t>
+        </is>
+      </c>
+      <c r="B35" s="5" t="n">
+        <v>7216</v>
+      </c>
+      <c r="C35" s="5" t="inlineStr">
+        <is>
+          <t>+250</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="4" t="inlineStr">
+        <is>
+          <t>Hanabi  Î±Î·Ð²Ï…</t>
+        </is>
+      </c>
+      <c r="B36" s="5" t="n">
+        <v>7062</v>
+      </c>
+      <c r="C36" s="5" t="inlineStr">
+        <is>
+          <t>+150</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="4" t="inlineStr">
+        <is>
+          <t>Saiyajin anbuâ„¢</t>
+        </is>
+      </c>
+      <c r="B37" s="5" t="n">
+        <v>4213</v>
+      </c>
+      <c r="C37" s="5" t="inlineStr">
+        <is>
+          <t>+150</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="4" t="inlineStr">
+        <is>
+          <t>Dummy</t>
+        </is>
+      </c>
+      <c r="B38" s="5" t="n">
+        <v>6572</v>
+      </c>
+      <c r="C38" s="5" t="inlineStr">
+        <is>
+          <t>+150</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="4" t="inlineStr">
+        <is>
+          <t>Cazador anbu â„¢</t>
+        </is>
+      </c>
+      <c r="B39" s="5" t="n">
+        <v>4136</v>
+      </c>
+      <c r="C39" s="5" t="inlineStr">
+        <is>
+          <t>+150</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="4" t="inlineStr">
+        <is>
+          <t>Besos Mojados</t>
+        </is>
+      </c>
+      <c r="B40" s="5" t="n">
+        <v>4425</v>
+      </c>
+      <c r="C40" s="5" t="inlineStr">
+        <is>
+          <t>+200</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="4" t="inlineStr">
+        <is>
+          <t>DarkFire</t>
+        </is>
+      </c>
+      <c r="B41" s="5" t="n">
+        <v>10546</v>
+      </c>
+      <c r="C41" s="5" t="inlineStr">
+        <is>
+          <t>+285</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="4" t="inlineStr">
+        <is>
+          <t>DarkSunny</t>
+        </is>
+      </c>
+      <c r="B42" s="5" t="n">
+        <v>10794</v>
+      </c>
+      <c r="C42" s="5" t="inlineStr">
+        <is>
+          <t>+275</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="4" t="inlineStr">
+        <is>
+          <t>Dairen Uchiha</t>
+        </is>
+      </c>
+      <c r="B43" s="5" t="n">
+        <v>11282</v>
+      </c>
+      <c r="C43" s="5" t="inlineStr">
+        <is>
+          <t>+275</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="4" t="inlineStr">
+        <is>
+          <t>LILI ZENIN®</t>
+        </is>
+      </c>
+      <c r="B44" s="5" t="n">
+        <v>6854</v>
+      </c>
+      <c r="C44" s="5" t="inlineStr">
+        <is>
+          <t>+300</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="4" t="inlineStr">
+        <is>
+          <t>ryumichel ZENIN ®</t>
+        </is>
+      </c>
+      <c r="B45" s="5" t="n">
+        <v>3068</v>
+      </c>
+      <c r="C45" s="5" t="inlineStr">
+        <is>
+          <t>+300</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="4" t="inlineStr">
+        <is>
+          <t>margot ZENIN ®</t>
+        </is>
+      </c>
+      <c r="B46" s="5" t="n">
+        <v>3100</v>
+      </c>
+      <c r="C46" s="5" t="inlineStr">
+        <is>
+          <t>+300</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="4" t="inlineStr">
+        <is>
+          <t>linda ZENIN ®</t>
+        </is>
+      </c>
+      <c r="B47" s="5" t="n">
+        <v>6961</v>
+      </c>
+      <c r="C47" s="5" t="inlineStr">
+        <is>
+          <t>+300</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="4" t="inlineStr">
+        <is>
+          <t>SHINRAIN ZENIN®</t>
+        </is>
+      </c>
+      <c r="B48" s="5" t="n">
+        <v>6727</v>
+      </c>
+      <c r="C48" s="5" t="inlineStr">
+        <is>
+          <t>+285</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="4" t="inlineStr">
+        <is>
+          <t>PlyRed-</t>
+        </is>
+      </c>
+      <c r="B49" s="5" t="n">
+        <v>5981</v>
+      </c>
+      <c r="C49" s="5" t="inlineStr">
+        <is>
+          <t>+200</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="4" t="inlineStr">
+        <is>
+          <t>equin0x</t>
+        </is>
+      </c>
+      <c r="B50" s="5" t="n">
+        <v>8466</v>
+      </c>
+      <c r="C50" s="5" t="inlineStr">
+        <is>
+          <t>+200</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="4" t="inlineStr">
+        <is>
+          <t>Jhayco - Mokai</t>
+        </is>
+      </c>
+      <c r="B51" s="5" t="n">
+        <v>10165</v>
+      </c>
+      <c r="C51" s="5" t="inlineStr">
+        <is>
+          <t>+250</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="4" t="inlineStr">
+        <is>
+          <t>Jhayco - Joe</t>
+        </is>
+      </c>
+      <c r="B52" s="5" t="n">
+        <v>10361</v>
+      </c>
+      <c r="C52" s="5" t="inlineStr">
+        <is>
+          <t>+250</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="4" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="B53" s="5" t="n">
+        <v>10232</v>
+      </c>
+      <c r="C53" s="5" t="inlineStr">
+        <is>
+          <t>+250</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="4" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="B54" s="5" t="n">
+        <v>10526</v>
+      </c>
+      <c r="C54" s="5" t="inlineStr">
+        <is>
+          <t>+250</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="4" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="B55" s="5" t="n">
+        <v>10211</v>
+      </c>
+      <c r="C55" s="5" t="inlineStr">
+        <is>
+          <t>+250</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="4" t="inlineStr">
+        <is>
+          <t>Go Go Juice</t>
+        </is>
+      </c>
+      <c r="B56" s="5" t="n">
+        <v>7930</v>
+      </c>
+      <c r="C56" s="5" t="inlineStr">
+        <is>
+          <t>+250</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="4" t="inlineStr">
+        <is>
+          <t>Jhayco - Imaginaste</t>
+        </is>
+      </c>
+      <c r="B57" s="5" t="n">
+        <v>4077</v>
+      </c>
+      <c r="C57" s="5" t="inlineStr">
+        <is>
+          <t>+150</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="4" t="inlineStr">
+        <is>
+          <t>PuNch</t>
+        </is>
+      </c>
+      <c r="B58" s="5" t="n">
+        <v>6865</v>
+      </c>
+      <c r="C58" s="5" t="inlineStr">
+        <is>
+          <t>+400</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A2:C2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
auto: snapshot 2026-07-31 13:31:00
</commit_message>
<xml_diff>
--- a/clan_3815.xlsx
+++ b/clan_3815.xlsx
@@ -6860,7 +6860,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Timestamp: 2026-07-31 13:01:00</t>
+          <t>Timestamp: 2026-07-31 13:31:00</t>
         </is>
       </c>
     </row>
@@ -6888,11 +6888,11 @@
         </is>
       </c>
       <c r="B4" s="5" t="n">
-        <v>7372</v>
+        <v>7422</v>
       </c>
       <c r="C4" s="5" t="inlineStr">
         <is>
-          <t>-2216</t>
+          <t>-2166</t>
         </is>
       </c>
     </row>
@@ -6903,11 +6903,11 @@
         </is>
       </c>
       <c r="B5" s="5" t="n">
-        <v>4164</v>
+        <v>4214</v>
       </c>
       <c r="C5" s="5" t="inlineStr">
         <is>
-          <t>+349</t>
+          <t>+399</t>
         </is>
       </c>
     </row>
@@ -6918,11 +6918,11 @@
         </is>
       </c>
       <c r="B6" s="5" t="n">
-        <v>4100</v>
+        <v>4150</v>
       </c>
       <c r="C6" s="5" t="inlineStr">
         <is>
-          <t>+285</t>
+          <t>+335</t>
         </is>
       </c>
     </row>
@@ -6933,11 +6933,11 @@
         </is>
       </c>
       <c r="B7" s="5" t="n">
-        <v>4048</v>
+        <v>4098</v>
       </c>
       <c r="C7" s="5" t="inlineStr">
         <is>
-          <t>+250</t>
+          <t>+300</t>
         </is>
       </c>
     </row>
@@ -6948,11 +6948,11 @@
         </is>
       </c>
       <c r="B8" s="5" t="n">
-        <v>5227</v>
+        <v>5327</v>
       </c>
       <c r="C8" s="5" t="inlineStr">
         <is>
-          <t>+200</t>
+          <t>+300</t>
         </is>
       </c>
     </row>
@@ -6963,11 +6963,11 @@
         </is>
       </c>
       <c r="B9" s="5" t="n">
-        <v>6897</v>
+        <v>6947</v>
       </c>
       <c r="C9" s="5" t="inlineStr">
         <is>
-          <t>+250</t>
+          <t>+300</t>
         </is>
       </c>
     </row>
@@ -6978,11 +6978,11 @@
         </is>
       </c>
       <c r="B10" s="5" t="n">
-        <v>7558</v>
+        <v>7608</v>
       </c>
       <c r="C10" s="5" t="inlineStr">
         <is>
-          <t>+250</t>
+          <t>+300</t>
         </is>
       </c>
     </row>
@@ -6993,11 +6993,11 @@
         </is>
       </c>
       <c r="B11" s="5" t="n">
-        <v>7410</v>
+        <v>7460</v>
       </c>
       <c r="C11" s="5" t="inlineStr">
         <is>
-          <t>+250</t>
+          <t>+300</t>
         </is>
       </c>
     </row>
@@ -7008,11 +7008,11 @@
         </is>
       </c>
       <c r="B12" s="5" t="n">
-        <v>4074</v>
+        <v>4124</v>
       </c>
       <c r="C12" s="5" t="inlineStr">
         <is>
-          <t>+259</t>
+          <t>+309</t>
         </is>
       </c>
     </row>
@@ -7023,11 +7023,11 @@
         </is>
       </c>
       <c r="B13" s="5" t="n">
-        <v>4015</v>
+        <v>4065</v>
       </c>
       <c r="C13" s="5" t="inlineStr">
         <is>
-          <t>+200</t>
+          <t>+250</t>
         </is>
       </c>
     </row>
@@ -7038,11 +7038,11 @@
         </is>
       </c>
       <c r="B14" s="5" t="n">
-        <v>4104</v>
+        <v>4154</v>
       </c>
       <c r="C14" s="5" t="inlineStr">
         <is>
-          <t>+200</t>
+          <t>+250</t>
         </is>
       </c>
     </row>
@@ -7068,11 +7068,11 @@
         </is>
       </c>
       <c r="B16" s="5" t="n">
-        <v>8412</v>
+        <v>8462</v>
       </c>
       <c r="C16" s="5" t="inlineStr">
         <is>
-          <t>+1134</t>
+          <t>+1184</t>
         </is>
       </c>
     </row>
@@ -7203,11 +7203,11 @@
         </is>
       </c>
       <c r="B25" s="5" t="n">
-        <v>6955</v>
+        <v>7005</v>
       </c>
       <c r="C25" s="5" t="inlineStr">
         <is>
-          <t>+250</t>
+          <t>+300</t>
         </is>
       </c>
     </row>
@@ -7308,11 +7308,11 @@
         </is>
       </c>
       <c r="B32" s="5" t="n">
-        <v>8251</v>
+        <v>8301</v>
       </c>
       <c r="C32" s="5" t="inlineStr">
         <is>
-          <t>+250</t>
+          <t>+300</t>
         </is>
       </c>
     </row>
@@ -7338,11 +7338,11 @@
         </is>
       </c>
       <c r="B34" s="5" t="n">
-        <v>9838</v>
+        <v>9888</v>
       </c>
       <c r="C34" s="5" t="inlineStr">
         <is>
-          <t>+250</t>
+          <t>+300</t>
         </is>
       </c>
     </row>
@@ -7368,11 +7368,11 @@
         </is>
       </c>
       <c r="B36" s="5" t="n">
-        <v>7062</v>
+        <v>7112</v>
       </c>
       <c r="C36" s="5" t="inlineStr">
         <is>
-          <t>+150</t>
+          <t>+200</t>
         </is>
       </c>
     </row>
@@ -7383,11 +7383,11 @@
         </is>
       </c>
       <c r="B37" s="5" t="n">
-        <v>4213</v>
+        <v>4263</v>
       </c>
       <c r="C37" s="5" t="inlineStr">
         <is>
-          <t>+150</t>
+          <t>+200</t>
         </is>
       </c>
     </row>
@@ -7398,11 +7398,11 @@
         </is>
       </c>
       <c r="B38" s="5" t="n">
-        <v>6572</v>
+        <v>6622</v>
       </c>
       <c r="C38" s="5" t="inlineStr">
         <is>
-          <t>+150</t>
+          <t>+200</t>
         </is>
       </c>
     </row>
@@ -7413,11 +7413,11 @@
         </is>
       </c>
       <c r="B39" s="5" t="n">
-        <v>4136</v>
+        <v>4186</v>
       </c>
       <c r="C39" s="5" t="inlineStr">
         <is>
-          <t>+150</t>
+          <t>+200</t>
         </is>
       </c>
     </row>
@@ -7443,11 +7443,11 @@
         </is>
       </c>
       <c r="B41" s="5" t="n">
-        <v>10546</v>
+        <v>10586</v>
       </c>
       <c r="C41" s="5" t="inlineStr">
         <is>
-          <t>+285</t>
+          <t>+325</t>
         </is>
       </c>
     </row>
@@ -7458,11 +7458,11 @@
         </is>
       </c>
       <c r="B42" s="5" t="n">
-        <v>10794</v>
+        <v>10844</v>
       </c>
       <c r="C42" s="5" t="inlineStr">
         <is>
-          <t>+275</t>
+          <t>+325</t>
         </is>
       </c>
     </row>
@@ -7473,11 +7473,11 @@
         </is>
       </c>
       <c r="B43" s="5" t="n">
-        <v>11282</v>
+        <v>11332</v>
       </c>
       <c r="C43" s="5" t="inlineStr">
         <is>
-          <t>+275</t>
+          <t>+325</t>
         </is>
       </c>
     </row>
@@ -7488,11 +7488,11 @@
         </is>
       </c>
       <c r="B44" s="5" t="n">
-        <v>6854</v>
+        <v>6904</v>
       </c>
       <c r="C44" s="5" t="inlineStr">
         <is>
-          <t>+300</t>
+          <t>+350</t>
         </is>
       </c>
     </row>
@@ -7503,11 +7503,11 @@
         </is>
       </c>
       <c r="B45" s="5" t="n">
-        <v>3068</v>
+        <v>3118</v>
       </c>
       <c r="C45" s="5" t="inlineStr">
         <is>
-          <t>+300</t>
+          <t>+350</t>
         </is>
       </c>
     </row>
@@ -7518,11 +7518,11 @@
         </is>
       </c>
       <c r="B46" s="5" t="n">
-        <v>3100</v>
+        <v>3150</v>
       </c>
       <c r="C46" s="5" t="inlineStr">
         <is>
-          <t>+300</t>
+          <t>+350</t>
         </is>
       </c>
     </row>
@@ -7533,11 +7533,11 @@
         </is>
       </c>
       <c r="B47" s="5" t="n">
-        <v>6961</v>
+        <v>7011</v>
       </c>
       <c r="C47" s="5" t="inlineStr">
         <is>
-          <t>+300</t>
+          <t>+350</t>
         </is>
       </c>
     </row>
@@ -7548,11 +7548,11 @@
         </is>
       </c>
       <c r="B48" s="5" t="n">
-        <v>6727</v>
+        <v>6777</v>
       </c>
       <c r="C48" s="5" t="inlineStr">
         <is>
-          <t>+285</t>
+          <t>+335</t>
         </is>
       </c>
     </row>
@@ -7563,11 +7563,11 @@
         </is>
       </c>
       <c r="B49" s="5" t="n">
-        <v>5981</v>
+        <v>6031</v>
       </c>
       <c r="C49" s="5" t="inlineStr">
         <is>
-          <t>+200</t>
+          <t>+250</t>
         </is>
       </c>
     </row>
@@ -7578,11 +7578,11 @@
         </is>
       </c>
       <c r="B50" s="5" t="n">
-        <v>8466</v>
+        <v>8516</v>
       </c>
       <c r="C50" s="5" t="inlineStr">
         <is>
-          <t>+200</t>
+          <t>+250</t>
         </is>
       </c>
     </row>
@@ -7698,11 +7698,11 @@
         </is>
       </c>
       <c r="B58" s="5" t="n">
-        <v>6865</v>
+        <v>6915</v>
       </c>
       <c r="C58" s="5" t="inlineStr">
         <is>
-          <t>+400</t>
+          <t>+450</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: snapshot 2026-08-01 13:01:00
</commit_message>
<xml_diff>
--- a/clan_3815.xlsx
+++ b/clan_3815.xlsx
@@ -24,6 +24,7 @@
     <sheet name="2026-07-29" sheetId="15" state="visible" r:id="rId15"/>
     <sheet name="2026-07-30" sheetId="16" state="visible" r:id="rId16"/>
     <sheet name="2026-07-31" sheetId="17" state="visible" r:id="rId17"/>
+    <sheet name="2026-08-01" sheetId="18" state="visible" r:id="rId18"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -7715,6 +7716,885 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C58"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="29" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Clan: Mans Best Friend (3815)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Timestamp: 2026-08-01 13:01:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>Total Reps</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>Daily Reps (+1d)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>Nobodys Son</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="n">
+        <v>7422</v>
+      </c>
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>-2466</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>Player</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="n">
+        <v>4314</v>
+      </c>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>+249</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>Player</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="n">
+        <v>4200</v>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>+135</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>X y L O T A</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="n">
+        <v>4098</v>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>AbdiHyde ID 13496</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="n">
+        <v>5427</v>
+      </c>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>+100</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>Create Character III</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="n">
+        <v>7047</v>
+      </c>
+      <c r="C9" s="5" t="inlineStr">
+        <is>
+          <t>+100</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>Create Character IV</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="n">
+        <v>7708</v>
+      </c>
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>+100</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>Create Character V</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="n">
+        <v>7560</v>
+      </c>
+      <c r="C11" s="5" t="inlineStr">
+        <is>
+          <t>+100</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t>Player</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="n">
+        <v>4174</v>
+      </c>
+      <c r="C12" s="5" t="inlineStr">
+        <is>
+          <t>+109</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="4" t="inlineStr">
+        <is>
+          <t>Player</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="n">
+        <v>4115</v>
+      </c>
+      <c r="C13" s="5" t="inlineStr">
+        <is>
+          <t>+50</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="4" t="inlineStr">
+        <is>
+          <t>hunry</t>
+        </is>
+      </c>
+      <c r="B14" s="5" t="n">
+        <v>4204</v>
+      </c>
+      <c r="C14" s="5" t="inlineStr">
+        <is>
+          <t>+50</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="4" t="inlineStr">
+        <is>
+          <t>Tears</t>
+        </is>
+      </c>
+      <c r="B15" s="5" t="n">
+        <v>7227</v>
+      </c>
+      <c r="C15" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="4" t="inlineStr">
+        <is>
+          <t>Sugar Talking</t>
+        </is>
+      </c>
+      <c r="B16" s="5" t="n">
+        <v>8462</v>
+      </c>
+      <c r="C16" s="5" t="inlineStr">
+        <is>
+          <t>+934</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="4" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B17" s="5" t="n">
+        <v>7523</v>
+      </c>
+      <c r="C17" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="4" t="inlineStr">
+        <is>
+          <t>Anti-Hero</t>
+        </is>
+      </c>
+      <c r="B18" s="5" t="n">
+        <v>8274</v>
+      </c>
+      <c r="C18" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="4" t="inlineStr">
+        <is>
+          <t>Vigilante Shit</t>
+        </is>
+      </c>
+      <c r="B19" s="5" t="n">
+        <v>8289</v>
+      </c>
+      <c r="C19" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="4" t="inlineStr">
+        <is>
+          <t>Sweet Nothing</t>
+        </is>
+      </c>
+      <c r="B20" s="5" t="n">
+        <v>8369</v>
+      </c>
+      <c r="C20" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="4" t="inlineStr">
+        <is>
+          <t>The Great War</t>
+        </is>
+      </c>
+      <c r="B21" s="5" t="n">
+        <v>8089</v>
+      </c>
+      <c r="C21" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">We Almost Broke Up </t>
+        </is>
+      </c>
+      <c r="B22" s="5" t="n">
+        <v>8343</v>
+      </c>
+      <c r="C22" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="4" t="inlineStr">
+        <is>
+          <t>When Did You Get Hot</t>
+        </is>
+      </c>
+      <c r="B23" s="5" t="n">
+        <v>8212</v>
+      </c>
+      <c r="C23" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="4" t="inlineStr">
+        <is>
+          <t>Dont Worry Ill Make</t>
+        </is>
+      </c>
+      <c r="B24" s="5" t="n">
+        <v>7554</v>
+      </c>
+      <c r="C24" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="4" t="inlineStr">
+        <is>
+          <t>Goodbye</t>
+        </is>
+      </c>
+      <c r="B25" s="5" t="n">
+        <v>7005</v>
+      </c>
+      <c r="C25" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="4" t="inlineStr">
+        <is>
+          <t>Mans Best Friend</t>
+        </is>
+      </c>
+      <c r="B26" s="5" t="n">
+        <v>6974</v>
+      </c>
+      <c r="C26" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="4" t="inlineStr">
+        <is>
+          <t>Lavender Haze</t>
+        </is>
+      </c>
+      <c r="B27" s="5" t="n">
+        <v>6962</v>
+      </c>
+      <c r="C27" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="4" t="inlineStr">
+        <is>
+          <t>Never Getting Laid</t>
+        </is>
+      </c>
+      <c r="B28" s="5" t="n">
+        <v>8493</v>
+      </c>
+      <c r="C28" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="4" t="inlineStr">
+        <is>
+          <t>My Man on Willpower</t>
+        </is>
+      </c>
+      <c r="B29" s="5" t="n">
+        <v>7480</v>
+      </c>
+      <c r="C29" s="5" t="inlineStr">
+        <is>
+          <t>-821</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="4" t="inlineStr">
+        <is>
+          <t>Manchild</t>
+        </is>
+      </c>
+      <c r="B30" s="5" t="n">
+        <v>8355</v>
+      </c>
+      <c r="C30" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="4" t="inlineStr">
+        <is>
+          <t>Sugar Talking</t>
+        </is>
+      </c>
+      <c r="B31" s="5" t="n">
+        <v>7528</v>
+      </c>
+      <c r="C31" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="4" t="inlineStr">
+        <is>
+          <t>My Man on Willpower</t>
+        </is>
+      </c>
+      <c r="B32" s="5" t="n">
+        <v>8301</v>
+      </c>
+      <c r="C32" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="4" t="inlineStr">
+        <is>
+          <t>Midnight Rain</t>
+        </is>
+      </c>
+      <c r="B33" s="5" t="n">
+        <v>6800</v>
+      </c>
+      <c r="C33" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="4" t="inlineStr">
+        <is>
+          <t>Nobodys Son</t>
+        </is>
+      </c>
+      <c r="B34" s="5" t="n">
+        <v>9888</v>
+      </c>
+      <c r="C34" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="4" t="inlineStr">
+        <is>
+          <t>House Tour</t>
+        </is>
+      </c>
+      <c r="B35" s="5" t="n">
+        <v>7216</v>
+      </c>
+      <c r="C35" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="4" t="inlineStr">
+        <is>
+          <t>Hanabi  Î±Î·Ð²Ï…</t>
+        </is>
+      </c>
+      <c r="B36" s="5" t="n">
+        <v>7212</v>
+      </c>
+      <c r="C36" s="5" t="inlineStr">
+        <is>
+          <t>+100</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="4" t="inlineStr">
+        <is>
+          <t>Saiyajin anbuâ„¢</t>
+        </is>
+      </c>
+      <c r="B37" s="5" t="n">
+        <v>4363</v>
+      </c>
+      <c r="C37" s="5" t="inlineStr">
+        <is>
+          <t>+100</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="4" t="inlineStr">
+        <is>
+          <t>Dummy</t>
+        </is>
+      </c>
+      <c r="B38" s="5" t="n">
+        <v>6736</v>
+      </c>
+      <c r="C38" s="5" t="inlineStr">
+        <is>
+          <t>+114</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="4" t="inlineStr">
+        <is>
+          <t>Cazador anbu â„¢</t>
+        </is>
+      </c>
+      <c r="B39" s="5" t="n">
+        <v>4336</v>
+      </c>
+      <c r="C39" s="5" t="inlineStr">
+        <is>
+          <t>+150</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="4" t="inlineStr">
+        <is>
+          <t>Besos Mojados</t>
+        </is>
+      </c>
+      <c r="B40" s="5" t="n">
+        <v>4425</v>
+      </c>
+      <c r="C40" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="4" t="inlineStr">
+        <is>
+          <t>DarkFire</t>
+        </is>
+      </c>
+      <c r="B41" s="5" t="n">
+        <v>10728</v>
+      </c>
+      <c r="C41" s="5" t="inlineStr">
+        <is>
+          <t>+142</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="4" t="inlineStr">
+        <is>
+          <t>DarkSunny</t>
+        </is>
+      </c>
+      <c r="B42" s="5" t="n">
+        <v>10994</v>
+      </c>
+      <c r="C42" s="5" t="inlineStr">
+        <is>
+          <t>+150</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="4" t="inlineStr">
+        <is>
+          <t>Dairen Uchiha</t>
+        </is>
+      </c>
+      <c r="B43" s="5" t="n">
+        <v>11482</v>
+      </c>
+      <c r="C43" s="5" t="inlineStr">
+        <is>
+          <t>+150</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="4" t="inlineStr">
+        <is>
+          <t>LILI ZENIN®</t>
+        </is>
+      </c>
+      <c r="B44" s="5" t="n">
+        <v>7004</v>
+      </c>
+      <c r="C44" s="5" t="inlineStr">
+        <is>
+          <t>+100</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="4" t="inlineStr">
+        <is>
+          <t>ryumichel ZENIN ®</t>
+        </is>
+      </c>
+      <c r="B45" s="5" t="n">
+        <v>3218</v>
+      </c>
+      <c r="C45" s="5" t="inlineStr">
+        <is>
+          <t>+100</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="4" t="inlineStr">
+        <is>
+          <t>margot ZENIN ®</t>
+        </is>
+      </c>
+      <c r="B46" s="5" t="n">
+        <v>3250</v>
+      </c>
+      <c r="C46" s="5" t="inlineStr">
+        <is>
+          <t>+100</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="4" t="inlineStr">
+        <is>
+          <t>linda ZENIN ®</t>
+        </is>
+      </c>
+      <c r="B47" s="5" t="n">
+        <v>7111</v>
+      </c>
+      <c r="C47" s="5" t="inlineStr">
+        <is>
+          <t>+100</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="4" t="inlineStr">
+        <is>
+          <t>SHINRAIN ZENIN®</t>
+        </is>
+      </c>
+      <c r="B48" s="5" t="n">
+        <v>6877</v>
+      </c>
+      <c r="C48" s="5" t="inlineStr">
+        <is>
+          <t>+100</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="4" t="inlineStr">
+        <is>
+          <t>PlyRed-</t>
+        </is>
+      </c>
+      <c r="B49" s="5" t="n">
+        <v>6031</v>
+      </c>
+      <c r="C49" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="4" t="inlineStr">
+        <is>
+          <t>equin0x</t>
+        </is>
+      </c>
+      <c r="B50" s="5" t="n">
+        <v>8516</v>
+      </c>
+      <c r="C50" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="4" t="inlineStr">
+        <is>
+          <t>Jhayco - Mokai</t>
+        </is>
+      </c>
+      <c r="B51" s="5" t="n">
+        <v>10165</v>
+      </c>
+      <c r="C51" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="4" t="inlineStr">
+        <is>
+          <t>Jhayco - Joe</t>
+        </is>
+      </c>
+      <c r="B52" s="5" t="n">
+        <v>10361</v>
+      </c>
+      <c r="C52" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="4" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="B53" s="5" t="n">
+        <v>10232</v>
+      </c>
+      <c r="C53" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="4" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="B54" s="5" t="n">
+        <v>10526</v>
+      </c>
+      <c r="C54" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="4" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="B55" s="5" t="n">
+        <v>10211</v>
+      </c>
+      <c r="C55" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="4" t="inlineStr">
+        <is>
+          <t>Go Go Juice</t>
+        </is>
+      </c>
+      <c r="B56" s="5" t="n">
+        <v>7930</v>
+      </c>
+      <c r="C56" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="4" t="inlineStr">
+        <is>
+          <t>Jhayco - Imaginaste</t>
+        </is>
+      </c>
+      <c r="B57" s="5" t="n">
+        <v>4077</v>
+      </c>
+      <c r="C57" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="4" t="inlineStr">
+        <is>
+          <t>PuNch</t>
+        </is>
+      </c>
+      <c r="B58" s="5" t="n">
+        <v>7065</v>
+      </c>
+      <c r="C58" s="5" t="inlineStr">
+        <is>
+          <t>+150</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A2:C2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
auto: snapshot 2026-08-02 13:01:01
</commit_message>
<xml_diff>
--- a/clan_3815.xlsx
+++ b/clan_3815.xlsx
@@ -25,6 +25,7 @@
     <sheet name="2026-07-30" sheetId="16" state="visible" r:id="rId16"/>
     <sheet name="2026-07-31" sheetId="17" state="visible" r:id="rId17"/>
     <sheet name="2026-08-01" sheetId="18" state="visible" r:id="rId18"/>
+    <sheet name="2026-08-02" sheetId="19" state="visible" r:id="rId19"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -8595,6 +8596,885 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C58"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="29" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Clan: Mans Best Friend (3815)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Timestamp: 2026-08-02 13:01:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>Total Reps</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>Daily Reps (+1d)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>Nobodys Son</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="n">
+        <v>7422</v>
+      </c>
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>-2466</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>Player</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="n">
+        <v>4314</v>
+      </c>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>+199</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>Player</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="n">
+        <v>4200</v>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>+85</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>X y L O T A</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="n">
+        <v>4098</v>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>AbdiHyde ID 13496</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="n">
+        <v>5427</v>
+      </c>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>Create Character III</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="n">
+        <v>7047</v>
+      </c>
+      <c r="C9" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>Create Character IV</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="n">
+        <v>7708</v>
+      </c>
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>Create Character V</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="n">
+        <v>7560</v>
+      </c>
+      <c r="C11" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t>Player</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="n">
+        <v>4174</v>
+      </c>
+      <c r="C12" s="5" t="inlineStr">
+        <is>
+          <t>+59</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="4" t="inlineStr">
+        <is>
+          <t>Player</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="n">
+        <v>4115</v>
+      </c>
+      <c r="C13" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="4" t="inlineStr">
+        <is>
+          <t>hunry</t>
+        </is>
+      </c>
+      <c r="B14" s="5" t="n">
+        <v>4204</v>
+      </c>
+      <c r="C14" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="4" t="inlineStr">
+        <is>
+          <t>Tears</t>
+        </is>
+      </c>
+      <c r="B15" s="5" t="n">
+        <v>7227</v>
+      </c>
+      <c r="C15" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="4" t="inlineStr">
+        <is>
+          <t>Sugar Talking</t>
+        </is>
+      </c>
+      <c r="B16" s="5" t="n">
+        <v>8462</v>
+      </c>
+      <c r="C16" s="5" t="inlineStr">
+        <is>
+          <t>+934</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="4" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B17" s="5" t="n">
+        <v>7523</v>
+      </c>
+      <c r="C17" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="4" t="inlineStr">
+        <is>
+          <t>Anti-Hero</t>
+        </is>
+      </c>
+      <c r="B18" s="5" t="n">
+        <v>8274</v>
+      </c>
+      <c r="C18" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="4" t="inlineStr">
+        <is>
+          <t>Vigilante Shit</t>
+        </is>
+      </c>
+      <c r="B19" s="5" t="n">
+        <v>8289</v>
+      </c>
+      <c r="C19" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="4" t="inlineStr">
+        <is>
+          <t>Sweet Nothing</t>
+        </is>
+      </c>
+      <c r="B20" s="5" t="n">
+        <v>8369</v>
+      </c>
+      <c r="C20" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="4" t="inlineStr">
+        <is>
+          <t>The Great War</t>
+        </is>
+      </c>
+      <c r="B21" s="5" t="n">
+        <v>8089</v>
+      </c>
+      <c r="C21" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">We Almost Broke Up </t>
+        </is>
+      </c>
+      <c r="B22" s="5" t="n">
+        <v>8343</v>
+      </c>
+      <c r="C22" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="4" t="inlineStr">
+        <is>
+          <t>When Did You Get Hot</t>
+        </is>
+      </c>
+      <c r="B23" s="5" t="n">
+        <v>8212</v>
+      </c>
+      <c r="C23" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="4" t="inlineStr">
+        <is>
+          <t>Dont Worry Ill Make</t>
+        </is>
+      </c>
+      <c r="B24" s="5" t="n">
+        <v>7554</v>
+      </c>
+      <c r="C24" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="4" t="inlineStr">
+        <is>
+          <t>Goodbye</t>
+        </is>
+      </c>
+      <c r="B25" s="5" t="n">
+        <v>7005</v>
+      </c>
+      <c r="C25" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="4" t="inlineStr">
+        <is>
+          <t>Mans Best Friend</t>
+        </is>
+      </c>
+      <c r="B26" s="5" t="n">
+        <v>6974</v>
+      </c>
+      <c r="C26" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="4" t="inlineStr">
+        <is>
+          <t>Lavender Haze</t>
+        </is>
+      </c>
+      <c r="B27" s="5" t="n">
+        <v>6962</v>
+      </c>
+      <c r="C27" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="4" t="inlineStr">
+        <is>
+          <t>Never Getting Laid</t>
+        </is>
+      </c>
+      <c r="B28" s="5" t="n">
+        <v>8493</v>
+      </c>
+      <c r="C28" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="4" t="inlineStr">
+        <is>
+          <t>My Man on Willpower</t>
+        </is>
+      </c>
+      <c r="B29" s="5" t="n">
+        <v>7480</v>
+      </c>
+      <c r="C29" s="5" t="inlineStr">
+        <is>
+          <t>-821</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="4" t="inlineStr">
+        <is>
+          <t>Manchild</t>
+        </is>
+      </c>
+      <c r="B30" s="5" t="n">
+        <v>8355</v>
+      </c>
+      <c r="C30" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="4" t="inlineStr">
+        <is>
+          <t>Sugar Talking</t>
+        </is>
+      </c>
+      <c r="B31" s="5" t="n">
+        <v>7528</v>
+      </c>
+      <c r="C31" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="4" t="inlineStr">
+        <is>
+          <t>My Man on Willpower</t>
+        </is>
+      </c>
+      <c r="B32" s="5" t="n">
+        <v>8301</v>
+      </c>
+      <c r="C32" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="4" t="inlineStr">
+        <is>
+          <t>Midnight Rain</t>
+        </is>
+      </c>
+      <c r="B33" s="5" t="n">
+        <v>6800</v>
+      </c>
+      <c r="C33" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="4" t="inlineStr">
+        <is>
+          <t>Nobodys Son</t>
+        </is>
+      </c>
+      <c r="B34" s="5" t="n">
+        <v>9888</v>
+      </c>
+      <c r="C34" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="4" t="inlineStr">
+        <is>
+          <t>House Tour</t>
+        </is>
+      </c>
+      <c r="B35" s="5" t="n">
+        <v>7216</v>
+      </c>
+      <c r="C35" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="4" t="inlineStr">
+        <is>
+          <t>Hanabi  Î±Î·Ð²Ï…</t>
+        </is>
+      </c>
+      <c r="B36" s="5" t="n">
+        <v>7212</v>
+      </c>
+      <c r="C36" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="4" t="inlineStr">
+        <is>
+          <t>Saiyajin anbuâ„¢</t>
+        </is>
+      </c>
+      <c r="B37" s="5" t="n">
+        <v>4363</v>
+      </c>
+      <c r="C37" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="4" t="inlineStr">
+        <is>
+          <t>Dummy</t>
+        </is>
+      </c>
+      <c r="B38" s="5" t="n">
+        <v>6736</v>
+      </c>
+      <c r="C38" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="4" t="inlineStr">
+        <is>
+          <t>Cazador anbu â„¢</t>
+        </is>
+      </c>
+      <c r="B39" s="5" t="n">
+        <v>4336</v>
+      </c>
+      <c r="C39" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="4" t="inlineStr">
+        <is>
+          <t>Besos Mojados</t>
+        </is>
+      </c>
+      <c r="B40" s="5" t="n">
+        <v>4425</v>
+      </c>
+      <c r="C40" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="4" t="inlineStr">
+        <is>
+          <t>DarkFire</t>
+        </is>
+      </c>
+      <c r="B41" s="5" t="n">
+        <v>10728</v>
+      </c>
+      <c r="C41" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="4" t="inlineStr">
+        <is>
+          <t>DarkSunny</t>
+        </is>
+      </c>
+      <c r="B42" s="5" t="n">
+        <v>10994</v>
+      </c>
+      <c r="C42" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="4" t="inlineStr">
+        <is>
+          <t>Dairen Uchiha</t>
+        </is>
+      </c>
+      <c r="B43" s="5" t="n">
+        <v>11482</v>
+      </c>
+      <c r="C43" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="4" t="inlineStr">
+        <is>
+          <t>LILI ZENIN®</t>
+        </is>
+      </c>
+      <c r="B44" s="5" t="n">
+        <v>7011</v>
+      </c>
+      <c r="C44" s="5" t="inlineStr">
+        <is>
+          <t>+7</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="4" t="inlineStr">
+        <is>
+          <t>ryumichel ZENIN ®</t>
+        </is>
+      </c>
+      <c r="B45" s="5" t="n">
+        <v>3218</v>
+      </c>
+      <c r="C45" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="4" t="inlineStr">
+        <is>
+          <t>margot ZENIN ®</t>
+        </is>
+      </c>
+      <c r="B46" s="5" t="n">
+        <v>3250</v>
+      </c>
+      <c r="C46" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="4" t="inlineStr">
+        <is>
+          <t>linda ZENIN ®</t>
+        </is>
+      </c>
+      <c r="B47" s="5" t="n">
+        <v>7111</v>
+      </c>
+      <c r="C47" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="4" t="inlineStr">
+        <is>
+          <t>SHINRAIN ZENIN®</t>
+        </is>
+      </c>
+      <c r="B48" s="5" t="n">
+        <v>6877</v>
+      </c>
+      <c r="C48" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="4" t="inlineStr">
+        <is>
+          <t>PlyRed-</t>
+        </is>
+      </c>
+      <c r="B49" s="5" t="n">
+        <v>6031</v>
+      </c>
+      <c r="C49" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="4" t="inlineStr">
+        <is>
+          <t>equin0x</t>
+        </is>
+      </c>
+      <c r="B50" s="5" t="n">
+        <v>8516</v>
+      </c>
+      <c r="C50" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="4" t="inlineStr">
+        <is>
+          <t>Jhayco - Mokai</t>
+        </is>
+      </c>
+      <c r="B51" s="5" t="n">
+        <v>10165</v>
+      </c>
+      <c r="C51" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="4" t="inlineStr">
+        <is>
+          <t>Jhayco - Joe</t>
+        </is>
+      </c>
+      <c r="B52" s="5" t="n">
+        <v>10361</v>
+      </c>
+      <c r="C52" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="4" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="B53" s="5" t="n">
+        <v>10232</v>
+      </c>
+      <c r="C53" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="4" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="B54" s="5" t="n">
+        <v>10526</v>
+      </c>
+      <c r="C54" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="4" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="B55" s="5" t="n">
+        <v>10211</v>
+      </c>
+      <c r="C55" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="4" t="inlineStr">
+        <is>
+          <t>Go Go Juice</t>
+        </is>
+      </c>
+      <c r="B56" s="5" t="n">
+        <v>7930</v>
+      </c>
+      <c r="C56" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="4" t="inlineStr">
+        <is>
+          <t>Jhayco - Imaginaste</t>
+        </is>
+      </c>
+      <c r="B57" s="5" t="n">
+        <v>4077</v>
+      </c>
+      <c r="C57" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="4" t="inlineStr">
+        <is>
+          <t>PuNch</t>
+        </is>
+      </c>
+      <c r="B58" s="5" t="n">
+        <v>7065</v>
+      </c>
+      <c r="C58" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A2:C2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
auto: snapshot 2026-08-03 13:01:00
</commit_message>
<xml_diff>
--- a/clan_3815.xlsx
+++ b/clan_3815.xlsx
@@ -26,6 +26,7 @@
     <sheet name="2026-07-31" sheetId="17" state="visible" r:id="rId17"/>
     <sheet name="2026-08-01" sheetId="18" state="visible" r:id="rId18"/>
     <sheet name="2026-08-02" sheetId="19" state="visible" r:id="rId19"/>
+    <sheet name="2026-08-03" sheetId="20" state="visible" r:id="rId20"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -9979,6 +9980,885 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet20.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C58"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="29" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Clan: Mans Best Friend (3815)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Timestamp: 2026-08-03 13:01:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>Total Reps</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>Daily Reps (+1d)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>Nobodys Son</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="n">
+        <v>7422</v>
+      </c>
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>-2466</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>Player</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="n">
+        <v>4314</v>
+      </c>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>+199</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>Player</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="n">
+        <v>4200</v>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>+85</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>X y L O T A</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="n">
+        <v>4098</v>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>AbdiHyde ID 13496</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="n">
+        <v>5427</v>
+      </c>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>Create Character III</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="n">
+        <v>7047</v>
+      </c>
+      <c r="C9" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>Create Character IV</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="n">
+        <v>7708</v>
+      </c>
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>Create Character V</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="n">
+        <v>7560</v>
+      </c>
+      <c r="C11" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t>Player</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="n">
+        <v>4174</v>
+      </c>
+      <c r="C12" s="5" t="inlineStr">
+        <is>
+          <t>+59</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="4" t="inlineStr">
+        <is>
+          <t>Player</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="n">
+        <v>4115</v>
+      </c>
+      <c r="C13" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="4" t="inlineStr">
+        <is>
+          <t>hunry</t>
+        </is>
+      </c>
+      <c r="B14" s="5" t="n">
+        <v>4204</v>
+      </c>
+      <c r="C14" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="4" t="inlineStr">
+        <is>
+          <t>Tears</t>
+        </is>
+      </c>
+      <c r="B15" s="5" t="n">
+        <v>7227</v>
+      </c>
+      <c r="C15" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="4" t="inlineStr">
+        <is>
+          <t>Sugar Talking</t>
+        </is>
+      </c>
+      <c r="B16" s="5" t="n">
+        <v>8462</v>
+      </c>
+      <c r="C16" s="5" t="inlineStr">
+        <is>
+          <t>+934</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="4" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B17" s="5" t="n">
+        <v>7523</v>
+      </c>
+      <c r="C17" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="4" t="inlineStr">
+        <is>
+          <t>Anti-Hero</t>
+        </is>
+      </c>
+      <c r="B18" s="5" t="n">
+        <v>8274</v>
+      </c>
+      <c r="C18" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="4" t="inlineStr">
+        <is>
+          <t>Vigilante Shit</t>
+        </is>
+      </c>
+      <c r="B19" s="5" t="n">
+        <v>8289</v>
+      </c>
+      <c r="C19" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="4" t="inlineStr">
+        <is>
+          <t>Sweet Nothing</t>
+        </is>
+      </c>
+      <c r="B20" s="5" t="n">
+        <v>8369</v>
+      </c>
+      <c r="C20" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="4" t="inlineStr">
+        <is>
+          <t>The Great War</t>
+        </is>
+      </c>
+      <c r="B21" s="5" t="n">
+        <v>8089</v>
+      </c>
+      <c r="C21" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">We Almost Broke Up </t>
+        </is>
+      </c>
+      <c r="B22" s="5" t="n">
+        <v>8343</v>
+      </c>
+      <c r="C22" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="4" t="inlineStr">
+        <is>
+          <t>When Did You Get Hot</t>
+        </is>
+      </c>
+      <c r="B23" s="5" t="n">
+        <v>8212</v>
+      </c>
+      <c r="C23" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="4" t="inlineStr">
+        <is>
+          <t>Dont Worry Ill Make</t>
+        </is>
+      </c>
+      <c r="B24" s="5" t="n">
+        <v>7554</v>
+      </c>
+      <c r="C24" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="4" t="inlineStr">
+        <is>
+          <t>Goodbye</t>
+        </is>
+      </c>
+      <c r="B25" s="5" t="n">
+        <v>7005</v>
+      </c>
+      <c r="C25" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="4" t="inlineStr">
+        <is>
+          <t>Mans Best Friend</t>
+        </is>
+      </c>
+      <c r="B26" s="5" t="n">
+        <v>6974</v>
+      </c>
+      <c r="C26" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="4" t="inlineStr">
+        <is>
+          <t>Lavender Haze</t>
+        </is>
+      </c>
+      <c r="B27" s="5" t="n">
+        <v>6962</v>
+      </c>
+      <c r="C27" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="4" t="inlineStr">
+        <is>
+          <t>Never Getting Laid</t>
+        </is>
+      </c>
+      <c r="B28" s="5" t="n">
+        <v>8493</v>
+      </c>
+      <c r="C28" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="4" t="inlineStr">
+        <is>
+          <t>My Man on Willpower</t>
+        </is>
+      </c>
+      <c r="B29" s="5" t="n">
+        <v>7480</v>
+      </c>
+      <c r="C29" s="5" t="inlineStr">
+        <is>
+          <t>-821</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="4" t="inlineStr">
+        <is>
+          <t>Manchild</t>
+        </is>
+      </c>
+      <c r="B30" s="5" t="n">
+        <v>8355</v>
+      </c>
+      <c r="C30" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="4" t="inlineStr">
+        <is>
+          <t>Sugar Talking</t>
+        </is>
+      </c>
+      <c r="B31" s="5" t="n">
+        <v>7528</v>
+      </c>
+      <c r="C31" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="4" t="inlineStr">
+        <is>
+          <t>My Man on Willpower</t>
+        </is>
+      </c>
+      <c r="B32" s="5" t="n">
+        <v>8301</v>
+      </c>
+      <c r="C32" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="4" t="inlineStr">
+        <is>
+          <t>Midnight Rain</t>
+        </is>
+      </c>
+      <c r="B33" s="5" t="n">
+        <v>6800</v>
+      </c>
+      <c r="C33" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="4" t="inlineStr">
+        <is>
+          <t>Nobodys Son</t>
+        </is>
+      </c>
+      <c r="B34" s="5" t="n">
+        <v>9888</v>
+      </c>
+      <c r="C34" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="4" t="inlineStr">
+        <is>
+          <t>House Tour</t>
+        </is>
+      </c>
+      <c r="B35" s="5" t="n">
+        <v>7216</v>
+      </c>
+      <c r="C35" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="4" t="inlineStr">
+        <is>
+          <t>Hanabi  Î±Î·Ð²Ï…</t>
+        </is>
+      </c>
+      <c r="B36" s="5" t="n">
+        <v>7212</v>
+      </c>
+      <c r="C36" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="4" t="inlineStr">
+        <is>
+          <t>Saiyajin anbuâ„¢</t>
+        </is>
+      </c>
+      <c r="B37" s="5" t="n">
+        <v>4363</v>
+      </c>
+      <c r="C37" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="4" t="inlineStr">
+        <is>
+          <t>Dummy</t>
+        </is>
+      </c>
+      <c r="B38" s="5" t="n">
+        <v>6736</v>
+      </c>
+      <c r="C38" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="4" t="inlineStr">
+        <is>
+          <t>Cazador anbu â„¢</t>
+        </is>
+      </c>
+      <c r="B39" s="5" t="n">
+        <v>4336</v>
+      </c>
+      <c r="C39" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="4" t="inlineStr">
+        <is>
+          <t>Besos Mojados</t>
+        </is>
+      </c>
+      <c r="B40" s="5" t="n">
+        <v>4425</v>
+      </c>
+      <c r="C40" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="4" t="inlineStr">
+        <is>
+          <t>DarkFire</t>
+        </is>
+      </c>
+      <c r="B41" s="5" t="n">
+        <v>10728</v>
+      </c>
+      <c r="C41" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="4" t="inlineStr">
+        <is>
+          <t>DarkSunny</t>
+        </is>
+      </c>
+      <c r="B42" s="5" t="n">
+        <v>10994</v>
+      </c>
+      <c r="C42" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="4" t="inlineStr">
+        <is>
+          <t>Dairen Uchiha</t>
+        </is>
+      </c>
+      <c r="B43" s="5" t="n">
+        <v>11482</v>
+      </c>
+      <c r="C43" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="4" t="inlineStr">
+        <is>
+          <t>LILI ZENIN®</t>
+        </is>
+      </c>
+      <c r="B44" s="5" t="n">
+        <v>7011</v>
+      </c>
+      <c r="C44" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="4" t="inlineStr">
+        <is>
+          <t>ryumichel ZENIN ®</t>
+        </is>
+      </c>
+      <c r="B45" s="5" t="n">
+        <v>3218</v>
+      </c>
+      <c r="C45" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="4" t="inlineStr">
+        <is>
+          <t>margot ZENIN ®</t>
+        </is>
+      </c>
+      <c r="B46" s="5" t="n">
+        <v>3250</v>
+      </c>
+      <c r="C46" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="4" t="inlineStr">
+        <is>
+          <t>linda ZENIN ®</t>
+        </is>
+      </c>
+      <c r="B47" s="5" t="n">
+        <v>7111</v>
+      </c>
+      <c r="C47" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="4" t="inlineStr">
+        <is>
+          <t>SHINRAIN ZENIN®</t>
+        </is>
+      </c>
+      <c r="B48" s="5" t="n">
+        <v>6877</v>
+      </c>
+      <c r="C48" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="4" t="inlineStr">
+        <is>
+          <t>PlyRed-</t>
+        </is>
+      </c>
+      <c r="B49" s="5" t="n">
+        <v>6031</v>
+      </c>
+      <c r="C49" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="4" t="inlineStr">
+        <is>
+          <t>equin0x</t>
+        </is>
+      </c>
+      <c r="B50" s="5" t="n">
+        <v>8516</v>
+      </c>
+      <c r="C50" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="4" t="inlineStr">
+        <is>
+          <t>Jhayco - Mokai</t>
+        </is>
+      </c>
+      <c r="B51" s="5" t="n">
+        <v>10165</v>
+      </c>
+      <c r="C51" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="4" t="inlineStr">
+        <is>
+          <t>Jhayco - Joe</t>
+        </is>
+      </c>
+      <c r="B52" s="5" t="n">
+        <v>10361</v>
+      </c>
+      <c r="C52" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="4" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="B53" s="5" t="n">
+        <v>10232</v>
+      </c>
+      <c r="C53" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="4" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="B54" s="5" t="n">
+        <v>10526</v>
+      </c>
+      <c r="C54" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="4" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="B55" s="5" t="n">
+        <v>10211</v>
+      </c>
+      <c r="C55" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="4" t="inlineStr">
+        <is>
+          <t>Go Go Juice</t>
+        </is>
+      </c>
+      <c r="B56" s="5" t="n">
+        <v>7930</v>
+      </c>
+      <c r="C56" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="4" t="inlineStr">
+        <is>
+          <t>Jhayco - Imaginaste</t>
+        </is>
+      </c>
+      <c r="B57" s="5" t="n">
+        <v>4077</v>
+      </c>
+      <c r="C57" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="4" t="inlineStr">
+        <is>
+          <t>PuNch</t>
+        </is>
+      </c>
+      <c r="B58" s="5" t="n">
+        <v>7065</v>
+      </c>
+      <c r="C58" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A2:C2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
auto: snapshot 2026-08-04 13:01:00
</commit_message>
<xml_diff>
--- a/clan_3815.xlsx
+++ b/clan_3815.xlsx
@@ -27,6 +27,7 @@
     <sheet name="2026-08-01" sheetId="18" state="visible" r:id="rId18"/>
     <sheet name="2026-08-02" sheetId="19" state="visible" r:id="rId19"/>
     <sheet name="2026-08-03" sheetId="20" state="visible" r:id="rId20"/>
+    <sheet name="2026-08-04" sheetId="21" state="visible" r:id="rId21"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -10859,6 +10860,885 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet21.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C58"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="29" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Clan: Mans Best Friend (3815)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Timestamp: 2026-08-04 13:01:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>Total Reps</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>Daily Reps (+1d)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>Nobodys Son</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="n">
+        <v>7422</v>
+      </c>
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>-2466</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>Player</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="n">
+        <v>4314</v>
+      </c>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>+199</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>Player</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="n">
+        <v>4200</v>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>+85</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>X y L O T A</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="n">
+        <v>4098</v>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>AbdiHyde ID 13496</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="n">
+        <v>5427</v>
+      </c>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>Create Character III</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="n">
+        <v>7047</v>
+      </c>
+      <c r="C9" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>Create Character IV</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="n">
+        <v>7708</v>
+      </c>
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>Create Character V</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="n">
+        <v>7560</v>
+      </c>
+      <c r="C11" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t>Player</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="n">
+        <v>4174</v>
+      </c>
+      <c r="C12" s="5" t="inlineStr">
+        <is>
+          <t>+59</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="4" t="inlineStr">
+        <is>
+          <t>Player</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="n">
+        <v>4115</v>
+      </c>
+      <c r="C13" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="4" t="inlineStr">
+        <is>
+          <t>hunry</t>
+        </is>
+      </c>
+      <c r="B14" s="5" t="n">
+        <v>4204</v>
+      </c>
+      <c r="C14" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="4" t="inlineStr">
+        <is>
+          <t>Tears</t>
+        </is>
+      </c>
+      <c r="B15" s="5" t="n">
+        <v>7227</v>
+      </c>
+      <c r="C15" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="4" t="inlineStr">
+        <is>
+          <t>Sugar Talking</t>
+        </is>
+      </c>
+      <c r="B16" s="5" t="n">
+        <v>8462</v>
+      </c>
+      <c r="C16" s="5" t="inlineStr">
+        <is>
+          <t>+934</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="4" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B17" s="5" t="n">
+        <v>7523</v>
+      </c>
+      <c r="C17" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="4" t="inlineStr">
+        <is>
+          <t>Anti-Hero</t>
+        </is>
+      </c>
+      <c r="B18" s="5" t="n">
+        <v>8274</v>
+      </c>
+      <c r="C18" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="4" t="inlineStr">
+        <is>
+          <t>Vigilante Shit</t>
+        </is>
+      </c>
+      <c r="B19" s="5" t="n">
+        <v>8289</v>
+      </c>
+      <c r="C19" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="4" t="inlineStr">
+        <is>
+          <t>Sweet Nothing</t>
+        </is>
+      </c>
+      <c r="B20" s="5" t="n">
+        <v>8369</v>
+      </c>
+      <c r="C20" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="4" t="inlineStr">
+        <is>
+          <t>The Great War</t>
+        </is>
+      </c>
+      <c r="B21" s="5" t="n">
+        <v>8089</v>
+      </c>
+      <c r="C21" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">We Almost Broke Up </t>
+        </is>
+      </c>
+      <c r="B22" s="5" t="n">
+        <v>8343</v>
+      </c>
+      <c r="C22" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="4" t="inlineStr">
+        <is>
+          <t>When Did You Get Hot</t>
+        </is>
+      </c>
+      <c r="B23" s="5" t="n">
+        <v>8212</v>
+      </c>
+      <c r="C23" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="4" t="inlineStr">
+        <is>
+          <t>Dont Worry Ill Make</t>
+        </is>
+      </c>
+      <c r="B24" s="5" t="n">
+        <v>7554</v>
+      </c>
+      <c r="C24" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="4" t="inlineStr">
+        <is>
+          <t>Goodbye</t>
+        </is>
+      </c>
+      <c r="B25" s="5" t="n">
+        <v>7005</v>
+      </c>
+      <c r="C25" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="4" t="inlineStr">
+        <is>
+          <t>Mans Best Friend</t>
+        </is>
+      </c>
+      <c r="B26" s="5" t="n">
+        <v>6974</v>
+      </c>
+      <c r="C26" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="4" t="inlineStr">
+        <is>
+          <t>Lavender Haze</t>
+        </is>
+      </c>
+      <c r="B27" s="5" t="n">
+        <v>6962</v>
+      </c>
+      <c r="C27" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="4" t="inlineStr">
+        <is>
+          <t>Never Getting Laid</t>
+        </is>
+      </c>
+      <c r="B28" s="5" t="n">
+        <v>8493</v>
+      </c>
+      <c r="C28" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="4" t="inlineStr">
+        <is>
+          <t>My Man on Willpower</t>
+        </is>
+      </c>
+      <c r="B29" s="5" t="n">
+        <v>7480</v>
+      </c>
+      <c r="C29" s="5" t="inlineStr">
+        <is>
+          <t>-821</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="4" t="inlineStr">
+        <is>
+          <t>Manchild</t>
+        </is>
+      </c>
+      <c r="B30" s="5" t="n">
+        <v>8355</v>
+      </c>
+      <c r="C30" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="4" t="inlineStr">
+        <is>
+          <t>Sugar Talking</t>
+        </is>
+      </c>
+      <c r="B31" s="5" t="n">
+        <v>7528</v>
+      </c>
+      <c r="C31" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="4" t="inlineStr">
+        <is>
+          <t>My Man on Willpower</t>
+        </is>
+      </c>
+      <c r="B32" s="5" t="n">
+        <v>8301</v>
+      </c>
+      <c r="C32" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="4" t="inlineStr">
+        <is>
+          <t>Midnight Rain</t>
+        </is>
+      </c>
+      <c r="B33" s="5" t="n">
+        <v>6800</v>
+      </c>
+      <c r="C33" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="4" t="inlineStr">
+        <is>
+          <t>Nobodys Son</t>
+        </is>
+      </c>
+      <c r="B34" s="5" t="n">
+        <v>9888</v>
+      </c>
+      <c r="C34" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="4" t="inlineStr">
+        <is>
+          <t>House Tour</t>
+        </is>
+      </c>
+      <c r="B35" s="5" t="n">
+        <v>7216</v>
+      </c>
+      <c r="C35" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="4" t="inlineStr">
+        <is>
+          <t>Hanabi  Î±Î·Ð²Ï…</t>
+        </is>
+      </c>
+      <c r="B36" s="5" t="n">
+        <v>7212</v>
+      </c>
+      <c r="C36" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="4" t="inlineStr">
+        <is>
+          <t>Saiyajin anbuâ„¢</t>
+        </is>
+      </c>
+      <c r="B37" s="5" t="n">
+        <v>4363</v>
+      </c>
+      <c r="C37" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="4" t="inlineStr">
+        <is>
+          <t>Dummy</t>
+        </is>
+      </c>
+      <c r="B38" s="5" t="n">
+        <v>6736</v>
+      </c>
+      <c r="C38" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="4" t="inlineStr">
+        <is>
+          <t>Cazador anbu â„¢</t>
+        </is>
+      </c>
+      <c r="B39" s="5" t="n">
+        <v>4336</v>
+      </c>
+      <c r="C39" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="4" t="inlineStr">
+        <is>
+          <t>Besos Mojados</t>
+        </is>
+      </c>
+      <c r="B40" s="5" t="n">
+        <v>4425</v>
+      </c>
+      <c r="C40" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="4" t="inlineStr">
+        <is>
+          <t>DarkFire</t>
+        </is>
+      </c>
+      <c r="B41" s="5" t="n">
+        <v>10728</v>
+      </c>
+      <c r="C41" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="4" t="inlineStr">
+        <is>
+          <t>DarkSunny</t>
+        </is>
+      </c>
+      <c r="B42" s="5" t="n">
+        <v>10994</v>
+      </c>
+      <c r="C42" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="4" t="inlineStr">
+        <is>
+          <t>Dairen Uchiha</t>
+        </is>
+      </c>
+      <c r="B43" s="5" t="n">
+        <v>11482</v>
+      </c>
+      <c r="C43" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="4" t="inlineStr">
+        <is>
+          <t>LILI ZENIN®</t>
+        </is>
+      </c>
+      <c r="B44" s="5" t="n">
+        <v>7019</v>
+      </c>
+      <c r="C44" s="5" t="inlineStr">
+        <is>
+          <t>+8</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="4" t="inlineStr">
+        <is>
+          <t>ryumichel ZENIN ®</t>
+        </is>
+      </c>
+      <c r="B45" s="5" t="n">
+        <v>3218</v>
+      </c>
+      <c r="C45" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="4" t="inlineStr">
+        <is>
+          <t>margot ZENIN ®</t>
+        </is>
+      </c>
+      <c r="B46" s="5" t="n">
+        <v>3250</v>
+      </c>
+      <c r="C46" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="4" t="inlineStr">
+        <is>
+          <t>linda ZENIN ®</t>
+        </is>
+      </c>
+      <c r="B47" s="5" t="n">
+        <v>7111</v>
+      </c>
+      <c r="C47" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="4" t="inlineStr">
+        <is>
+          <t>SHINRAIN ZENIN®</t>
+        </is>
+      </c>
+      <c r="B48" s="5" t="n">
+        <v>6877</v>
+      </c>
+      <c r="C48" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="4" t="inlineStr">
+        <is>
+          <t>PlyRed-</t>
+        </is>
+      </c>
+      <c r="B49" s="5" t="n">
+        <v>6031</v>
+      </c>
+      <c r="C49" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="4" t="inlineStr">
+        <is>
+          <t>equin0x</t>
+        </is>
+      </c>
+      <c r="B50" s="5" t="n">
+        <v>8516</v>
+      </c>
+      <c r="C50" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="4" t="inlineStr">
+        <is>
+          <t>Jhayco - Mokai</t>
+        </is>
+      </c>
+      <c r="B51" s="5" t="n">
+        <v>10165</v>
+      </c>
+      <c r="C51" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="4" t="inlineStr">
+        <is>
+          <t>Jhayco - Joe</t>
+        </is>
+      </c>
+      <c r="B52" s="5" t="n">
+        <v>10361</v>
+      </c>
+      <c r="C52" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="4" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="B53" s="5" t="n">
+        <v>10232</v>
+      </c>
+      <c r="C53" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="4" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="B54" s="5" t="n">
+        <v>10526</v>
+      </c>
+      <c r="C54" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="4" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="B55" s="5" t="n">
+        <v>10211</v>
+      </c>
+      <c r="C55" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="4" t="inlineStr">
+        <is>
+          <t>Go Go Juice</t>
+        </is>
+      </c>
+      <c r="B56" s="5" t="n">
+        <v>7930</v>
+      </c>
+      <c r="C56" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="4" t="inlineStr">
+        <is>
+          <t>Jhayco - Imaginaste</t>
+        </is>
+      </c>
+      <c r="B57" s="5" t="n">
+        <v>4077</v>
+      </c>
+      <c r="C57" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="4" t="inlineStr">
+        <is>
+          <t>PuNch</t>
+        </is>
+      </c>
+      <c r="B58" s="5" t="n">
+        <v>7065</v>
+      </c>
+      <c r="C58" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A2:C2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
auto: snapshot 2026-08-05 13:01:00
</commit_message>
<xml_diff>
--- a/clan_3815.xlsx
+++ b/clan_3815.xlsx
@@ -28,6 +28,7 @@
     <sheet name="2026-08-02" sheetId="19" state="visible" r:id="rId19"/>
     <sheet name="2026-08-03" sheetId="20" state="visible" r:id="rId20"/>
     <sheet name="2026-08-04" sheetId="21" state="visible" r:id="rId21"/>
+    <sheet name="2026-08-05" sheetId="22" state="visible" r:id="rId22"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -11739,6 +11740,885 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet22.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C58"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="29" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Clan: Mans Best Friend (3815)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Timestamp: 2026-08-05 13:01:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>Total Reps</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>Daily Reps (+1d)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>Nobodys Son</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="n">
+        <v>7422</v>
+      </c>
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>-2466</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>Player</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="n">
+        <v>4314</v>
+      </c>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>+199</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>Player</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="n">
+        <v>4200</v>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>+85</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>X y L O T A</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="n">
+        <v>4098</v>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>AbdiHyde ID 13496</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="n">
+        <v>5427</v>
+      </c>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>Create Character III</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="n">
+        <v>7047</v>
+      </c>
+      <c r="C9" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>Create Character IV</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="n">
+        <v>7708</v>
+      </c>
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>Create Character V</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="n">
+        <v>7560</v>
+      </c>
+      <c r="C11" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t>Player</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="n">
+        <v>4174</v>
+      </c>
+      <c r="C12" s="5" t="inlineStr">
+        <is>
+          <t>+59</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="4" t="inlineStr">
+        <is>
+          <t>Player</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="n">
+        <v>4115</v>
+      </c>
+      <c r="C13" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="4" t="inlineStr">
+        <is>
+          <t>hunry</t>
+        </is>
+      </c>
+      <c r="B14" s="5" t="n">
+        <v>4204</v>
+      </c>
+      <c r="C14" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="4" t="inlineStr">
+        <is>
+          <t>Tears</t>
+        </is>
+      </c>
+      <c r="B15" s="5" t="n">
+        <v>7227</v>
+      </c>
+      <c r="C15" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="4" t="inlineStr">
+        <is>
+          <t>Sugar Talking</t>
+        </is>
+      </c>
+      <c r="B16" s="5" t="n">
+        <v>8462</v>
+      </c>
+      <c r="C16" s="5" t="inlineStr">
+        <is>
+          <t>+934</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="4" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B17" s="5" t="n">
+        <v>7523</v>
+      </c>
+      <c r="C17" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="4" t="inlineStr">
+        <is>
+          <t>Anti-Hero</t>
+        </is>
+      </c>
+      <c r="B18" s="5" t="n">
+        <v>8274</v>
+      </c>
+      <c r="C18" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="4" t="inlineStr">
+        <is>
+          <t>Vigilante Shit</t>
+        </is>
+      </c>
+      <c r="B19" s="5" t="n">
+        <v>8289</v>
+      </c>
+      <c r="C19" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="4" t="inlineStr">
+        <is>
+          <t>Sweet Nothing</t>
+        </is>
+      </c>
+      <c r="B20" s="5" t="n">
+        <v>8369</v>
+      </c>
+      <c r="C20" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="4" t="inlineStr">
+        <is>
+          <t>The Great War</t>
+        </is>
+      </c>
+      <c r="B21" s="5" t="n">
+        <v>8089</v>
+      </c>
+      <c r="C21" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">We Almost Broke Up </t>
+        </is>
+      </c>
+      <c r="B22" s="5" t="n">
+        <v>8343</v>
+      </c>
+      <c r="C22" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="4" t="inlineStr">
+        <is>
+          <t>When Did You Get Hot</t>
+        </is>
+      </c>
+      <c r="B23" s="5" t="n">
+        <v>8212</v>
+      </c>
+      <c r="C23" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="4" t="inlineStr">
+        <is>
+          <t>Dont Worry Ill Make</t>
+        </is>
+      </c>
+      <c r="B24" s="5" t="n">
+        <v>7554</v>
+      </c>
+      <c r="C24" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="4" t="inlineStr">
+        <is>
+          <t>Goodbye</t>
+        </is>
+      </c>
+      <c r="B25" s="5" t="n">
+        <v>7005</v>
+      </c>
+      <c r="C25" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="4" t="inlineStr">
+        <is>
+          <t>Mans Best Friend</t>
+        </is>
+      </c>
+      <c r="B26" s="5" t="n">
+        <v>6974</v>
+      </c>
+      <c r="C26" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="4" t="inlineStr">
+        <is>
+          <t>Lavender Haze</t>
+        </is>
+      </c>
+      <c r="B27" s="5" t="n">
+        <v>6962</v>
+      </c>
+      <c r="C27" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="4" t="inlineStr">
+        <is>
+          <t>Never Getting Laid</t>
+        </is>
+      </c>
+      <c r="B28" s="5" t="n">
+        <v>8493</v>
+      </c>
+      <c r="C28" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="4" t="inlineStr">
+        <is>
+          <t>My Man on Willpower</t>
+        </is>
+      </c>
+      <c r="B29" s="5" t="n">
+        <v>7480</v>
+      </c>
+      <c r="C29" s="5" t="inlineStr">
+        <is>
+          <t>-821</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="4" t="inlineStr">
+        <is>
+          <t>Manchild</t>
+        </is>
+      </c>
+      <c r="B30" s="5" t="n">
+        <v>8355</v>
+      </c>
+      <c r="C30" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="4" t="inlineStr">
+        <is>
+          <t>Sugar Talking</t>
+        </is>
+      </c>
+      <c r="B31" s="5" t="n">
+        <v>7528</v>
+      </c>
+      <c r="C31" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="4" t="inlineStr">
+        <is>
+          <t>My Man on Willpower</t>
+        </is>
+      </c>
+      <c r="B32" s="5" t="n">
+        <v>8301</v>
+      </c>
+      <c r="C32" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="4" t="inlineStr">
+        <is>
+          <t>Midnight Rain</t>
+        </is>
+      </c>
+      <c r="B33" s="5" t="n">
+        <v>6800</v>
+      </c>
+      <c r="C33" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="4" t="inlineStr">
+        <is>
+          <t>Nobodys Son</t>
+        </is>
+      </c>
+      <c r="B34" s="5" t="n">
+        <v>9888</v>
+      </c>
+      <c r="C34" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="4" t="inlineStr">
+        <is>
+          <t>House Tour</t>
+        </is>
+      </c>
+      <c r="B35" s="5" t="n">
+        <v>7216</v>
+      </c>
+      <c r="C35" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="4" t="inlineStr">
+        <is>
+          <t>Hanabi  Î±Î·Ð²Ï…</t>
+        </is>
+      </c>
+      <c r="B36" s="5" t="n">
+        <v>7212</v>
+      </c>
+      <c r="C36" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="4" t="inlineStr">
+        <is>
+          <t>Saiyajin anbuâ„¢</t>
+        </is>
+      </c>
+      <c r="B37" s="5" t="n">
+        <v>4363</v>
+      </c>
+      <c r="C37" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="4" t="inlineStr">
+        <is>
+          <t>Dummy</t>
+        </is>
+      </c>
+      <c r="B38" s="5" t="n">
+        <v>6736</v>
+      </c>
+      <c r="C38" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="4" t="inlineStr">
+        <is>
+          <t>Cazador anbu â„¢</t>
+        </is>
+      </c>
+      <c r="B39" s="5" t="n">
+        <v>4336</v>
+      </c>
+      <c r="C39" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="4" t="inlineStr">
+        <is>
+          <t>Besos Mojados</t>
+        </is>
+      </c>
+      <c r="B40" s="5" t="n">
+        <v>4425</v>
+      </c>
+      <c r="C40" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="4" t="inlineStr">
+        <is>
+          <t>DarkFire</t>
+        </is>
+      </c>
+      <c r="B41" s="5" t="n">
+        <v>10728</v>
+      </c>
+      <c r="C41" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="4" t="inlineStr">
+        <is>
+          <t>DarkSunny</t>
+        </is>
+      </c>
+      <c r="B42" s="5" t="n">
+        <v>10994</v>
+      </c>
+      <c r="C42" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="4" t="inlineStr">
+        <is>
+          <t>Dairen Uchiha</t>
+        </is>
+      </c>
+      <c r="B43" s="5" t="n">
+        <v>11482</v>
+      </c>
+      <c r="C43" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="4" t="inlineStr">
+        <is>
+          <t>LILI ZENIN®</t>
+        </is>
+      </c>
+      <c r="B44" s="5" t="n">
+        <v>7019</v>
+      </c>
+      <c r="C44" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="4" t="inlineStr">
+        <is>
+          <t>ryumichel ZENIN ®</t>
+        </is>
+      </c>
+      <c r="B45" s="5" t="n">
+        <v>3218</v>
+      </c>
+      <c r="C45" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="4" t="inlineStr">
+        <is>
+          <t>margot ZENIN ®</t>
+        </is>
+      </c>
+      <c r="B46" s="5" t="n">
+        <v>3250</v>
+      </c>
+      <c r="C46" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="4" t="inlineStr">
+        <is>
+          <t>linda ZENIN ®</t>
+        </is>
+      </c>
+      <c r="B47" s="5" t="n">
+        <v>7111</v>
+      </c>
+      <c r="C47" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="4" t="inlineStr">
+        <is>
+          <t>SHINRAIN ZENIN®</t>
+        </is>
+      </c>
+      <c r="B48" s="5" t="n">
+        <v>6877</v>
+      </c>
+      <c r="C48" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="4" t="inlineStr">
+        <is>
+          <t>PlyRed-</t>
+        </is>
+      </c>
+      <c r="B49" s="5" t="n">
+        <v>6031</v>
+      </c>
+      <c r="C49" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="4" t="inlineStr">
+        <is>
+          <t>equin0x</t>
+        </is>
+      </c>
+      <c r="B50" s="5" t="n">
+        <v>8516</v>
+      </c>
+      <c r="C50" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="4" t="inlineStr">
+        <is>
+          <t>Jhayco - Mokai</t>
+        </is>
+      </c>
+      <c r="B51" s="5" t="n">
+        <v>10165</v>
+      </c>
+      <c r="C51" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="4" t="inlineStr">
+        <is>
+          <t>Jhayco - Joe</t>
+        </is>
+      </c>
+      <c r="B52" s="5" t="n">
+        <v>10361</v>
+      </c>
+      <c r="C52" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="4" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="B53" s="5" t="n">
+        <v>10232</v>
+      </c>
+      <c r="C53" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="4" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="B54" s="5" t="n">
+        <v>10526</v>
+      </c>
+      <c r="C54" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="4" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="B55" s="5" t="n">
+        <v>10211</v>
+      </c>
+      <c r="C55" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="4" t="inlineStr">
+        <is>
+          <t>Go Go Juice</t>
+        </is>
+      </c>
+      <c r="B56" s="5" t="n">
+        <v>7930</v>
+      </c>
+      <c r="C56" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="4" t="inlineStr">
+        <is>
+          <t>Jhayco - Imaginaste</t>
+        </is>
+      </c>
+      <c r="B57" s="5" t="n">
+        <v>4077</v>
+      </c>
+      <c r="C57" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="4" t="inlineStr">
+        <is>
+          <t>PuNch</t>
+        </is>
+      </c>
+      <c r="B58" s="5" t="n">
+        <v>7065</v>
+      </c>
+      <c r="C58" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A2:C2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
auto: snapshot 2026-08-06 13:01:00
</commit_message>
<xml_diff>
--- a/clan_3815.xlsx
+++ b/clan_3815.xlsx
@@ -29,6 +29,7 @@
     <sheet name="2026-08-03" sheetId="20" state="visible" r:id="rId20"/>
     <sheet name="2026-08-04" sheetId="21" state="visible" r:id="rId21"/>
     <sheet name="2026-08-05" sheetId="22" state="visible" r:id="rId22"/>
+    <sheet name="2026-08-06" sheetId="23" state="visible" r:id="rId23"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -12619,6 +12620,885 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet23.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C58"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="29" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Clan: Mans Best Friend (3815)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Timestamp: 2026-08-06 13:01:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>Total Reps</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>Daily Reps (+1d)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>Nobodys Son</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="n">
+        <v>7422</v>
+      </c>
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>-2466</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>Player</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="n">
+        <v>4314</v>
+      </c>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>+199</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>Player</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="n">
+        <v>4200</v>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>+85</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>X y L O T A</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="n">
+        <v>4098</v>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>AbdiHyde ID 13496</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="n">
+        <v>5427</v>
+      </c>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>Create Character III</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="n">
+        <v>7047</v>
+      </c>
+      <c r="C9" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>Create Character IV</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="n">
+        <v>7708</v>
+      </c>
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>Create Character V</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="n">
+        <v>7560</v>
+      </c>
+      <c r="C11" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t>Player</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="n">
+        <v>4174</v>
+      </c>
+      <c r="C12" s="5" t="inlineStr">
+        <is>
+          <t>+59</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="4" t="inlineStr">
+        <is>
+          <t>Player</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="n">
+        <v>4115</v>
+      </c>
+      <c r="C13" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="4" t="inlineStr">
+        <is>
+          <t>hunry</t>
+        </is>
+      </c>
+      <c r="B14" s="5" t="n">
+        <v>4204</v>
+      </c>
+      <c r="C14" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="4" t="inlineStr">
+        <is>
+          <t>Tears</t>
+        </is>
+      </c>
+      <c r="B15" s="5" t="n">
+        <v>7227</v>
+      </c>
+      <c r="C15" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="4" t="inlineStr">
+        <is>
+          <t>Sugar Talking</t>
+        </is>
+      </c>
+      <c r="B16" s="5" t="n">
+        <v>8462</v>
+      </c>
+      <c r="C16" s="5" t="inlineStr">
+        <is>
+          <t>+934</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="4" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B17" s="5" t="n">
+        <v>7523</v>
+      </c>
+      <c r="C17" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="4" t="inlineStr">
+        <is>
+          <t>Anti-Hero</t>
+        </is>
+      </c>
+      <c r="B18" s="5" t="n">
+        <v>8274</v>
+      </c>
+      <c r="C18" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="4" t="inlineStr">
+        <is>
+          <t>Vigilante Shit</t>
+        </is>
+      </c>
+      <c r="B19" s="5" t="n">
+        <v>8289</v>
+      </c>
+      <c r="C19" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="4" t="inlineStr">
+        <is>
+          <t>Sweet Nothing</t>
+        </is>
+      </c>
+      <c r="B20" s="5" t="n">
+        <v>8369</v>
+      </c>
+      <c r="C20" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="4" t="inlineStr">
+        <is>
+          <t>The Great War</t>
+        </is>
+      </c>
+      <c r="B21" s="5" t="n">
+        <v>8089</v>
+      </c>
+      <c r="C21" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">We Almost Broke Up </t>
+        </is>
+      </c>
+      <c r="B22" s="5" t="n">
+        <v>8343</v>
+      </c>
+      <c r="C22" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="4" t="inlineStr">
+        <is>
+          <t>When Did You Get Hot</t>
+        </is>
+      </c>
+      <c r="B23" s="5" t="n">
+        <v>8212</v>
+      </c>
+      <c r="C23" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="4" t="inlineStr">
+        <is>
+          <t>Dont Worry Ill Make</t>
+        </is>
+      </c>
+      <c r="B24" s="5" t="n">
+        <v>7554</v>
+      </c>
+      <c r="C24" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="4" t="inlineStr">
+        <is>
+          <t>Goodbye</t>
+        </is>
+      </c>
+      <c r="B25" s="5" t="n">
+        <v>7005</v>
+      </c>
+      <c r="C25" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="4" t="inlineStr">
+        <is>
+          <t>Mans Best Friend</t>
+        </is>
+      </c>
+      <c r="B26" s="5" t="n">
+        <v>6974</v>
+      </c>
+      <c r="C26" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="4" t="inlineStr">
+        <is>
+          <t>Lavender Haze</t>
+        </is>
+      </c>
+      <c r="B27" s="5" t="n">
+        <v>6962</v>
+      </c>
+      <c r="C27" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="4" t="inlineStr">
+        <is>
+          <t>Never Getting Laid</t>
+        </is>
+      </c>
+      <c r="B28" s="5" t="n">
+        <v>8493</v>
+      </c>
+      <c r="C28" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="4" t="inlineStr">
+        <is>
+          <t>My Man on Willpower</t>
+        </is>
+      </c>
+      <c r="B29" s="5" t="n">
+        <v>7480</v>
+      </c>
+      <c r="C29" s="5" t="inlineStr">
+        <is>
+          <t>-821</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="4" t="inlineStr">
+        <is>
+          <t>Manchild</t>
+        </is>
+      </c>
+      <c r="B30" s="5" t="n">
+        <v>8355</v>
+      </c>
+      <c r="C30" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="4" t="inlineStr">
+        <is>
+          <t>Sugar Talking</t>
+        </is>
+      </c>
+      <c r="B31" s="5" t="n">
+        <v>7528</v>
+      </c>
+      <c r="C31" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="4" t="inlineStr">
+        <is>
+          <t>My Man on Willpower</t>
+        </is>
+      </c>
+      <c r="B32" s="5" t="n">
+        <v>8301</v>
+      </c>
+      <c r="C32" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="4" t="inlineStr">
+        <is>
+          <t>Midnight Rain</t>
+        </is>
+      </c>
+      <c r="B33" s="5" t="n">
+        <v>6800</v>
+      </c>
+      <c r="C33" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="4" t="inlineStr">
+        <is>
+          <t>Nobodys Son</t>
+        </is>
+      </c>
+      <c r="B34" s="5" t="n">
+        <v>9888</v>
+      </c>
+      <c r="C34" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="4" t="inlineStr">
+        <is>
+          <t>House Tour</t>
+        </is>
+      </c>
+      <c r="B35" s="5" t="n">
+        <v>7216</v>
+      </c>
+      <c r="C35" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="4" t="inlineStr">
+        <is>
+          <t>Hanabi  Î±Î·Ð²Ï…</t>
+        </is>
+      </c>
+      <c r="B36" s="5" t="n">
+        <v>7212</v>
+      </c>
+      <c r="C36" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="4" t="inlineStr">
+        <is>
+          <t>Saiyajin anbuâ„¢</t>
+        </is>
+      </c>
+      <c r="B37" s="5" t="n">
+        <v>4363</v>
+      </c>
+      <c r="C37" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="4" t="inlineStr">
+        <is>
+          <t>Dummy</t>
+        </is>
+      </c>
+      <c r="B38" s="5" t="n">
+        <v>6736</v>
+      </c>
+      <c r="C38" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="4" t="inlineStr">
+        <is>
+          <t>Cazador anbu â„¢</t>
+        </is>
+      </c>
+      <c r="B39" s="5" t="n">
+        <v>4336</v>
+      </c>
+      <c r="C39" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="4" t="inlineStr">
+        <is>
+          <t>Besos Mojados</t>
+        </is>
+      </c>
+      <c r="B40" s="5" t="n">
+        <v>4425</v>
+      </c>
+      <c r="C40" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="4" t="inlineStr">
+        <is>
+          <t>DarkFire</t>
+        </is>
+      </c>
+      <c r="B41" s="5" t="n">
+        <v>10728</v>
+      </c>
+      <c r="C41" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="4" t="inlineStr">
+        <is>
+          <t>DarkSunny</t>
+        </is>
+      </c>
+      <c r="B42" s="5" t="n">
+        <v>10994</v>
+      </c>
+      <c r="C42" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="4" t="inlineStr">
+        <is>
+          <t>Dairen Uchiha</t>
+        </is>
+      </c>
+      <c r="B43" s="5" t="n">
+        <v>11482</v>
+      </c>
+      <c r="C43" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="4" t="inlineStr">
+        <is>
+          <t>LILI ZENIN®</t>
+        </is>
+      </c>
+      <c r="B44" s="5" t="n">
+        <v>7019</v>
+      </c>
+      <c r="C44" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="4" t="inlineStr">
+        <is>
+          <t>ryumichel ZENIN ®</t>
+        </is>
+      </c>
+      <c r="B45" s="5" t="n">
+        <v>3218</v>
+      </c>
+      <c r="C45" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="4" t="inlineStr">
+        <is>
+          <t>margot ZENIN ®</t>
+        </is>
+      </c>
+      <c r="B46" s="5" t="n">
+        <v>3250</v>
+      </c>
+      <c r="C46" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="4" t="inlineStr">
+        <is>
+          <t>linda ZENIN ®</t>
+        </is>
+      </c>
+      <c r="B47" s="5" t="n">
+        <v>7111</v>
+      </c>
+      <c r="C47" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="4" t="inlineStr">
+        <is>
+          <t>SHINRAIN ZENIN®</t>
+        </is>
+      </c>
+      <c r="B48" s="5" t="n">
+        <v>6877</v>
+      </c>
+      <c r="C48" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="4" t="inlineStr">
+        <is>
+          <t>PlyRed-</t>
+        </is>
+      </c>
+      <c r="B49" s="5" t="n">
+        <v>6031</v>
+      </c>
+      <c r="C49" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="4" t="inlineStr">
+        <is>
+          <t>equin0x</t>
+        </is>
+      </c>
+      <c r="B50" s="5" t="n">
+        <v>8516</v>
+      </c>
+      <c r="C50" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="4" t="inlineStr">
+        <is>
+          <t>Jhayco - Mokai</t>
+        </is>
+      </c>
+      <c r="B51" s="5" t="n">
+        <v>10165</v>
+      </c>
+      <c r="C51" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="4" t="inlineStr">
+        <is>
+          <t>Jhayco - Joe</t>
+        </is>
+      </c>
+      <c r="B52" s="5" t="n">
+        <v>10361</v>
+      </c>
+      <c r="C52" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="4" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="B53" s="5" t="n">
+        <v>10232</v>
+      </c>
+      <c r="C53" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="4" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="B54" s="5" t="n">
+        <v>10526</v>
+      </c>
+      <c r="C54" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="4" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="B55" s="5" t="n">
+        <v>10211</v>
+      </c>
+      <c r="C55" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="4" t="inlineStr">
+        <is>
+          <t>Go Go Juice</t>
+        </is>
+      </c>
+      <c r="B56" s="5" t="n">
+        <v>7930</v>
+      </c>
+      <c r="C56" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="4" t="inlineStr">
+        <is>
+          <t>Jhayco - Imaginaste</t>
+        </is>
+      </c>
+      <c r="B57" s="5" t="n">
+        <v>4077</v>
+      </c>
+      <c r="C57" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="4" t="inlineStr">
+        <is>
+          <t>PuNch</t>
+        </is>
+      </c>
+      <c r="B58" s="5" t="n">
+        <v>7065</v>
+      </c>
+      <c r="C58" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A2:C2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
auto: snapshot 2026-08-07 13:01:00
</commit_message>
<xml_diff>
--- a/clan_3815.xlsx
+++ b/clan_3815.xlsx
@@ -30,6 +30,7 @@
     <sheet name="2026-08-04" sheetId="21" state="visible" r:id="rId21"/>
     <sheet name="2026-08-05" sheetId="22" state="visible" r:id="rId22"/>
     <sheet name="2026-08-06" sheetId="23" state="visible" r:id="rId23"/>
+    <sheet name="2026-08-07" sheetId="24" state="visible" r:id="rId24"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -13499,6 +13500,870 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet24.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C57"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="29" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Clan: Mans Best Friend (3815)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Timestamp: 2026-08-07 13:01:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>Total Reps</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>Daily Reps (+1d)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>Nobodys Son</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="n">
+        <v>7422</v>
+      </c>
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>-2466</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>Player</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="n">
+        <v>4314</v>
+      </c>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>+199</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>Player</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="n">
+        <v>4200</v>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>+85</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>X y L O T A</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="n">
+        <v>4098</v>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>AbdiHyde ID 13496</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="n">
+        <v>5427</v>
+      </c>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>Create Character III</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="n">
+        <v>7047</v>
+      </c>
+      <c r="C9" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>Create Character IV</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="n">
+        <v>7708</v>
+      </c>
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>Create Character V</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="n">
+        <v>7560</v>
+      </c>
+      <c r="C11" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t>Player</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="n">
+        <v>4174</v>
+      </c>
+      <c r="C12" s="5" t="inlineStr">
+        <is>
+          <t>+59</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="4" t="inlineStr">
+        <is>
+          <t>Player</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="n">
+        <v>4115</v>
+      </c>
+      <c r="C13" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="4" t="inlineStr">
+        <is>
+          <t>hunry</t>
+        </is>
+      </c>
+      <c r="B14" s="5" t="n">
+        <v>4204</v>
+      </c>
+      <c r="C14" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="4" t="inlineStr">
+        <is>
+          <t>Tears</t>
+        </is>
+      </c>
+      <c r="B15" s="5" t="n">
+        <v>7227</v>
+      </c>
+      <c r="C15" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="4" t="inlineStr">
+        <is>
+          <t>Sugar Talking</t>
+        </is>
+      </c>
+      <c r="B16" s="5" t="n">
+        <v>8462</v>
+      </c>
+      <c r="C16" s="5" t="inlineStr">
+        <is>
+          <t>+934</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="4" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B17" s="5" t="n">
+        <v>7523</v>
+      </c>
+      <c r="C17" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="4" t="inlineStr">
+        <is>
+          <t>Anti-Hero</t>
+        </is>
+      </c>
+      <c r="B18" s="5" t="n">
+        <v>8274</v>
+      </c>
+      <c r="C18" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="4" t="inlineStr">
+        <is>
+          <t>Vigilante Shit</t>
+        </is>
+      </c>
+      <c r="B19" s="5" t="n">
+        <v>8289</v>
+      </c>
+      <c r="C19" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="4" t="inlineStr">
+        <is>
+          <t>Sweet Nothing</t>
+        </is>
+      </c>
+      <c r="B20" s="5" t="n">
+        <v>8369</v>
+      </c>
+      <c r="C20" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="4" t="inlineStr">
+        <is>
+          <t>The Great War</t>
+        </is>
+      </c>
+      <c r="B21" s="5" t="n">
+        <v>8089</v>
+      </c>
+      <c r="C21" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">We Almost Broke Up </t>
+        </is>
+      </c>
+      <c r="B22" s="5" t="n">
+        <v>8343</v>
+      </c>
+      <c r="C22" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="4" t="inlineStr">
+        <is>
+          <t>When Did You Get Hot</t>
+        </is>
+      </c>
+      <c r="B23" s="5" t="n">
+        <v>8212</v>
+      </c>
+      <c r="C23" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="4" t="inlineStr">
+        <is>
+          <t>Dont Worry Ill Make</t>
+        </is>
+      </c>
+      <c r="B24" s="5" t="n">
+        <v>7554</v>
+      </c>
+      <c r="C24" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="4" t="inlineStr">
+        <is>
+          <t>Goodbye</t>
+        </is>
+      </c>
+      <c r="B25" s="5" t="n">
+        <v>7005</v>
+      </c>
+      <c r="C25" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="4" t="inlineStr">
+        <is>
+          <t>Mans Best Friend</t>
+        </is>
+      </c>
+      <c r="B26" s="5" t="n">
+        <v>6974</v>
+      </c>
+      <c r="C26" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="4" t="inlineStr">
+        <is>
+          <t>Lavender Haze</t>
+        </is>
+      </c>
+      <c r="B27" s="5" t="n">
+        <v>6962</v>
+      </c>
+      <c r="C27" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="4" t="inlineStr">
+        <is>
+          <t>Never Getting Laid</t>
+        </is>
+      </c>
+      <c r="B28" s="5" t="n">
+        <v>8493</v>
+      </c>
+      <c r="C28" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="4" t="inlineStr">
+        <is>
+          <t>My Man on Willpower</t>
+        </is>
+      </c>
+      <c r="B29" s="5" t="n">
+        <v>7480</v>
+      </c>
+      <c r="C29" s="5" t="inlineStr">
+        <is>
+          <t>-821</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="4" t="inlineStr">
+        <is>
+          <t>Manchild</t>
+        </is>
+      </c>
+      <c r="B30" s="5" t="n">
+        <v>8355</v>
+      </c>
+      <c r="C30" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="4" t="inlineStr">
+        <is>
+          <t>Sugar Talking</t>
+        </is>
+      </c>
+      <c r="B31" s="5" t="n">
+        <v>7528</v>
+      </c>
+      <c r="C31" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="4" t="inlineStr">
+        <is>
+          <t>My Man on Willpower</t>
+        </is>
+      </c>
+      <c r="B32" s="5" t="n">
+        <v>8301</v>
+      </c>
+      <c r="C32" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="4" t="inlineStr">
+        <is>
+          <t>Midnight Rain</t>
+        </is>
+      </c>
+      <c r="B33" s="5" t="n">
+        <v>6800</v>
+      </c>
+      <c r="C33" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="4" t="inlineStr">
+        <is>
+          <t>Nobodys Son</t>
+        </is>
+      </c>
+      <c r="B34" s="5" t="n">
+        <v>9888</v>
+      </c>
+      <c r="C34" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="4" t="inlineStr">
+        <is>
+          <t>House Tour</t>
+        </is>
+      </c>
+      <c r="B35" s="5" t="n">
+        <v>7216</v>
+      </c>
+      <c r="C35" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="4" t="inlineStr">
+        <is>
+          <t>Hanabi  Î±Î·Ð²Ï…</t>
+        </is>
+      </c>
+      <c r="B36" s="5" t="n">
+        <v>7212</v>
+      </c>
+      <c r="C36" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="4" t="inlineStr">
+        <is>
+          <t>Saiyajin anbuâ„¢</t>
+        </is>
+      </c>
+      <c r="B37" s="5" t="n">
+        <v>4363</v>
+      </c>
+      <c r="C37" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="4" t="inlineStr">
+        <is>
+          <t>Dummy</t>
+        </is>
+      </c>
+      <c r="B38" s="5" t="n">
+        <v>6736</v>
+      </c>
+      <c r="C38" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="4" t="inlineStr">
+        <is>
+          <t>Cazador anbu â„¢</t>
+        </is>
+      </c>
+      <c r="B39" s="5" t="n">
+        <v>4336</v>
+      </c>
+      <c r="C39" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="4" t="inlineStr">
+        <is>
+          <t>Besos Mojados</t>
+        </is>
+      </c>
+      <c r="B40" s="5" t="n">
+        <v>4425</v>
+      </c>
+      <c r="C40" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="4" t="inlineStr">
+        <is>
+          <t>DarkFire</t>
+        </is>
+      </c>
+      <c r="B41" s="5" t="n">
+        <v>10728</v>
+      </c>
+      <c r="C41" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="4" t="inlineStr">
+        <is>
+          <t>DarkSunny</t>
+        </is>
+      </c>
+      <c r="B42" s="5" t="n">
+        <v>10994</v>
+      </c>
+      <c r="C42" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="4" t="inlineStr">
+        <is>
+          <t>Dairen Uchiha</t>
+        </is>
+      </c>
+      <c r="B43" s="5" t="n">
+        <v>11482</v>
+      </c>
+      <c r="C43" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="4" t="inlineStr">
+        <is>
+          <t>LILI ZENIN®</t>
+        </is>
+      </c>
+      <c r="B44" s="5" t="n">
+        <v>7019</v>
+      </c>
+      <c r="C44" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="4" t="inlineStr">
+        <is>
+          <t>ryumichel ZENIN ®</t>
+        </is>
+      </c>
+      <c r="B45" s="5" t="n">
+        <v>3218</v>
+      </c>
+      <c r="C45" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="4" t="inlineStr">
+        <is>
+          <t>margot ZENIN ®</t>
+        </is>
+      </c>
+      <c r="B46" s="5" t="n">
+        <v>3250</v>
+      </c>
+      <c r="C46" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="4" t="inlineStr">
+        <is>
+          <t>linda ZENIN ®</t>
+        </is>
+      </c>
+      <c r="B47" s="5" t="n">
+        <v>7111</v>
+      </c>
+      <c r="C47" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="4" t="inlineStr">
+        <is>
+          <t>PlyRed-</t>
+        </is>
+      </c>
+      <c r="B48" s="5" t="n">
+        <v>6031</v>
+      </c>
+      <c r="C48" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="4" t="inlineStr">
+        <is>
+          <t>equin0x</t>
+        </is>
+      </c>
+      <c r="B49" s="5" t="n">
+        <v>8516</v>
+      </c>
+      <c r="C49" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="4" t="inlineStr">
+        <is>
+          <t>Jhayco - Mokai</t>
+        </is>
+      </c>
+      <c r="B50" s="5" t="n">
+        <v>10165</v>
+      </c>
+      <c r="C50" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="4" t="inlineStr">
+        <is>
+          <t>Jhayco - Joe</t>
+        </is>
+      </c>
+      <c r="B51" s="5" t="n">
+        <v>10361</v>
+      </c>
+      <c r="C51" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="4" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="B52" s="5" t="n">
+        <v>10232</v>
+      </c>
+      <c r="C52" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="4" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="B53" s="5" t="n">
+        <v>10526</v>
+      </c>
+      <c r="C53" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="4" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="B54" s="5" t="n">
+        <v>10211</v>
+      </c>
+      <c r="C54" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="4" t="inlineStr">
+        <is>
+          <t>Go Go Juice</t>
+        </is>
+      </c>
+      <c r="B55" s="5" t="n">
+        <v>7930</v>
+      </c>
+      <c r="C55" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="4" t="inlineStr">
+        <is>
+          <t>Jhayco - Imaginaste</t>
+        </is>
+      </c>
+      <c r="B56" s="5" t="n">
+        <v>4077</v>
+      </c>
+      <c r="C56" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="4" t="inlineStr">
+        <is>
+          <t>PuNch</t>
+        </is>
+      </c>
+      <c r="B57" s="5" t="n">
+        <v>7065</v>
+      </c>
+      <c r="C57" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A2:C2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
auto: snapshot 2026-08-08 13:01:00
</commit_message>
<xml_diff>
--- a/clan_3815.xlsx
+++ b/clan_3815.xlsx
@@ -31,6 +31,7 @@
     <sheet name="2026-08-05" sheetId="22" state="visible" r:id="rId22"/>
     <sheet name="2026-08-06" sheetId="23" state="visible" r:id="rId23"/>
     <sheet name="2026-08-07" sheetId="24" state="visible" r:id="rId24"/>
+    <sheet name="2026-08-08" sheetId="25" state="visible" r:id="rId25"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -14364,6 +14365,870 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet25.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C57"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="29" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Clan: Mans Best Friend (3815)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Timestamp: 2026-08-08 13:01:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>Total Reps</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>Daily Reps (+1d)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>Nobodys Son</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="n">
+        <v>7422</v>
+      </c>
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>-2466</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>Player</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="n">
+        <v>4314</v>
+      </c>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>+199</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>Player</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="n">
+        <v>4200</v>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>+85</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>X y L O T A</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="n">
+        <v>4098</v>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>AbdiHyde ID 13496</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="n">
+        <v>5427</v>
+      </c>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>Create Character III</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="n">
+        <v>7047</v>
+      </c>
+      <c r="C9" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>Create Character IV</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="n">
+        <v>7708</v>
+      </c>
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>Create Character V</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="n">
+        <v>7560</v>
+      </c>
+      <c r="C11" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t>Player</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="n">
+        <v>4174</v>
+      </c>
+      <c r="C12" s="5" t="inlineStr">
+        <is>
+          <t>+59</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="4" t="inlineStr">
+        <is>
+          <t>Player</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="n">
+        <v>4115</v>
+      </c>
+      <c r="C13" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="4" t="inlineStr">
+        <is>
+          <t>hunry</t>
+        </is>
+      </c>
+      <c r="B14" s="5" t="n">
+        <v>4204</v>
+      </c>
+      <c r="C14" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="4" t="inlineStr">
+        <is>
+          <t>Tears</t>
+        </is>
+      </c>
+      <c r="B15" s="5" t="n">
+        <v>7227</v>
+      </c>
+      <c r="C15" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="4" t="inlineStr">
+        <is>
+          <t>Sugar Talking</t>
+        </is>
+      </c>
+      <c r="B16" s="5" t="n">
+        <v>8462</v>
+      </c>
+      <c r="C16" s="5" t="inlineStr">
+        <is>
+          <t>+934</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="4" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B17" s="5" t="n">
+        <v>7523</v>
+      </c>
+      <c r="C17" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="4" t="inlineStr">
+        <is>
+          <t>Anti-Hero</t>
+        </is>
+      </c>
+      <c r="B18" s="5" t="n">
+        <v>8274</v>
+      </c>
+      <c r="C18" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="4" t="inlineStr">
+        <is>
+          <t>Vigilante Shit</t>
+        </is>
+      </c>
+      <c r="B19" s="5" t="n">
+        <v>8289</v>
+      </c>
+      <c r="C19" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="4" t="inlineStr">
+        <is>
+          <t>Sweet Nothing</t>
+        </is>
+      </c>
+      <c r="B20" s="5" t="n">
+        <v>8369</v>
+      </c>
+      <c r="C20" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="4" t="inlineStr">
+        <is>
+          <t>The Great War</t>
+        </is>
+      </c>
+      <c r="B21" s="5" t="n">
+        <v>8089</v>
+      </c>
+      <c r="C21" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">We Almost Broke Up </t>
+        </is>
+      </c>
+      <c r="B22" s="5" t="n">
+        <v>8343</v>
+      </c>
+      <c r="C22" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="4" t="inlineStr">
+        <is>
+          <t>When Did You Get Hot</t>
+        </is>
+      </c>
+      <c r="B23" s="5" t="n">
+        <v>8212</v>
+      </c>
+      <c r="C23" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="4" t="inlineStr">
+        <is>
+          <t>Dont Worry Ill Make</t>
+        </is>
+      </c>
+      <c r="B24" s="5" t="n">
+        <v>7554</v>
+      </c>
+      <c r="C24" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="4" t="inlineStr">
+        <is>
+          <t>Goodbye</t>
+        </is>
+      </c>
+      <c r="B25" s="5" t="n">
+        <v>7005</v>
+      </c>
+      <c r="C25" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="4" t="inlineStr">
+        <is>
+          <t>Mans Best Friend</t>
+        </is>
+      </c>
+      <c r="B26" s="5" t="n">
+        <v>6974</v>
+      </c>
+      <c r="C26" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="4" t="inlineStr">
+        <is>
+          <t>Lavender Haze</t>
+        </is>
+      </c>
+      <c r="B27" s="5" t="n">
+        <v>6962</v>
+      </c>
+      <c r="C27" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="4" t="inlineStr">
+        <is>
+          <t>Never Getting Laid</t>
+        </is>
+      </c>
+      <c r="B28" s="5" t="n">
+        <v>8493</v>
+      </c>
+      <c r="C28" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="4" t="inlineStr">
+        <is>
+          <t>My Man on Willpower</t>
+        </is>
+      </c>
+      <c r="B29" s="5" t="n">
+        <v>7480</v>
+      </c>
+      <c r="C29" s="5" t="inlineStr">
+        <is>
+          <t>-821</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="4" t="inlineStr">
+        <is>
+          <t>Manchild</t>
+        </is>
+      </c>
+      <c r="B30" s="5" t="n">
+        <v>8355</v>
+      </c>
+      <c r="C30" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="4" t="inlineStr">
+        <is>
+          <t>Sugar Talking</t>
+        </is>
+      </c>
+      <c r="B31" s="5" t="n">
+        <v>7528</v>
+      </c>
+      <c r="C31" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="4" t="inlineStr">
+        <is>
+          <t>My Man on Willpower</t>
+        </is>
+      </c>
+      <c r="B32" s="5" t="n">
+        <v>8301</v>
+      </c>
+      <c r="C32" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="4" t="inlineStr">
+        <is>
+          <t>Midnight Rain</t>
+        </is>
+      </c>
+      <c r="B33" s="5" t="n">
+        <v>6800</v>
+      </c>
+      <c r="C33" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="4" t="inlineStr">
+        <is>
+          <t>Nobodys Son</t>
+        </is>
+      </c>
+      <c r="B34" s="5" t="n">
+        <v>9888</v>
+      </c>
+      <c r="C34" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="4" t="inlineStr">
+        <is>
+          <t>House Tour</t>
+        </is>
+      </c>
+      <c r="B35" s="5" t="n">
+        <v>7216</v>
+      </c>
+      <c r="C35" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="4" t="inlineStr">
+        <is>
+          <t>Hanabi  Î±Î·Ð²Ï…</t>
+        </is>
+      </c>
+      <c r="B36" s="5" t="n">
+        <v>7212</v>
+      </c>
+      <c r="C36" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="4" t="inlineStr">
+        <is>
+          <t>Saiyajin anbuâ„¢</t>
+        </is>
+      </c>
+      <c r="B37" s="5" t="n">
+        <v>4363</v>
+      </c>
+      <c r="C37" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="4" t="inlineStr">
+        <is>
+          <t>Dummy</t>
+        </is>
+      </c>
+      <c r="B38" s="5" t="n">
+        <v>6736</v>
+      </c>
+      <c r="C38" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="4" t="inlineStr">
+        <is>
+          <t>Cazador anbu â„¢</t>
+        </is>
+      </c>
+      <c r="B39" s="5" t="n">
+        <v>4336</v>
+      </c>
+      <c r="C39" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="4" t="inlineStr">
+        <is>
+          <t>Besos Mojados</t>
+        </is>
+      </c>
+      <c r="B40" s="5" t="n">
+        <v>4425</v>
+      </c>
+      <c r="C40" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="4" t="inlineStr">
+        <is>
+          <t>DarkFire</t>
+        </is>
+      </c>
+      <c r="B41" s="5" t="n">
+        <v>10728</v>
+      </c>
+      <c r="C41" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="4" t="inlineStr">
+        <is>
+          <t>DarkSunny</t>
+        </is>
+      </c>
+      <c r="B42" s="5" t="n">
+        <v>10994</v>
+      </c>
+      <c r="C42" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="4" t="inlineStr">
+        <is>
+          <t>Dairen Uchiha</t>
+        </is>
+      </c>
+      <c r="B43" s="5" t="n">
+        <v>11482</v>
+      </c>
+      <c r="C43" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="4" t="inlineStr">
+        <is>
+          <t>LILI ZENIN®</t>
+        </is>
+      </c>
+      <c r="B44" s="5" t="n">
+        <v>7019</v>
+      </c>
+      <c r="C44" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="4" t="inlineStr">
+        <is>
+          <t>ryumichel ZENIN ®</t>
+        </is>
+      </c>
+      <c r="B45" s="5" t="n">
+        <v>3218</v>
+      </c>
+      <c r="C45" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="4" t="inlineStr">
+        <is>
+          <t>margot ZENIN ®</t>
+        </is>
+      </c>
+      <c r="B46" s="5" t="n">
+        <v>3250</v>
+      </c>
+      <c r="C46" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="4" t="inlineStr">
+        <is>
+          <t>linda ZENIN ®</t>
+        </is>
+      </c>
+      <c r="B47" s="5" t="n">
+        <v>7111</v>
+      </c>
+      <c r="C47" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="4" t="inlineStr">
+        <is>
+          <t>PlyRed-</t>
+        </is>
+      </c>
+      <c r="B48" s="5" t="n">
+        <v>6031</v>
+      </c>
+      <c r="C48" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="4" t="inlineStr">
+        <is>
+          <t>equin0x</t>
+        </is>
+      </c>
+      <c r="B49" s="5" t="n">
+        <v>8516</v>
+      </c>
+      <c r="C49" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="4" t="inlineStr">
+        <is>
+          <t>Jhayco - Mokai</t>
+        </is>
+      </c>
+      <c r="B50" s="5" t="n">
+        <v>10165</v>
+      </c>
+      <c r="C50" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="4" t="inlineStr">
+        <is>
+          <t>Jhayco - Joe</t>
+        </is>
+      </c>
+      <c r="B51" s="5" t="n">
+        <v>10361</v>
+      </c>
+      <c r="C51" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="4" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="B52" s="5" t="n">
+        <v>10232</v>
+      </c>
+      <c r="C52" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="4" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="B53" s="5" t="n">
+        <v>10526</v>
+      </c>
+      <c r="C53" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="4" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="B54" s="5" t="n">
+        <v>10211</v>
+      </c>
+      <c r="C54" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="4" t="inlineStr">
+        <is>
+          <t>Go Go Juice</t>
+        </is>
+      </c>
+      <c r="B55" s="5" t="n">
+        <v>7930</v>
+      </c>
+      <c r="C55" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="4" t="inlineStr">
+        <is>
+          <t>Jhayco - Imaginaste</t>
+        </is>
+      </c>
+      <c r="B56" s="5" t="n">
+        <v>4077</v>
+      </c>
+      <c r="C56" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="4" t="inlineStr">
+        <is>
+          <t>PuNch</t>
+        </is>
+      </c>
+      <c r="B57" s="5" t="n">
+        <v>7065</v>
+      </c>
+      <c r="C57" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A2:C2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
auto: snapshot 2026-08-09 13:01:01
</commit_message>
<xml_diff>
--- a/clan_3815.xlsx
+++ b/clan_3815.xlsx
@@ -32,6 +32,7 @@
     <sheet name="2026-08-06" sheetId="23" state="visible" r:id="rId23"/>
     <sheet name="2026-08-07" sheetId="24" state="visible" r:id="rId24"/>
     <sheet name="2026-08-08" sheetId="25" state="visible" r:id="rId25"/>
+    <sheet name="2026-08-09" sheetId="26" state="visible" r:id="rId26"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -15229,6 +15230,870 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet26.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C57"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="29" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Clan: Mans Best Friend (3815)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Timestamp: 2026-08-09 13:01:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>Total Reps</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>Daily Reps (+1d)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>Nobodys Son</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="n">
+        <v>7422</v>
+      </c>
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>-2466</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>Player</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="n">
+        <v>4314</v>
+      </c>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>+199</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>Player</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="n">
+        <v>4200</v>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>+85</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>X y L O T A</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="n">
+        <v>4098</v>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>AbdiHyde ID 13496</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="n">
+        <v>5427</v>
+      </c>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>Create Character III</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="n">
+        <v>7047</v>
+      </c>
+      <c r="C9" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>Create Character IV</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="n">
+        <v>7708</v>
+      </c>
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>Create Character V</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="n">
+        <v>7560</v>
+      </c>
+      <c r="C11" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t>Player</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="n">
+        <v>4174</v>
+      </c>
+      <c r="C12" s="5" t="inlineStr">
+        <is>
+          <t>+59</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="4" t="inlineStr">
+        <is>
+          <t>Player</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="n">
+        <v>4115</v>
+      </c>
+      <c r="C13" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="4" t="inlineStr">
+        <is>
+          <t>hunry</t>
+        </is>
+      </c>
+      <c r="B14" s="5" t="n">
+        <v>4204</v>
+      </c>
+      <c r="C14" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="4" t="inlineStr">
+        <is>
+          <t>BlacKRin O</t>
+        </is>
+      </c>
+      <c r="B15" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C15" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="4" t="inlineStr">
+        <is>
+          <t>Tears</t>
+        </is>
+      </c>
+      <c r="B16" s="5" t="n">
+        <v>7227</v>
+      </c>
+      <c r="C16" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="4" t="inlineStr">
+        <is>
+          <t>Sugar Talking</t>
+        </is>
+      </c>
+      <c r="B17" s="5" t="n">
+        <v>8462</v>
+      </c>
+      <c r="C17" s="5" t="inlineStr">
+        <is>
+          <t>+934</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="4" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B18" s="5" t="n">
+        <v>7523</v>
+      </c>
+      <c r="C18" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="4" t="inlineStr">
+        <is>
+          <t>Anti-Hero</t>
+        </is>
+      </c>
+      <c r="B19" s="5" t="n">
+        <v>8274</v>
+      </c>
+      <c r="C19" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="4" t="inlineStr">
+        <is>
+          <t>Vigilante Shit</t>
+        </is>
+      </c>
+      <c r="B20" s="5" t="n">
+        <v>8289</v>
+      </c>
+      <c r="C20" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="4" t="inlineStr">
+        <is>
+          <t>Sweet Nothing</t>
+        </is>
+      </c>
+      <c r="B21" s="5" t="n">
+        <v>8369</v>
+      </c>
+      <c r="C21" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="4" t="inlineStr">
+        <is>
+          <t>The Great War</t>
+        </is>
+      </c>
+      <c r="B22" s="5" t="n">
+        <v>8089</v>
+      </c>
+      <c r="C22" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">We Almost Broke Up </t>
+        </is>
+      </c>
+      <c r="B23" s="5" t="n">
+        <v>8343</v>
+      </c>
+      <c r="C23" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="4" t="inlineStr">
+        <is>
+          <t>When Did You Get Hot</t>
+        </is>
+      </c>
+      <c r="B24" s="5" t="n">
+        <v>8212</v>
+      </c>
+      <c r="C24" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="4" t="inlineStr">
+        <is>
+          <t>Dont Worry Ill Make</t>
+        </is>
+      </c>
+      <c r="B25" s="5" t="n">
+        <v>7554</v>
+      </c>
+      <c r="C25" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="4" t="inlineStr">
+        <is>
+          <t>Goodbye</t>
+        </is>
+      </c>
+      <c r="B26" s="5" t="n">
+        <v>7005</v>
+      </c>
+      <c r="C26" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="4" t="inlineStr">
+        <is>
+          <t>Mans Best Friend</t>
+        </is>
+      </c>
+      <c r="B27" s="5" t="n">
+        <v>6974</v>
+      </c>
+      <c r="C27" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="4" t="inlineStr">
+        <is>
+          <t>Lavender Haze</t>
+        </is>
+      </c>
+      <c r="B28" s="5" t="n">
+        <v>6962</v>
+      </c>
+      <c r="C28" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="4" t="inlineStr">
+        <is>
+          <t>Never Getting Laid</t>
+        </is>
+      </c>
+      <c r="B29" s="5" t="n">
+        <v>8493</v>
+      </c>
+      <c r="C29" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="4" t="inlineStr">
+        <is>
+          <t>My Man on Willpower</t>
+        </is>
+      </c>
+      <c r="B30" s="5" t="n">
+        <v>7480</v>
+      </c>
+      <c r="C30" s="5" t="inlineStr">
+        <is>
+          <t>-821</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="4" t="inlineStr">
+        <is>
+          <t>Manchild</t>
+        </is>
+      </c>
+      <c r="B31" s="5" t="n">
+        <v>8355</v>
+      </c>
+      <c r="C31" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="4" t="inlineStr">
+        <is>
+          <t>Sugar Talking</t>
+        </is>
+      </c>
+      <c r="B32" s="5" t="n">
+        <v>7528</v>
+      </c>
+      <c r="C32" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="4" t="inlineStr">
+        <is>
+          <t>My Man on Willpower</t>
+        </is>
+      </c>
+      <c r="B33" s="5" t="n">
+        <v>8301</v>
+      </c>
+      <c r="C33" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="4" t="inlineStr">
+        <is>
+          <t>Midnight Rain</t>
+        </is>
+      </c>
+      <c r="B34" s="5" t="n">
+        <v>6800</v>
+      </c>
+      <c r="C34" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="4" t="inlineStr">
+        <is>
+          <t>Nobodys Son</t>
+        </is>
+      </c>
+      <c r="B35" s="5" t="n">
+        <v>9888</v>
+      </c>
+      <c r="C35" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="4" t="inlineStr">
+        <is>
+          <t>House Tour</t>
+        </is>
+      </c>
+      <c r="B36" s="5" t="n">
+        <v>7216</v>
+      </c>
+      <c r="C36" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="4" t="inlineStr">
+        <is>
+          <t>Hanabi  Î±Î·Ð²Ï…</t>
+        </is>
+      </c>
+      <c r="B37" s="5" t="n">
+        <v>7212</v>
+      </c>
+      <c r="C37" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="4" t="inlineStr">
+        <is>
+          <t>Saiyajin anbuâ„¢</t>
+        </is>
+      </c>
+      <c r="B38" s="5" t="n">
+        <v>4363</v>
+      </c>
+      <c r="C38" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="4" t="inlineStr">
+        <is>
+          <t>Dummy</t>
+        </is>
+      </c>
+      <c r="B39" s="5" t="n">
+        <v>6736</v>
+      </c>
+      <c r="C39" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="4" t="inlineStr">
+        <is>
+          <t>Cazador anbu â„¢</t>
+        </is>
+      </c>
+      <c r="B40" s="5" t="n">
+        <v>4336</v>
+      </c>
+      <c r="C40" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="4" t="inlineStr">
+        <is>
+          <t>Besos Mojados</t>
+        </is>
+      </c>
+      <c r="B41" s="5" t="n">
+        <v>4425</v>
+      </c>
+      <c r="C41" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="4" t="inlineStr">
+        <is>
+          <t>DarkFire</t>
+        </is>
+      </c>
+      <c r="B42" s="5" t="n">
+        <v>10728</v>
+      </c>
+      <c r="C42" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="4" t="inlineStr">
+        <is>
+          <t>DarkSunny</t>
+        </is>
+      </c>
+      <c r="B43" s="5" t="n">
+        <v>10994</v>
+      </c>
+      <c r="C43" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="4" t="inlineStr">
+        <is>
+          <t>Dairen Uchiha</t>
+        </is>
+      </c>
+      <c r="B44" s="5" t="n">
+        <v>11482</v>
+      </c>
+      <c r="C44" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="4" t="inlineStr">
+        <is>
+          <t>LILI ZENIN®</t>
+        </is>
+      </c>
+      <c r="B45" s="5" t="n">
+        <v>7019</v>
+      </c>
+      <c r="C45" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="4" t="inlineStr">
+        <is>
+          <t>ryumichel ZENIN ®</t>
+        </is>
+      </c>
+      <c r="B46" s="5" t="n">
+        <v>3218</v>
+      </c>
+      <c r="C46" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="4" t="inlineStr">
+        <is>
+          <t>margot ZENIN ®</t>
+        </is>
+      </c>
+      <c r="B47" s="5" t="n">
+        <v>3250</v>
+      </c>
+      <c r="C47" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="4" t="inlineStr">
+        <is>
+          <t>linda ZENIN ®</t>
+        </is>
+      </c>
+      <c r="B48" s="5" t="n">
+        <v>7111</v>
+      </c>
+      <c r="C48" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="4" t="inlineStr">
+        <is>
+          <t>equin0x</t>
+        </is>
+      </c>
+      <c r="B49" s="5" t="n">
+        <v>8516</v>
+      </c>
+      <c r="C49" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="4" t="inlineStr">
+        <is>
+          <t>Jhayco - Mokai</t>
+        </is>
+      </c>
+      <c r="B50" s="5" t="n">
+        <v>10165</v>
+      </c>
+      <c r="C50" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="4" t="inlineStr">
+        <is>
+          <t>Jhayco - Joe</t>
+        </is>
+      </c>
+      <c r="B51" s="5" t="n">
+        <v>10361</v>
+      </c>
+      <c r="C51" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="4" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="B52" s="5" t="n">
+        <v>10232</v>
+      </c>
+      <c r="C52" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="4" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="B53" s="5" t="n">
+        <v>10526</v>
+      </c>
+      <c r="C53" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="4" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="B54" s="5" t="n">
+        <v>10211</v>
+      </c>
+      <c r="C54" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="4" t="inlineStr">
+        <is>
+          <t>Go Go Juice</t>
+        </is>
+      </c>
+      <c r="B55" s="5" t="n">
+        <v>7930</v>
+      </c>
+      <c r="C55" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="4" t="inlineStr">
+        <is>
+          <t>Jhayco - Imaginaste</t>
+        </is>
+      </c>
+      <c r="B56" s="5" t="n">
+        <v>4077</v>
+      </c>
+      <c r="C56" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="4" t="inlineStr">
+        <is>
+          <t>PuNch</t>
+        </is>
+      </c>
+      <c r="B57" s="5" t="n">
+        <v>7065</v>
+      </c>
+      <c r="C57" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A2:C2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
auto: snapshot 2026-08-10 13:01:00
</commit_message>
<xml_diff>
--- a/clan_3815.xlsx
+++ b/clan_3815.xlsx
@@ -33,6 +33,7 @@
     <sheet name="2026-08-07" sheetId="24" state="visible" r:id="rId24"/>
     <sheet name="2026-08-08" sheetId="25" state="visible" r:id="rId25"/>
     <sheet name="2026-08-09" sheetId="26" state="visible" r:id="rId26"/>
+    <sheet name="2026-08-10" sheetId="27" state="visible" r:id="rId27"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -16094,6 +16095,870 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet27.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C57"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="29" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Clan: Mans Best Friend (3815)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Timestamp: 2026-08-10 13:01:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>Total Reps</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>Daily Reps (+1d)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>Nobodys Son</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>-9888</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>Player</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>-4115</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>Player</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>-4115</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>X y L O T A</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>-4098</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>AbdiHyde ID 13496</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>-5427</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>Create Character III</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C9" s="5" t="inlineStr">
+        <is>
+          <t>-7047</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>Create Character IV</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>-7708</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>Create Character V</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C11" s="5" t="inlineStr">
+        <is>
+          <t>-7560</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t>Player</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C12" s="5" t="inlineStr">
+        <is>
+          <t>-4115</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="4" t="inlineStr">
+        <is>
+          <t>Player</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C13" s="5" t="inlineStr">
+        <is>
+          <t>-4115</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="4" t="inlineStr">
+        <is>
+          <t>hunry</t>
+        </is>
+      </c>
+      <c r="B14" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C14" s="5" t="inlineStr">
+        <is>
+          <t>-4204</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="4" t="inlineStr">
+        <is>
+          <t>BlacKRin O</t>
+        </is>
+      </c>
+      <c r="B15" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C15" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="4" t="inlineStr">
+        <is>
+          <t>Tears</t>
+        </is>
+      </c>
+      <c r="B16" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C16" s="5" t="inlineStr">
+        <is>
+          <t>-7227</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="4" t="inlineStr">
+        <is>
+          <t>Sugar Talking</t>
+        </is>
+      </c>
+      <c r="B17" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C17" s="5" t="inlineStr">
+        <is>
+          <t>-7528</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="4" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B18" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C18" s="5" t="inlineStr">
+        <is>
+          <t>-7523</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="4" t="inlineStr">
+        <is>
+          <t>Anti-Hero</t>
+        </is>
+      </c>
+      <c r="B19" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C19" s="5" t="inlineStr">
+        <is>
+          <t>-8274</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="4" t="inlineStr">
+        <is>
+          <t>Vigilante Shit</t>
+        </is>
+      </c>
+      <c r="B20" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C20" s="5" t="inlineStr">
+        <is>
+          <t>-8289</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="4" t="inlineStr">
+        <is>
+          <t>Sweet Nothing</t>
+        </is>
+      </c>
+      <c r="B21" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C21" s="5" t="inlineStr">
+        <is>
+          <t>-8369</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="4" t="inlineStr">
+        <is>
+          <t>The Great War</t>
+        </is>
+      </c>
+      <c r="B22" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C22" s="5" t="inlineStr">
+        <is>
+          <t>-8089</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">We Almost Broke Up </t>
+        </is>
+      </c>
+      <c r="B23" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C23" s="5" t="inlineStr">
+        <is>
+          <t>-8343</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="4" t="inlineStr">
+        <is>
+          <t>When Did You Get Hot</t>
+        </is>
+      </c>
+      <c r="B24" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C24" s="5" t="inlineStr">
+        <is>
+          <t>-8212</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="4" t="inlineStr">
+        <is>
+          <t>Dont Worry Ill Make</t>
+        </is>
+      </c>
+      <c r="B25" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C25" s="5" t="inlineStr">
+        <is>
+          <t>-7554</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="4" t="inlineStr">
+        <is>
+          <t>Goodbye</t>
+        </is>
+      </c>
+      <c r="B26" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C26" s="5" t="inlineStr">
+        <is>
+          <t>-7005</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="4" t="inlineStr">
+        <is>
+          <t>Mans Best Friend</t>
+        </is>
+      </c>
+      <c r="B27" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C27" s="5" t="inlineStr">
+        <is>
+          <t>-6974</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="4" t="inlineStr">
+        <is>
+          <t>Lavender Haze</t>
+        </is>
+      </c>
+      <c r="B28" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C28" s="5" t="inlineStr">
+        <is>
+          <t>-6962</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="4" t="inlineStr">
+        <is>
+          <t>Never Getting Laid</t>
+        </is>
+      </c>
+      <c r="B29" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C29" s="5" t="inlineStr">
+        <is>
+          <t>-8493</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="4" t="inlineStr">
+        <is>
+          <t>My Man on Willpower</t>
+        </is>
+      </c>
+      <c r="B30" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C30" s="5" t="inlineStr">
+        <is>
+          <t>-8301</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="4" t="inlineStr">
+        <is>
+          <t>Manchild</t>
+        </is>
+      </c>
+      <c r="B31" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C31" s="5" t="inlineStr">
+        <is>
+          <t>-8355</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="4" t="inlineStr">
+        <is>
+          <t>Sugar Talking</t>
+        </is>
+      </c>
+      <c r="B32" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C32" s="5" t="inlineStr">
+        <is>
+          <t>-7528</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="4" t="inlineStr">
+        <is>
+          <t>My Man on Willpower</t>
+        </is>
+      </c>
+      <c r="B33" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C33" s="5" t="inlineStr">
+        <is>
+          <t>-8301</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="4" t="inlineStr">
+        <is>
+          <t>Midnight Rain</t>
+        </is>
+      </c>
+      <c r="B34" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C34" s="5" t="inlineStr">
+        <is>
+          <t>-6800</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="4" t="inlineStr">
+        <is>
+          <t>Nobodys Son</t>
+        </is>
+      </c>
+      <c r="B35" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C35" s="5" t="inlineStr">
+        <is>
+          <t>-9888</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="4" t="inlineStr">
+        <is>
+          <t>House Tour</t>
+        </is>
+      </c>
+      <c r="B36" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C36" s="5" t="inlineStr">
+        <is>
+          <t>-7216</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="4" t="inlineStr">
+        <is>
+          <t>Hanabi  Î±Î·Ð²Ï…</t>
+        </is>
+      </c>
+      <c r="B37" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C37" s="5" t="inlineStr">
+        <is>
+          <t>-7212</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="4" t="inlineStr">
+        <is>
+          <t>Saiyajin anbuâ„¢</t>
+        </is>
+      </c>
+      <c r="B38" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C38" s="5" t="inlineStr">
+        <is>
+          <t>-4363</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="4" t="inlineStr">
+        <is>
+          <t>Dummy</t>
+        </is>
+      </c>
+      <c r="B39" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C39" s="5" t="inlineStr">
+        <is>
+          <t>-6736</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="4" t="inlineStr">
+        <is>
+          <t>Cazador anbu â„¢</t>
+        </is>
+      </c>
+      <c r="B40" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C40" s="5" t="inlineStr">
+        <is>
+          <t>-4336</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="4" t="inlineStr">
+        <is>
+          <t>Besos Mojados</t>
+        </is>
+      </c>
+      <c r="B41" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C41" s="5" t="inlineStr">
+        <is>
+          <t>-4425</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="4" t="inlineStr">
+        <is>
+          <t>DarkFire</t>
+        </is>
+      </c>
+      <c r="B42" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C42" s="5" t="inlineStr">
+        <is>
+          <t>-10728</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="4" t="inlineStr">
+        <is>
+          <t>DarkSunny</t>
+        </is>
+      </c>
+      <c r="B43" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C43" s="5" t="inlineStr">
+        <is>
+          <t>-10994</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="4" t="inlineStr">
+        <is>
+          <t>Dairen Uchiha</t>
+        </is>
+      </c>
+      <c r="B44" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C44" s="5" t="inlineStr">
+        <is>
+          <t>-11482</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="4" t="inlineStr">
+        <is>
+          <t>LILI ZENIN®</t>
+        </is>
+      </c>
+      <c r="B45" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C45" s="5" t="inlineStr">
+        <is>
+          <t>-7019</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="4" t="inlineStr">
+        <is>
+          <t>ryumichel ZENIN ®</t>
+        </is>
+      </c>
+      <c r="B46" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C46" s="5" t="inlineStr">
+        <is>
+          <t>-3218</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="4" t="inlineStr">
+        <is>
+          <t>margot ZENIN ®</t>
+        </is>
+      </c>
+      <c r="B47" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C47" s="5" t="inlineStr">
+        <is>
+          <t>-3250</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="4" t="inlineStr">
+        <is>
+          <t>linda ZENIN ®</t>
+        </is>
+      </c>
+      <c r="B48" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C48" s="5" t="inlineStr">
+        <is>
+          <t>-7111</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="4" t="inlineStr">
+        <is>
+          <t>equin0x</t>
+        </is>
+      </c>
+      <c r="B49" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C49" s="5" t="inlineStr">
+        <is>
+          <t>-8516</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="4" t="inlineStr">
+        <is>
+          <t>Jhayco - Mokai</t>
+        </is>
+      </c>
+      <c r="B50" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C50" s="5" t="inlineStr">
+        <is>
+          <t>-10165</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="4" t="inlineStr">
+        <is>
+          <t>Jhayco - Joe</t>
+        </is>
+      </c>
+      <c r="B51" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C51" s="5" t="inlineStr">
+        <is>
+          <t>-10361</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="4" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="B52" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C52" s="5" t="inlineStr">
+        <is>
+          <t>-10232</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="4" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="B53" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C53" s="5" t="inlineStr">
+        <is>
+          <t>-10526</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="4" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="B54" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C54" s="5" t="inlineStr">
+        <is>
+          <t>-10211</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="4" t="inlineStr">
+        <is>
+          <t>Go Go Juice</t>
+        </is>
+      </c>
+      <c r="B55" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C55" s="5" t="inlineStr">
+        <is>
+          <t>-7930</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="4" t="inlineStr">
+        <is>
+          <t>Jhayco - Imaginaste</t>
+        </is>
+      </c>
+      <c r="B56" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C56" s="5" t="inlineStr">
+        <is>
+          <t>-4077</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="4" t="inlineStr">
+        <is>
+          <t>PuNch</t>
+        </is>
+      </c>
+      <c r="B57" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C57" s="5" t="inlineStr">
+        <is>
+          <t>-7065</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A2:C2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
auto: snapshot 2026-08-11 13:01:01
</commit_message>
<xml_diff>
--- a/clan_3815.xlsx
+++ b/clan_3815.xlsx
@@ -34,6 +34,7 @@
     <sheet name="2026-08-08" sheetId="25" state="visible" r:id="rId25"/>
     <sheet name="2026-08-09" sheetId="26" state="visible" r:id="rId26"/>
     <sheet name="2026-08-10" sheetId="27" state="visible" r:id="rId27"/>
+    <sheet name="2026-08-11" sheetId="28" state="visible" r:id="rId28"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -16959,6 +16960,870 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet28.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C57"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="29" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Clan: Mans Best Friend (3815)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Timestamp: 2026-08-11 13:01:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>Total Reps</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>Daily Reps (+1d)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>Nobodys Son</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>Player</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>Player</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>X y L O T A</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>AbdiHyde ID 13496</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>Create Character III</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C9" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>Create Character IV</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>Create Character V</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C11" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t>Player</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C12" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="4" t="inlineStr">
+        <is>
+          <t>Player</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C13" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="4" t="inlineStr">
+        <is>
+          <t>hunry</t>
+        </is>
+      </c>
+      <c r="B14" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C14" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="4" t="inlineStr">
+        <is>
+          <t>BlacKRin O</t>
+        </is>
+      </c>
+      <c r="B15" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C15" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="4" t="inlineStr">
+        <is>
+          <t>Tears</t>
+        </is>
+      </c>
+      <c r="B16" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C16" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="4" t="inlineStr">
+        <is>
+          <t>Sugar Talking</t>
+        </is>
+      </c>
+      <c r="B17" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C17" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="4" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B18" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C18" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="4" t="inlineStr">
+        <is>
+          <t>Anti-Hero</t>
+        </is>
+      </c>
+      <c r="B19" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C19" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="4" t="inlineStr">
+        <is>
+          <t>Vigilante Shit</t>
+        </is>
+      </c>
+      <c r="B20" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C20" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="4" t="inlineStr">
+        <is>
+          <t>Sweet Nothing</t>
+        </is>
+      </c>
+      <c r="B21" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C21" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="4" t="inlineStr">
+        <is>
+          <t>The Great War</t>
+        </is>
+      </c>
+      <c r="B22" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C22" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">We Almost Broke Up </t>
+        </is>
+      </c>
+      <c r="B23" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C23" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="4" t="inlineStr">
+        <is>
+          <t>When Did You Get Hot</t>
+        </is>
+      </c>
+      <c r="B24" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C24" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="4" t="inlineStr">
+        <is>
+          <t>Dont Worry Ill Make</t>
+        </is>
+      </c>
+      <c r="B25" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C25" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="4" t="inlineStr">
+        <is>
+          <t>Goodbye</t>
+        </is>
+      </c>
+      <c r="B26" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C26" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="4" t="inlineStr">
+        <is>
+          <t>Mans Best Friend</t>
+        </is>
+      </c>
+      <c r="B27" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C27" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="4" t="inlineStr">
+        <is>
+          <t>Lavender Haze</t>
+        </is>
+      </c>
+      <c r="B28" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C28" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="4" t="inlineStr">
+        <is>
+          <t>Never Getting Laid</t>
+        </is>
+      </c>
+      <c r="B29" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C29" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="4" t="inlineStr">
+        <is>
+          <t>My Man on Willpower</t>
+        </is>
+      </c>
+      <c r="B30" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C30" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="4" t="inlineStr">
+        <is>
+          <t>Manchild</t>
+        </is>
+      </c>
+      <c r="B31" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C31" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="4" t="inlineStr">
+        <is>
+          <t>Sugar Talking</t>
+        </is>
+      </c>
+      <c r="B32" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C32" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="4" t="inlineStr">
+        <is>
+          <t>My Man on Willpower</t>
+        </is>
+      </c>
+      <c r="B33" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C33" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="4" t="inlineStr">
+        <is>
+          <t>Midnight Rain</t>
+        </is>
+      </c>
+      <c r="B34" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C34" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="4" t="inlineStr">
+        <is>
+          <t>Nobodys Son</t>
+        </is>
+      </c>
+      <c r="B35" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C35" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="4" t="inlineStr">
+        <is>
+          <t>House Tour</t>
+        </is>
+      </c>
+      <c r="B36" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C36" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="4" t="inlineStr">
+        <is>
+          <t>Hanabi  Î±Î·Ð²Ï…</t>
+        </is>
+      </c>
+      <c r="B37" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C37" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="4" t="inlineStr">
+        <is>
+          <t>Saiyajin anbuâ„¢</t>
+        </is>
+      </c>
+      <c r="B38" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C38" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="4" t="inlineStr">
+        <is>
+          <t>Dummy</t>
+        </is>
+      </c>
+      <c r="B39" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C39" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="4" t="inlineStr">
+        <is>
+          <t>Cazador anbu â„¢</t>
+        </is>
+      </c>
+      <c r="B40" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C40" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="4" t="inlineStr">
+        <is>
+          <t>Besos Mojados</t>
+        </is>
+      </c>
+      <c r="B41" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C41" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="4" t="inlineStr">
+        <is>
+          <t>DarkFire</t>
+        </is>
+      </c>
+      <c r="B42" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C42" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="4" t="inlineStr">
+        <is>
+          <t>DarkSunny</t>
+        </is>
+      </c>
+      <c r="B43" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C43" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="4" t="inlineStr">
+        <is>
+          <t>Dairen Uchiha</t>
+        </is>
+      </c>
+      <c r="B44" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C44" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="4" t="inlineStr">
+        <is>
+          <t>LILI ZENIN®</t>
+        </is>
+      </c>
+      <c r="B45" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C45" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="4" t="inlineStr">
+        <is>
+          <t>ryumichel ZENIN ®</t>
+        </is>
+      </c>
+      <c r="B46" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C46" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="4" t="inlineStr">
+        <is>
+          <t>margot ZENIN ®</t>
+        </is>
+      </c>
+      <c r="B47" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C47" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="4" t="inlineStr">
+        <is>
+          <t>linda ZENIN ®</t>
+        </is>
+      </c>
+      <c r="B48" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C48" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="4" t="inlineStr">
+        <is>
+          <t>equin0x</t>
+        </is>
+      </c>
+      <c r="B49" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C49" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="4" t="inlineStr">
+        <is>
+          <t>Jhayco - Mokai</t>
+        </is>
+      </c>
+      <c r="B50" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C50" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="4" t="inlineStr">
+        <is>
+          <t>Jhayco - Joe</t>
+        </is>
+      </c>
+      <c r="B51" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C51" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="4" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="B52" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C52" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="4" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="B53" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C53" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="4" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="B54" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C54" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="4" t="inlineStr">
+        <is>
+          <t>Go Go Juice</t>
+        </is>
+      </c>
+      <c r="B55" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C55" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="4" t="inlineStr">
+        <is>
+          <t>Jhayco - Imaginaste</t>
+        </is>
+      </c>
+      <c r="B56" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C56" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="4" t="inlineStr">
+        <is>
+          <t>PuNch</t>
+        </is>
+      </c>
+      <c r="B57" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C57" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A2:C2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
auto: snapshot 2026-08-12 13:01:00
</commit_message>
<xml_diff>
--- a/clan_3815.xlsx
+++ b/clan_3815.xlsx
@@ -35,6 +35,7 @@
     <sheet name="2026-08-09" sheetId="26" state="visible" r:id="rId26"/>
     <sheet name="2026-08-10" sheetId="27" state="visible" r:id="rId27"/>
     <sheet name="2026-08-11" sheetId="28" state="visible" r:id="rId28"/>
+    <sheet name="2026-08-12" sheetId="29" state="visible" r:id="rId29"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -17824,6 +17825,870 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet29.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C57"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="29" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Clan: Mans Best Friend (3815)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Timestamp: 2026-08-12 13:01:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>Total Reps</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>Daily Reps (+1d)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>Nobodys Son</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>Player</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>Player</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>X y L O T A</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>AbdiHyde ID 13496</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>Create Character III</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C9" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>Create Character IV</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>Create Character V</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C11" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t>Player</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C12" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="4" t="inlineStr">
+        <is>
+          <t>Player</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C13" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="4" t="inlineStr">
+        <is>
+          <t>hunry</t>
+        </is>
+      </c>
+      <c r="B14" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C14" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="4" t="inlineStr">
+        <is>
+          <t>BlacKRin O</t>
+        </is>
+      </c>
+      <c r="B15" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C15" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="4" t="inlineStr">
+        <is>
+          <t>Tears</t>
+        </is>
+      </c>
+      <c r="B16" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C16" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="4" t="inlineStr">
+        <is>
+          <t>Sugar Talking</t>
+        </is>
+      </c>
+      <c r="B17" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C17" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="4" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B18" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C18" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="4" t="inlineStr">
+        <is>
+          <t>Anti-Hero</t>
+        </is>
+      </c>
+      <c r="B19" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C19" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="4" t="inlineStr">
+        <is>
+          <t>Vigilante Shit</t>
+        </is>
+      </c>
+      <c r="B20" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C20" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="4" t="inlineStr">
+        <is>
+          <t>Sweet Nothing</t>
+        </is>
+      </c>
+      <c r="B21" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C21" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="4" t="inlineStr">
+        <is>
+          <t>The Great War</t>
+        </is>
+      </c>
+      <c r="B22" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C22" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">We Almost Broke Up </t>
+        </is>
+      </c>
+      <c r="B23" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C23" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="4" t="inlineStr">
+        <is>
+          <t>When Did You Get Hot</t>
+        </is>
+      </c>
+      <c r="B24" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C24" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="4" t="inlineStr">
+        <is>
+          <t>Dont Worry Ill Make</t>
+        </is>
+      </c>
+      <c r="B25" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C25" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="4" t="inlineStr">
+        <is>
+          <t>Goodbye</t>
+        </is>
+      </c>
+      <c r="B26" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C26" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="4" t="inlineStr">
+        <is>
+          <t>Mans Best Friend</t>
+        </is>
+      </c>
+      <c r="B27" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C27" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="4" t="inlineStr">
+        <is>
+          <t>Lavender Haze</t>
+        </is>
+      </c>
+      <c r="B28" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C28" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="4" t="inlineStr">
+        <is>
+          <t>Never Getting Laid</t>
+        </is>
+      </c>
+      <c r="B29" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C29" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="4" t="inlineStr">
+        <is>
+          <t>My Man on Willpower</t>
+        </is>
+      </c>
+      <c r="B30" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C30" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="4" t="inlineStr">
+        <is>
+          <t>Manchild</t>
+        </is>
+      </c>
+      <c r="B31" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C31" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="4" t="inlineStr">
+        <is>
+          <t>Sugar Talking</t>
+        </is>
+      </c>
+      <c r="B32" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C32" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="4" t="inlineStr">
+        <is>
+          <t>My Man on Willpower</t>
+        </is>
+      </c>
+      <c r="B33" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C33" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="4" t="inlineStr">
+        <is>
+          <t>Midnight Rain</t>
+        </is>
+      </c>
+      <c r="B34" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C34" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="4" t="inlineStr">
+        <is>
+          <t>Nobodys Son</t>
+        </is>
+      </c>
+      <c r="B35" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C35" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="4" t="inlineStr">
+        <is>
+          <t>House Tour</t>
+        </is>
+      </c>
+      <c r="B36" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C36" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="4" t="inlineStr">
+        <is>
+          <t>Hanabi  Î±Î·Ð²Ï…</t>
+        </is>
+      </c>
+      <c r="B37" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C37" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="4" t="inlineStr">
+        <is>
+          <t>Saiyajin anbuâ„¢</t>
+        </is>
+      </c>
+      <c r="B38" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C38" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="4" t="inlineStr">
+        <is>
+          <t>Dummy</t>
+        </is>
+      </c>
+      <c r="B39" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C39" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="4" t="inlineStr">
+        <is>
+          <t>Cazador anbu â„¢</t>
+        </is>
+      </c>
+      <c r="B40" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C40" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="4" t="inlineStr">
+        <is>
+          <t>Besos Mojados</t>
+        </is>
+      </c>
+      <c r="B41" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C41" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="4" t="inlineStr">
+        <is>
+          <t>DarkFire</t>
+        </is>
+      </c>
+      <c r="B42" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C42" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="4" t="inlineStr">
+        <is>
+          <t>DarkSunny</t>
+        </is>
+      </c>
+      <c r="B43" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C43" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="4" t="inlineStr">
+        <is>
+          <t>Dairen Uchiha</t>
+        </is>
+      </c>
+      <c r="B44" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C44" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="4" t="inlineStr">
+        <is>
+          <t>LILI ZENIN®</t>
+        </is>
+      </c>
+      <c r="B45" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C45" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="4" t="inlineStr">
+        <is>
+          <t>ryumichel ZENIN ®</t>
+        </is>
+      </c>
+      <c r="B46" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C46" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="4" t="inlineStr">
+        <is>
+          <t>margot ZENIN ®</t>
+        </is>
+      </c>
+      <c r="B47" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C47" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="4" t="inlineStr">
+        <is>
+          <t>linda ZENIN ®</t>
+        </is>
+      </c>
+      <c r="B48" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C48" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="4" t="inlineStr">
+        <is>
+          <t>equin0x</t>
+        </is>
+      </c>
+      <c r="B49" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C49" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="4" t="inlineStr">
+        <is>
+          <t>Jhayco - Mokai</t>
+        </is>
+      </c>
+      <c r="B50" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C50" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="4" t="inlineStr">
+        <is>
+          <t>Jhayco - Joe</t>
+        </is>
+      </c>
+      <c r="B51" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C51" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="4" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="B52" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C52" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="4" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="B53" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C53" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="4" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="B54" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C54" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="4" t="inlineStr">
+        <is>
+          <t>Go Go Juice</t>
+        </is>
+      </c>
+      <c r="B55" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C55" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="4" t="inlineStr">
+        <is>
+          <t>Jhayco - Imaginaste</t>
+        </is>
+      </c>
+      <c r="B56" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C56" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="4" t="inlineStr">
+        <is>
+          <t>PuNch</t>
+        </is>
+      </c>
+      <c r="B57" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C57" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A2:C2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
auto: snapshot 2026-08-13 13:01:01
</commit_message>
<xml_diff>
--- a/clan_3815.xlsx
+++ b/clan_3815.xlsx
@@ -36,6 +36,7 @@
     <sheet name="2026-08-10" sheetId="27" state="visible" r:id="rId27"/>
     <sheet name="2026-08-11" sheetId="28" state="visible" r:id="rId28"/>
     <sheet name="2026-08-12" sheetId="29" state="visible" r:id="rId29"/>
+    <sheet name="2026-08-13" sheetId="30" state="visible" r:id="rId30"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -19193,6 +19194,870 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet30.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C57"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="29" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Clan: Mans Best Friend (3815)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Timestamp: 2026-08-13 13:01:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>Total Reps</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>Daily Reps (+1d)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>Nobodys Son</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>Player</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>Player</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>X y L O T A</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>AbdiHyde ID 13496</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>Create Character III</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C9" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>Create Character IV</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>Create Character V</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C11" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t>Player</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C12" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="4" t="inlineStr">
+        <is>
+          <t>Player</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C13" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="4" t="inlineStr">
+        <is>
+          <t>hunry</t>
+        </is>
+      </c>
+      <c r="B14" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C14" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="4" t="inlineStr">
+        <is>
+          <t>BlacKRin O</t>
+        </is>
+      </c>
+      <c r="B15" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C15" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="4" t="inlineStr">
+        <is>
+          <t>Tears</t>
+        </is>
+      </c>
+      <c r="B16" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C16" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="4" t="inlineStr">
+        <is>
+          <t>Sugar Talking</t>
+        </is>
+      </c>
+      <c r="B17" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C17" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="4" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B18" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C18" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="4" t="inlineStr">
+        <is>
+          <t>Anti-Hero</t>
+        </is>
+      </c>
+      <c r="B19" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C19" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="4" t="inlineStr">
+        <is>
+          <t>Vigilante Shit</t>
+        </is>
+      </c>
+      <c r="B20" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C20" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="4" t="inlineStr">
+        <is>
+          <t>Sweet Nothing</t>
+        </is>
+      </c>
+      <c r="B21" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C21" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="4" t="inlineStr">
+        <is>
+          <t>The Great War</t>
+        </is>
+      </c>
+      <c r="B22" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C22" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">We Almost Broke Up </t>
+        </is>
+      </c>
+      <c r="B23" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C23" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="4" t="inlineStr">
+        <is>
+          <t>When Did You Get Hot</t>
+        </is>
+      </c>
+      <c r="B24" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C24" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="4" t="inlineStr">
+        <is>
+          <t>Dont Worry Ill Make</t>
+        </is>
+      </c>
+      <c r="B25" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C25" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="4" t="inlineStr">
+        <is>
+          <t>Goodbye</t>
+        </is>
+      </c>
+      <c r="B26" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C26" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="4" t="inlineStr">
+        <is>
+          <t>Mans Best Friend</t>
+        </is>
+      </c>
+      <c r="B27" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C27" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="4" t="inlineStr">
+        <is>
+          <t>Lavender Haze</t>
+        </is>
+      </c>
+      <c r="B28" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C28" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="4" t="inlineStr">
+        <is>
+          <t>Never Getting Laid</t>
+        </is>
+      </c>
+      <c r="B29" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C29" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="4" t="inlineStr">
+        <is>
+          <t>My Man on Willpower</t>
+        </is>
+      </c>
+      <c r="B30" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C30" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="4" t="inlineStr">
+        <is>
+          <t>Manchild</t>
+        </is>
+      </c>
+      <c r="B31" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C31" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="4" t="inlineStr">
+        <is>
+          <t>Sugar Talking</t>
+        </is>
+      </c>
+      <c r="B32" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C32" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="4" t="inlineStr">
+        <is>
+          <t>My Man on Willpower</t>
+        </is>
+      </c>
+      <c r="B33" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C33" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="4" t="inlineStr">
+        <is>
+          <t>Midnight Rain</t>
+        </is>
+      </c>
+      <c r="B34" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C34" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="4" t="inlineStr">
+        <is>
+          <t>Nobodys Son</t>
+        </is>
+      </c>
+      <c r="B35" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C35" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="4" t="inlineStr">
+        <is>
+          <t>House Tour</t>
+        </is>
+      </c>
+      <c r="B36" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C36" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="4" t="inlineStr">
+        <is>
+          <t>Hanabi  Î±Î·Ð²Ï…</t>
+        </is>
+      </c>
+      <c r="B37" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C37" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="4" t="inlineStr">
+        <is>
+          <t>Saiyajin anbuâ„¢</t>
+        </is>
+      </c>
+      <c r="B38" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C38" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="4" t="inlineStr">
+        <is>
+          <t>Dummy</t>
+        </is>
+      </c>
+      <c r="B39" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C39" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="4" t="inlineStr">
+        <is>
+          <t>Cazador anbu â„¢</t>
+        </is>
+      </c>
+      <c r="B40" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C40" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="4" t="inlineStr">
+        <is>
+          <t>Besos Mojados</t>
+        </is>
+      </c>
+      <c r="B41" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C41" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="4" t="inlineStr">
+        <is>
+          <t>DarkFire</t>
+        </is>
+      </c>
+      <c r="B42" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C42" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="4" t="inlineStr">
+        <is>
+          <t>DarkSunny</t>
+        </is>
+      </c>
+      <c r="B43" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C43" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="4" t="inlineStr">
+        <is>
+          <t>Dairen Uchiha</t>
+        </is>
+      </c>
+      <c r="B44" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C44" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="4" t="inlineStr">
+        <is>
+          <t>LILI ZENIN®</t>
+        </is>
+      </c>
+      <c r="B45" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C45" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="4" t="inlineStr">
+        <is>
+          <t>ryumichel ZENIN ®</t>
+        </is>
+      </c>
+      <c r="B46" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C46" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="4" t="inlineStr">
+        <is>
+          <t>margot ZENIN ®</t>
+        </is>
+      </c>
+      <c r="B47" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C47" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="4" t="inlineStr">
+        <is>
+          <t>linda ZENIN ®</t>
+        </is>
+      </c>
+      <c r="B48" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C48" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="4" t="inlineStr">
+        <is>
+          <t>equin0x</t>
+        </is>
+      </c>
+      <c r="B49" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C49" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="4" t="inlineStr">
+        <is>
+          <t>Jhayco - Mokai</t>
+        </is>
+      </c>
+      <c r="B50" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C50" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="4" t="inlineStr">
+        <is>
+          <t>Jhayco - Joe</t>
+        </is>
+      </c>
+      <c r="B51" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C51" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="4" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="B52" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C52" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="4" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="B53" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C53" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="4" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="B54" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C54" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="4" t="inlineStr">
+        <is>
+          <t>Go Go Juice</t>
+        </is>
+      </c>
+      <c r="B55" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C55" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="4" t="inlineStr">
+        <is>
+          <t>Jhayco - Imaginaste</t>
+        </is>
+      </c>
+      <c r="B56" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C56" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="4" t="inlineStr">
+        <is>
+          <t>PuNch</t>
+        </is>
+      </c>
+      <c r="B57" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C57" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A2:C2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
auto: snapshot 2026-08-14 13:01:01
</commit_message>
<xml_diff>
--- a/clan_3815.xlsx
+++ b/clan_3815.xlsx
@@ -37,6 +37,7 @@
     <sheet name="2026-08-11" sheetId="28" state="visible" r:id="rId28"/>
     <sheet name="2026-08-12" sheetId="29" state="visible" r:id="rId29"/>
     <sheet name="2026-08-13" sheetId="30" state="visible" r:id="rId30"/>
+    <sheet name="2026-08-14" sheetId="31" state="visible" r:id="rId31"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -20058,6 +20059,870 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet31.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C57"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="29" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Clan: Mans Best Friend (3815)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Timestamp: 2026-08-14 13:01:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>Total Reps</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>Daily Reps (+1d)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>Nobodys Son</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>Player</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>Player</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>X y L O T A</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>AbdiHyde ID 13496</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>Create Character III</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C9" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>Create Character IV</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>Create Character V</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C11" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t>Player</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C12" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="4" t="inlineStr">
+        <is>
+          <t>Player</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C13" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="4" t="inlineStr">
+        <is>
+          <t>hunry</t>
+        </is>
+      </c>
+      <c r="B14" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C14" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="4" t="inlineStr">
+        <is>
+          <t>BlacKRin O</t>
+        </is>
+      </c>
+      <c r="B15" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C15" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="4" t="inlineStr">
+        <is>
+          <t>Tears</t>
+        </is>
+      </c>
+      <c r="B16" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C16" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="4" t="inlineStr">
+        <is>
+          <t>Sugar Talking</t>
+        </is>
+      </c>
+      <c r="B17" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C17" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="4" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B18" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C18" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="4" t="inlineStr">
+        <is>
+          <t>Anti-Hero</t>
+        </is>
+      </c>
+      <c r="B19" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C19" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="4" t="inlineStr">
+        <is>
+          <t>Vigilante Shit</t>
+        </is>
+      </c>
+      <c r="B20" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C20" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="4" t="inlineStr">
+        <is>
+          <t>Sweet Nothing</t>
+        </is>
+      </c>
+      <c r="B21" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C21" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="4" t="inlineStr">
+        <is>
+          <t>The Great War</t>
+        </is>
+      </c>
+      <c r="B22" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C22" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">We Almost Broke Up </t>
+        </is>
+      </c>
+      <c r="B23" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C23" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="4" t="inlineStr">
+        <is>
+          <t>When Did You Get Hot</t>
+        </is>
+      </c>
+      <c r="B24" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C24" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="4" t="inlineStr">
+        <is>
+          <t>Dont Worry Ill Make</t>
+        </is>
+      </c>
+      <c r="B25" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C25" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="4" t="inlineStr">
+        <is>
+          <t>Goodbye</t>
+        </is>
+      </c>
+      <c r="B26" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C26" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="4" t="inlineStr">
+        <is>
+          <t>Mans Best Friend</t>
+        </is>
+      </c>
+      <c r="B27" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C27" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="4" t="inlineStr">
+        <is>
+          <t>Lavender Haze</t>
+        </is>
+      </c>
+      <c r="B28" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C28" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="4" t="inlineStr">
+        <is>
+          <t>Never Getting Laid</t>
+        </is>
+      </c>
+      <c r="B29" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C29" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="4" t="inlineStr">
+        <is>
+          <t>My Man on Willpower</t>
+        </is>
+      </c>
+      <c r="B30" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C30" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="4" t="inlineStr">
+        <is>
+          <t>Manchild</t>
+        </is>
+      </c>
+      <c r="B31" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C31" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="4" t="inlineStr">
+        <is>
+          <t>Sugar Talking</t>
+        </is>
+      </c>
+      <c r="B32" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C32" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="4" t="inlineStr">
+        <is>
+          <t>My Man on Willpower</t>
+        </is>
+      </c>
+      <c r="B33" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C33" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="4" t="inlineStr">
+        <is>
+          <t>Midnight Rain</t>
+        </is>
+      </c>
+      <c r="B34" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C34" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="4" t="inlineStr">
+        <is>
+          <t>Nobodys Son</t>
+        </is>
+      </c>
+      <c r="B35" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C35" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="4" t="inlineStr">
+        <is>
+          <t>House Tour</t>
+        </is>
+      </c>
+      <c r="B36" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C36" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="4" t="inlineStr">
+        <is>
+          <t>Hanabi  Î±Î·Ð²Ï…</t>
+        </is>
+      </c>
+      <c r="B37" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C37" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="4" t="inlineStr">
+        <is>
+          <t>Saiyajin anbuâ„¢</t>
+        </is>
+      </c>
+      <c r="B38" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C38" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="4" t="inlineStr">
+        <is>
+          <t>Dummy</t>
+        </is>
+      </c>
+      <c r="B39" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C39" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="4" t="inlineStr">
+        <is>
+          <t>Cazador anbu â„¢</t>
+        </is>
+      </c>
+      <c r="B40" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C40" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="4" t="inlineStr">
+        <is>
+          <t>Besos Mojados</t>
+        </is>
+      </c>
+      <c r="B41" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C41" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="4" t="inlineStr">
+        <is>
+          <t>DarkFire</t>
+        </is>
+      </c>
+      <c r="B42" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C42" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="4" t="inlineStr">
+        <is>
+          <t>DarkSunny</t>
+        </is>
+      </c>
+      <c r="B43" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C43" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="4" t="inlineStr">
+        <is>
+          <t>Dairen Uchiha</t>
+        </is>
+      </c>
+      <c r="B44" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C44" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="4" t="inlineStr">
+        <is>
+          <t>LILI ZENIN®</t>
+        </is>
+      </c>
+      <c r="B45" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C45" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="4" t="inlineStr">
+        <is>
+          <t>ryumichel ZENIN ®</t>
+        </is>
+      </c>
+      <c r="B46" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C46" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="4" t="inlineStr">
+        <is>
+          <t>margot ZENIN ®</t>
+        </is>
+      </c>
+      <c r="B47" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C47" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="4" t="inlineStr">
+        <is>
+          <t>linda ZENIN ®</t>
+        </is>
+      </c>
+      <c r="B48" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C48" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="4" t="inlineStr">
+        <is>
+          <t>equin0x</t>
+        </is>
+      </c>
+      <c r="B49" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C49" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="4" t="inlineStr">
+        <is>
+          <t>Jhayco - Mokai</t>
+        </is>
+      </c>
+      <c r="B50" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C50" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="4" t="inlineStr">
+        <is>
+          <t>Jhayco - Joe</t>
+        </is>
+      </c>
+      <c r="B51" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C51" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="4" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="B52" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C52" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="4" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="B53" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C53" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="4" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="B54" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C54" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="4" t="inlineStr">
+        <is>
+          <t>Go Go Juice</t>
+        </is>
+      </c>
+      <c r="B55" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C55" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="4" t="inlineStr">
+        <is>
+          <t>Jhayco - Imaginaste</t>
+        </is>
+      </c>
+      <c r="B56" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C56" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="4" t="inlineStr">
+        <is>
+          <t>PuNch</t>
+        </is>
+      </c>
+      <c r="B57" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C57" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A2:C2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
auto: snapshot 2026-08-15 13:01:01
</commit_message>
<xml_diff>
--- a/clan_3815.xlsx
+++ b/clan_3815.xlsx
@@ -38,6 +38,7 @@
     <sheet name="2026-08-12" sheetId="29" state="visible" r:id="rId29"/>
     <sheet name="2026-08-13" sheetId="30" state="visible" r:id="rId30"/>
     <sheet name="2026-08-14" sheetId="31" state="visible" r:id="rId31"/>
+    <sheet name="2026-08-15" sheetId="32" state="visible" r:id="rId32"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -20923,6 +20924,870 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet32.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C57"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="29" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Clan: Mans Best Friend (3815)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Timestamp: 2026-08-15 13:01:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>Total Reps</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>Daily Reps (+1d)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>Nobodys Son</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>Player</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>Player</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>X y L O T A</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>AbdiHyde ID 13496</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>Create Character III</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C9" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>Create Character IV</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>Create Character V</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C11" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t>Player</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C12" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="4" t="inlineStr">
+        <is>
+          <t>Player</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C13" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="4" t="inlineStr">
+        <is>
+          <t>hunry</t>
+        </is>
+      </c>
+      <c r="B14" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C14" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="4" t="inlineStr">
+        <is>
+          <t>BlacKRin O</t>
+        </is>
+      </c>
+      <c r="B15" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C15" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="4" t="inlineStr">
+        <is>
+          <t>Tears</t>
+        </is>
+      </c>
+      <c r="B16" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C16" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="4" t="inlineStr">
+        <is>
+          <t>Sugar Talking</t>
+        </is>
+      </c>
+      <c r="B17" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C17" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="4" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B18" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C18" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="4" t="inlineStr">
+        <is>
+          <t>Anti-Hero</t>
+        </is>
+      </c>
+      <c r="B19" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C19" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="4" t="inlineStr">
+        <is>
+          <t>Vigilante Shit</t>
+        </is>
+      </c>
+      <c r="B20" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C20" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="4" t="inlineStr">
+        <is>
+          <t>Sweet Nothing</t>
+        </is>
+      </c>
+      <c r="B21" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C21" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="4" t="inlineStr">
+        <is>
+          <t>The Great War</t>
+        </is>
+      </c>
+      <c r="B22" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C22" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">We Almost Broke Up </t>
+        </is>
+      </c>
+      <c r="B23" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C23" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="4" t="inlineStr">
+        <is>
+          <t>When Did You Get Hot</t>
+        </is>
+      </c>
+      <c r="B24" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C24" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="4" t="inlineStr">
+        <is>
+          <t>Dont Worry Ill Make</t>
+        </is>
+      </c>
+      <c r="B25" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C25" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="4" t="inlineStr">
+        <is>
+          <t>Goodbye</t>
+        </is>
+      </c>
+      <c r="B26" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C26" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="4" t="inlineStr">
+        <is>
+          <t>Mans Best Friend</t>
+        </is>
+      </c>
+      <c r="B27" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C27" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="4" t="inlineStr">
+        <is>
+          <t>Lavender Haze</t>
+        </is>
+      </c>
+      <c r="B28" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C28" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="4" t="inlineStr">
+        <is>
+          <t>Never Getting Laid</t>
+        </is>
+      </c>
+      <c r="B29" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C29" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="4" t="inlineStr">
+        <is>
+          <t>My Man on Willpower</t>
+        </is>
+      </c>
+      <c r="B30" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C30" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="4" t="inlineStr">
+        <is>
+          <t>Manchild</t>
+        </is>
+      </c>
+      <c r="B31" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C31" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="4" t="inlineStr">
+        <is>
+          <t>Sugar Talking</t>
+        </is>
+      </c>
+      <c r="B32" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C32" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="4" t="inlineStr">
+        <is>
+          <t>My Man on Willpower</t>
+        </is>
+      </c>
+      <c r="B33" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C33" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="4" t="inlineStr">
+        <is>
+          <t>Midnight Rain</t>
+        </is>
+      </c>
+      <c r="B34" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C34" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="4" t="inlineStr">
+        <is>
+          <t>Nobodys Son</t>
+        </is>
+      </c>
+      <c r="B35" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C35" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="4" t="inlineStr">
+        <is>
+          <t>House Tour</t>
+        </is>
+      </c>
+      <c r="B36" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C36" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="4" t="inlineStr">
+        <is>
+          <t>Hanabi  Î±Î·Ð²Ï…</t>
+        </is>
+      </c>
+      <c r="B37" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C37" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="4" t="inlineStr">
+        <is>
+          <t>Saiyajin anbuâ„¢</t>
+        </is>
+      </c>
+      <c r="B38" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C38" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="4" t="inlineStr">
+        <is>
+          <t>Dummy</t>
+        </is>
+      </c>
+      <c r="B39" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C39" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="4" t="inlineStr">
+        <is>
+          <t>Cazador anbu â„¢</t>
+        </is>
+      </c>
+      <c r="B40" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C40" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="4" t="inlineStr">
+        <is>
+          <t>Besos Mojados</t>
+        </is>
+      </c>
+      <c r="B41" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C41" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="4" t="inlineStr">
+        <is>
+          <t>DarkFire</t>
+        </is>
+      </c>
+      <c r="B42" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C42" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="4" t="inlineStr">
+        <is>
+          <t>DarkSunny</t>
+        </is>
+      </c>
+      <c r="B43" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C43" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="4" t="inlineStr">
+        <is>
+          <t>Dairen Uchiha</t>
+        </is>
+      </c>
+      <c r="B44" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C44" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="4" t="inlineStr">
+        <is>
+          <t>LILI ZENIN®</t>
+        </is>
+      </c>
+      <c r="B45" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C45" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="4" t="inlineStr">
+        <is>
+          <t>ryumichel ZENIN ®</t>
+        </is>
+      </c>
+      <c r="B46" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C46" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="4" t="inlineStr">
+        <is>
+          <t>margot ZENIN ®</t>
+        </is>
+      </c>
+      <c r="B47" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C47" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="4" t="inlineStr">
+        <is>
+          <t>linda ZENIN ®</t>
+        </is>
+      </c>
+      <c r="B48" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C48" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="4" t="inlineStr">
+        <is>
+          <t>equin0x</t>
+        </is>
+      </c>
+      <c r="B49" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C49" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="4" t="inlineStr">
+        <is>
+          <t>Jhayco - Mokai</t>
+        </is>
+      </c>
+      <c r="B50" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C50" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="4" t="inlineStr">
+        <is>
+          <t>Jhayco - Joe</t>
+        </is>
+      </c>
+      <c r="B51" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C51" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="4" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="B52" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C52" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="4" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="B53" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C53" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="4" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="B54" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C54" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="4" t="inlineStr">
+        <is>
+          <t>Go Go Juice</t>
+        </is>
+      </c>
+      <c r="B55" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C55" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="4" t="inlineStr">
+        <is>
+          <t>Jhayco - Imaginaste</t>
+        </is>
+      </c>
+      <c r="B56" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C56" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="4" t="inlineStr">
+        <is>
+          <t>PuNch</t>
+        </is>
+      </c>
+      <c r="B57" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C57" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A2:C2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
auto: snapshot 2026-08-16 13:01:00
</commit_message>
<xml_diff>
--- a/clan_3815.xlsx
+++ b/clan_3815.xlsx
@@ -39,6 +39,7 @@
     <sheet name="2026-08-13" sheetId="30" state="visible" r:id="rId30"/>
     <sheet name="2026-08-14" sheetId="31" state="visible" r:id="rId31"/>
     <sheet name="2026-08-15" sheetId="32" state="visible" r:id="rId32"/>
+    <sheet name="2026-08-16" sheetId="33" state="visible" r:id="rId33"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -21788,6 +21789,870 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet33.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C57"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="29" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Clan: Mans Best Friend (3815)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Timestamp: 2026-08-16 13:01:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>Total Reps</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>Daily Reps (+1d)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>Nobodys Son</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>Player</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>Player</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>X y L O T A</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>AbdiHyde ID 13496</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>Create Character III</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C9" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>Create Character IV</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>Create Character V</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C11" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t>Player</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C12" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="4" t="inlineStr">
+        <is>
+          <t>Player</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C13" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="4" t="inlineStr">
+        <is>
+          <t>hunry</t>
+        </is>
+      </c>
+      <c r="B14" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C14" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="4" t="inlineStr">
+        <is>
+          <t>BlacKRin O</t>
+        </is>
+      </c>
+      <c r="B15" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C15" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="4" t="inlineStr">
+        <is>
+          <t>Tears</t>
+        </is>
+      </c>
+      <c r="B16" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C16" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="4" t="inlineStr">
+        <is>
+          <t>Sugar Talking</t>
+        </is>
+      </c>
+      <c r="B17" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C17" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="4" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B18" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C18" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="4" t="inlineStr">
+        <is>
+          <t>Anti-Hero</t>
+        </is>
+      </c>
+      <c r="B19" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C19" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="4" t="inlineStr">
+        <is>
+          <t>Vigilante Shit</t>
+        </is>
+      </c>
+      <c r="B20" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C20" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="4" t="inlineStr">
+        <is>
+          <t>Sweet Nothing</t>
+        </is>
+      </c>
+      <c r="B21" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C21" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="4" t="inlineStr">
+        <is>
+          <t>The Great War</t>
+        </is>
+      </c>
+      <c r="B22" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C22" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">We Almost Broke Up </t>
+        </is>
+      </c>
+      <c r="B23" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C23" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="4" t="inlineStr">
+        <is>
+          <t>When Did You Get Hot</t>
+        </is>
+      </c>
+      <c r="B24" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C24" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="4" t="inlineStr">
+        <is>
+          <t>Dont Worry Ill Make</t>
+        </is>
+      </c>
+      <c r="B25" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C25" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="4" t="inlineStr">
+        <is>
+          <t>Goodbye</t>
+        </is>
+      </c>
+      <c r="B26" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C26" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="4" t="inlineStr">
+        <is>
+          <t>Mans Best Friend</t>
+        </is>
+      </c>
+      <c r="B27" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C27" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="4" t="inlineStr">
+        <is>
+          <t>Lavender Haze</t>
+        </is>
+      </c>
+      <c r="B28" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C28" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="4" t="inlineStr">
+        <is>
+          <t>Never Getting Laid</t>
+        </is>
+      </c>
+      <c r="B29" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C29" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="4" t="inlineStr">
+        <is>
+          <t>My Man on Willpower</t>
+        </is>
+      </c>
+      <c r="B30" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C30" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="4" t="inlineStr">
+        <is>
+          <t>Manchild</t>
+        </is>
+      </c>
+      <c r="B31" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C31" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="4" t="inlineStr">
+        <is>
+          <t>Sugar Talking</t>
+        </is>
+      </c>
+      <c r="B32" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C32" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="4" t="inlineStr">
+        <is>
+          <t>My Man on Willpower</t>
+        </is>
+      </c>
+      <c r="B33" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C33" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="4" t="inlineStr">
+        <is>
+          <t>Midnight Rain</t>
+        </is>
+      </c>
+      <c r="B34" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C34" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="4" t="inlineStr">
+        <is>
+          <t>Nobodys Son</t>
+        </is>
+      </c>
+      <c r="B35" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C35" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="4" t="inlineStr">
+        <is>
+          <t>House Tour</t>
+        </is>
+      </c>
+      <c r="B36" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C36" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="4" t="inlineStr">
+        <is>
+          <t>Hanabi  Î±Î·Ð²Ï…</t>
+        </is>
+      </c>
+      <c r="B37" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C37" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="4" t="inlineStr">
+        <is>
+          <t>Saiyajin anbuâ„¢</t>
+        </is>
+      </c>
+      <c r="B38" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C38" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="4" t="inlineStr">
+        <is>
+          <t>Dummy</t>
+        </is>
+      </c>
+      <c r="B39" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C39" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="4" t="inlineStr">
+        <is>
+          <t>Cazador anbu â„¢</t>
+        </is>
+      </c>
+      <c r="B40" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C40" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="4" t="inlineStr">
+        <is>
+          <t>Besos Mojados</t>
+        </is>
+      </c>
+      <c r="B41" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C41" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="4" t="inlineStr">
+        <is>
+          <t>DarkFire</t>
+        </is>
+      </c>
+      <c r="B42" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C42" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="4" t="inlineStr">
+        <is>
+          <t>DarkSunny</t>
+        </is>
+      </c>
+      <c r="B43" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C43" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="4" t="inlineStr">
+        <is>
+          <t>Dairen Uchiha</t>
+        </is>
+      </c>
+      <c r="B44" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C44" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="4" t="inlineStr">
+        <is>
+          <t>LILI ZENIN®</t>
+        </is>
+      </c>
+      <c r="B45" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C45" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="4" t="inlineStr">
+        <is>
+          <t>ryumichel ZENIN ®</t>
+        </is>
+      </c>
+      <c r="B46" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C46" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="4" t="inlineStr">
+        <is>
+          <t>margot ZENIN ®</t>
+        </is>
+      </c>
+      <c r="B47" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C47" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="4" t="inlineStr">
+        <is>
+          <t>linda ZENIN ®</t>
+        </is>
+      </c>
+      <c r="B48" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C48" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="4" t="inlineStr">
+        <is>
+          <t>equin0x</t>
+        </is>
+      </c>
+      <c r="B49" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C49" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="4" t="inlineStr">
+        <is>
+          <t>Jhayco - Mokai</t>
+        </is>
+      </c>
+      <c r="B50" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C50" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="4" t="inlineStr">
+        <is>
+          <t>Jhayco - Joe</t>
+        </is>
+      </c>
+      <c r="B51" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C51" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="4" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="B52" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C52" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="4" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="B53" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C53" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="4" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="B54" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C54" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="4" t="inlineStr">
+        <is>
+          <t>Go Go Juice</t>
+        </is>
+      </c>
+      <c r="B55" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C55" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="4" t="inlineStr">
+        <is>
+          <t>Jhayco - Imaginaste</t>
+        </is>
+      </c>
+      <c r="B56" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C56" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="4" t="inlineStr">
+        <is>
+          <t>PuNch</t>
+        </is>
+      </c>
+      <c r="B57" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C57" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A2:C2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
auto: snapshot 2026-08-17 13:01:01
</commit_message>
<xml_diff>
--- a/clan_3815.xlsx
+++ b/clan_3815.xlsx
@@ -40,6 +40,7 @@
     <sheet name="2026-08-14" sheetId="31" state="visible" r:id="rId31"/>
     <sheet name="2026-08-15" sheetId="32" state="visible" r:id="rId32"/>
     <sheet name="2026-08-16" sheetId="33" state="visible" r:id="rId33"/>
+    <sheet name="2026-08-17" sheetId="34" state="visible" r:id="rId34"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -22653,6 +22654,870 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet34.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C57"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="29" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Clan: Mans Best Friend (3815)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Timestamp: 2026-08-17 13:01:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>Total Reps</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>Daily Reps (+1d)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>Nobodys Son</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>Player</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>Player</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>X y L O T A</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>AbdiHyde ID 13496</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>Create Character III</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C9" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>Create Character IV</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>Create Character V</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C11" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t>Player</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C12" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="4" t="inlineStr">
+        <is>
+          <t>Player</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C13" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="4" t="inlineStr">
+        <is>
+          <t>hunry</t>
+        </is>
+      </c>
+      <c r="B14" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C14" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="4" t="inlineStr">
+        <is>
+          <t>BlacKRin O</t>
+        </is>
+      </c>
+      <c r="B15" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C15" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="4" t="inlineStr">
+        <is>
+          <t>Tears</t>
+        </is>
+      </c>
+      <c r="B16" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C16" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="4" t="inlineStr">
+        <is>
+          <t>Sugar Talking</t>
+        </is>
+      </c>
+      <c r="B17" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C17" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="4" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B18" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C18" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="4" t="inlineStr">
+        <is>
+          <t>Anti-Hero</t>
+        </is>
+      </c>
+      <c r="B19" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C19" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="4" t="inlineStr">
+        <is>
+          <t>Vigilante Shit</t>
+        </is>
+      </c>
+      <c r="B20" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C20" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="4" t="inlineStr">
+        <is>
+          <t>Sweet Nothing</t>
+        </is>
+      </c>
+      <c r="B21" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C21" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="4" t="inlineStr">
+        <is>
+          <t>The Great War</t>
+        </is>
+      </c>
+      <c r="B22" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C22" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">We Almost Broke Up </t>
+        </is>
+      </c>
+      <c r="B23" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C23" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="4" t="inlineStr">
+        <is>
+          <t>When Did You Get Hot</t>
+        </is>
+      </c>
+      <c r="B24" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C24" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="4" t="inlineStr">
+        <is>
+          <t>Dont Worry Ill Make</t>
+        </is>
+      </c>
+      <c r="B25" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C25" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="4" t="inlineStr">
+        <is>
+          <t>Goodbye</t>
+        </is>
+      </c>
+      <c r="B26" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C26" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="4" t="inlineStr">
+        <is>
+          <t>Mans Best Friend</t>
+        </is>
+      </c>
+      <c r="B27" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C27" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="4" t="inlineStr">
+        <is>
+          <t>Lavender Haze</t>
+        </is>
+      </c>
+      <c r="B28" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C28" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="4" t="inlineStr">
+        <is>
+          <t>Never Getting Laid</t>
+        </is>
+      </c>
+      <c r="B29" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C29" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="4" t="inlineStr">
+        <is>
+          <t>My Man on Willpower</t>
+        </is>
+      </c>
+      <c r="B30" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C30" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="4" t="inlineStr">
+        <is>
+          <t>Manchild</t>
+        </is>
+      </c>
+      <c r="B31" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C31" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="4" t="inlineStr">
+        <is>
+          <t>Sugar Talking</t>
+        </is>
+      </c>
+      <c r="B32" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C32" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="4" t="inlineStr">
+        <is>
+          <t>My Man on Willpower</t>
+        </is>
+      </c>
+      <c r="B33" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C33" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="4" t="inlineStr">
+        <is>
+          <t>Midnight Rain</t>
+        </is>
+      </c>
+      <c r="B34" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C34" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="4" t="inlineStr">
+        <is>
+          <t>Nobodys Son</t>
+        </is>
+      </c>
+      <c r="B35" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C35" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="4" t="inlineStr">
+        <is>
+          <t>House Tour</t>
+        </is>
+      </c>
+      <c r="B36" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C36" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="4" t="inlineStr">
+        <is>
+          <t>Hanabi  Î±Î·Ð²Ï…</t>
+        </is>
+      </c>
+      <c r="B37" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C37" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="4" t="inlineStr">
+        <is>
+          <t>Saiyajin anbuâ„¢</t>
+        </is>
+      </c>
+      <c r="B38" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C38" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="4" t="inlineStr">
+        <is>
+          <t>Dummy</t>
+        </is>
+      </c>
+      <c r="B39" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C39" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="4" t="inlineStr">
+        <is>
+          <t>Cazador anbu â„¢</t>
+        </is>
+      </c>
+      <c r="B40" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C40" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="4" t="inlineStr">
+        <is>
+          <t>Besos Mojados</t>
+        </is>
+      </c>
+      <c r="B41" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C41" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="4" t="inlineStr">
+        <is>
+          <t>DarkFire</t>
+        </is>
+      </c>
+      <c r="B42" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C42" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="4" t="inlineStr">
+        <is>
+          <t>DarkSunny</t>
+        </is>
+      </c>
+      <c r="B43" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C43" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="4" t="inlineStr">
+        <is>
+          <t>Dairen Uchiha</t>
+        </is>
+      </c>
+      <c r="B44" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C44" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="4" t="inlineStr">
+        <is>
+          <t>LILI ZENIN®</t>
+        </is>
+      </c>
+      <c r="B45" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C45" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="4" t="inlineStr">
+        <is>
+          <t>ryumichel ZENIN ®</t>
+        </is>
+      </c>
+      <c r="B46" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C46" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="4" t="inlineStr">
+        <is>
+          <t>margot ZENIN ®</t>
+        </is>
+      </c>
+      <c r="B47" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C47" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="4" t="inlineStr">
+        <is>
+          <t>linda ZENIN ®</t>
+        </is>
+      </c>
+      <c r="B48" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C48" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="4" t="inlineStr">
+        <is>
+          <t>equin0x</t>
+        </is>
+      </c>
+      <c r="B49" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C49" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="4" t="inlineStr">
+        <is>
+          <t>Jhayco - Mokai</t>
+        </is>
+      </c>
+      <c r="B50" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C50" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="4" t="inlineStr">
+        <is>
+          <t>Jhayco - Joe</t>
+        </is>
+      </c>
+      <c r="B51" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C51" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="4" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="B52" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C52" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="4" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="B53" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C53" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="4" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="B54" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C54" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="4" t="inlineStr">
+        <is>
+          <t>Go Go Juice</t>
+        </is>
+      </c>
+      <c r="B55" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C55" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="4" t="inlineStr">
+        <is>
+          <t>Jhayco - Imaginaste</t>
+        </is>
+      </c>
+      <c r="B56" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C56" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="4" t="inlineStr">
+        <is>
+          <t>PuNch</t>
+        </is>
+      </c>
+      <c r="B57" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C57" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A2:C2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
auto: snapshot 2026-08-18 13:01:00
</commit_message>
<xml_diff>
--- a/clan_3815.xlsx
+++ b/clan_3815.xlsx
@@ -41,6 +41,7 @@
     <sheet name="2026-08-15" sheetId="32" state="visible" r:id="rId32"/>
     <sheet name="2026-08-16" sheetId="33" state="visible" r:id="rId33"/>
     <sheet name="2026-08-17" sheetId="34" state="visible" r:id="rId34"/>
+    <sheet name="2026-08-18" sheetId="35" state="visible" r:id="rId35"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -23518,6 +23519,870 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet35.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C57"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="29" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Clan: Mans Best Friend (3815)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Timestamp: 2026-08-18 13:01:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>Total Reps</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>Daily Reps (+1d)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>Nobodys Son</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>Player</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>Player</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>X y L O T A</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>AbdiHyde ID 13496</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>Create Character III</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C9" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>Create Character IV</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>Create Character V</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C11" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t>Player</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C12" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="4" t="inlineStr">
+        <is>
+          <t>Player</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C13" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="4" t="inlineStr">
+        <is>
+          <t>hunry</t>
+        </is>
+      </c>
+      <c r="B14" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C14" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="4" t="inlineStr">
+        <is>
+          <t>BlacKRin O</t>
+        </is>
+      </c>
+      <c r="B15" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C15" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="4" t="inlineStr">
+        <is>
+          <t>Tears</t>
+        </is>
+      </c>
+      <c r="B16" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C16" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="4" t="inlineStr">
+        <is>
+          <t>Sugar Talking</t>
+        </is>
+      </c>
+      <c r="B17" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C17" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="4" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B18" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C18" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="4" t="inlineStr">
+        <is>
+          <t>Anti-Hero</t>
+        </is>
+      </c>
+      <c r="B19" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C19" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="4" t="inlineStr">
+        <is>
+          <t>Vigilante Shit</t>
+        </is>
+      </c>
+      <c r="B20" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C20" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="4" t="inlineStr">
+        <is>
+          <t>Sweet Nothing</t>
+        </is>
+      </c>
+      <c r="B21" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C21" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="4" t="inlineStr">
+        <is>
+          <t>The Great War</t>
+        </is>
+      </c>
+      <c r="B22" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C22" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">We Almost Broke Up </t>
+        </is>
+      </c>
+      <c r="B23" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C23" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="4" t="inlineStr">
+        <is>
+          <t>When Did You Get Hot</t>
+        </is>
+      </c>
+      <c r="B24" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C24" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="4" t="inlineStr">
+        <is>
+          <t>Dont Worry Ill Make</t>
+        </is>
+      </c>
+      <c r="B25" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C25" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="4" t="inlineStr">
+        <is>
+          <t>Goodbye</t>
+        </is>
+      </c>
+      <c r="B26" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C26" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="4" t="inlineStr">
+        <is>
+          <t>Mans Best Friend</t>
+        </is>
+      </c>
+      <c r="B27" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C27" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="4" t="inlineStr">
+        <is>
+          <t>Lavender Haze</t>
+        </is>
+      </c>
+      <c r="B28" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C28" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="4" t="inlineStr">
+        <is>
+          <t>Never Getting Laid</t>
+        </is>
+      </c>
+      <c r="B29" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C29" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="4" t="inlineStr">
+        <is>
+          <t>My Man on Willpower</t>
+        </is>
+      </c>
+      <c r="B30" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C30" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="4" t="inlineStr">
+        <is>
+          <t>Manchild</t>
+        </is>
+      </c>
+      <c r="B31" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C31" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="4" t="inlineStr">
+        <is>
+          <t>Sugar Talking</t>
+        </is>
+      </c>
+      <c r="B32" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C32" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="4" t="inlineStr">
+        <is>
+          <t>My Man on Willpower</t>
+        </is>
+      </c>
+      <c r="B33" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C33" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="4" t="inlineStr">
+        <is>
+          <t>Midnight Rain</t>
+        </is>
+      </c>
+      <c r="B34" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C34" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="4" t="inlineStr">
+        <is>
+          <t>Nobodys Son</t>
+        </is>
+      </c>
+      <c r="B35" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C35" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="4" t="inlineStr">
+        <is>
+          <t>House Tour</t>
+        </is>
+      </c>
+      <c r="B36" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C36" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="4" t="inlineStr">
+        <is>
+          <t>Hanabi  Î±Î·Ð²Ï…</t>
+        </is>
+      </c>
+      <c r="B37" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C37" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="4" t="inlineStr">
+        <is>
+          <t>Saiyajin anbuâ„¢</t>
+        </is>
+      </c>
+      <c r="B38" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C38" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="4" t="inlineStr">
+        <is>
+          <t>Dummy</t>
+        </is>
+      </c>
+      <c r="B39" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C39" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="4" t="inlineStr">
+        <is>
+          <t>Cazador anbu â„¢</t>
+        </is>
+      </c>
+      <c r="B40" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C40" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="4" t="inlineStr">
+        <is>
+          <t>Besos Mojados</t>
+        </is>
+      </c>
+      <c r="B41" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C41" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="4" t="inlineStr">
+        <is>
+          <t>DarkFire</t>
+        </is>
+      </c>
+      <c r="B42" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C42" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="4" t="inlineStr">
+        <is>
+          <t>DarkSunny</t>
+        </is>
+      </c>
+      <c r="B43" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C43" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="4" t="inlineStr">
+        <is>
+          <t>Dairen Uchiha</t>
+        </is>
+      </c>
+      <c r="B44" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C44" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="4" t="inlineStr">
+        <is>
+          <t>LILI ZENIN®</t>
+        </is>
+      </c>
+      <c r="B45" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C45" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="4" t="inlineStr">
+        <is>
+          <t>ryumichel ZENIN ®</t>
+        </is>
+      </c>
+      <c r="B46" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C46" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="4" t="inlineStr">
+        <is>
+          <t>margot ZENIN ®</t>
+        </is>
+      </c>
+      <c r="B47" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C47" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="4" t="inlineStr">
+        <is>
+          <t>linda ZENIN ®</t>
+        </is>
+      </c>
+      <c r="B48" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C48" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="4" t="inlineStr">
+        <is>
+          <t>equin0x</t>
+        </is>
+      </c>
+      <c r="B49" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C49" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="4" t="inlineStr">
+        <is>
+          <t>Jhayco - Mokai</t>
+        </is>
+      </c>
+      <c r="B50" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C50" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="4" t="inlineStr">
+        <is>
+          <t>Jhayco - Joe</t>
+        </is>
+      </c>
+      <c r="B51" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C51" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="4" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="B52" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C52" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="4" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="B53" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C53" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="4" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="B54" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C54" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="4" t="inlineStr">
+        <is>
+          <t>Go Go Juice</t>
+        </is>
+      </c>
+      <c r="B55" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C55" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="4" t="inlineStr">
+        <is>
+          <t>Jhayco - Imaginaste</t>
+        </is>
+      </c>
+      <c r="B56" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C56" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="4" t="inlineStr">
+        <is>
+          <t>PuNch</t>
+        </is>
+      </c>
+      <c r="B57" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C57" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A2:C2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
auto: snapshot 2026-08-19 13:01:01
</commit_message>
<xml_diff>
--- a/clan_3815.xlsx
+++ b/clan_3815.xlsx
@@ -42,6 +42,7 @@
     <sheet name="2026-08-16" sheetId="33" state="visible" r:id="rId33"/>
     <sheet name="2026-08-17" sheetId="34" state="visible" r:id="rId34"/>
     <sheet name="2026-08-18" sheetId="35" state="visible" r:id="rId35"/>
+    <sheet name="2026-08-19" sheetId="36" state="visible" r:id="rId36"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -24383,6 +24384,870 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet36.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C57"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="29" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Clan: Mans Best Friend (3815)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Timestamp: 2026-08-19 13:01:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>Total Reps</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>Daily Reps (+1d)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>Nobodys Son</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>Player</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>Player</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>X y L O T A</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>AbdiHyde ID 13496</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>Create Character III</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C9" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>Create Character IV</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>Create Character V</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C11" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t>Player</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C12" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="4" t="inlineStr">
+        <is>
+          <t>Player</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C13" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="4" t="inlineStr">
+        <is>
+          <t>hunry</t>
+        </is>
+      </c>
+      <c r="B14" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C14" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="4" t="inlineStr">
+        <is>
+          <t>BlacKRin O</t>
+        </is>
+      </c>
+      <c r="B15" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C15" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="4" t="inlineStr">
+        <is>
+          <t>Tears</t>
+        </is>
+      </c>
+      <c r="B16" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C16" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="4" t="inlineStr">
+        <is>
+          <t>Sugar Talking</t>
+        </is>
+      </c>
+      <c r="B17" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C17" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="4" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B18" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C18" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="4" t="inlineStr">
+        <is>
+          <t>Anti-Hero</t>
+        </is>
+      </c>
+      <c r="B19" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C19" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="4" t="inlineStr">
+        <is>
+          <t>Vigilante Shit</t>
+        </is>
+      </c>
+      <c r="B20" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C20" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="4" t="inlineStr">
+        <is>
+          <t>Sweet Nothing</t>
+        </is>
+      </c>
+      <c r="B21" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C21" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="4" t="inlineStr">
+        <is>
+          <t>The Great War</t>
+        </is>
+      </c>
+      <c r="B22" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C22" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">We Almost Broke Up </t>
+        </is>
+      </c>
+      <c r="B23" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C23" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="4" t="inlineStr">
+        <is>
+          <t>When Did You Get Hot</t>
+        </is>
+      </c>
+      <c r="B24" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C24" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="4" t="inlineStr">
+        <is>
+          <t>Dont Worry Ill Make</t>
+        </is>
+      </c>
+      <c r="B25" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C25" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="4" t="inlineStr">
+        <is>
+          <t>Goodbye</t>
+        </is>
+      </c>
+      <c r="B26" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C26" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="4" t="inlineStr">
+        <is>
+          <t>Mans Best Friend</t>
+        </is>
+      </c>
+      <c r="B27" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C27" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="4" t="inlineStr">
+        <is>
+          <t>Lavender Haze</t>
+        </is>
+      </c>
+      <c r="B28" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C28" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="4" t="inlineStr">
+        <is>
+          <t>Never Getting Laid</t>
+        </is>
+      </c>
+      <c r="B29" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C29" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="4" t="inlineStr">
+        <is>
+          <t>My Man on Willpower</t>
+        </is>
+      </c>
+      <c r="B30" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C30" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="4" t="inlineStr">
+        <is>
+          <t>Manchild</t>
+        </is>
+      </c>
+      <c r="B31" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C31" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="4" t="inlineStr">
+        <is>
+          <t>Sugar Talking</t>
+        </is>
+      </c>
+      <c r="B32" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C32" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="4" t="inlineStr">
+        <is>
+          <t>My Man on Willpower</t>
+        </is>
+      </c>
+      <c r="B33" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C33" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="4" t="inlineStr">
+        <is>
+          <t>Midnight Rain</t>
+        </is>
+      </c>
+      <c r="B34" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C34" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="4" t="inlineStr">
+        <is>
+          <t>Nobodys Son</t>
+        </is>
+      </c>
+      <c r="B35" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C35" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="4" t="inlineStr">
+        <is>
+          <t>House Tour</t>
+        </is>
+      </c>
+      <c r="B36" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C36" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="4" t="inlineStr">
+        <is>
+          <t>Hanabi  Î±Î·Ð²Ï…</t>
+        </is>
+      </c>
+      <c r="B37" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C37" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="4" t="inlineStr">
+        <is>
+          <t>Saiyajin anbuâ„¢</t>
+        </is>
+      </c>
+      <c r="B38" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C38" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="4" t="inlineStr">
+        <is>
+          <t>Dummy</t>
+        </is>
+      </c>
+      <c r="B39" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C39" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="4" t="inlineStr">
+        <is>
+          <t>Cazador anbu â„¢</t>
+        </is>
+      </c>
+      <c r="B40" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C40" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="4" t="inlineStr">
+        <is>
+          <t>Besos Mojados</t>
+        </is>
+      </c>
+      <c r="B41" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C41" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="4" t="inlineStr">
+        <is>
+          <t>DarkFire</t>
+        </is>
+      </c>
+      <c r="B42" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C42" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="4" t="inlineStr">
+        <is>
+          <t>DarkSunny</t>
+        </is>
+      </c>
+      <c r="B43" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C43" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="4" t="inlineStr">
+        <is>
+          <t>Dairen Uchiha</t>
+        </is>
+      </c>
+      <c r="B44" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C44" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="4" t="inlineStr">
+        <is>
+          <t>LILI ZENIN®</t>
+        </is>
+      </c>
+      <c r="B45" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C45" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="4" t="inlineStr">
+        <is>
+          <t>ryumichel ZENIN ®</t>
+        </is>
+      </c>
+      <c r="B46" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C46" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="4" t="inlineStr">
+        <is>
+          <t>margot ZENIN ®</t>
+        </is>
+      </c>
+      <c r="B47" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C47" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="4" t="inlineStr">
+        <is>
+          <t>linda ZENIN ®</t>
+        </is>
+      </c>
+      <c r="B48" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C48" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="4" t="inlineStr">
+        <is>
+          <t>equin0x</t>
+        </is>
+      </c>
+      <c r="B49" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C49" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="4" t="inlineStr">
+        <is>
+          <t>Jhayco - Mokai</t>
+        </is>
+      </c>
+      <c r="B50" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C50" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="4" t="inlineStr">
+        <is>
+          <t>Jhayco - Joe</t>
+        </is>
+      </c>
+      <c r="B51" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C51" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="4" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="B52" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C52" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="4" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="B53" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C53" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="4" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="B54" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C54" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="4" t="inlineStr">
+        <is>
+          <t>Go Go Juice</t>
+        </is>
+      </c>
+      <c r="B55" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C55" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="4" t="inlineStr">
+        <is>
+          <t>Jhayco - Imaginaste</t>
+        </is>
+      </c>
+      <c r="B56" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C56" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="4" t="inlineStr">
+        <is>
+          <t>PuNch</t>
+        </is>
+      </c>
+      <c r="B57" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C57" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A2:C2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
auto: snapshot 2026-08-20 13:01:01
</commit_message>
<xml_diff>
--- a/clan_3815.xlsx
+++ b/clan_3815.xlsx
@@ -43,6 +43,7 @@
     <sheet name="2026-08-17" sheetId="34" state="visible" r:id="rId34"/>
     <sheet name="2026-08-18" sheetId="35" state="visible" r:id="rId35"/>
     <sheet name="2026-08-19" sheetId="36" state="visible" r:id="rId36"/>
+    <sheet name="2026-08-20" sheetId="37" state="visible" r:id="rId37"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -25248,6 +25249,870 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet37.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C57"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="29" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Clan: Mans Best Friend (3815)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Timestamp: 2026-08-20 13:01:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>Total Reps</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>Daily Reps (+1d)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>Nobodys Son</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>Player</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>Player</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>X y L O T A</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>AbdiHyde ID 13496</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>Create Character III</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C9" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>Create Character IV</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>Create Character V</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C11" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t>Player</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C12" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="4" t="inlineStr">
+        <is>
+          <t>Player</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C13" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="4" t="inlineStr">
+        <is>
+          <t>hunry</t>
+        </is>
+      </c>
+      <c r="B14" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C14" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="4" t="inlineStr">
+        <is>
+          <t>BlacKRin O</t>
+        </is>
+      </c>
+      <c r="B15" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C15" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="4" t="inlineStr">
+        <is>
+          <t>Tears</t>
+        </is>
+      </c>
+      <c r="B16" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C16" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="4" t="inlineStr">
+        <is>
+          <t>Sugar Talking</t>
+        </is>
+      </c>
+      <c r="B17" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C17" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="4" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B18" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C18" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="4" t="inlineStr">
+        <is>
+          <t>Anti-Hero</t>
+        </is>
+      </c>
+      <c r="B19" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C19" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="4" t="inlineStr">
+        <is>
+          <t>Vigilante Shit</t>
+        </is>
+      </c>
+      <c r="B20" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C20" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="4" t="inlineStr">
+        <is>
+          <t>Sweet Nothing</t>
+        </is>
+      </c>
+      <c r="B21" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C21" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="4" t="inlineStr">
+        <is>
+          <t>The Great War</t>
+        </is>
+      </c>
+      <c r="B22" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C22" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">We Almost Broke Up </t>
+        </is>
+      </c>
+      <c r="B23" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C23" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="4" t="inlineStr">
+        <is>
+          <t>When Did You Get Hot</t>
+        </is>
+      </c>
+      <c r="B24" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C24" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="4" t="inlineStr">
+        <is>
+          <t>Dont Worry Ill Make</t>
+        </is>
+      </c>
+      <c r="B25" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C25" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="4" t="inlineStr">
+        <is>
+          <t>Goodbye</t>
+        </is>
+      </c>
+      <c r="B26" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C26" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="4" t="inlineStr">
+        <is>
+          <t>Mans Best Friend</t>
+        </is>
+      </c>
+      <c r="B27" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C27" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="4" t="inlineStr">
+        <is>
+          <t>Lavender Haze</t>
+        </is>
+      </c>
+      <c r="B28" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C28" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="4" t="inlineStr">
+        <is>
+          <t>Never Getting Laid</t>
+        </is>
+      </c>
+      <c r="B29" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C29" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="4" t="inlineStr">
+        <is>
+          <t>My Man on Willpower</t>
+        </is>
+      </c>
+      <c r="B30" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C30" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="4" t="inlineStr">
+        <is>
+          <t>Manchild</t>
+        </is>
+      </c>
+      <c r="B31" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C31" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="4" t="inlineStr">
+        <is>
+          <t>Sugar Talking</t>
+        </is>
+      </c>
+      <c r="B32" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C32" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="4" t="inlineStr">
+        <is>
+          <t>My Man on Willpower</t>
+        </is>
+      </c>
+      <c r="B33" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C33" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="4" t="inlineStr">
+        <is>
+          <t>Midnight Rain</t>
+        </is>
+      </c>
+      <c r="B34" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C34" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="4" t="inlineStr">
+        <is>
+          <t>Nobodys Son</t>
+        </is>
+      </c>
+      <c r="B35" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C35" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="4" t="inlineStr">
+        <is>
+          <t>House Tour</t>
+        </is>
+      </c>
+      <c r="B36" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C36" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="4" t="inlineStr">
+        <is>
+          <t>Hanabi  Î±Î·Ð²Ï…</t>
+        </is>
+      </c>
+      <c r="B37" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C37" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="4" t="inlineStr">
+        <is>
+          <t>Saiyajin anbuâ„¢</t>
+        </is>
+      </c>
+      <c r="B38" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C38" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="4" t="inlineStr">
+        <is>
+          <t>Dummy</t>
+        </is>
+      </c>
+      <c r="B39" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C39" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="4" t="inlineStr">
+        <is>
+          <t>Cazador anbu â„¢</t>
+        </is>
+      </c>
+      <c r="B40" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C40" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="4" t="inlineStr">
+        <is>
+          <t>Besos Mojados</t>
+        </is>
+      </c>
+      <c r="B41" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C41" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="4" t="inlineStr">
+        <is>
+          <t>DarkFire</t>
+        </is>
+      </c>
+      <c r="B42" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C42" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="4" t="inlineStr">
+        <is>
+          <t>DarkSunny</t>
+        </is>
+      </c>
+      <c r="B43" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C43" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="4" t="inlineStr">
+        <is>
+          <t>Dairen Uchiha</t>
+        </is>
+      </c>
+      <c r="B44" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C44" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="4" t="inlineStr">
+        <is>
+          <t>LILI ZENIN®</t>
+        </is>
+      </c>
+      <c r="B45" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C45" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="4" t="inlineStr">
+        <is>
+          <t>ryumichel ZENIN ®</t>
+        </is>
+      </c>
+      <c r="B46" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C46" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="4" t="inlineStr">
+        <is>
+          <t>margot ZENIN ®</t>
+        </is>
+      </c>
+      <c r="B47" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C47" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="4" t="inlineStr">
+        <is>
+          <t>linda ZENIN ®</t>
+        </is>
+      </c>
+      <c r="B48" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C48" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="4" t="inlineStr">
+        <is>
+          <t>equin0x</t>
+        </is>
+      </c>
+      <c r="B49" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C49" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="4" t="inlineStr">
+        <is>
+          <t>Jhayco - Mokai</t>
+        </is>
+      </c>
+      <c r="B50" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C50" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="4" t="inlineStr">
+        <is>
+          <t>Jhayco - Joe</t>
+        </is>
+      </c>
+      <c r="B51" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C51" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="4" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="B52" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C52" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="4" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="B53" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C53" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="4" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="B54" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C54" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="4" t="inlineStr">
+        <is>
+          <t>Go Go Juice</t>
+        </is>
+      </c>
+      <c r="B55" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C55" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="4" t="inlineStr">
+        <is>
+          <t>Jhayco - Imaginaste</t>
+        </is>
+      </c>
+      <c r="B56" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C56" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="4" t="inlineStr">
+        <is>
+          <t>PuNch</t>
+        </is>
+      </c>
+      <c r="B57" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C57" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A2:C2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
auto: snapshot 2026-08-21 13:01:00
</commit_message>
<xml_diff>
--- a/clan_3815.xlsx
+++ b/clan_3815.xlsx
@@ -44,6 +44,7 @@
     <sheet name="2026-08-18" sheetId="35" state="visible" r:id="rId35"/>
     <sheet name="2026-08-19" sheetId="36" state="visible" r:id="rId36"/>
     <sheet name="2026-08-20" sheetId="37" state="visible" r:id="rId37"/>
+    <sheet name="2026-08-21" sheetId="38" state="visible" r:id="rId38"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -26113,6 +26114,870 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet38.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C57"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="29" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Clan: Mans Best Friend (3815)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Timestamp: 2026-08-21 13:01:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>Total Reps</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>Daily Reps (+1d)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>Nobodys Son</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>Player</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>Player</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>X y L O T A</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>AbdiHyde ID 13496</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>Create Character III</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C9" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>Create Character IV</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>Create Character V</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C11" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t>Player</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C12" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="4" t="inlineStr">
+        <is>
+          <t>Player</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C13" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="4" t="inlineStr">
+        <is>
+          <t>hunry</t>
+        </is>
+      </c>
+      <c r="B14" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C14" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="4" t="inlineStr">
+        <is>
+          <t>BlacKRin O</t>
+        </is>
+      </c>
+      <c r="B15" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C15" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="4" t="inlineStr">
+        <is>
+          <t>Tears</t>
+        </is>
+      </c>
+      <c r="B16" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C16" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="4" t="inlineStr">
+        <is>
+          <t>Sugar Talking</t>
+        </is>
+      </c>
+      <c r="B17" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C17" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="4" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B18" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C18" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="4" t="inlineStr">
+        <is>
+          <t>Anti-Hero</t>
+        </is>
+      </c>
+      <c r="B19" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C19" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="4" t="inlineStr">
+        <is>
+          <t>Vigilante Shit</t>
+        </is>
+      </c>
+      <c r="B20" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C20" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="4" t="inlineStr">
+        <is>
+          <t>Sweet Nothing</t>
+        </is>
+      </c>
+      <c r="B21" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C21" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="4" t="inlineStr">
+        <is>
+          <t>The Great War</t>
+        </is>
+      </c>
+      <c r="B22" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C22" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">We Almost Broke Up </t>
+        </is>
+      </c>
+      <c r="B23" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C23" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="4" t="inlineStr">
+        <is>
+          <t>When Did You Get Hot</t>
+        </is>
+      </c>
+      <c r="B24" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C24" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="4" t="inlineStr">
+        <is>
+          <t>Dont Worry Ill Make</t>
+        </is>
+      </c>
+      <c r="B25" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C25" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="4" t="inlineStr">
+        <is>
+          <t>Goodbye</t>
+        </is>
+      </c>
+      <c r="B26" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C26" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="4" t="inlineStr">
+        <is>
+          <t>Mans Best Friend</t>
+        </is>
+      </c>
+      <c r="B27" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C27" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="4" t="inlineStr">
+        <is>
+          <t>Lavender Haze</t>
+        </is>
+      </c>
+      <c r="B28" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C28" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="4" t="inlineStr">
+        <is>
+          <t>Never Getting Laid</t>
+        </is>
+      </c>
+      <c r="B29" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C29" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="4" t="inlineStr">
+        <is>
+          <t>My Man on Willpower</t>
+        </is>
+      </c>
+      <c r="B30" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C30" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="4" t="inlineStr">
+        <is>
+          <t>Manchild</t>
+        </is>
+      </c>
+      <c r="B31" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C31" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="4" t="inlineStr">
+        <is>
+          <t>Sugar Talking</t>
+        </is>
+      </c>
+      <c r="B32" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C32" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="4" t="inlineStr">
+        <is>
+          <t>My Man on Willpower</t>
+        </is>
+      </c>
+      <c r="B33" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C33" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="4" t="inlineStr">
+        <is>
+          <t>Midnight Rain</t>
+        </is>
+      </c>
+      <c r="B34" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C34" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="4" t="inlineStr">
+        <is>
+          <t>Nobodys Son</t>
+        </is>
+      </c>
+      <c r="B35" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C35" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="4" t="inlineStr">
+        <is>
+          <t>House Tour</t>
+        </is>
+      </c>
+      <c r="B36" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C36" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="4" t="inlineStr">
+        <is>
+          <t>Hanabi  Î±Î·Ð²Ï…</t>
+        </is>
+      </c>
+      <c r="B37" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C37" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="4" t="inlineStr">
+        <is>
+          <t>Saiyajin anbuâ„¢</t>
+        </is>
+      </c>
+      <c r="B38" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C38" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="4" t="inlineStr">
+        <is>
+          <t>Dummy</t>
+        </is>
+      </c>
+      <c r="B39" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C39" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="4" t="inlineStr">
+        <is>
+          <t>Cazador anbu â„¢</t>
+        </is>
+      </c>
+      <c r="B40" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C40" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="4" t="inlineStr">
+        <is>
+          <t>Besos Mojados</t>
+        </is>
+      </c>
+      <c r="B41" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C41" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="4" t="inlineStr">
+        <is>
+          <t>DarkFire</t>
+        </is>
+      </c>
+      <c r="B42" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C42" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="4" t="inlineStr">
+        <is>
+          <t>DarkSunny</t>
+        </is>
+      </c>
+      <c r="B43" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C43" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="4" t="inlineStr">
+        <is>
+          <t>Dairen Uchiha</t>
+        </is>
+      </c>
+      <c r="B44" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C44" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="4" t="inlineStr">
+        <is>
+          <t>LILI ZENIN®</t>
+        </is>
+      </c>
+      <c r="B45" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C45" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="4" t="inlineStr">
+        <is>
+          <t>ryumichel ZENIN ®</t>
+        </is>
+      </c>
+      <c r="B46" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C46" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="4" t="inlineStr">
+        <is>
+          <t>margot ZENIN ®</t>
+        </is>
+      </c>
+      <c r="B47" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C47" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="4" t="inlineStr">
+        <is>
+          <t>linda ZENIN ®</t>
+        </is>
+      </c>
+      <c r="B48" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C48" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="4" t="inlineStr">
+        <is>
+          <t>equin0x</t>
+        </is>
+      </c>
+      <c r="B49" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C49" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="4" t="inlineStr">
+        <is>
+          <t>Jhayco - Mokai</t>
+        </is>
+      </c>
+      <c r="B50" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C50" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="4" t="inlineStr">
+        <is>
+          <t>Jhayco - Joe</t>
+        </is>
+      </c>
+      <c r="B51" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C51" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="4" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="B52" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C52" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="4" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="B53" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C53" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="4" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="B54" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C54" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="4" t="inlineStr">
+        <is>
+          <t>Go Go Juice</t>
+        </is>
+      </c>
+      <c r="B55" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C55" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="4" t="inlineStr">
+        <is>
+          <t>Jhayco - Imaginaste</t>
+        </is>
+      </c>
+      <c r="B56" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C56" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="4" t="inlineStr">
+        <is>
+          <t>PuNch</t>
+        </is>
+      </c>
+      <c r="B57" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C57" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A2:C2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
auto: snapshot 2026-08-22 13:01:02
</commit_message>
<xml_diff>
--- a/clan_3815.xlsx
+++ b/clan_3815.xlsx
@@ -45,6 +45,7 @@
     <sheet name="2026-08-19" sheetId="36" state="visible" r:id="rId36"/>
     <sheet name="2026-08-20" sheetId="37" state="visible" r:id="rId37"/>
     <sheet name="2026-08-21" sheetId="38" state="visible" r:id="rId38"/>
+    <sheet name="2026-08-22" sheetId="39" state="visible" r:id="rId39"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -26978,6 +26979,870 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet39.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C57"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="29" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Clan: Mans Best Friend (3815)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Timestamp: 2026-08-22 13:01:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>Total Reps</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>Daily Reps (+1d)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>Nobodys Son</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>Player</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>Player</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>X y L O T A</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>AbdiHyde ID 13496</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>Create Character III</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C9" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>Create Character IV</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>Create Character V</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C11" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t>Player</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C12" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="4" t="inlineStr">
+        <is>
+          <t>Player</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C13" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="4" t="inlineStr">
+        <is>
+          <t>hunry</t>
+        </is>
+      </c>
+      <c r="B14" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C14" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="4" t="inlineStr">
+        <is>
+          <t>BlacKRin O</t>
+        </is>
+      </c>
+      <c r="B15" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C15" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="4" t="inlineStr">
+        <is>
+          <t>Tears</t>
+        </is>
+      </c>
+      <c r="B16" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C16" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="4" t="inlineStr">
+        <is>
+          <t>Sugar Talking</t>
+        </is>
+      </c>
+      <c r="B17" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C17" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="4" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B18" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C18" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="4" t="inlineStr">
+        <is>
+          <t>Anti-Hero</t>
+        </is>
+      </c>
+      <c r="B19" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C19" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="4" t="inlineStr">
+        <is>
+          <t>Vigilante Shit</t>
+        </is>
+      </c>
+      <c r="B20" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C20" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="4" t="inlineStr">
+        <is>
+          <t>Sweet Nothing</t>
+        </is>
+      </c>
+      <c r="B21" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C21" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="4" t="inlineStr">
+        <is>
+          <t>The Great War</t>
+        </is>
+      </c>
+      <c r="B22" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C22" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">We Almost Broke Up </t>
+        </is>
+      </c>
+      <c r="B23" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C23" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="4" t="inlineStr">
+        <is>
+          <t>When Did You Get Hot</t>
+        </is>
+      </c>
+      <c r="B24" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C24" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="4" t="inlineStr">
+        <is>
+          <t>Dont Worry Ill Make</t>
+        </is>
+      </c>
+      <c r="B25" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C25" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="4" t="inlineStr">
+        <is>
+          <t>Goodbye</t>
+        </is>
+      </c>
+      <c r="B26" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C26" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="4" t="inlineStr">
+        <is>
+          <t>Mans Best Friend</t>
+        </is>
+      </c>
+      <c r="B27" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C27" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="4" t="inlineStr">
+        <is>
+          <t>Lavender Haze</t>
+        </is>
+      </c>
+      <c r="B28" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C28" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="4" t="inlineStr">
+        <is>
+          <t>Never Getting Laid</t>
+        </is>
+      </c>
+      <c r="B29" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C29" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="4" t="inlineStr">
+        <is>
+          <t>My Man on Willpower</t>
+        </is>
+      </c>
+      <c r="B30" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C30" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="4" t="inlineStr">
+        <is>
+          <t>Manchild</t>
+        </is>
+      </c>
+      <c r="B31" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C31" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="4" t="inlineStr">
+        <is>
+          <t>Sugar Talking</t>
+        </is>
+      </c>
+      <c r="B32" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C32" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="4" t="inlineStr">
+        <is>
+          <t>My Man on Willpower</t>
+        </is>
+      </c>
+      <c r="B33" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C33" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="4" t="inlineStr">
+        <is>
+          <t>Midnight Rain</t>
+        </is>
+      </c>
+      <c r="B34" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C34" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="4" t="inlineStr">
+        <is>
+          <t>Nobodys Son</t>
+        </is>
+      </c>
+      <c r="B35" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C35" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="4" t="inlineStr">
+        <is>
+          <t>House Tour</t>
+        </is>
+      </c>
+      <c r="B36" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C36" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="4" t="inlineStr">
+        <is>
+          <t>Hanabi  Î±Î·Ð²Ï…</t>
+        </is>
+      </c>
+      <c r="B37" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C37" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="4" t="inlineStr">
+        <is>
+          <t>Saiyajin anbuâ„¢</t>
+        </is>
+      </c>
+      <c r="B38" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C38" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="4" t="inlineStr">
+        <is>
+          <t>Dummy</t>
+        </is>
+      </c>
+      <c r="B39" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C39" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="4" t="inlineStr">
+        <is>
+          <t>Cazador anbu â„¢</t>
+        </is>
+      </c>
+      <c r="B40" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C40" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="4" t="inlineStr">
+        <is>
+          <t>Besos Mojados</t>
+        </is>
+      </c>
+      <c r="B41" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C41" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="4" t="inlineStr">
+        <is>
+          <t>DarkFire</t>
+        </is>
+      </c>
+      <c r="B42" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C42" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="4" t="inlineStr">
+        <is>
+          <t>DarkSunny</t>
+        </is>
+      </c>
+      <c r="B43" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C43" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="4" t="inlineStr">
+        <is>
+          <t>Dairen Uchiha</t>
+        </is>
+      </c>
+      <c r="B44" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C44" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="4" t="inlineStr">
+        <is>
+          <t>LILI ZENIN®</t>
+        </is>
+      </c>
+      <c r="B45" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C45" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="4" t="inlineStr">
+        <is>
+          <t>ryumichel ZENIN ®</t>
+        </is>
+      </c>
+      <c r="B46" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C46" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="4" t="inlineStr">
+        <is>
+          <t>margot ZENIN ®</t>
+        </is>
+      </c>
+      <c r="B47" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C47" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="4" t="inlineStr">
+        <is>
+          <t>linda ZENIN ®</t>
+        </is>
+      </c>
+      <c r="B48" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C48" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="4" t="inlineStr">
+        <is>
+          <t>equin0x</t>
+        </is>
+      </c>
+      <c r="B49" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C49" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="4" t="inlineStr">
+        <is>
+          <t>Jhayco - Mokai</t>
+        </is>
+      </c>
+      <c r="B50" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C50" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="4" t="inlineStr">
+        <is>
+          <t>Jhayco - Joe</t>
+        </is>
+      </c>
+      <c r="B51" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C51" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="4" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="B52" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C52" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="4" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="B53" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C53" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="4" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="B54" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C54" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="4" t="inlineStr">
+        <is>
+          <t>Go Go Juice</t>
+        </is>
+      </c>
+      <c r="B55" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C55" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="4" t="inlineStr">
+        <is>
+          <t>Jhayco - Imaginaste</t>
+        </is>
+      </c>
+      <c r="B56" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C56" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="4" t="inlineStr">
+        <is>
+          <t>PuNch</t>
+        </is>
+      </c>
+      <c r="B57" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C57" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A2:C2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
auto: snapshot 2026-08-23 13:01:01
</commit_message>
<xml_diff>
--- a/clan_3815.xlsx
+++ b/clan_3815.xlsx
@@ -46,6 +46,7 @@
     <sheet name="2026-08-20" sheetId="37" state="visible" r:id="rId37"/>
     <sheet name="2026-08-21" sheetId="38" state="visible" r:id="rId38"/>
     <sheet name="2026-08-22" sheetId="39" state="visible" r:id="rId39"/>
+    <sheet name="2026-08-23" sheetId="40" state="visible" r:id="rId40"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -28347,6 +28348,870 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet40.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C57"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="29" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Clan: Mans Best Friend (3815)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Timestamp: 2026-08-23 13:01:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>Total Reps</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>Daily Reps (+1d)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>Nobodys Son</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>Player</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>Player</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>X y L O T A</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>AbdiHyde ID 13496</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>Create Character III</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C9" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>Create Character IV</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>Create Character V</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C11" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t>Player</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C12" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="4" t="inlineStr">
+        <is>
+          <t>Player</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C13" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="4" t="inlineStr">
+        <is>
+          <t>hunry</t>
+        </is>
+      </c>
+      <c r="B14" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C14" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="4" t="inlineStr">
+        <is>
+          <t>BlacKRin O</t>
+        </is>
+      </c>
+      <c r="B15" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C15" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="4" t="inlineStr">
+        <is>
+          <t>Tears</t>
+        </is>
+      </c>
+      <c r="B16" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C16" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="4" t="inlineStr">
+        <is>
+          <t>Sugar Talking</t>
+        </is>
+      </c>
+      <c r="B17" s="5" t="n">
+        <v>50</v>
+      </c>
+      <c r="C17" s="5" t="inlineStr">
+        <is>
+          <t>+50</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="4" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B18" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C18" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="4" t="inlineStr">
+        <is>
+          <t>Anti-Hero</t>
+        </is>
+      </c>
+      <c r="B19" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C19" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="4" t="inlineStr">
+        <is>
+          <t>Vigilante Shit</t>
+        </is>
+      </c>
+      <c r="B20" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C20" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="4" t="inlineStr">
+        <is>
+          <t>Sweet Nothing</t>
+        </is>
+      </c>
+      <c r="B21" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C21" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="4" t="inlineStr">
+        <is>
+          <t>The Great War</t>
+        </is>
+      </c>
+      <c r="B22" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C22" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">We Almost Broke Up </t>
+        </is>
+      </c>
+      <c r="B23" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C23" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="4" t="inlineStr">
+        <is>
+          <t>When Did You Get Hot</t>
+        </is>
+      </c>
+      <c r="B24" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C24" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="4" t="inlineStr">
+        <is>
+          <t>Dont Worry Ill Make</t>
+        </is>
+      </c>
+      <c r="B25" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C25" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="4" t="inlineStr">
+        <is>
+          <t>Goodbye</t>
+        </is>
+      </c>
+      <c r="B26" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C26" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="4" t="inlineStr">
+        <is>
+          <t>Mans Best Friend</t>
+        </is>
+      </c>
+      <c r="B27" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C27" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="4" t="inlineStr">
+        <is>
+          <t>Lavender Haze</t>
+        </is>
+      </c>
+      <c r="B28" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C28" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="4" t="inlineStr">
+        <is>
+          <t>Never Getting Laid</t>
+        </is>
+      </c>
+      <c r="B29" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C29" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="4" t="inlineStr">
+        <is>
+          <t>My Man on Willpower</t>
+        </is>
+      </c>
+      <c r="B30" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C30" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="4" t="inlineStr">
+        <is>
+          <t>Manchild</t>
+        </is>
+      </c>
+      <c r="B31" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C31" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="4" t="inlineStr">
+        <is>
+          <t>Sugar Talking</t>
+        </is>
+      </c>
+      <c r="B32" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C32" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="4" t="inlineStr">
+        <is>
+          <t>My Man on Willpower</t>
+        </is>
+      </c>
+      <c r="B33" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C33" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="4" t="inlineStr">
+        <is>
+          <t>Midnight Rain</t>
+        </is>
+      </c>
+      <c r="B34" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C34" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="4" t="inlineStr">
+        <is>
+          <t>Nobodys Son</t>
+        </is>
+      </c>
+      <c r="B35" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C35" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="4" t="inlineStr">
+        <is>
+          <t>House Tour</t>
+        </is>
+      </c>
+      <c r="B36" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C36" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="4" t="inlineStr">
+        <is>
+          <t>Hanabi  Î±Î·Ð²Ï…</t>
+        </is>
+      </c>
+      <c r="B37" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C37" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="4" t="inlineStr">
+        <is>
+          <t>Saiyajin anbuâ„¢</t>
+        </is>
+      </c>
+      <c r="B38" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C38" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="4" t="inlineStr">
+        <is>
+          <t>Dummy</t>
+        </is>
+      </c>
+      <c r="B39" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C39" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="4" t="inlineStr">
+        <is>
+          <t>Cazador anbu â„¢</t>
+        </is>
+      </c>
+      <c r="B40" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C40" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="4" t="inlineStr">
+        <is>
+          <t>Besos Mojados</t>
+        </is>
+      </c>
+      <c r="B41" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C41" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="4" t="inlineStr">
+        <is>
+          <t>DarkFire</t>
+        </is>
+      </c>
+      <c r="B42" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C42" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="4" t="inlineStr">
+        <is>
+          <t>DarkSunny</t>
+        </is>
+      </c>
+      <c r="B43" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C43" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="4" t="inlineStr">
+        <is>
+          <t>Dairen Uchiha</t>
+        </is>
+      </c>
+      <c r="B44" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C44" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="4" t="inlineStr">
+        <is>
+          <t>LILI ZENIN®</t>
+        </is>
+      </c>
+      <c r="B45" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C45" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="4" t="inlineStr">
+        <is>
+          <t>ryumichel ZENIN ®</t>
+        </is>
+      </c>
+      <c r="B46" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C46" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="4" t="inlineStr">
+        <is>
+          <t>margot ZENIN ®</t>
+        </is>
+      </c>
+      <c r="B47" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C47" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="4" t="inlineStr">
+        <is>
+          <t>linda ZENIN ®</t>
+        </is>
+      </c>
+      <c r="B48" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C48" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="4" t="inlineStr">
+        <is>
+          <t>equin0x</t>
+        </is>
+      </c>
+      <c r="B49" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C49" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="4" t="inlineStr">
+        <is>
+          <t>Jhayco - Mokai</t>
+        </is>
+      </c>
+      <c r="B50" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C50" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="4" t="inlineStr">
+        <is>
+          <t>Jhayco - Joe</t>
+        </is>
+      </c>
+      <c r="B51" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C51" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="4" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="B52" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C52" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="4" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="B53" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C53" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="4" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="B54" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C54" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="4" t="inlineStr">
+        <is>
+          <t>Go Go Juice</t>
+        </is>
+      </c>
+      <c r="B55" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C55" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="4" t="inlineStr">
+        <is>
+          <t>Jhayco - Imaginaste</t>
+        </is>
+      </c>
+      <c r="B56" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C56" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="4" t="inlineStr">
+        <is>
+          <t>PuNch</t>
+        </is>
+      </c>
+      <c r="B57" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C57" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A2:C2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
auto: snapshot 2026-08-24 13:01:01
</commit_message>
<xml_diff>
--- a/clan_3815.xlsx
+++ b/clan_3815.xlsx
@@ -47,6 +47,7 @@
     <sheet name="2026-08-21" sheetId="38" state="visible" r:id="rId38"/>
     <sheet name="2026-08-22" sheetId="39" state="visible" r:id="rId39"/>
     <sheet name="2026-08-23" sheetId="40" state="visible" r:id="rId40"/>
+    <sheet name="2026-08-24" sheetId="41" state="visible" r:id="rId41"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -29212,6 +29213,870 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet41.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C57"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="29" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Clan: Mans Best Friend (3815)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Timestamp: 2026-08-24 13:01:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>Total Reps</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>Daily Reps (+1d)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>Nobodys Son</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>Player</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>Player</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>X y L O T A</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>AbdiHyde ID 13496</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>Create Character III</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C9" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>Create Character IV</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>Create Character V</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C11" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t>Player</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C12" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="4" t="inlineStr">
+        <is>
+          <t>Player</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C13" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="4" t="inlineStr">
+        <is>
+          <t>hunry</t>
+        </is>
+      </c>
+      <c r="B14" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C14" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="4" t="inlineStr">
+        <is>
+          <t>BlacKRin O</t>
+        </is>
+      </c>
+      <c r="B15" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C15" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="4" t="inlineStr">
+        <is>
+          <t>Tears</t>
+        </is>
+      </c>
+      <c r="B16" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C16" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="4" t="inlineStr">
+        <is>
+          <t>Sugar Talking</t>
+        </is>
+      </c>
+      <c r="B17" s="5" t="n">
+        <v>50</v>
+      </c>
+      <c r="C17" s="5" t="inlineStr">
+        <is>
+          <t>+50</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="4" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B18" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C18" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="4" t="inlineStr">
+        <is>
+          <t>Anti-Hero</t>
+        </is>
+      </c>
+      <c r="B19" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C19" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="4" t="inlineStr">
+        <is>
+          <t>Vigilante Shit</t>
+        </is>
+      </c>
+      <c r="B20" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C20" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="4" t="inlineStr">
+        <is>
+          <t>Sweet Nothing</t>
+        </is>
+      </c>
+      <c r="B21" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C21" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="4" t="inlineStr">
+        <is>
+          <t>The Great War</t>
+        </is>
+      </c>
+      <c r="B22" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C22" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">We Almost Broke Up </t>
+        </is>
+      </c>
+      <c r="B23" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C23" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="4" t="inlineStr">
+        <is>
+          <t>When Did You Get Hot</t>
+        </is>
+      </c>
+      <c r="B24" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C24" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="4" t="inlineStr">
+        <is>
+          <t>Dont Worry Ill Make</t>
+        </is>
+      </c>
+      <c r="B25" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C25" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="4" t="inlineStr">
+        <is>
+          <t>Goodbye</t>
+        </is>
+      </c>
+      <c r="B26" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C26" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="4" t="inlineStr">
+        <is>
+          <t>Mans Best Friend</t>
+        </is>
+      </c>
+      <c r="B27" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C27" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="4" t="inlineStr">
+        <is>
+          <t>Lavender Haze</t>
+        </is>
+      </c>
+      <c r="B28" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C28" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="4" t="inlineStr">
+        <is>
+          <t>Never Getting Laid</t>
+        </is>
+      </c>
+      <c r="B29" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C29" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="4" t="inlineStr">
+        <is>
+          <t>My Man on Willpower</t>
+        </is>
+      </c>
+      <c r="B30" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C30" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="4" t="inlineStr">
+        <is>
+          <t>Manchild</t>
+        </is>
+      </c>
+      <c r="B31" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C31" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="4" t="inlineStr">
+        <is>
+          <t>Sugar Talking</t>
+        </is>
+      </c>
+      <c r="B32" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C32" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="4" t="inlineStr">
+        <is>
+          <t>My Man on Willpower</t>
+        </is>
+      </c>
+      <c r="B33" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C33" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="4" t="inlineStr">
+        <is>
+          <t>Midnight Rain</t>
+        </is>
+      </c>
+      <c r="B34" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C34" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="4" t="inlineStr">
+        <is>
+          <t>Nobodys Son</t>
+        </is>
+      </c>
+      <c r="B35" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C35" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="4" t="inlineStr">
+        <is>
+          <t>House Tour</t>
+        </is>
+      </c>
+      <c r="B36" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C36" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="4" t="inlineStr">
+        <is>
+          <t>Hanabi  Î±Î·Ð²Ï…</t>
+        </is>
+      </c>
+      <c r="B37" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C37" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="4" t="inlineStr">
+        <is>
+          <t>Saiyajin anbuâ„¢</t>
+        </is>
+      </c>
+      <c r="B38" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C38" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="4" t="inlineStr">
+        <is>
+          <t>Dummy</t>
+        </is>
+      </c>
+      <c r="B39" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C39" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="4" t="inlineStr">
+        <is>
+          <t>Cazador anbu â„¢</t>
+        </is>
+      </c>
+      <c r="B40" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C40" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="4" t="inlineStr">
+        <is>
+          <t>Besos Mojados</t>
+        </is>
+      </c>
+      <c r="B41" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C41" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="4" t="inlineStr">
+        <is>
+          <t>DarkFire</t>
+        </is>
+      </c>
+      <c r="B42" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C42" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="4" t="inlineStr">
+        <is>
+          <t>DarkSunny</t>
+        </is>
+      </c>
+      <c r="B43" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C43" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="4" t="inlineStr">
+        <is>
+          <t>Dairen Uchiha</t>
+        </is>
+      </c>
+      <c r="B44" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C44" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="4" t="inlineStr">
+        <is>
+          <t>LILI ZENIN®</t>
+        </is>
+      </c>
+      <c r="B45" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C45" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="4" t="inlineStr">
+        <is>
+          <t>ryumichel ZENIN ®</t>
+        </is>
+      </c>
+      <c r="B46" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C46" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="4" t="inlineStr">
+        <is>
+          <t>margot ZENIN ®</t>
+        </is>
+      </c>
+      <c r="B47" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C47" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="4" t="inlineStr">
+        <is>
+          <t>linda ZENIN ®</t>
+        </is>
+      </c>
+      <c r="B48" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C48" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="4" t="inlineStr">
+        <is>
+          <t>equin0x</t>
+        </is>
+      </c>
+      <c r="B49" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C49" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="4" t="inlineStr">
+        <is>
+          <t>Jhayco - Mokai</t>
+        </is>
+      </c>
+      <c r="B50" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C50" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="4" t="inlineStr">
+        <is>
+          <t>Jhayco - Joe</t>
+        </is>
+      </c>
+      <c r="B51" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C51" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="4" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="B52" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C52" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="4" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="B53" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C53" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="4" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="B54" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C54" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="4" t="inlineStr">
+        <is>
+          <t>Go Go Juice</t>
+        </is>
+      </c>
+      <c r="B55" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C55" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="4" t="inlineStr">
+        <is>
+          <t>Jhayco - Imaginaste</t>
+        </is>
+      </c>
+      <c r="B56" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C56" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="4" t="inlineStr">
+        <is>
+          <t>PuNch</t>
+        </is>
+      </c>
+      <c r="B57" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C57" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A2:C2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
auto: snapshot 2026-08-25 13:01:01
</commit_message>
<xml_diff>
--- a/clan_3815.xlsx
+++ b/clan_3815.xlsx
@@ -48,6 +48,7 @@
     <sheet name="2026-08-22" sheetId="39" state="visible" r:id="rId39"/>
     <sheet name="2026-08-23" sheetId="40" state="visible" r:id="rId40"/>
     <sheet name="2026-08-24" sheetId="41" state="visible" r:id="rId41"/>
+    <sheet name="2026-08-25" sheetId="42" state="visible" r:id="rId42"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -30077,6 +30078,870 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet42.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C57"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="29" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Clan: Mans Best Friend (3815)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Timestamp: 2026-08-25 13:01:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>Total Reps</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>Daily Reps (+1d)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>Nobodys Son</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>Player</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>Player</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>X y L O T A</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>AbdiHyde ID 13496</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>Create Character III</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C9" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>Create Character IV</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>Create Character V</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C11" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t>Player</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C12" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="4" t="inlineStr">
+        <is>
+          <t>Player</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C13" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="4" t="inlineStr">
+        <is>
+          <t>hunry</t>
+        </is>
+      </c>
+      <c r="B14" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C14" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="4" t="inlineStr">
+        <is>
+          <t>BlacKRin O</t>
+        </is>
+      </c>
+      <c r="B15" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C15" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="4" t="inlineStr">
+        <is>
+          <t>Tears</t>
+        </is>
+      </c>
+      <c r="B16" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C16" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="4" t="inlineStr">
+        <is>
+          <t>Sugar Talking</t>
+        </is>
+      </c>
+      <c r="B17" s="5" t="n">
+        <v>50</v>
+      </c>
+      <c r="C17" s="5" t="inlineStr">
+        <is>
+          <t>+50</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="4" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B18" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C18" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="4" t="inlineStr">
+        <is>
+          <t>Anti-Hero</t>
+        </is>
+      </c>
+      <c r="B19" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C19" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="4" t="inlineStr">
+        <is>
+          <t>Vigilante Shit</t>
+        </is>
+      </c>
+      <c r="B20" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C20" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="4" t="inlineStr">
+        <is>
+          <t>Sweet Nothing</t>
+        </is>
+      </c>
+      <c r="B21" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C21" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="4" t="inlineStr">
+        <is>
+          <t>The Great War</t>
+        </is>
+      </c>
+      <c r="B22" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C22" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">We Almost Broke Up </t>
+        </is>
+      </c>
+      <c r="B23" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C23" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="4" t="inlineStr">
+        <is>
+          <t>When Did You Get Hot</t>
+        </is>
+      </c>
+      <c r="B24" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C24" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="4" t="inlineStr">
+        <is>
+          <t>Dont Worry Ill Make</t>
+        </is>
+      </c>
+      <c r="B25" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C25" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="4" t="inlineStr">
+        <is>
+          <t>Goodbye</t>
+        </is>
+      </c>
+      <c r="B26" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C26" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="4" t="inlineStr">
+        <is>
+          <t>Mans Best Friend</t>
+        </is>
+      </c>
+      <c r="B27" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C27" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="4" t="inlineStr">
+        <is>
+          <t>Lavender Haze</t>
+        </is>
+      </c>
+      <c r="B28" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C28" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="4" t="inlineStr">
+        <is>
+          <t>Never Getting Laid</t>
+        </is>
+      </c>
+      <c r="B29" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C29" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="4" t="inlineStr">
+        <is>
+          <t>My Man on Willpower</t>
+        </is>
+      </c>
+      <c r="B30" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C30" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="4" t="inlineStr">
+        <is>
+          <t>Manchild</t>
+        </is>
+      </c>
+      <c r="B31" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C31" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="4" t="inlineStr">
+        <is>
+          <t>Sugar Talking</t>
+        </is>
+      </c>
+      <c r="B32" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C32" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="4" t="inlineStr">
+        <is>
+          <t>My Man on Willpower</t>
+        </is>
+      </c>
+      <c r="B33" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C33" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="4" t="inlineStr">
+        <is>
+          <t>Midnight Rain</t>
+        </is>
+      </c>
+      <c r="B34" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C34" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="4" t="inlineStr">
+        <is>
+          <t>Nobodys Son</t>
+        </is>
+      </c>
+      <c r="B35" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C35" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="4" t="inlineStr">
+        <is>
+          <t>House Tour</t>
+        </is>
+      </c>
+      <c r="B36" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C36" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="4" t="inlineStr">
+        <is>
+          <t>Hanabi  Î±Î·Ð²Ï…</t>
+        </is>
+      </c>
+      <c r="B37" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C37" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="4" t="inlineStr">
+        <is>
+          <t>Saiyajin anbuâ„¢</t>
+        </is>
+      </c>
+      <c r="B38" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C38" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="4" t="inlineStr">
+        <is>
+          <t>Dummy</t>
+        </is>
+      </c>
+      <c r="B39" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C39" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="4" t="inlineStr">
+        <is>
+          <t>Cazador anbu â„¢</t>
+        </is>
+      </c>
+      <c r="B40" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C40" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="4" t="inlineStr">
+        <is>
+          <t>Besos Mojados</t>
+        </is>
+      </c>
+      <c r="B41" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C41" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="4" t="inlineStr">
+        <is>
+          <t>DarkFire</t>
+        </is>
+      </c>
+      <c r="B42" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C42" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="4" t="inlineStr">
+        <is>
+          <t>DarkSunny</t>
+        </is>
+      </c>
+      <c r="B43" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C43" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="4" t="inlineStr">
+        <is>
+          <t>Dairen Uchiha</t>
+        </is>
+      </c>
+      <c r="B44" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C44" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="4" t="inlineStr">
+        <is>
+          <t>LILI ZENIN®</t>
+        </is>
+      </c>
+      <c r="B45" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C45" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="4" t="inlineStr">
+        <is>
+          <t>ryumichel ZENIN ®</t>
+        </is>
+      </c>
+      <c r="B46" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C46" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="4" t="inlineStr">
+        <is>
+          <t>margot ZENIN ®</t>
+        </is>
+      </c>
+      <c r="B47" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C47" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="4" t="inlineStr">
+        <is>
+          <t>linda ZENIN ®</t>
+        </is>
+      </c>
+      <c r="B48" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C48" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="4" t="inlineStr">
+        <is>
+          <t>equin0x</t>
+        </is>
+      </c>
+      <c r="B49" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C49" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="4" t="inlineStr">
+        <is>
+          <t>Jhayco - Mokai</t>
+        </is>
+      </c>
+      <c r="B50" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C50" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="4" t="inlineStr">
+        <is>
+          <t>Jhayco - Joe</t>
+        </is>
+      </c>
+      <c r="B51" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C51" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="4" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="B52" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C52" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="4" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="B53" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C53" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="4" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="B54" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C54" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="4" t="inlineStr">
+        <is>
+          <t>Go Go Juice</t>
+        </is>
+      </c>
+      <c r="B55" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C55" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="4" t="inlineStr">
+        <is>
+          <t>Jhayco - Imaginaste</t>
+        </is>
+      </c>
+      <c r="B56" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C56" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="4" t="inlineStr">
+        <is>
+          <t>PuNch</t>
+        </is>
+      </c>
+      <c r="B57" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C57" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A2:C2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
auto: snapshot 2026-08-26 13:01:01
</commit_message>
<xml_diff>
--- a/clan_3815.xlsx
+++ b/clan_3815.xlsx
@@ -49,6 +49,7 @@
     <sheet name="2026-08-23" sheetId="40" state="visible" r:id="rId40"/>
     <sheet name="2026-08-24" sheetId="41" state="visible" r:id="rId41"/>
     <sheet name="2026-08-25" sheetId="42" state="visible" r:id="rId42"/>
+    <sheet name="2026-08-26" sheetId="43" state="visible" r:id="rId43"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -30942,6 +30943,870 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet43.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C57"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="29" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Clan: Mans Best Friend (3815)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Timestamp: 2026-08-26 13:01:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>Total Reps</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>Daily Reps (+1d)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>Nobodys Son</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>Player</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>Player</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>X y L O T A</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>AbdiHyde ID 13496</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>Create Character III</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C9" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>Create Character IV</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>Create Character V</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C11" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t>Player</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C12" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="4" t="inlineStr">
+        <is>
+          <t>Player</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C13" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="4" t="inlineStr">
+        <is>
+          <t>hunry</t>
+        </is>
+      </c>
+      <c r="B14" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C14" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="4" t="inlineStr">
+        <is>
+          <t>BlacKRin O</t>
+        </is>
+      </c>
+      <c r="B15" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C15" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="4" t="inlineStr">
+        <is>
+          <t>Tears</t>
+        </is>
+      </c>
+      <c r="B16" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C16" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="4" t="inlineStr">
+        <is>
+          <t>Sugar Talking</t>
+        </is>
+      </c>
+      <c r="B17" s="5" t="n">
+        <v>50</v>
+      </c>
+      <c r="C17" s="5" t="inlineStr">
+        <is>
+          <t>+50</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="4" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B18" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C18" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="4" t="inlineStr">
+        <is>
+          <t>Anti-Hero</t>
+        </is>
+      </c>
+      <c r="B19" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C19" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="4" t="inlineStr">
+        <is>
+          <t>Vigilante Shit</t>
+        </is>
+      </c>
+      <c r="B20" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C20" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="4" t="inlineStr">
+        <is>
+          <t>Sweet Nothing</t>
+        </is>
+      </c>
+      <c r="B21" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C21" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="4" t="inlineStr">
+        <is>
+          <t>The Great War</t>
+        </is>
+      </c>
+      <c r="B22" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C22" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">We Almost Broke Up </t>
+        </is>
+      </c>
+      <c r="B23" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C23" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="4" t="inlineStr">
+        <is>
+          <t>When Did You Get Hot</t>
+        </is>
+      </c>
+      <c r="B24" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C24" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="4" t="inlineStr">
+        <is>
+          <t>Dont Worry Ill Make</t>
+        </is>
+      </c>
+      <c r="B25" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C25" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="4" t="inlineStr">
+        <is>
+          <t>Goodbye</t>
+        </is>
+      </c>
+      <c r="B26" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C26" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="4" t="inlineStr">
+        <is>
+          <t>Mans Best Friend</t>
+        </is>
+      </c>
+      <c r="B27" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C27" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="4" t="inlineStr">
+        <is>
+          <t>Lavender Haze</t>
+        </is>
+      </c>
+      <c r="B28" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C28" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="4" t="inlineStr">
+        <is>
+          <t>Never Getting Laid</t>
+        </is>
+      </c>
+      <c r="B29" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C29" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="4" t="inlineStr">
+        <is>
+          <t>My Man on Willpower</t>
+        </is>
+      </c>
+      <c r="B30" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C30" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="4" t="inlineStr">
+        <is>
+          <t>Manchild</t>
+        </is>
+      </c>
+      <c r="B31" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C31" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="4" t="inlineStr">
+        <is>
+          <t>Sugar Talking</t>
+        </is>
+      </c>
+      <c r="B32" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C32" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="4" t="inlineStr">
+        <is>
+          <t>My Man on Willpower</t>
+        </is>
+      </c>
+      <c r="B33" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C33" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="4" t="inlineStr">
+        <is>
+          <t>Midnight Rain</t>
+        </is>
+      </c>
+      <c r="B34" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C34" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="4" t="inlineStr">
+        <is>
+          <t>Nobodys Son</t>
+        </is>
+      </c>
+      <c r="B35" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C35" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="4" t="inlineStr">
+        <is>
+          <t>House Tour</t>
+        </is>
+      </c>
+      <c r="B36" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C36" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="4" t="inlineStr">
+        <is>
+          <t>Hanabi  Î±Î·Ð²Ï…</t>
+        </is>
+      </c>
+      <c r="B37" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C37" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="4" t="inlineStr">
+        <is>
+          <t>Saiyajin anbuâ„¢</t>
+        </is>
+      </c>
+      <c r="B38" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C38" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="4" t="inlineStr">
+        <is>
+          <t>Dummy</t>
+        </is>
+      </c>
+      <c r="B39" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C39" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="4" t="inlineStr">
+        <is>
+          <t>Cazador anbu â„¢</t>
+        </is>
+      </c>
+      <c r="B40" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C40" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="4" t="inlineStr">
+        <is>
+          <t>Besos Mojados</t>
+        </is>
+      </c>
+      <c r="B41" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C41" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="4" t="inlineStr">
+        <is>
+          <t>DarkFire</t>
+        </is>
+      </c>
+      <c r="B42" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C42" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="4" t="inlineStr">
+        <is>
+          <t>DarkSunny</t>
+        </is>
+      </c>
+      <c r="B43" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C43" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="4" t="inlineStr">
+        <is>
+          <t>Dairen Uchiha</t>
+        </is>
+      </c>
+      <c r="B44" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C44" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="4" t="inlineStr">
+        <is>
+          <t>LILI ZENIN®</t>
+        </is>
+      </c>
+      <c r="B45" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C45" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="4" t="inlineStr">
+        <is>
+          <t>ryumichel ZENIN ®</t>
+        </is>
+      </c>
+      <c r="B46" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C46" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="4" t="inlineStr">
+        <is>
+          <t>margot ZENIN ®</t>
+        </is>
+      </c>
+      <c r="B47" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C47" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="4" t="inlineStr">
+        <is>
+          <t>linda ZENIN ®</t>
+        </is>
+      </c>
+      <c r="B48" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C48" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="4" t="inlineStr">
+        <is>
+          <t>equin0x</t>
+        </is>
+      </c>
+      <c r="B49" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C49" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="4" t="inlineStr">
+        <is>
+          <t>Jhayco - Mokai</t>
+        </is>
+      </c>
+      <c r="B50" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C50" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="4" t="inlineStr">
+        <is>
+          <t>Jhayco - Joe</t>
+        </is>
+      </c>
+      <c r="B51" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C51" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="4" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="B52" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C52" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="4" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="B53" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C53" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="4" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="B54" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C54" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="4" t="inlineStr">
+        <is>
+          <t>Go Go Juice</t>
+        </is>
+      </c>
+      <c r="B55" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C55" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="4" t="inlineStr">
+        <is>
+          <t>Jhayco - Imaginaste</t>
+        </is>
+      </c>
+      <c r="B56" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C56" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="4" t="inlineStr">
+        <is>
+          <t>PuNch</t>
+        </is>
+      </c>
+      <c r="B57" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C57" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A2:C2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
auto: snapshot 2026-08-27 13:01:01
</commit_message>
<xml_diff>
--- a/clan_3815.xlsx
+++ b/clan_3815.xlsx
@@ -50,6 +50,7 @@
     <sheet name="2026-08-24" sheetId="41" state="visible" r:id="rId41"/>
     <sheet name="2026-08-25" sheetId="42" state="visible" r:id="rId42"/>
     <sheet name="2026-08-26" sheetId="43" state="visible" r:id="rId43"/>
+    <sheet name="2026-08-27" sheetId="44" state="visible" r:id="rId44"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -31807,6 +31808,870 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet44.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C57"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="29" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Clan: Mans Best Friend (3815)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Timestamp: 2026-08-27 13:01:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>Total Reps</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>Daily Reps (+1d)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>Nobodys Son</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="n">
+        <v>750</v>
+      </c>
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>+750</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>Player</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>Player</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>X y L O T A</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>AbdiHyde ID 13496</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>Create Character III</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C9" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>Create Character IV</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>Create Character V</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C11" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t>Player</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C12" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="4" t="inlineStr">
+        <is>
+          <t>Player</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C13" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="4" t="inlineStr">
+        <is>
+          <t>hunry</t>
+        </is>
+      </c>
+      <c r="B14" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C14" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="4" t="inlineStr">
+        <is>
+          <t>BlacKRin O</t>
+        </is>
+      </c>
+      <c r="B15" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C15" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="4" t="inlineStr">
+        <is>
+          <t>Tears</t>
+        </is>
+      </c>
+      <c r="B16" s="5" t="n">
+        <v>750</v>
+      </c>
+      <c r="C16" s="5" t="inlineStr">
+        <is>
+          <t>+750</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="4" t="inlineStr">
+        <is>
+          <t>Sugar Talking</t>
+        </is>
+      </c>
+      <c r="B17" s="5" t="n">
+        <v>1050</v>
+      </c>
+      <c r="C17" s="5" t="inlineStr">
+        <is>
+          <t>+1050</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="4" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B18" s="5" t="n">
+        <v>750</v>
+      </c>
+      <c r="C18" s="5" t="inlineStr">
+        <is>
+          <t>+750</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="4" t="inlineStr">
+        <is>
+          <t>Anti-Hero</t>
+        </is>
+      </c>
+      <c r="B19" s="5" t="n">
+        <v>750</v>
+      </c>
+      <c r="C19" s="5" t="inlineStr">
+        <is>
+          <t>+750</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="4" t="inlineStr">
+        <is>
+          <t>Vigilante Shit</t>
+        </is>
+      </c>
+      <c r="B20" s="5" t="n">
+        <v>750</v>
+      </c>
+      <c r="C20" s="5" t="inlineStr">
+        <is>
+          <t>+750</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="4" t="inlineStr">
+        <is>
+          <t>Sweet Nothing</t>
+        </is>
+      </c>
+      <c r="B21" s="5" t="n">
+        <v>750</v>
+      </c>
+      <c r="C21" s="5" t="inlineStr">
+        <is>
+          <t>+750</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="4" t="inlineStr">
+        <is>
+          <t>The Great War</t>
+        </is>
+      </c>
+      <c r="B22" s="5" t="n">
+        <v>750</v>
+      </c>
+      <c r="C22" s="5" t="inlineStr">
+        <is>
+          <t>+750</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">We Almost Broke Up </t>
+        </is>
+      </c>
+      <c r="B23" s="5" t="n">
+        <v>750</v>
+      </c>
+      <c r="C23" s="5" t="inlineStr">
+        <is>
+          <t>+750</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="4" t="inlineStr">
+        <is>
+          <t>When Did You Get Hot</t>
+        </is>
+      </c>
+      <c r="B24" s="5" t="n">
+        <v>750</v>
+      </c>
+      <c r="C24" s="5" t="inlineStr">
+        <is>
+          <t>+750</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="4" t="inlineStr">
+        <is>
+          <t>Dont Worry Ill Make</t>
+        </is>
+      </c>
+      <c r="B25" s="5" t="n">
+        <v>750</v>
+      </c>
+      <c r="C25" s="5" t="inlineStr">
+        <is>
+          <t>+750</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="4" t="inlineStr">
+        <is>
+          <t>Goodbye</t>
+        </is>
+      </c>
+      <c r="B26" s="5" t="n">
+        <v>750</v>
+      </c>
+      <c r="C26" s="5" t="inlineStr">
+        <is>
+          <t>+750</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="4" t="inlineStr">
+        <is>
+          <t>Mans Best Friend</t>
+        </is>
+      </c>
+      <c r="B27" s="5" t="n">
+        <v>750</v>
+      </c>
+      <c r="C27" s="5" t="inlineStr">
+        <is>
+          <t>+750</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="4" t="inlineStr">
+        <is>
+          <t>Lavender Haze</t>
+        </is>
+      </c>
+      <c r="B28" s="5" t="n">
+        <v>750</v>
+      </c>
+      <c r="C28" s="5" t="inlineStr">
+        <is>
+          <t>+750</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="4" t="inlineStr">
+        <is>
+          <t>Never Getting Laid</t>
+        </is>
+      </c>
+      <c r="B29" s="5" t="n">
+        <v>750</v>
+      </c>
+      <c r="C29" s="5" t="inlineStr">
+        <is>
+          <t>+750</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="4" t="inlineStr">
+        <is>
+          <t>My Man on Willpower</t>
+        </is>
+      </c>
+      <c r="B30" s="5" t="n">
+        <v>500</v>
+      </c>
+      <c r="C30" s="5" t="inlineStr">
+        <is>
+          <t>+500</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="4" t="inlineStr">
+        <is>
+          <t>Manchild</t>
+        </is>
+      </c>
+      <c r="B31" s="5" t="n">
+        <v>750</v>
+      </c>
+      <c r="C31" s="5" t="inlineStr">
+        <is>
+          <t>+750</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="4" t="inlineStr">
+        <is>
+          <t>Sugar Talking</t>
+        </is>
+      </c>
+      <c r="B32" s="5" t="n">
+        <v>750</v>
+      </c>
+      <c r="C32" s="5" t="inlineStr">
+        <is>
+          <t>+750</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="4" t="inlineStr">
+        <is>
+          <t>My Man on Willpower</t>
+        </is>
+      </c>
+      <c r="B33" s="5" t="n">
+        <v>1000</v>
+      </c>
+      <c r="C33" s="5" t="inlineStr">
+        <is>
+          <t>+1000</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="4" t="inlineStr">
+        <is>
+          <t>Midnight Rain</t>
+        </is>
+      </c>
+      <c r="B34" s="5" t="n">
+        <v>750</v>
+      </c>
+      <c r="C34" s="5" t="inlineStr">
+        <is>
+          <t>+750</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="4" t="inlineStr">
+        <is>
+          <t>Nobodys Son</t>
+        </is>
+      </c>
+      <c r="B35" s="5" t="n">
+        <v>1000</v>
+      </c>
+      <c r="C35" s="5" t="inlineStr">
+        <is>
+          <t>+1000</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="4" t="inlineStr">
+        <is>
+          <t>House Tour</t>
+        </is>
+      </c>
+      <c r="B36" s="5" t="n">
+        <v>750</v>
+      </c>
+      <c r="C36" s="5" t="inlineStr">
+        <is>
+          <t>+750</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="4" t="inlineStr">
+        <is>
+          <t>Hanabi  Î±Î·Ð²Ï…</t>
+        </is>
+      </c>
+      <c r="B37" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C37" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="4" t="inlineStr">
+        <is>
+          <t>Saiyajin anbuâ„¢</t>
+        </is>
+      </c>
+      <c r="B38" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C38" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="4" t="inlineStr">
+        <is>
+          <t>Dummy</t>
+        </is>
+      </c>
+      <c r="B39" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C39" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="4" t="inlineStr">
+        <is>
+          <t>Cazador anbu â„¢</t>
+        </is>
+      </c>
+      <c r="B40" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C40" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="4" t="inlineStr">
+        <is>
+          <t>Besos Mojados</t>
+        </is>
+      </c>
+      <c r="B41" s="5" t="n">
+        <v>750</v>
+      </c>
+      <c r="C41" s="5" t="inlineStr">
+        <is>
+          <t>+750</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="4" t="inlineStr">
+        <is>
+          <t>DarkFire</t>
+        </is>
+      </c>
+      <c r="B42" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C42" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="4" t="inlineStr">
+        <is>
+          <t>DarkSunny</t>
+        </is>
+      </c>
+      <c r="B43" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C43" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="4" t="inlineStr">
+        <is>
+          <t>Dairen Uchiha</t>
+        </is>
+      </c>
+      <c r="B44" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C44" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="4" t="inlineStr">
+        <is>
+          <t>LILI ZENIN®</t>
+        </is>
+      </c>
+      <c r="B45" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C45" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="4" t="inlineStr">
+        <is>
+          <t>ryumichel ZENIN ®</t>
+        </is>
+      </c>
+      <c r="B46" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C46" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="4" t="inlineStr">
+        <is>
+          <t>margot ZENIN ®</t>
+        </is>
+      </c>
+      <c r="B47" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C47" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="4" t="inlineStr">
+        <is>
+          <t>linda ZENIN ®</t>
+        </is>
+      </c>
+      <c r="B48" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C48" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="4" t="inlineStr">
+        <is>
+          <t>equin0x</t>
+        </is>
+      </c>
+      <c r="B49" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C49" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="4" t="inlineStr">
+        <is>
+          <t>Jhayco - Mokai</t>
+        </is>
+      </c>
+      <c r="B50" s="5" t="n">
+        <v>1000</v>
+      </c>
+      <c r="C50" s="5" t="inlineStr">
+        <is>
+          <t>+1000</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="4" t="inlineStr">
+        <is>
+          <t>Jhayco - Joe</t>
+        </is>
+      </c>
+      <c r="B51" s="5" t="n">
+        <v>1000</v>
+      </c>
+      <c r="C51" s="5" t="inlineStr">
+        <is>
+          <t>+1000</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="4" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="B52" s="5" t="n">
+        <v>1000</v>
+      </c>
+      <c r="C52" s="5" t="inlineStr">
+        <is>
+          <t>+1000</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="4" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="B53" s="5" t="n">
+        <v>750</v>
+      </c>
+      <c r="C53" s="5" t="inlineStr">
+        <is>
+          <t>+750</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="4" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="B54" s="5" t="n">
+        <v>750</v>
+      </c>
+      <c r="C54" s="5" t="inlineStr">
+        <is>
+          <t>+750</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="4" t="inlineStr">
+        <is>
+          <t>Go Go Juice</t>
+        </is>
+      </c>
+      <c r="B55" s="5" t="n">
+        <v>750</v>
+      </c>
+      <c r="C55" s="5" t="inlineStr">
+        <is>
+          <t>+750</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="4" t="inlineStr">
+        <is>
+          <t>Jhayco - Imaginaste</t>
+        </is>
+      </c>
+      <c r="B56" s="5" t="n">
+        <v>750</v>
+      </c>
+      <c r="C56" s="5" t="inlineStr">
+        <is>
+          <t>+750</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="4" t="inlineStr">
+        <is>
+          <t>PuNch</t>
+        </is>
+      </c>
+      <c r="B57" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C57" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A2:C2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
auto: snapshot 2026-08-27 13:31:01
</commit_message>
<xml_diff>
--- a/clan_3815.xlsx
+++ b/clan_3815.xlsx
@@ -31832,7 +31832,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Timestamp: 2026-08-27 13:01:00</t>
+          <t>Timestamp: 2026-08-27 13:31:00</t>
         </is>
       </c>
     </row>
@@ -31860,11 +31860,11 @@
         </is>
       </c>
       <c r="B4" s="5" t="n">
-        <v>750</v>
+        <v>1250</v>
       </c>
       <c r="C4" s="5" t="inlineStr">
         <is>
-          <t>+750</t>
+          <t>+1250</t>
         </is>
       </c>
     </row>
@@ -32040,11 +32040,11 @@
         </is>
       </c>
       <c r="B16" s="5" t="n">
-        <v>750</v>
+        <v>1000</v>
       </c>
       <c r="C16" s="5" t="inlineStr">
         <is>
-          <t>+750</t>
+          <t>+1000</t>
         </is>
       </c>
     </row>
@@ -32070,11 +32070,11 @@
         </is>
       </c>
       <c r="B18" s="5" t="n">
-        <v>750</v>
+        <v>1250</v>
       </c>
       <c r="C18" s="5" t="inlineStr">
         <is>
-          <t>+750</t>
+          <t>+1250</t>
         </is>
       </c>
     </row>
@@ -32085,11 +32085,11 @@
         </is>
       </c>
       <c r="B19" s="5" t="n">
-        <v>750</v>
+        <v>1000</v>
       </c>
       <c r="C19" s="5" t="inlineStr">
         <is>
-          <t>+750</t>
+          <t>+1000</t>
         </is>
       </c>
     </row>
@@ -32100,11 +32100,11 @@
         </is>
       </c>
       <c r="B20" s="5" t="n">
-        <v>750</v>
+        <v>1000</v>
       </c>
       <c r="C20" s="5" t="inlineStr">
         <is>
-          <t>+750</t>
+          <t>+1000</t>
         </is>
       </c>
     </row>
@@ -32115,11 +32115,11 @@
         </is>
       </c>
       <c r="B21" s="5" t="n">
-        <v>750</v>
+        <v>1000</v>
       </c>
       <c r="C21" s="5" t="inlineStr">
         <is>
-          <t>+750</t>
+          <t>+1000</t>
         </is>
       </c>
     </row>
@@ -32130,11 +32130,11 @@
         </is>
       </c>
       <c r="B22" s="5" t="n">
-        <v>750</v>
+        <v>1000</v>
       </c>
       <c r="C22" s="5" t="inlineStr">
         <is>
-          <t>+750</t>
+          <t>+1000</t>
         </is>
       </c>
     </row>
@@ -32145,11 +32145,11 @@
         </is>
       </c>
       <c r="B23" s="5" t="n">
-        <v>750</v>
+        <v>1000</v>
       </c>
       <c r="C23" s="5" t="inlineStr">
         <is>
-          <t>+750</t>
+          <t>+1000</t>
         </is>
       </c>
     </row>
@@ -32160,11 +32160,11 @@
         </is>
       </c>
       <c r="B24" s="5" t="n">
-        <v>750</v>
+        <v>1000</v>
       </c>
       <c r="C24" s="5" t="inlineStr">
         <is>
-          <t>+750</t>
+          <t>+1000</t>
         </is>
       </c>
     </row>
@@ -32175,11 +32175,11 @@
         </is>
       </c>
       <c r="B25" s="5" t="n">
-        <v>750</v>
+        <v>1000</v>
       </c>
       <c r="C25" s="5" t="inlineStr">
         <is>
-          <t>+750</t>
+          <t>+1000</t>
         </is>
       </c>
     </row>
@@ -32190,11 +32190,11 @@
         </is>
       </c>
       <c r="B26" s="5" t="n">
-        <v>750</v>
+        <v>1250</v>
       </c>
       <c r="C26" s="5" t="inlineStr">
         <is>
-          <t>+750</t>
+          <t>+1250</t>
         </is>
       </c>
     </row>
@@ -32205,11 +32205,11 @@
         </is>
       </c>
       <c r="B27" s="5" t="n">
-        <v>750</v>
+        <v>1250</v>
       </c>
       <c r="C27" s="5" t="inlineStr">
         <is>
-          <t>+750</t>
+          <t>+1250</t>
         </is>
       </c>
     </row>
@@ -32220,11 +32220,11 @@
         </is>
       </c>
       <c r="B28" s="5" t="n">
-        <v>750</v>
+        <v>1250</v>
       </c>
       <c r="C28" s="5" t="inlineStr">
         <is>
-          <t>+750</t>
+          <t>+1250</t>
         </is>
       </c>
     </row>
@@ -32235,11 +32235,11 @@
         </is>
       </c>
       <c r="B29" s="5" t="n">
-        <v>750</v>
+        <v>1000</v>
       </c>
       <c r="C29" s="5" t="inlineStr">
         <is>
-          <t>+750</t>
+          <t>+1000</t>
         </is>
       </c>
     </row>
@@ -32250,11 +32250,11 @@
         </is>
       </c>
       <c r="B30" s="5" t="n">
-        <v>500</v>
+        <v>750</v>
       </c>
       <c r="C30" s="5" t="inlineStr">
         <is>
-          <t>+500</t>
+          <t>+750</t>
         </is>
       </c>
     </row>
@@ -32265,11 +32265,11 @@
         </is>
       </c>
       <c r="B31" s="5" t="n">
-        <v>750</v>
+        <v>1000</v>
       </c>
       <c r="C31" s="5" t="inlineStr">
         <is>
-          <t>+750</t>
+          <t>+1000</t>
         </is>
       </c>
     </row>
@@ -32280,11 +32280,11 @@
         </is>
       </c>
       <c r="B32" s="5" t="n">
-        <v>750</v>
+        <v>1000</v>
       </c>
       <c r="C32" s="5" t="inlineStr">
         <is>
-          <t>+750</t>
+          <t>+1000</t>
         </is>
       </c>
     </row>
@@ -32310,11 +32310,11 @@
         </is>
       </c>
       <c r="B34" s="5" t="n">
-        <v>750</v>
+        <v>1250</v>
       </c>
       <c r="C34" s="5" t="inlineStr">
         <is>
-          <t>+750</t>
+          <t>+1250</t>
         </is>
       </c>
     </row>
@@ -32340,11 +32340,11 @@
         </is>
       </c>
       <c r="B36" s="5" t="n">
-        <v>750</v>
+        <v>1000</v>
       </c>
       <c r="C36" s="5" t="inlineStr">
         <is>
-          <t>+750</t>
+          <t>+1000</t>
         </is>
       </c>
     </row>
@@ -32415,11 +32415,11 @@
         </is>
       </c>
       <c r="B41" s="5" t="n">
-        <v>750</v>
+        <v>1201</v>
       </c>
       <c r="C41" s="5" t="inlineStr">
         <is>
-          <t>+750</t>
+          <t>+1201</t>
         </is>
       </c>
     </row>
@@ -32595,11 +32595,11 @@
         </is>
       </c>
       <c r="B53" s="5" t="n">
-        <v>750</v>
+        <v>1250</v>
       </c>
       <c r="C53" s="5" t="inlineStr">
         <is>
-          <t>+750</t>
+          <t>+1250</t>
         </is>
       </c>
     </row>
@@ -32610,11 +32610,11 @@
         </is>
       </c>
       <c r="B54" s="5" t="n">
-        <v>750</v>
+        <v>1250</v>
       </c>
       <c r="C54" s="5" t="inlineStr">
         <is>
-          <t>+750</t>
+          <t>+1250</t>
         </is>
       </c>
     </row>
@@ -32625,11 +32625,11 @@
         </is>
       </c>
       <c r="B55" s="5" t="n">
-        <v>750</v>
+        <v>1000</v>
       </c>
       <c r="C55" s="5" t="inlineStr">
         <is>
-          <t>+750</t>
+          <t>+1000</t>
         </is>
       </c>
     </row>
@@ -32640,11 +32640,11 @@
         </is>
       </c>
       <c r="B56" s="5" t="n">
-        <v>750</v>
+        <v>1250</v>
       </c>
       <c r="C56" s="5" t="inlineStr">
         <is>
-          <t>+750</t>
+          <t>+1250</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: snapshot 2026-08-28 13:01:01
</commit_message>
<xml_diff>
--- a/clan_3815.xlsx
+++ b/clan_3815.xlsx
@@ -51,6 +51,7 @@
     <sheet name="2026-08-25" sheetId="42" state="visible" r:id="rId42"/>
     <sheet name="2026-08-26" sheetId="43" state="visible" r:id="rId43"/>
     <sheet name="2026-08-27" sheetId="44" state="visible" r:id="rId44"/>
+    <sheet name="2026-08-28" sheetId="45" state="visible" r:id="rId45"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -32672,6 +32673,870 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet45.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C57"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="29" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Clan: Mans Best Friend (3815)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Timestamp: 2026-08-28 13:01:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>Total Reps</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>Daily Reps (+1d)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>Nobodys Son</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="n">
+        <v>3250</v>
+      </c>
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>+2250</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>Player</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>Player</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>X y L O T A</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>AbdiHyde ID 13496</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>Create Character III</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C9" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>Create Character IV</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>Create Character V</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C11" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t>Player</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C12" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="4" t="inlineStr">
+        <is>
+          <t>Player</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C13" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="4" t="inlineStr">
+        <is>
+          <t>hunry</t>
+        </is>
+      </c>
+      <c r="B14" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C14" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="4" t="inlineStr">
+        <is>
+          <t>BlacKRin O</t>
+        </is>
+      </c>
+      <c r="B15" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C15" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="4" t="inlineStr">
+        <is>
+          <t>Tears</t>
+        </is>
+      </c>
+      <c r="B16" s="5" t="n">
+        <v>3750</v>
+      </c>
+      <c r="C16" s="5" t="inlineStr">
+        <is>
+          <t>+2750</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="4" t="inlineStr">
+        <is>
+          <t>Sugar Talking</t>
+        </is>
+      </c>
+      <c r="B17" s="5" t="n">
+        <v>4756</v>
+      </c>
+      <c r="C17" s="5" t="inlineStr">
+        <is>
+          <t>+3756</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="4" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B18" s="5" t="n">
+        <v>4250</v>
+      </c>
+      <c r="C18" s="5" t="inlineStr">
+        <is>
+          <t>+3000</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="4" t="inlineStr">
+        <is>
+          <t>Anti-Hero</t>
+        </is>
+      </c>
+      <c r="B19" s="5" t="n">
+        <v>3804</v>
+      </c>
+      <c r="C19" s="5" t="inlineStr">
+        <is>
+          <t>+2804</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="4" t="inlineStr">
+        <is>
+          <t>Vigilante Shit</t>
+        </is>
+      </c>
+      <c r="B20" s="5" t="n">
+        <v>4000</v>
+      </c>
+      <c r="C20" s="5" t="inlineStr">
+        <is>
+          <t>+3000</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="4" t="inlineStr">
+        <is>
+          <t>Sweet Nothing</t>
+        </is>
+      </c>
+      <c r="B21" s="5" t="n">
+        <v>4000</v>
+      </c>
+      <c r="C21" s="5" t="inlineStr">
+        <is>
+          <t>+3000</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="4" t="inlineStr">
+        <is>
+          <t>The Great War</t>
+        </is>
+      </c>
+      <c r="B22" s="5" t="n">
+        <v>4000</v>
+      </c>
+      <c r="C22" s="5" t="inlineStr">
+        <is>
+          <t>+3000</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">We Almost Broke Up </t>
+        </is>
+      </c>
+      <c r="B23" s="5" t="n">
+        <v>3103</v>
+      </c>
+      <c r="C23" s="5" t="inlineStr">
+        <is>
+          <t>+2103</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="4" t="inlineStr">
+        <is>
+          <t>When Did You Get Hot</t>
+        </is>
+      </c>
+      <c r="B24" s="5" t="n">
+        <v>3103</v>
+      </c>
+      <c r="C24" s="5" t="inlineStr">
+        <is>
+          <t>+2103</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="4" t="inlineStr">
+        <is>
+          <t>Dont Worry Ill Make</t>
+        </is>
+      </c>
+      <c r="B25" s="5" t="n">
+        <v>3152</v>
+      </c>
+      <c r="C25" s="5" t="inlineStr">
+        <is>
+          <t>+2152</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="4" t="inlineStr">
+        <is>
+          <t>Goodbye</t>
+        </is>
+      </c>
+      <c r="B26" s="5" t="n">
+        <v>3250</v>
+      </c>
+      <c r="C26" s="5" t="inlineStr">
+        <is>
+          <t>+2000</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="4" t="inlineStr">
+        <is>
+          <t>Mans Best Friend</t>
+        </is>
+      </c>
+      <c r="B27" s="5" t="n">
+        <v>3250</v>
+      </c>
+      <c r="C27" s="5" t="inlineStr">
+        <is>
+          <t>+2000</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="4" t="inlineStr">
+        <is>
+          <t>Lavender Haze</t>
+        </is>
+      </c>
+      <c r="B28" s="5" t="n">
+        <v>3250</v>
+      </c>
+      <c r="C28" s="5" t="inlineStr">
+        <is>
+          <t>+2000</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="4" t="inlineStr">
+        <is>
+          <t>Never Getting Laid</t>
+        </is>
+      </c>
+      <c r="B29" s="5" t="n">
+        <v>3750</v>
+      </c>
+      <c r="C29" s="5" t="inlineStr">
+        <is>
+          <t>+2750</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="4" t="inlineStr">
+        <is>
+          <t>My Man on Willpower</t>
+        </is>
+      </c>
+      <c r="B30" s="5" t="n">
+        <v>3000</v>
+      </c>
+      <c r="C30" s="5" t="inlineStr">
+        <is>
+          <t>+2000</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="4" t="inlineStr">
+        <is>
+          <t>Manchild</t>
+        </is>
+      </c>
+      <c r="B31" s="5" t="n">
+        <v>3750</v>
+      </c>
+      <c r="C31" s="5" t="inlineStr">
+        <is>
+          <t>+2750</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="4" t="inlineStr">
+        <is>
+          <t>Sugar Talking</t>
+        </is>
+      </c>
+      <c r="B32" s="5" t="n">
+        <v>3000</v>
+      </c>
+      <c r="C32" s="5" t="inlineStr">
+        <is>
+          <t>+2000</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="4" t="inlineStr">
+        <is>
+          <t>My Man on Willpower</t>
+        </is>
+      </c>
+      <c r="B33" s="5" t="n">
+        <v>4750</v>
+      </c>
+      <c r="C33" s="5" t="inlineStr">
+        <is>
+          <t>+3750</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="4" t="inlineStr">
+        <is>
+          <t>Midnight Rain</t>
+        </is>
+      </c>
+      <c r="B34" s="5" t="n">
+        <v>3250</v>
+      </c>
+      <c r="C34" s="5" t="inlineStr">
+        <is>
+          <t>+2000</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="4" t="inlineStr">
+        <is>
+          <t>Nobodys Son</t>
+        </is>
+      </c>
+      <c r="B35" s="5" t="n">
+        <v>4750</v>
+      </c>
+      <c r="C35" s="5" t="inlineStr">
+        <is>
+          <t>+3750</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="4" t="inlineStr">
+        <is>
+          <t>House Tour</t>
+        </is>
+      </c>
+      <c r="B36" s="5" t="n">
+        <v>3000</v>
+      </c>
+      <c r="C36" s="5" t="inlineStr">
+        <is>
+          <t>+2000</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="4" t="inlineStr">
+        <is>
+          <t>Hanabi  Î±Î·Ð²Ï…</t>
+        </is>
+      </c>
+      <c r="B37" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C37" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="4" t="inlineStr">
+        <is>
+          <t>Saiyajin anbuâ„¢</t>
+        </is>
+      </c>
+      <c r="B38" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C38" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="4" t="inlineStr">
+        <is>
+          <t>Dummy</t>
+        </is>
+      </c>
+      <c r="B39" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C39" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="4" t="inlineStr">
+        <is>
+          <t>Cazador anbu â„¢</t>
+        </is>
+      </c>
+      <c r="B40" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C40" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="4" t="inlineStr">
+        <is>
+          <t>Besos Mojados</t>
+        </is>
+      </c>
+      <c r="B41" s="5" t="n">
+        <v>2201</v>
+      </c>
+      <c r="C41" s="5" t="inlineStr">
+        <is>
+          <t>+1000</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="4" t="inlineStr">
+        <is>
+          <t>DarkFire</t>
+        </is>
+      </c>
+      <c r="B42" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C42" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="4" t="inlineStr">
+        <is>
+          <t>DarkSunny</t>
+        </is>
+      </c>
+      <c r="B43" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C43" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="4" t="inlineStr">
+        <is>
+          <t>Dairen Uchiha</t>
+        </is>
+      </c>
+      <c r="B44" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C44" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="4" t="inlineStr">
+        <is>
+          <t>LILI ZENIN®</t>
+        </is>
+      </c>
+      <c r="B45" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C45" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="4" t="inlineStr">
+        <is>
+          <t>ryumichel ZENIN ®</t>
+        </is>
+      </c>
+      <c r="B46" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C46" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="4" t="inlineStr">
+        <is>
+          <t>margot ZENIN ®</t>
+        </is>
+      </c>
+      <c r="B47" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C47" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="4" t="inlineStr">
+        <is>
+          <t>linda ZENIN ®</t>
+        </is>
+      </c>
+      <c r="B48" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C48" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="4" t="inlineStr">
+        <is>
+          <t>equin0x</t>
+        </is>
+      </c>
+      <c r="B49" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C49" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="4" t="inlineStr">
+        <is>
+          <t>Jhayco - Mokai</t>
+        </is>
+      </c>
+      <c r="B50" s="5" t="n">
+        <v>5250</v>
+      </c>
+      <c r="C50" s="5" t="inlineStr">
+        <is>
+          <t>+4250</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="4" t="inlineStr">
+        <is>
+          <t>Jhayco - Joe</t>
+        </is>
+      </c>
+      <c r="B51" s="5" t="n">
+        <v>4901</v>
+      </c>
+      <c r="C51" s="5" t="inlineStr">
+        <is>
+          <t>+3901</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="4" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="B52" s="5" t="n">
+        <v>4206</v>
+      </c>
+      <c r="C52" s="5" t="inlineStr">
+        <is>
+          <t>+3206</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="4" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="B53" s="5" t="n">
+        <v>4500</v>
+      </c>
+      <c r="C53" s="5" t="inlineStr">
+        <is>
+          <t>+3250</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="4" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="B54" s="5" t="n">
+        <v>4500</v>
+      </c>
+      <c r="C54" s="5" t="inlineStr">
+        <is>
+          <t>+3250</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="4" t="inlineStr">
+        <is>
+          <t>Go Go Juice</t>
+        </is>
+      </c>
+      <c r="B55" s="5" t="n">
+        <v>3750</v>
+      </c>
+      <c r="C55" s="5" t="inlineStr">
+        <is>
+          <t>+2750</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="4" t="inlineStr">
+        <is>
+          <t>Jhayco - Imaginaste</t>
+        </is>
+      </c>
+      <c r="B56" s="5" t="n">
+        <v>2157</v>
+      </c>
+      <c r="C56" s="5" t="inlineStr">
+        <is>
+          <t>+907</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="4" t="inlineStr">
+        <is>
+          <t>PuNch</t>
+        </is>
+      </c>
+      <c r="B57" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C57" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A2:C2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
auto: snapshot 2026-08-29 13:01:01
</commit_message>
<xml_diff>
--- a/clan_3815.xlsx
+++ b/clan_3815.xlsx
@@ -52,6 +52,7 @@
     <sheet name="2026-08-26" sheetId="43" state="visible" r:id="rId43"/>
     <sheet name="2026-08-27" sheetId="44" state="visible" r:id="rId44"/>
     <sheet name="2026-08-28" sheetId="45" state="visible" r:id="rId45"/>
+    <sheet name="2026-08-29" sheetId="46" state="visible" r:id="rId46"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -33537,6 +33538,885 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet46.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C58"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="29" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Clan: Mans Best Friend (3815)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Timestamp: 2026-08-29 13:01:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>Total Reps</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>Daily Reps (+1d)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>Nobodys Son</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="n">
+        <v>3250</v>
+      </c>
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>-1500</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>Player</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>Player</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>X y L O T A</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>AbdiHyde ID 13496</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>Create Character III</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C9" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>Create Character IV</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>Create Character V</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C11" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t>Player</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C12" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="4" t="inlineStr">
+        <is>
+          <t>Player</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C13" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="4" t="inlineStr">
+        <is>
+          <t>hunry</t>
+        </is>
+      </c>
+      <c r="B14" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C14" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="4" t="inlineStr">
+        <is>
+          <t>BlacKRin O</t>
+        </is>
+      </c>
+      <c r="B15" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C15" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="4" t="inlineStr">
+        <is>
+          <t>Tears</t>
+        </is>
+      </c>
+      <c r="B16" s="5" t="n">
+        <v>3750</v>
+      </c>
+      <c r="C16" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="4" t="inlineStr">
+        <is>
+          <t>NPC | SNOOPY</t>
+        </is>
+      </c>
+      <c r="B17" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C17" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="4" t="inlineStr">
+        <is>
+          <t>Sugar Talking</t>
+        </is>
+      </c>
+      <c r="B18" s="5" t="n">
+        <v>5506</v>
+      </c>
+      <c r="C18" s="5" t="inlineStr">
+        <is>
+          <t>+2506</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="4" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B19" s="5" t="n">
+        <v>4250</v>
+      </c>
+      <c r="C19" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="4" t="inlineStr">
+        <is>
+          <t>Anti-Hero</t>
+        </is>
+      </c>
+      <c r="B20" s="5" t="n">
+        <v>3804</v>
+      </c>
+      <c r="C20" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="4" t="inlineStr">
+        <is>
+          <t>Vigilante Shit</t>
+        </is>
+      </c>
+      <c r="B21" s="5" t="n">
+        <v>4000</v>
+      </c>
+      <c r="C21" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="4" t="inlineStr">
+        <is>
+          <t>Sweet Nothing</t>
+        </is>
+      </c>
+      <c r="B22" s="5" t="n">
+        <v>4000</v>
+      </c>
+      <c r="C22" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="4" t="inlineStr">
+        <is>
+          <t>The Great War</t>
+        </is>
+      </c>
+      <c r="B23" s="5" t="n">
+        <v>4000</v>
+      </c>
+      <c r="C23" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">We Almost Broke Up </t>
+        </is>
+      </c>
+      <c r="B24" s="5" t="n">
+        <v>4603</v>
+      </c>
+      <c r="C24" s="5" t="inlineStr">
+        <is>
+          <t>+1500</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="4" t="inlineStr">
+        <is>
+          <t>When Did You Get Hot</t>
+        </is>
+      </c>
+      <c r="B25" s="5" t="n">
+        <v>4603</v>
+      </c>
+      <c r="C25" s="5" t="inlineStr">
+        <is>
+          <t>+1500</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="4" t="inlineStr">
+        <is>
+          <t>Dont Worry Ill Make</t>
+        </is>
+      </c>
+      <c r="B26" s="5" t="n">
+        <v>4603</v>
+      </c>
+      <c r="C26" s="5" t="inlineStr">
+        <is>
+          <t>+1451</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="4" t="inlineStr">
+        <is>
+          <t>Goodbye</t>
+        </is>
+      </c>
+      <c r="B27" s="5" t="n">
+        <v>3250</v>
+      </c>
+      <c r="C27" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="4" t="inlineStr">
+        <is>
+          <t>Mans Best Friend</t>
+        </is>
+      </c>
+      <c r="B28" s="5" t="n">
+        <v>3250</v>
+      </c>
+      <c r="C28" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="4" t="inlineStr">
+        <is>
+          <t>Lavender Haze</t>
+        </is>
+      </c>
+      <c r="B29" s="5" t="n">
+        <v>3250</v>
+      </c>
+      <c r="C29" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="4" t="inlineStr">
+        <is>
+          <t>Never Getting Laid</t>
+        </is>
+      </c>
+      <c r="B30" s="5" t="n">
+        <v>3750</v>
+      </c>
+      <c r="C30" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="4" t="inlineStr">
+        <is>
+          <t>My Man on Willpower</t>
+        </is>
+      </c>
+      <c r="B31" s="5" t="n">
+        <v>3000</v>
+      </c>
+      <c r="C31" s="5" t="inlineStr">
+        <is>
+          <t>-1750</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="4" t="inlineStr">
+        <is>
+          <t>Manchild</t>
+        </is>
+      </c>
+      <c r="B32" s="5" t="n">
+        <v>3750</v>
+      </c>
+      <c r="C32" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="4" t="inlineStr">
+        <is>
+          <t>Sugar Talking</t>
+        </is>
+      </c>
+      <c r="B33" s="5" t="n">
+        <v>4250</v>
+      </c>
+      <c r="C33" s="5" t="inlineStr">
+        <is>
+          <t>+1250</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="4" t="inlineStr">
+        <is>
+          <t>My Man on Willpower</t>
+        </is>
+      </c>
+      <c r="B34" s="5" t="n">
+        <v>5750</v>
+      </c>
+      <c r="C34" s="5" t="inlineStr">
+        <is>
+          <t>+1000</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="4" t="inlineStr">
+        <is>
+          <t>Midnight Rain</t>
+        </is>
+      </c>
+      <c r="B35" s="5" t="n">
+        <v>3250</v>
+      </c>
+      <c r="C35" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="4" t="inlineStr">
+        <is>
+          <t>Nobodys Son</t>
+        </is>
+      </c>
+      <c r="B36" s="5" t="n">
+        <v>5750</v>
+      </c>
+      <c r="C36" s="5" t="inlineStr">
+        <is>
+          <t>+1000</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="4" t="inlineStr">
+        <is>
+          <t>House Tour</t>
+        </is>
+      </c>
+      <c r="B37" s="5" t="n">
+        <v>4250</v>
+      </c>
+      <c r="C37" s="5" t="inlineStr">
+        <is>
+          <t>+1250</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="4" t="inlineStr">
+        <is>
+          <t>Hanabi  Î±Î·Ð²Ï…</t>
+        </is>
+      </c>
+      <c r="B38" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C38" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="4" t="inlineStr">
+        <is>
+          <t>Saiyajin anbuâ„¢</t>
+        </is>
+      </c>
+      <c r="B39" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C39" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="4" t="inlineStr">
+        <is>
+          <t>Dummy</t>
+        </is>
+      </c>
+      <c r="B40" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C40" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="4" t="inlineStr">
+        <is>
+          <t>Cazador anbu â„¢</t>
+        </is>
+      </c>
+      <c r="B41" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C41" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="4" t="inlineStr">
+        <is>
+          <t>Besos Mojados</t>
+        </is>
+      </c>
+      <c r="B42" s="5" t="n">
+        <v>2201</v>
+      </c>
+      <c r="C42" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="4" t="inlineStr">
+        <is>
+          <t>DarkFire</t>
+        </is>
+      </c>
+      <c r="B43" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C43" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="4" t="inlineStr">
+        <is>
+          <t>DarkSunny</t>
+        </is>
+      </c>
+      <c r="B44" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C44" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="4" t="inlineStr">
+        <is>
+          <t>Dairen Uchiha</t>
+        </is>
+      </c>
+      <c r="B45" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C45" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="4" t="inlineStr">
+        <is>
+          <t>LILI ZENIN®</t>
+        </is>
+      </c>
+      <c r="B46" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C46" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="4" t="inlineStr">
+        <is>
+          <t>ryumichel ZENIN ®</t>
+        </is>
+      </c>
+      <c r="B47" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C47" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="4" t="inlineStr">
+        <is>
+          <t>margot ZENIN ®</t>
+        </is>
+      </c>
+      <c r="B48" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C48" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="4" t="inlineStr">
+        <is>
+          <t>linda ZENIN ®</t>
+        </is>
+      </c>
+      <c r="B49" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C49" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="4" t="inlineStr">
+        <is>
+          <t>equin0x</t>
+        </is>
+      </c>
+      <c r="B50" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C50" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="4" t="inlineStr">
+        <is>
+          <t>Jhayco - Mokai</t>
+        </is>
+      </c>
+      <c r="B51" s="5" t="n">
+        <v>8500</v>
+      </c>
+      <c r="C51" s="5" t="inlineStr">
+        <is>
+          <t>+3250</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="4" t="inlineStr">
+        <is>
+          <t>Jhayco - Joe</t>
+        </is>
+      </c>
+      <c r="B52" s="5" t="n">
+        <v>8651</v>
+      </c>
+      <c r="C52" s="5" t="inlineStr">
+        <is>
+          <t>+3750</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="4" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="B53" s="5" t="n">
+        <v>7461</v>
+      </c>
+      <c r="C53" s="5" t="inlineStr">
+        <is>
+          <t>+3255</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="4" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="B54" s="5" t="n">
+        <v>7853</v>
+      </c>
+      <c r="C54" s="5" t="inlineStr">
+        <is>
+          <t>+3353</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="4" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="B55" s="5" t="n">
+        <v>8000</v>
+      </c>
+      <c r="C55" s="5" t="inlineStr">
+        <is>
+          <t>+3500</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="4" t="inlineStr">
+        <is>
+          <t>Go Go Juice</t>
+        </is>
+      </c>
+      <c r="B56" s="5" t="n">
+        <v>3750</v>
+      </c>
+      <c r="C56" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="4" t="inlineStr">
+        <is>
+          <t>Jhayco - Imaginaste</t>
+        </is>
+      </c>
+      <c r="B57" s="5" t="n">
+        <v>2157</v>
+      </c>
+      <c r="C57" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="4" t="inlineStr">
+        <is>
+          <t>PuNch</t>
+        </is>
+      </c>
+      <c r="B58" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C58" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A2:C2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
auto: snapshot 2026-08-30 13:01:00
</commit_message>
<xml_diff>
--- a/clan_3815.xlsx
+++ b/clan_3815.xlsx
@@ -53,6 +53,7 @@
     <sheet name="2026-08-27" sheetId="44" state="visible" r:id="rId44"/>
     <sheet name="2026-08-28" sheetId="45" state="visible" r:id="rId45"/>
     <sheet name="2026-08-29" sheetId="46" state="visible" r:id="rId46"/>
+    <sheet name="2026-08-30" sheetId="47" state="visible" r:id="rId47"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -34417,6 +34418,885 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet47.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C58"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="29" customWidth="1" min="1" max="1"/>
+    <col width="9" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Clan: Mans Best Friend (3815)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Timestamp: 2026-08-30 13:01:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>Total Reps</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>Daily Reps (+1d)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>Nobodys Son</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="n">
+        <v>57880</v>
+      </c>
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>+52130</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>Player</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>Player</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>X y L O T A</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>AbdiHyde ID 13496</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>Create Character III</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C9" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>Create Character IV</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>Create Character V</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C11" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t>Player</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C12" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="4" t="inlineStr">
+        <is>
+          <t>Player</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C13" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="4" t="inlineStr">
+        <is>
+          <t>hunry</t>
+        </is>
+      </c>
+      <c r="B14" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C14" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="4" t="inlineStr">
+        <is>
+          <t>BlacKRin O</t>
+        </is>
+      </c>
+      <c r="B15" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C15" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="4" t="inlineStr">
+        <is>
+          <t>Tears</t>
+        </is>
+      </c>
+      <c r="B16" s="5" t="n">
+        <v>32550</v>
+      </c>
+      <c r="C16" s="5" t="inlineStr">
+        <is>
+          <t>+28800</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="4" t="inlineStr">
+        <is>
+          <t>NPC | SNOOPY</t>
+        </is>
+      </c>
+      <c r="B17" s="5" t="n">
+        <v>86158</v>
+      </c>
+      <c r="C17" s="5" t="inlineStr">
+        <is>
+          <t>+86158</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="4" t="inlineStr">
+        <is>
+          <t>Sugar Talking</t>
+        </is>
+      </c>
+      <c r="B18" s="5" t="n">
+        <v>43311</v>
+      </c>
+      <c r="C18" s="5" t="inlineStr">
+        <is>
+          <t>+39061</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="4" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B19" s="5" t="n">
+        <v>21095</v>
+      </c>
+      <c r="C19" s="5" t="inlineStr">
+        <is>
+          <t>+16845</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="4" t="inlineStr">
+        <is>
+          <t>Anti-Hero</t>
+        </is>
+      </c>
+      <c r="B20" s="5" t="n">
+        <v>20061</v>
+      </c>
+      <c r="C20" s="5" t="inlineStr">
+        <is>
+          <t>+16257</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="4" t="inlineStr">
+        <is>
+          <t>Vigilante Shit</t>
+        </is>
+      </c>
+      <c r="B21" s="5" t="n">
+        <v>46794</v>
+      </c>
+      <c r="C21" s="5" t="inlineStr">
+        <is>
+          <t>+42794</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="4" t="inlineStr">
+        <is>
+          <t>Sweet Nothing</t>
+        </is>
+      </c>
+      <c r="B22" s="5" t="n">
+        <v>8590</v>
+      </c>
+      <c r="C22" s="5" t="inlineStr">
+        <is>
+          <t>+4590</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="4" t="inlineStr">
+        <is>
+          <t>The Great War</t>
+        </is>
+      </c>
+      <c r="B23" s="5" t="n">
+        <v>8590</v>
+      </c>
+      <c r="C23" s="5" t="inlineStr">
+        <is>
+          <t>+4590</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">We Almost Broke Up </t>
+        </is>
+      </c>
+      <c r="B24" s="5" t="n">
+        <v>8983</v>
+      </c>
+      <c r="C24" s="5" t="inlineStr">
+        <is>
+          <t>+4380</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="4" t="inlineStr">
+        <is>
+          <t>When Did You Get Hot</t>
+        </is>
+      </c>
+      <c r="B25" s="5" t="n">
+        <v>135825</v>
+      </c>
+      <c r="C25" s="5" t="inlineStr">
+        <is>
+          <t>+131222</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="4" t="inlineStr">
+        <is>
+          <t>Dont Worry Ill Make</t>
+        </is>
+      </c>
+      <c r="B26" s="5" t="n">
+        <v>8943</v>
+      </c>
+      <c r="C26" s="5" t="inlineStr">
+        <is>
+          <t>+4340</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="4" t="inlineStr">
+        <is>
+          <t>Goodbye</t>
+        </is>
+      </c>
+      <c r="B27" s="5" t="n">
+        <v>22895</v>
+      </c>
+      <c r="C27" s="5" t="inlineStr">
+        <is>
+          <t>+19645</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="4" t="inlineStr">
+        <is>
+          <t>Mans Best Friend</t>
+        </is>
+      </c>
+      <c r="B28" s="5" t="n">
+        <v>19870</v>
+      </c>
+      <c r="C28" s="5" t="inlineStr">
+        <is>
+          <t>+16620</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="4" t="inlineStr">
+        <is>
+          <t>Lavender Haze</t>
+        </is>
+      </c>
+      <c r="B29" s="5" t="n">
+        <v>11620</v>
+      </c>
+      <c r="C29" s="5" t="inlineStr">
+        <is>
+          <t>+8370</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="4" t="inlineStr">
+        <is>
+          <t>Never Getting Laid</t>
+        </is>
+      </c>
+      <c r="B30" s="5" t="n">
+        <v>9099</v>
+      </c>
+      <c r="C30" s="5" t="inlineStr">
+        <is>
+          <t>+5349</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="4" t="inlineStr">
+        <is>
+          <t>My Man on Willpower</t>
+        </is>
+      </c>
+      <c r="B31" s="5" t="n">
+        <v>8290</v>
+      </c>
+      <c r="C31" s="5" t="inlineStr">
+        <is>
+          <t>+2540</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="4" t="inlineStr">
+        <is>
+          <t>Manchild</t>
+        </is>
+      </c>
+      <c r="B32" s="5" t="n">
+        <v>9540</v>
+      </c>
+      <c r="C32" s="5" t="inlineStr">
+        <is>
+          <t>+5790</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="4" t="inlineStr">
+        <is>
+          <t>Sugar Talking</t>
+        </is>
+      </c>
+      <c r="B33" s="5" t="n">
+        <v>8633</v>
+      </c>
+      <c r="C33" s="5" t="inlineStr">
+        <is>
+          <t>+4383</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="4" t="inlineStr">
+        <is>
+          <t>My Man on Willpower</t>
+        </is>
+      </c>
+      <c r="B34" s="5" t="n">
+        <v>10675</v>
+      </c>
+      <c r="C34" s="5" t="inlineStr">
+        <is>
+          <t>+4925</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="4" t="inlineStr">
+        <is>
+          <t>Midnight Rain</t>
+        </is>
+      </c>
+      <c r="B35" s="5" t="n">
+        <v>11382</v>
+      </c>
+      <c r="C35" s="5" t="inlineStr">
+        <is>
+          <t>+8132</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="4" t="inlineStr">
+        <is>
+          <t>Nobodys Son</t>
+        </is>
+      </c>
+      <c r="B36" s="5" t="n">
+        <v>11090</v>
+      </c>
+      <c r="C36" s="5" t="inlineStr">
+        <is>
+          <t>+5340</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="4" t="inlineStr">
+        <is>
+          <t>House Tour</t>
+        </is>
+      </c>
+      <c r="B37" s="5" t="n">
+        <v>8514</v>
+      </c>
+      <c r="C37" s="5" t="inlineStr">
+        <is>
+          <t>+4264</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="4" t="inlineStr">
+        <is>
+          <t>Hanabi  Î±Î·Ð²Ï…</t>
+        </is>
+      </c>
+      <c r="B38" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C38" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="4" t="inlineStr">
+        <is>
+          <t>Saiyajin anbuâ„¢</t>
+        </is>
+      </c>
+      <c r="B39" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C39" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="4" t="inlineStr">
+        <is>
+          <t>Dummy</t>
+        </is>
+      </c>
+      <c r="B40" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C40" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="4" t="inlineStr">
+        <is>
+          <t>Cazador anbu â„¢</t>
+        </is>
+      </c>
+      <c r="B41" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C41" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="4" t="inlineStr">
+        <is>
+          <t>Besos Mojados</t>
+        </is>
+      </c>
+      <c r="B42" s="5" t="n">
+        <v>5171</v>
+      </c>
+      <c r="C42" s="5" t="inlineStr">
+        <is>
+          <t>+2970</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="4" t="inlineStr">
+        <is>
+          <t>DarkFire</t>
+        </is>
+      </c>
+      <c r="B43" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C43" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="4" t="inlineStr">
+        <is>
+          <t>DarkSunny</t>
+        </is>
+      </c>
+      <c r="B44" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C44" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="4" t="inlineStr">
+        <is>
+          <t>Dairen Uchiha</t>
+        </is>
+      </c>
+      <c r="B45" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C45" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="4" t="inlineStr">
+        <is>
+          <t>LILI ZENIN®</t>
+        </is>
+      </c>
+      <c r="B46" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C46" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="4" t="inlineStr">
+        <is>
+          <t>ryumichel ZENIN ®</t>
+        </is>
+      </c>
+      <c r="B47" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C47" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="4" t="inlineStr">
+        <is>
+          <t>margot ZENIN ®</t>
+        </is>
+      </c>
+      <c r="B48" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C48" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="4" t="inlineStr">
+        <is>
+          <t>linda ZENIN ®</t>
+        </is>
+      </c>
+      <c r="B49" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C49" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="4" t="inlineStr">
+        <is>
+          <t>equin0x</t>
+        </is>
+      </c>
+      <c r="B50" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C50" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="4" t="inlineStr">
+        <is>
+          <t>Jhayco - Mokai</t>
+        </is>
+      </c>
+      <c r="B51" s="5" t="n">
+        <v>30090</v>
+      </c>
+      <c r="C51" s="5" t="inlineStr">
+        <is>
+          <t>+21590</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="4" t="inlineStr">
+        <is>
+          <t>Jhayco - Joe</t>
+        </is>
+      </c>
+      <c r="B52" s="5" t="n">
+        <v>27217</v>
+      </c>
+      <c r="C52" s="5" t="inlineStr">
+        <is>
+          <t>+18566</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="4" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="B53" s="5" t="n">
+        <v>22946</v>
+      </c>
+      <c r="C53" s="5" t="inlineStr">
+        <is>
+          <t>+15485</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="4" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="B54" s="5" t="n">
+        <v>15193</v>
+      </c>
+      <c r="C54" s="5" t="inlineStr">
+        <is>
+          <t>+7340</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="4" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="B55" s="5" t="n">
+        <v>15130</v>
+      </c>
+      <c r="C55" s="5" t="inlineStr">
+        <is>
+          <t>+7130</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="4" t="inlineStr">
+        <is>
+          <t>Go Go Juice</t>
+        </is>
+      </c>
+      <c r="B56" s="5" t="n">
+        <v>9040</v>
+      </c>
+      <c r="C56" s="5" t="inlineStr">
+        <is>
+          <t>+5290</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="4" t="inlineStr">
+        <is>
+          <t>Jhayco - Imaginaste</t>
+        </is>
+      </c>
+      <c r="B57" s="5" t="n">
+        <v>5127</v>
+      </c>
+      <c r="C57" s="5" t="inlineStr">
+        <is>
+          <t>+2970</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="4" t="inlineStr">
+        <is>
+          <t>PuNch</t>
+        </is>
+      </c>
+      <c r="B58" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C58" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A2:C2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
auto: snapshot 2026-08-31 13:01:01
</commit_message>
<xml_diff>
--- a/clan_3815.xlsx
+++ b/clan_3815.xlsx
@@ -54,6 +54,7 @@
     <sheet name="2026-08-28" sheetId="45" state="visible" r:id="rId45"/>
     <sheet name="2026-08-29" sheetId="46" state="visible" r:id="rId46"/>
     <sheet name="2026-08-30" sheetId="47" state="visible" r:id="rId47"/>
+    <sheet name="2026-08-31" sheetId="48" state="visible" r:id="rId48"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -35297,6 +35298,885 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet48.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C58"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="29" customWidth="1" min="1" max="1"/>
+    <col width="9" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Clan: Mans Best Friend (3815)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Timestamp: 2026-08-31 13:01:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>Total Reps</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>Daily Reps (+1d)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>Nobodys Son</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="n">
+        <v>57880</v>
+      </c>
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>+46790</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>Player</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>Player</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>X y L O T A</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>AbdiHyde ID 13496</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>Create Character III</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C9" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>Create Character IV</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>Create Character V</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C11" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t>Player</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C12" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="4" t="inlineStr">
+        <is>
+          <t>Player</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C13" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="4" t="inlineStr">
+        <is>
+          <t>hunry</t>
+        </is>
+      </c>
+      <c r="B14" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C14" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="4" t="inlineStr">
+        <is>
+          <t>BlacKRin O</t>
+        </is>
+      </c>
+      <c r="B15" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C15" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="4" t="inlineStr">
+        <is>
+          <t>Tears</t>
+        </is>
+      </c>
+      <c r="B16" s="5" t="n">
+        <v>32550</v>
+      </c>
+      <c r="C16" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="4" t="inlineStr">
+        <is>
+          <t>NPC | SNOOPY</t>
+        </is>
+      </c>
+      <c r="B17" s="5" t="n">
+        <v>86158</v>
+      </c>
+      <c r="C17" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="4" t="inlineStr">
+        <is>
+          <t>Sugar Talking</t>
+        </is>
+      </c>
+      <c r="B18" s="5" t="n">
+        <v>43311</v>
+      </c>
+      <c r="C18" s="5" t="inlineStr">
+        <is>
+          <t>+34678</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="4" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B19" s="5" t="n">
+        <v>21095</v>
+      </c>
+      <c r="C19" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="4" t="inlineStr">
+        <is>
+          <t>Anti-Hero</t>
+        </is>
+      </c>
+      <c r="B20" s="5" t="n">
+        <v>20061</v>
+      </c>
+      <c r="C20" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="4" t="inlineStr">
+        <is>
+          <t>Vigilante Shit</t>
+        </is>
+      </c>
+      <c r="B21" s="5" t="n">
+        <v>46794</v>
+      </c>
+      <c r="C21" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="4" t="inlineStr">
+        <is>
+          <t>Sweet Nothing</t>
+        </is>
+      </c>
+      <c r="B22" s="5" t="n">
+        <v>8590</v>
+      </c>
+      <c r="C22" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="4" t="inlineStr">
+        <is>
+          <t>The Great War</t>
+        </is>
+      </c>
+      <c r="B23" s="5" t="n">
+        <v>8590</v>
+      </c>
+      <c r="C23" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">We Almost Broke Up </t>
+        </is>
+      </c>
+      <c r="B24" s="5" t="n">
+        <v>8983</v>
+      </c>
+      <c r="C24" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="4" t="inlineStr">
+        <is>
+          <t>When Did You Get Hot</t>
+        </is>
+      </c>
+      <c r="B25" s="5" t="n">
+        <v>135825</v>
+      </c>
+      <c r="C25" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="4" t="inlineStr">
+        <is>
+          <t>Dont Worry Ill Make</t>
+        </is>
+      </c>
+      <c r="B26" s="5" t="n">
+        <v>8943</v>
+      </c>
+      <c r="C26" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="4" t="inlineStr">
+        <is>
+          <t>Goodbye</t>
+        </is>
+      </c>
+      <c r="B27" s="5" t="n">
+        <v>22895</v>
+      </c>
+      <c r="C27" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="4" t="inlineStr">
+        <is>
+          <t>Mans Best Friend</t>
+        </is>
+      </c>
+      <c r="B28" s="5" t="n">
+        <v>19870</v>
+      </c>
+      <c r="C28" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="4" t="inlineStr">
+        <is>
+          <t>Lavender Haze</t>
+        </is>
+      </c>
+      <c r="B29" s="5" t="n">
+        <v>11620</v>
+      </c>
+      <c r="C29" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="4" t="inlineStr">
+        <is>
+          <t>Never Getting Laid</t>
+        </is>
+      </c>
+      <c r="B30" s="5" t="n">
+        <v>9099</v>
+      </c>
+      <c r="C30" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="4" t="inlineStr">
+        <is>
+          <t>My Man on Willpower</t>
+        </is>
+      </c>
+      <c r="B31" s="5" t="n">
+        <v>8290</v>
+      </c>
+      <c r="C31" s="5" t="inlineStr">
+        <is>
+          <t>-2385</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="4" t="inlineStr">
+        <is>
+          <t>Manchild</t>
+        </is>
+      </c>
+      <c r="B32" s="5" t="n">
+        <v>9540</v>
+      </c>
+      <c r="C32" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="4" t="inlineStr">
+        <is>
+          <t>Sugar Talking</t>
+        </is>
+      </c>
+      <c r="B33" s="5" t="n">
+        <v>8633</v>
+      </c>
+      <c r="C33" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="4" t="inlineStr">
+        <is>
+          <t>My Man on Willpower</t>
+        </is>
+      </c>
+      <c r="B34" s="5" t="n">
+        <v>10675</v>
+      </c>
+      <c r="C34" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="4" t="inlineStr">
+        <is>
+          <t>Midnight Rain</t>
+        </is>
+      </c>
+      <c r="B35" s="5" t="n">
+        <v>11382</v>
+      </c>
+      <c r="C35" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="4" t="inlineStr">
+        <is>
+          <t>Nobodys Son</t>
+        </is>
+      </c>
+      <c r="B36" s="5" t="n">
+        <v>11090</v>
+      </c>
+      <c r="C36" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="4" t="inlineStr">
+        <is>
+          <t>House Tour</t>
+        </is>
+      </c>
+      <c r="B37" s="5" t="n">
+        <v>8514</v>
+      </c>
+      <c r="C37" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="4" t="inlineStr">
+        <is>
+          <t>Hanabi  Î±Î·Ð²Ï…</t>
+        </is>
+      </c>
+      <c r="B38" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C38" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="4" t="inlineStr">
+        <is>
+          <t>Saiyajin anbuâ„¢</t>
+        </is>
+      </c>
+      <c r="B39" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C39" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="4" t="inlineStr">
+        <is>
+          <t>Dummy</t>
+        </is>
+      </c>
+      <c r="B40" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C40" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="4" t="inlineStr">
+        <is>
+          <t>Cazador anbu â„¢</t>
+        </is>
+      </c>
+      <c r="B41" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C41" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="4" t="inlineStr">
+        <is>
+          <t>Besos Mojados</t>
+        </is>
+      </c>
+      <c r="B42" s="5" t="n">
+        <v>5171</v>
+      </c>
+      <c r="C42" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="4" t="inlineStr">
+        <is>
+          <t>DarkFire</t>
+        </is>
+      </c>
+      <c r="B43" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C43" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="4" t="inlineStr">
+        <is>
+          <t>DarkSunny</t>
+        </is>
+      </c>
+      <c r="B44" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C44" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="4" t="inlineStr">
+        <is>
+          <t>Dairen Uchiha</t>
+        </is>
+      </c>
+      <c r="B45" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C45" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="4" t="inlineStr">
+        <is>
+          <t>LILI ZENIN®</t>
+        </is>
+      </c>
+      <c r="B46" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C46" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="4" t="inlineStr">
+        <is>
+          <t>ryumichel ZENIN ®</t>
+        </is>
+      </c>
+      <c r="B47" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C47" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="4" t="inlineStr">
+        <is>
+          <t>margot ZENIN ®</t>
+        </is>
+      </c>
+      <c r="B48" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C48" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="4" t="inlineStr">
+        <is>
+          <t>linda ZENIN ®</t>
+        </is>
+      </c>
+      <c r="B49" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C49" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="4" t="inlineStr">
+        <is>
+          <t>equin0x</t>
+        </is>
+      </c>
+      <c r="B50" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C50" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="4" t="inlineStr">
+        <is>
+          <t>Jhayco - Mokai</t>
+        </is>
+      </c>
+      <c r="B51" s="5" t="n">
+        <v>30090</v>
+      </c>
+      <c r="C51" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="4" t="inlineStr">
+        <is>
+          <t>Jhayco - Joe</t>
+        </is>
+      </c>
+      <c r="B52" s="5" t="n">
+        <v>27217</v>
+      </c>
+      <c r="C52" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="4" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="B53" s="5" t="n">
+        <v>22946</v>
+      </c>
+      <c r="C53" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="4" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="B54" s="5" t="n">
+        <v>15193</v>
+      </c>
+      <c r="C54" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="4" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="B55" s="5" t="n">
+        <v>15130</v>
+      </c>
+      <c r="C55" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="4" t="inlineStr">
+        <is>
+          <t>Go Go Juice</t>
+        </is>
+      </c>
+      <c r="B56" s="5" t="n">
+        <v>9040</v>
+      </c>
+      <c r="C56" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="4" t="inlineStr">
+        <is>
+          <t>Jhayco - Imaginaste</t>
+        </is>
+      </c>
+      <c r="B57" s="5" t="n">
+        <v>5127</v>
+      </c>
+      <c r="C57" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="4" t="inlineStr">
+        <is>
+          <t>PuNch</t>
+        </is>
+      </c>
+      <c r="B58" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C58" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A2:C2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
auto: snapshot 2026-09-01 13:01:01
</commit_message>
<xml_diff>
--- a/clan_3815.xlsx
+++ b/clan_3815.xlsx
@@ -55,6 +55,7 @@
     <sheet name="2026-08-29" sheetId="46" state="visible" r:id="rId46"/>
     <sheet name="2026-08-30" sheetId="47" state="visible" r:id="rId47"/>
     <sheet name="2026-08-31" sheetId="48" state="visible" r:id="rId48"/>
+    <sheet name="2026-09-01" sheetId="49" state="visible" r:id="rId49"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -36177,6 +36178,885 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet49.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C58"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="29" customWidth="1" min="1" max="1"/>
+    <col width="9" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Clan: Mans Best Friend (3815)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Timestamp: 2026-09-01 13:01:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>Total Reps</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>Daily Reps (+1d)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>Nobodys Son</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="n">
+        <v>57880</v>
+      </c>
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>+46790</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>Player</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>Player</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>X y L O T A</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>AbdiHyde ID 13496</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>Create Character III</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C9" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>Create Character IV</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>Create Character V</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C11" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t>Player</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C12" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="4" t="inlineStr">
+        <is>
+          <t>Player</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C13" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="4" t="inlineStr">
+        <is>
+          <t>hunry</t>
+        </is>
+      </c>
+      <c r="B14" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C14" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="4" t="inlineStr">
+        <is>
+          <t>BlacKRin O</t>
+        </is>
+      </c>
+      <c r="B15" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C15" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="4" t="inlineStr">
+        <is>
+          <t>Tears</t>
+        </is>
+      </c>
+      <c r="B16" s="5" t="n">
+        <v>32550</v>
+      </c>
+      <c r="C16" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="4" t="inlineStr">
+        <is>
+          <t>NPC | SNOOPY</t>
+        </is>
+      </c>
+      <c r="B17" s="5" t="n">
+        <v>86158</v>
+      </c>
+      <c r="C17" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="4" t="inlineStr">
+        <is>
+          <t>Sugar Talking</t>
+        </is>
+      </c>
+      <c r="B18" s="5" t="n">
+        <v>43311</v>
+      </c>
+      <c r="C18" s="5" t="inlineStr">
+        <is>
+          <t>+34678</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="4" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B19" s="5" t="n">
+        <v>21095</v>
+      </c>
+      <c r="C19" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="4" t="inlineStr">
+        <is>
+          <t>Anti-Hero</t>
+        </is>
+      </c>
+      <c r="B20" s="5" t="n">
+        <v>20061</v>
+      </c>
+      <c r="C20" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="4" t="inlineStr">
+        <is>
+          <t>Vigilante Shit</t>
+        </is>
+      </c>
+      <c r="B21" s="5" t="n">
+        <v>46794</v>
+      </c>
+      <c r="C21" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="4" t="inlineStr">
+        <is>
+          <t>Sweet Nothing</t>
+        </is>
+      </c>
+      <c r="B22" s="5" t="n">
+        <v>8590</v>
+      </c>
+      <c r="C22" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="4" t="inlineStr">
+        <is>
+          <t>The Great War</t>
+        </is>
+      </c>
+      <c r="B23" s="5" t="n">
+        <v>8590</v>
+      </c>
+      <c r="C23" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">We Almost Broke Up </t>
+        </is>
+      </c>
+      <c r="B24" s="5" t="n">
+        <v>8983</v>
+      </c>
+      <c r="C24" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="4" t="inlineStr">
+        <is>
+          <t>When Did You Get Hot</t>
+        </is>
+      </c>
+      <c r="B25" s="5" t="n">
+        <v>135825</v>
+      </c>
+      <c r="C25" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="4" t="inlineStr">
+        <is>
+          <t>Dont Worry Ill Make</t>
+        </is>
+      </c>
+      <c r="B26" s="5" t="n">
+        <v>8943</v>
+      </c>
+      <c r="C26" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="4" t="inlineStr">
+        <is>
+          <t>Goodbye</t>
+        </is>
+      </c>
+      <c r="B27" s="5" t="n">
+        <v>22895</v>
+      </c>
+      <c r="C27" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="4" t="inlineStr">
+        <is>
+          <t>Mans Best Friend</t>
+        </is>
+      </c>
+      <c r="B28" s="5" t="n">
+        <v>19870</v>
+      </c>
+      <c r="C28" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="4" t="inlineStr">
+        <is>
+          <t>Lavender Haze</t>
+        </is>
+      </c>
+      <c r="B29" s="5" t="n">
+        <v>11620</v>
+      </c>
+      <c r="C29" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="4" t="inlineStr">
+        <is>
+          <t>Never Getting Laid</t>
+        </is>
+      </c>
+      <c r="B30" s="5" t="n">
+        <v>9099</v>
+      </c>
+      <c r="C30" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="4" t="inlineStr">
+        <is>
+          <t>My Man on Willpower</t>
+        </is>
+      </c>
+      <c r="B31" s="5" t="n">
+        <v>8290</v>
+      </c>
+      <c r="C31" s="5" t="inlineStr">
+        <is>
+          <t>-2385</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="4" t="inlineStr">
+        <is>
+          <t>Manchild</t>
+        </is>
+      </c>
+      <c r="B32" s="5" t="n">
+        <v>9540</v>
+      </c>
+      <c r="C32" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="4" t="inlineStr">
+        <is>
+          <t>Sugar Talking</t>
+        </is>
+      </c>
+      <c r="B33" s="5" t="n">
+        <v>8633</v>
+      </c>
+      <c r="C33" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="4" t="inlineStr">
+        <is>
+          <t>My Man on Willpower</t>
+        </is>
+      </c>
+      <c r="B34" s="5" t="n">
+        <v>10675</v>
+      </c>
+      <c r="C34" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="4" t="inlineStr">
+        <is>
+          <t>Midnight Rain</t>
+        </is>
+      </c>
+      <c r="B35" s="5" t="n">
+        <v>11382</v>
+      </c>
+      <c r="C35" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="4" t="inlineStr">
+        <is>
+          <t>Nobodys Son</t>
+        </is>
+      </c>
+      <c r="B36" s="5" t="n">
+        <v>11090</v>
+      </c>
+      <c r="C36" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="4" t="inlineStr">
+        <is>
+          <t>House Tour</t>
+        </is>
+      </c>
+      <c r="B37" s="5" t="n">
+        <v>8514</v>
+      </c>
+      <c r="C37" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="4" t="inlineStr">
+        <is>
+          <t>Hanabi  Î±Î·Ð²Ï…</t>
+        </is>
+      </c>
+      <c r="B38" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C38" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="4" t="inlineStr">
+        <is>
+          <t>Saiyajin anbuâ„¢</t>
+        </is>
+      </c>
+      <c r="B39" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C39" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="4" t="inlineStr">
+        <is>
+          <t>Dummy</t>
+        </is>
+      </c>
+      <c r="B40" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C40" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="4" t="inlineStr">
+        <is>
+          <t>Cazador anbu â„¢</t>
+        </is>
+      </c>
+      <c r="B41" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C41" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="4" t="inlineStr">
+        <is>
+          <t>Besos Mojados</t>
+        </is>
+      </c>
+      <c r="B42" s="5" t="n">
+        <v>5171</v>
+      </c>
+      <c r="C42" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="4" t="inlineStr">
+        <is>
+          <t>DarkFire</t>
+        </is>
+      </c>
+      <c r="B43" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C43" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="4" t="inlineStr">
+        <is>
+          <t>DarkSunny</t>
+        </is>
+      </c>
+      <c r="B44" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C44" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="4" t="inlineStr">
+        <is>
+          <t>Dairen Uchiha</t>
+        </is>
+      </c>
+      <c r="B45" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C45" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="4" t="inlineStr">
+        <is>
+          <t>LILI ZENIN®</t>
+        </is>
+      </c>
+      <c r="B46" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C46" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="4" t="inlineStr">
+        <is>
+          <t>ryumichel ZENIN ®</t>
+        </is>
+      </c>
+      <c r="B47" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C47" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="4" t="inlineStr">
+        <is>
+          <t>margot ZENIN ®</t>
+        </is>
+      </c>
+      <c r="B48" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C48" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="4" t="inlineStr">
+        <is>
+          <t>linda ZENIN ®</t>
+        </is>
+      </c>
+      <c r="B49" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C49" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="4" t="inlineStr">
+        <is>
+          <t>equin0x</t>
+        </is>
+      </c>
+      <c r="B50" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C50" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="4" t="inlineStr">
+        <is>
+          <t>Jhayco - Mokai</t>
+        </is>
+      </c>
+      <c r="B51" s="5" t="n">
+        <v>30090</v>
+      </c>
+      <c r="C51" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="4" t="inlineStr">
+        <is>
+          <t>Jhayco - Joe</t>
+        </is>
+      </c>
+      <c r="B52" s="5" t="n">
+        <v>27217</v>
+      </c>
+      <c r="C52" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="4" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="B53" s="5" t="n">
+        <v>22946</v>
+      </c>
+      <c r="C53" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="4" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="B54" s="5" t="n">
+        <v>15193</v>
+      </c>
+      <c r="C54" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="4" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="B55" s="5" t="n">
+        <v>15130</v>
+      </c>
+      <c r="C55" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="4" t="inlineStr">
+        <is>
+          <t>Go Go Juice</t>
+        </is>
+      </c>
+      <c r="B56" s="5" t="n">
+        <v>9040</v>
+      </c>
+      <c r="C56" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="4" t="inlineStr">
+        <is>
+          <t>Jhayco - Imaginaste</t>
+        </is>
+      </c>
+      <c r="B57" s="5" t="n">
+        <v>5127</v>
+      </c>
+      <c r="C57" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="4" t="inlineStr">
+        <is>
+          <t>PuNch</t>
+        </is>
+      </c>
+      <c r="B58" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C58" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A2:C2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
auto: snapshot 2026-09-02 13:01:01
</commit_message>
<xml_diff>
--- a/clan_3815.xlsx
+++ b/clan_3815.xlsx
@@ -56,6 +56,7 @@
     <sheet name="2026-08-30" sheetId="47" state="visible" r:id="rId47"/>
     <sheet name="2026-08-31" sheetId="48" state="visible" r:id="rId48"/>
     <sheet name="2026-09-01" sheetId="49" state="visible" r:id="rId49"/>
+    <sheet name="2026-09-02" sheetId="50" state="visible" r:id="rId50"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -37561,6 +37562,885 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet50.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C58"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="29" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Clan: Mans Best Friend (3815)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Timestamp: 2026-09-02 13:01:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>Total Reps</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>Daily Reps (+1d)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>Nobodys Son</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="n">
+        <v>553</v>
+      </c>
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>-10537</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>Player</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>Player</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>X y L O T A</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>AbdiHyde ID 13496</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>Create Character III</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C9" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>Create Character IV</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>Create Character V</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C11" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t>Player</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C12" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="4" t="inlineStr">
+        <is>
+          <t>Player</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C13" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="4" t="inlineStr">
+        <is>
+          <t>hunry</t>
+        </is>
+      </c>
+      <c r="B14" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C14" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="4" t="inlineStr">
+        <is>
+          <t>BlacKRin O</t>
+        </is>
+      </c>
+      <c r="B15" s="5" t="n">
+        <v>106</v>
+      </c>
+      <c r="C15" s="5" t="inlineStr">
+        <is>
+          <t>+106</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="4" t="inlineStr">
+        <is>
+          <t>Tears</t>
+        </is>
+      </c>
+      <c r="B16" s="5" t="n">
+        <v>218</v>
+      </c>
+      <c r="C16" s="5" t="inlineStr">
+        <is>
+          <t>-32332</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="4" t="inlineStr">
+        <is>
+          <t>NPC | SNOOPY</t>
+        </is>
+      </c>
+      <c r="B17" s="5" t="n">
+        <v>45</v>
+      </c>
+      <c r="C17" s="5" t="inlineStr">
+        <is>
+          <t>-86113</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="4" t="inlineStr">
+        <is>
+          <t>Sugar Talking</t>
+        </is>
+      </c>
+      <c r="B18" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C18" s="5" t="inlineStr">
+        <is>
+          <t>-8633</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="4" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B19" s="5" t="n">
+        <v>15</v>
+      </c>
+      <c r="C19" s="5" t="inlineStr">
+        <is>
+          <t>-21080</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="4" t="inlineStr">
+        <is>
+          <t>Anti-Hero</t>
+        </is>
+      </c>
+      <c r="B20" s="5" t="n">
+        <v>225</v>
+      </c>
+      <c r="C20" s="5" t="inlineStr">
+        <is>
+          <t>-19836</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="4" t="inlineStr">
+        <is>
+          <t>Vigilante Shit</t>
+        </is>
+      </c>
+      <c r="B21" s="5" t="n">
+        <v>130</v>
+      </c>
+      <c r="C21" s="5" t="inlineStr">
+        <is>
+          <t>-46664</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="4" t="inlineStr">
+        <is>
+          <t>Sweet Nothing</t>
+        </is>
+      </c>
+      <c r="B22" s="5" t="n">
+        <v>57</v>
+      </c>
+      <c r="C22" s="5" t="inlineStr">
+        <is>
+          <t>-8533</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="4" t="inlineStr">
+        <is>
+          <t>The Great War</t>
+        </is>
+      </c>
+      <c r="B23" s="5" t="n">
+        <v>45</v>
+      </c>
+      <c r="C23" s="5" t="inlineStr">
+        <is>
+          <t>-8545</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">We Almost Broke Up </t>
+        </is>
+      </c>
+      <c r="B24" s="5" t="n">
+        <v>45</v>
+      </c>
+      <c r="C24" s="5" t="inlineStr">
+        <is>
+          <t>-8938</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="4" t="inlineStr">
+        <is>
+          <t>When Did You Get Hot</t>
+        </is>
+      </c>
+      <c r="B25" s="5" t="n">
+        <v>45</v>
+      </c>
+      <c r="C25" s="5" t="inlineStr">
+        <is>
+          <t>-135780</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="4" t="inlineStr">
+        <is>
+          <t>Dont Worry Ill Make</t>
+        </is>
+      </c>
+      <c r="B26" s="5" t="n">
+        <v>45</v>
+      </c>
+      <c r="C26" s="5" t="inlineStr">
+        <is>
+          <t>-8898</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="4" t="inlineStr">
+        <is>
+          <t>Goodbye</t>
+        </is>
+      </c>
+      <c r="B27" s="5" t="n">
+        <v>21</v>
+      </c>
+      <c r="C27" s="5" t="inlineStr">
+        <is>
+          <t>-22874</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="4" t="inlineStr">
+        <is>
+          <t>Mans Best Friend</t>
+        </is>
+      </c>
+      <c r="B28" s="5" t="n">
+        <v>21</v>
+      </c>
+      <c r="C28" s="5" t="inlineStr">
+        <is>
+          <t>-19849</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="4" t="inlineStr">
+        <is>
+          <t>Lavender Haze</t>
+        </is>
+      </c>
+      <c r="B29" s="5" t="n">
+        <v>21</v>
+      </c>
+      <c r="C29" s="5" t="inlineStr">
+        <is>
+          <t>-11599</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="4" t="inlineStr">
+        <is>
+          <t>Never Getting Laid</t>
+        </is>
+      </c>
+      <c r="B30" s="5" t="n">
+        <v>115</v>
+      </c>
+      <c r="C30" s="5" t="inlineStr">
+        <is>
+          <t>-8984</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="4" t="inlineStr">
+        <is>
+          <t>My Man on Willpower</t>
+        </is>
+      </c>
+      <c r="B31" s="5" t="n">
+        <v>32</v>
+      </c>
+      <c r="C31" s="5" t="inlineStr">
+        <is>
+          <t>-10643</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="4" t="inlineStr">
+        <is>
+          <t>Manchild</t>
+        </is>
+      </c>
+      <c r="B32" s="5" t="n">
+        <v>45</v>
+      </c>
+      <c r="C32" s="5" t="inlineStr">
+        <is>
+          <t>-9495</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="4" t="inlineStr">
+        <is>
+          <t>Sugar Talking</t>
+        </is>
+      </c>
+      <c r="B33" s="5" t="n">
+        <v>45</v>
+      </c>
+      <c r="C33" s="5" t="inlineStr">
+        <is>
+          <t>-8588</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="4" t="inlineStr">
+        <is>
+          <t>My Man on Willpower</t>
+        </is>
+      </c>
+      <c r="B34" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C34" s="5" t="inlineStr">
+        <is>
+          <t>-10675</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="4" t="inlineStr">
+        <is>
+          <t>Midnight Rain</t>
+        </is>
+      </c>
+      <c r="B35" s="5" t="n">
+        <v>21</v>
+      </c>
+      <c r="C35" s="5" t="inlineStr">
+        <is>
+          <t>-11361</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="4" t="inlineStr">
+        <is>
+          <t>Nobodys Son</t>
+        </is>
+      </c>
+      <c r="B36" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C36" s="5" t="inlineStr">
+        <is>
+          <t>-11090</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="4" t="inlineStr">
+        <is>
+          <t>House Tour</t>
+        </is>
+      </c>
+      <c r="B37" s="5" t="n">
+        <v>45</v>
+      </c>
+      <c r="C37" s="5" t="inlineStr">
+        <is>
+          <t>-8469</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="4" t="inlineStr">
+        <is>
+          <t>Hanabi  Î±Î·Ð²Ï…</t>
+        </is>
+      </c>
+      <c r="B38" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C38" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="4" t="inlineStr">
+        <is>
+          <t>Saiyajin anbuâ„¢</t>
+        </is>
+      </c>
+      <c r="B39" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C39" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="4" t="inlineStr">
+        <is>
+          <t>Dummy</t>
+        </is>
+      </c>
+      <c r="B40" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C40" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="4" t="inlineStr">
+        <is>
+          <t>Cazador anbu â„¢</t>
+        </is>
+      </c>
+      <c r="B41" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C41" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="4" t="inlineStr">
+        <is>
+          <t>Besos Mojados</t>
+        </is>
+      </c>
+      <c r="B42" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C42" s="5" t="inlineStr">
+        <is>
+          <t>-5171</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="4" t="inlineStr">
+        <is>
+          <t>DarkFire</t>
+        </is>
+      </c>
+      <c r="B43" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C43" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="4" t="inlineStr">
+        <is>
+          <t>DarkSunny</t>
+        </is>
+      </c>
+      <c r="B44" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C44" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="4" t="inlineStr">
+        <is>
+          <t>Dairen Uchiha</t>
+        </is>
+      </c>
+      <c r="B45" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C45" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="4" t="inlineStr">
+        <is>
+          <t>LILI ZENIN®</t>
+        </is>
+      </c>
+      <c r="B46" s="5" t="n">
+        <v>64</v>
+      </c>
+      <c r="C46" s="5" t="inlineStr">
+        <is>
+          <t>+64</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="4" t="inlineStr">
+        <is>
+          <t>ryumichel ZENIN ®</t>
+        </is>
+      </c>
+      <c r="B47" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C47" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="4" t="inlineStr">
+        <is>
+          <t>margot ZENIN ®</t>
+        </is>
+      </c>
+      <c r="B48" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C48" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="4" t="inlineStr">
+        <is>
+          <t>linda ZENIN ®</t>
+        </is>
+      </c>
+      <c r="B49" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C49" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="4" t="inlineStr">
+        <is>
+          <t>equin0x</t>
+        </is>
+      </c>
+      <c r="B50" s="5" t="n">
+        <v>30</v>
+      </c>
+      <c r="C50" s="5" t="inlineStr">
+        <is>
+          <t>+30</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="4" t="inlineStr">
+        <is>
+          <t>Jhayco - Mokai</t>
+        </is>
+      </c>
+      <c r="B51" s="5" t="n">
+        <v>182</v>
+      </c>
+      <c r="C51" s="5" t="inlineStr">
+        <is>
+          <t>-29908</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="4" t="inlineStr">
+        <is>
+          <t>Jhayco - Joe</t>
+        </is>
+      </c>
+      <c r="B52" s="5" t="n">
+        <v>85</v>
+      </c>
+      <c r="C52" s="5" t="inlineStr">
+        <is>
+          <t>-27132</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="4" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="B53" s="5" t="n">
+        <v>45</v>
+      </c>
+      <c r="C53" s="5" t="inlineStr">
+        <is>
+          <t>-22901</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="4" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="B54" s="5" t="n">
+        <v>45</v>
+      </c>
+      <c r="C54" s="5" t="inlineStr">
+        <is>
+          <t>-15148</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="4" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="B55" s="5" t="n">
+        <v>45</v>
+      </c>
+      <c r="C55" s="5" t="inlineStr">
+        <is>
+          <t>-15085</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="4" t="inlineStr">
+        <is>
+          <t>Go Go Juice</t>
+        </is>
+      </c>
+      <c r="B56" s="5" t="n">
+        <v>45</v>
+      </c>
+      <c r="C56" s="5" t="inlineStr">
+        <is>
+          <t>-8995</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="4" t="inlineStr">
+        <is>
+          <t>Jhayco - Imaginaste</t>
+        </is>
+      </c>
+      <c r="B57" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C57" s="5" t="inlineStr">
+        <is>
+          <t>-5127</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="4" t="inlineStr">
+        <is>
+          <t>PuNch</t>
+        </is>
+      </c>
+      <c r="B58" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C58" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A2:C2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
auto: snapshot 2026-09-02 13:31:01
</commit_message>
<xml_diff>
--- a/clan_3815.xlsx
+++ b/clan_3815.xlsx
@@ -37586,7 +37586,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Timestamp: 2026-09-02 13:01:00</t>
+          <t>Timestamp: 2026-09-02 13:31:00</t>
         </is>
       </c>
     </row>
@@ -37839,11 +37839,11 @@
         </is>
       </c>
       <c r="B19" s="5" t="n">
-        <v>15</v>
+        <v>25</v>
       </c>
       <c r="C19" s="5" t="inlineStr">
         <is>
-          <t>-21080</t>
+          <t>-21070</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: snapshot 2026-09-03 13:01:01
</commit_message>
<xml_diff>
--- a/clan_3815.xlsx
+++ b/clan_3815.xlsx
@@ -57,6 +57,7 @@
     <sheet name="2026-08-31" sheetId="48" state="visible" r:id="rId48"/>
     <sheet name="2026-09-01" sheetId="49" state="visible" r:id="rId49"/>
     <sheet name="2026-09-02" sheetId="50" state="visible" r:id="rId50"/>
+    <sheet name="2026-09-03" sheetId="51" state="visible" r:id="rId51"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -38441,6 +38442,885 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet51.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C58"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="29" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Clan: Mans Best Friend (3815)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Timestamp: 2026-09-03 13:01:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>Total Reps</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>Daily Reps (+1d)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>Nobodys Son</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="n">
+        <v>553</v>
+      </c>
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>+553</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>Player</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>Player</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>X y L O T A</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>AbdiHyde ID 13496</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>Create Character III</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C9" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>Create Character IV</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>Create Character V</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C11" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t>Player</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C12" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="4" t="inlineStr">
+        <is>
+          <t>Player</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C13" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="4" t="inlineStr">
+        <is>
+          <t>hunry</t>
+        </is>
+      </c>
+      <c r="B14" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C14" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="4" t="inlineStr">
+        <is>
+          <t>BlacKRin O</t>
+        </is>
+      </c>
+      <c r="B15" s="5" t="n">
+        <v>106</v>
+      </c>
+      <c r="C15" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="4" t="inlineStr">
+        <is>
+          <t>Tears</t>
+        </is>
+      </c>
+      <c r="B16" s="5" t="n">
+        <v>218</v>
+      </c>
+      <c r="C16" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="4" t="inlineStr">
+        <is>
+          <t>NPC | SNOOPY</t>
+        </is>
+      </c>
+      <c r="B17" s="5" t="n">
+        <v>45</v>
+      </c>
+      <c r="C17" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="4" t="inlineStr">
+        <is>
+          <t>Sugar Talking</t>
+        </is>
+      </c>
+      <c r="B18" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C18" s="5" t="inlineStr">
+        <is>
+          <t>-45</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="4" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B19" s="5" t="n">
+        <v>25</v>
+      </c>
+      <c r="C19" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="4" t="inlineStr">
+        <is>
+          <t>Anti-Hero</t>
+        </is>
+      </c>
+      <c r="B20" s="5" t="n">
+        <v>225</v>
+      </c>
+      <c r="C20" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="4" t="inlineStr">
+        <is>
+          <t>Vigilante Shit</t>
+        </is>
+      </c>
+      <c r="B21" s="5" t="n">
+        <v>130</v>
+      </c>
+      <c r="C21" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="4" t="inlineStr">
+        <is>
+          <t>Sweet Nothing</t>
+        </is>
+      </c>
+      <c r="B22" s="5" t="n">
+        <v>57</v>
+      </c>
+      <c r="C22" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="4" t="inlineStr">
+        <is>
+          <t>The Great War</t>
+        </is>
+      </c>
+      <c r="B23" s="5" t="n">
+        <v>45</v>
+      </c>
+      <c r="C23" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">We Almost Broke Up </t>
+        </is>
+      </c>
+      <c r="B24" s="5" t="n">
+        <v>45</v>
+      </c>
+      <c r="C24" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="4" t="inlineStr">
+        <is>
+          <t>When Did You Get Hot</t>
+        </is>
+      </c>
+      <c r="B25" s="5" t="n">
+        <v>45</v>
+      </c>
+      <c r="C25" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="4" t="inlineStr">
+        <is>
+          <t>Dont Worry Ill Make</t>
+        </is>
+      </c>
+      <c r="B26" s="5" t="n">
+        <v>45</v>
+      </c>
+      <c r="C26" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="4" t="inlineStr">
+        <is>
+          <t>Goodbye</t>
+        </is>
+      </c>
+      <c r="B27" s="5" t="n">
+        <v>21</v>
+      </c>
+      <c r="C27" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="4" t="inlineStr">
+        <is>
+          <t>Mans Best Friend</t>
+        </is>
+      </c>
+      <c r="B28" s="5" t="n">
+        <v>21</v>
+      </c>
+      <c r="C28" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="4" t="inlineStr">
+        <is>
+          <t>Lavender Haze</t>
+        </is>
+      </c>
+      <c r="B29" s="5" t="n">
+        <v>21</v>
+      </c>
+      <c r="C29" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="4" t="inlineStr">
+        <is>
+          <t>Never Getting Laid</t>
+        </is>
+      </c>
+      <c r="B30" s="5" t="n">
+        <v>115</v>
+      </c>
+      <c r="C30" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="4" t="inlineStr">
+        <is>
+          <t>My Man on Willpower</t>
+        </is>
+      </c>
+      <c r="B31" s="5" t="n">
+        <v>32</v>
+      </c>
+      <c r="C31" s="5" t="inlineStr">
+        <is>
+          <t>+32</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="4" t="inlineStr">
+        <is>
+          <t>Manchild</t>
+        </is>
+      </c>
+      <c r="B32" s="5" t="n">
+        <v>45</v>
+      </c>
+      <c r="C32" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="4" t="inlineStr">
+        <is>
+          <t>Sugar Talking</t>
+        </is>
+      </c>
+      <c r="B33" s="5" t="n">
+        <v>45</v>
+      </c>
+      <c r="C33" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="4" t="inlineStr">
+        <is>
+          <t>My Man on Willpower</t>
+        </is>
+      </c>
+      <c r="B34" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C34" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="4" t="inlineStr">
+        <is>
+          <t>Midnight Rain</t>
+        </is>
+      </c>
+      <c r="B35" s="5" t="n">
+        <v>21</v>
+      </c>
+      <c r="C35" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="4" t="inlineStr">
+        <is>
+          <t>Nobodys Son</t>
+        </is>
+      </c>
+      <c r="B36" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C36" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="4" t="inlineStr">
+        <is>
+          <t>House Tour</t>
+        </is>
+      </c>
+      <c r="B37" s="5" t="n">
+        <v>45</v>
+      </c>
+      <c r="C37" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="4" t="inlineStr">
+        <is>
+          <t>Hanabi  Î±Î·Ð²Ï…</t>
+        </is>
+      </c>
+      <c r="B38" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C38" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="4" t="inlineStr">
+        <is>
+          <t>Saiyajin anbuâ„¢</t>
+        </is>
+      </c>
+      <c r="B39" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C39" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="4" t="inlineStr">
+        <is>
+          <t>Dummy</t>
+        </is>
+      </c>
+      <c r="B40" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C40" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="4" t="inlineStr">
+        <is>
+          <t>Cazador anbu â„¢</t>
+        </is>
+      </c>
+      <c r="B41" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C41" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="4" t="inlineStr">
+        <is>
+          <t>Besos Mojados</t>
+        </is>
+      </c>
+      <c r="B42" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C42" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="4" t="inlineStr">
+        <is>
+          <t>DarkFire</t>
+        </is>
+      </c>
+      <c r="B43" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C43" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="4" t="inlineStr">
+        <is>
+          <t>DarkSunny</t>
+        </is>
+      </c>
+      <c r="B44" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C44" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="4" t="inlineStr">
+        <is>
+          <t>Dairen Uchiha</t>
+        </is>
+      </c>
+      <c r="B45" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C45" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="4" t="inlineStr">
+        <is>
+          <t>LILI ZENIN®</t>
+        </is>
+      </c>
+      <c r="B46" s="5" t="n">
+        <v>64</v>
+      </c>
+      <c r="C46" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="4" t="inlineStr">
+        <is>
+          <t>ryumichel ZENIN ®</t>
+        </is>
+      </c>
+      <c r="B47" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C47" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="4" t="inlineStr">
+        <is>
+          <t>margot ZENIN ®</t>
+        </is>
+      </c>
+      <c r="B48" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C48" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="4" t="inlineStr">
+        <is>
+          <t>linda ZENIN ®</t>
+        </is>
+      </c>
+      <c r="B49" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C49" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="4" t="inlineStr">
+        <is>
+          <t>equin0x</t>
+        </is>
+      </c>
+      <c r="B50" s="5" t="n">
+        <v>30</v>
+      </c>
+      <c r="C50" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="4" t="inlineStr">
+        <is>
+          <t>Jhayco - Mokai</t>
+        </is>
+      </c>
+      <c r="B51" s="5" t="n">
+        <v>182</v>
+      </c>
+      <c r="C51" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="4" t="inlineStr">
+        <is>
+          <t>Jhayco - Joe</t>
+        </is>
+      </c>
+      <c r="B52" s="5" t="n">
+        <v>85</v>
+      </c>
+      <c r="C52" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="4" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="B53" s="5" t="n">
+        <v>45</v>
+      </c>
+      <c r="C53" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="4" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="B54" s="5" t="n">
+        <v>45</v>
+      </c>
+      <c r="C54" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="4" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="B55" s="5" t="n">
+        <v>45</v>
+      </c>
+      <c r="C55" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="4" t="inlineStr">
+        <is>
+          <t>Go Go Juice</t>
+        </is>
+      </c>
+      <c r="B56" s="5" t="n">
+        <v>45</v>
+      </c>
+      <c r="C56" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="4" t="inlineStr">
+        <is>
+          <t>Jhayco - Imaginaste</t>
+        </is>
+      </c>
+      <c r="B57" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C57" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="4" t="inlineStr">
+        <is>
+          <t>PuNch</t>
+        </is>
+      </c>
+      <c r="B58" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C58" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A2:C2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
auto: snapshot 2026-09-04 13:01:01
</commit_message>
<xml_diff>
--- a/clan_3815.xlsx
+++ b/clan_3815.xlsx
@@ -58,6 +58,7 @@
     <sheet name="2026-09-01" sheetId="49" state="visible" r:id="rId49"/>
     <sheet name="2026-09-02" sheetId="50" state="visible" r:id="rId50"/>
     <sheet name="2026-09-03" sheetId="51" state="visible" r:id="rId51"/>
+    <sheet name="2026-09-04" sheetId="52" state="visible" r:id="rId52"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -39321,6 +39322,885 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet52.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C58"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="29" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Clan: Mans Best Friend (3815)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Timestamp: 2026-09-04 13:01:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>Total Reps</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>Daily Reps (+1d)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>Nobodys Son</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="n">
+        <v>553</v>
+      </c>
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>+553</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>Player</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>Player</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>X y L O T A</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>AbdiHyde ID 13496</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>Create Character III</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C9" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>Create Character IV</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>Create Character V</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C11" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t>Player</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C12" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="4" t="inlineStr">
+        <is>
+          <t>Player</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C13" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="4" t="inlineStr">
+        <is>
+          <t>hunry</t>
+        </is>
+      </c>
+      <c r="B14" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C14" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="4" t="inlineStr">
+        <is>
+          <t>BlacKRin O</t>
+        </is>
+      </c>
+      <c r="B15" s="5" t="n">
+        <v>106</v>
+      </c>
+      <c r="C15" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="4" t="inlineStr">
+        <is>
+          <t>Tears</t>
+        </is>
+      </c>
+      <c r="B16" s="5" t="n">
+        <v>218</v>
+      </c>
+      <c r="C16" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="4" t="inlineStr">
+        <is>
+          <t>NPC | SNOOPY</t>
+        </is>
+      </c>
+      <c r="B17" s="5" t="n">
+        <v>45</v>
+      </c>
+      <c r="C17" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="4" t="inlineStr">
+        <is>
+          <t>Sugar Talking</t>
+        </is>
+      </c>
+      <c r="B18" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C18" s="5" t="inlineStr">
+        <is>
+          <t>-45</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="4" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B19" s="5" t="n">
+        <v>25</v>
+      </c>
+      <c r="C19" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="4" t="inlineStr">
+        <is>
+          <t>Anti-Hero</t>
+        </is>
+      </c>
+      <c r="B20" s="5" t="n">
+        <v>225</v>
+      </c>
+      <c r="C20" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="4" t="inlineStr">
+        <is>
+          <t>Vigilante Shit</t>
+        </is>
+      </c>
+      <c r="B21" s="5" t="n">
+        <v>130</v>
+      </c>
+      <c r="C21" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="4" t="inlineStr">
+        <is>
+          <t>Sweet Nothing</t>
+        </is>
+      </c>
+      <c r="B22" s="5" t="n">
+        <v>57</v>
+      </c>
+      <c r="C22" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="4" t="inlineStr">
+        <is>
+          <t>The Great War</t>
+        </is>
+      </c>
+      <c r="B23" s="5" t="n">
+        <v>45</v>
+      </c>
+      <c r="C23" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">We Almost Broke Up </t>
+        </is>
+      </c>
+      <c r="B24" s="5" t="n">
+        <v>45</v>
+      </c>
+      <c r="C24" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="4" t="inlineStr">
+        <is>
+          <t>When Did You Get Hot</t>
+        </is>
+      </c>
+      <c r="B25" s="5" t="n">
+        <v>45</v>
+      </c>
+      <c r="C25" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="4" t="inlineStr">
+        <is>
+          <t>Dont Worry Ill Make</t>
+        </is>
+      </c>
+      <c r="B26" s="5" t="n">
+        <v>45</v>
+      </c>
+      <c r="C26" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="4" t="inlineStr">
+        <is>
+          <t>Goodbye</t>
+        </is>
+      </c>
+      <c r="B27" s="5" t="n">
+        <v>21</v>
+      </c>
+      <c r="C27" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="4" t="inlineStr">
+        <is>
+          <t>Mans Best Friend</t>
+        </is>
+      </c>
+      <c r="B28" s="5" t="n">
+        <v>21</v>
+      </c>
+      <c r="C28" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="4" t="inlineStr">
+        <is>
+          <t>Lavender Haze</t>
+        </is>
+      </c>
+      <c r="B29" s="5" t="n">
+        <v>21</v>
+      </c>
+      <c r="C29" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="4" t="inlineStr">
+        <is>
+          <t>Never Getting Laid</t>
+        </is>
+      </c>
+      <c r="B30" s="5" t="n">
+        <v>115</v>
+      </c>
+      <c r="C30" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="4" t="inlineStr">
+        <is>
+          <t>My Man on Willpower</t>
+        </is>
+      </c>
+      <c r="B31" s="5" t="n">
+        <v>32</v>
+      </c>
+      <c r="C31" s="5" t="inlineStr">
+        <is>
+          <t>+32</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="4" t="inlineStr">
+        <is>
+          <t>Manchild</t>
+        </is>
+      </c>
+      <c r="B32" s="5" t="n">
+        <v>45</v>
+      </c>
+      <c r="C32" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="4" t="inlineStr">
+        <is>
+          <t>Sugar Talking</t>
+        </is>
+      </c>
+      <c r="B33" s="5" t="n">
+        <v>45</v>
+      </c>
+      <c r="C33" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="4" t="inlineStr">
+        <is>
+          <t>My Man on Willpower</t>
+        </is>
+      </c>
+      <c r="B34" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C34" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="4" t="inlineStr">
+        <is>
+          <t>Midnight Rain</t>
+        </is>
+      </c>
+      <c r="B35" s="5" t="n">
+        <v>21</v>
+      </c>
+      <c r="C35" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="4" t="inlineStr">
+        <is>
+          <t>Nobodys Son</t>
+        </is>
+      </c>
+      <c r="B36" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C36" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="4" t="inlineStr">
+        <is>
+          <t>House Tour</t>
+        </is>
+      </c>
+      <c r="B37" s="5" t="n">
+        <v>45</v>
+      </c>
+      <c r="C37" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="4" t="inlineStr">
+        <is>
+          <t>Hanabi  Î±Î·Ð²Ï…</t>
+        </is>
+      </c>
+      <c r="B38" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C38" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="4" t="inlineStr">
+        <is>
+          <t>Saiyajin anbuâ„¢</t>
+        </is>
+      </c>
+      <c r="B39" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C39" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="4" t="inlineStr">
+        <is>
+          <t>Dummy</t>
+        </is>
+      </c>
+      <c r="B40" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C40" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="4" t="inlineStr">
+        <is>
+          <t>Cazador anbu â„¢</t>
+        </is>
+      </c>
+      <c r="B41" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C41" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="4" t="inlineStr">
+        <is>
+          <t>Besos Mojados</t>
+        </is>
+      </c>
+      <c r="B42" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C42" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="4" t="inlineStr">
+        <is>
+          <t>DarkFire</t>
+        </is>
+      </c>
+      <c r="B43" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C43" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="4" t="inlineStr">
+        <is>
+          <t>DarkSunny</t>
+        </is>
+      </c>
+      <c r="B44" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C44" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="4" t="inlineStr">
+        <is>
+          <t>Dairen Uchiha</t>
+        </is>
+      </c>
+      <c r="B45" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C45" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="4" t="inlineStr">
+        <is>
+          <t>LILI ZENIN®</t>
+        </is>
+      </c>
+      <c r="B46" s="5" t="n">
+        <v>64</v>
+      </c>
+      <c r="C46" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="4" t="inlineStr">
+        <is>
+          <t>ryumichel ZENIN ®</t>
+        </is>
+      </c>
+      <c r="B47" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C47" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="4" t="inlineStr">
+        <is>
+          <t>margot ZENIN ®</t>
+        </is>
+      </c>
+      <c r="B48" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C48" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="4" t="inlineStr">
+        <is>
+          <t>linda ZENIN ®</t>
+        </is>
+      </c>
+      <c r="B49" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C49" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="4" t="inlineStr">
+        <is>
+          <t>equin0x</t>
+        </is>
+      </c>
+      <c r="B50" s="5" t="n">
+        <v>30</v>
+      </c>
+      <c r="C50" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="4" t="inlineStr">
+        <is>
+          <t>Jhayco - Mokai</t>
+        </is>
+      </c>
+      <c r="B51" s="5" t="n">
+        <v>182</v>
+      </c>
+      <c r="C51" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="4" t="inlineStr">
+        <is>
+          <t>Jhayco - Joe</t>
+        </is>
+      </c>
+      <c r="B52" s="5" t="n">
+        <v>85</v>
+      </c>
+      <c r="C52" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="4" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="B53" s="5" t="n">
+        <v>45</v>
+      </c>
+      <c r="C53" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="4" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="B54" s="5" t="n">
+        <v>45</v>
+      </c>
+      <c r="C54" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="4" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="B55" s="5" t="n">
+        <v>45</v>
+      </c>
+      <c r="C55" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="4" t="inlineStr">
+        <is>
+          <t>Go Go Juice</t>
+        </is>
+      </c>
+      <c r="B56" s="5" t="n">
+        <v>45</v>
+      </c>
+      <c r="C56" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="4" t="inlineStr">
+        <is>
+          <t>Jhayco - Imaginaste</t>
+        </is>
+      </c>
+      <c r="B57" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C57" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="4" t="inlineStr">
+        <is>
+          <t>PuNch</t>
+        </is>
+      </c>
+      <c r="B58" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C58" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A2:C2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
auto: snapshot 2026-09-05 13:01:01
</commit_message>
<xml_diff>
--- a/clan_3815.xlsx
+++ b/clan_3815.xlsx
@@ -59,6 +59,7 @@
     <sheet name="2026-09-02" sheetId="50" state="visible" r:id="rId50"/>
     <sheet name="2026-09-03" sheetId="51" state="visible" r:id="rId51"/>
     <sheet name="2026-09-04" sheetId="52" state="visible" r:id="rId52"/>
+    <sheet name="2026-09-05" sheetId="53" state="visible" r:id="rId53"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -40201,6 +40202,885 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet53.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C58"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="29" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Clan: Mans Best Friend (3815)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Timestamp: 2026-09-05 13:01:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>Total Reps</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>Daily Reps (+1d)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>Nobodys Son</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="n">
+        <v>553</v>
+      </c>
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>+553</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>Player</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>Player</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>X y L O T A</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>AbdiHyde ID 13496</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>Create Character III</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C9" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>Create Character IV</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>Create Character V</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C11" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t>Player</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C12" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="4" t="inlineStr">
+        <is>
+          <t>Player</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C13" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="4" t="inlineStr">
+        <is>
+          <t>hunry</t>
+        </is>
+      </c>
+      <c r="B14" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C14" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="4" t="inlineStr">
+        <is>
+          <t>BlacKRin O</t>
+        </is>
+      </c>
+      <c r="B15" s="5" t="n">
+        <v>106</v>
+      </c>
+      <c r="C15" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="4" t="inlineStr">
+        <is>
+          <t>Tears</t>
+        </is>
+      </c>
+      <c r="B16" s="5" t="n">
+        <v>218</v>
+      </c>
+      <c r="C16" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="4" t="inlineStr">
+        <is>
+          <t>NPC | SNOOPY</t>
+        </is>
+      </c>
+      <c r="B17" s="5" t="n">
+        <v>45</v>
+      </c>
+      <c r="C17" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="4" t="inlineStr">
+        <is>
+          <t>Sugar Talking</t>
+        </is>
+      </c>
+      <c r="B18" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C18" s="5" t="inlineStr">
+        <is>
+          <t>-45</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="4" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B19" s="5" t="n">
+        <v>25</v>
+      </c>
+      <c r="C19" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="4" t="inlineStr">
+        <is>
+          <t>Anti-Hero</t>
+        </is>
+      </c>
+      <c r="B20" s="5" t="n">
+        <v>225</v>
+      </c>
+      <c r="C20" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="4" t="inlineStr">
+        <is>
+          <t>Vigilante Shit</t>
+        </is>
+      </c>
+      <c r="B21" s="5" t="n">
+        <v>130</v>
+      </c>
+      <c r="C21" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="4" t="inlineStr">
+        <is>
+          <t>Sweet Nothing</t>
+        </is>
+      </c>
+      <c r="B22" s="5" t="n">
+        <v>57</v>
+      </c>
+      <c r="C22" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="4" t="inlineStr">
+        <is>
+          <t>The Great War</t>
+        </is>
+      </c>
+      <c r="B23" s="5" t="n">
+        <v>45</v>
+      </c>
+      <c r="C23" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">We Almost Broke Up </t>
+        </is>
+      </c>
+      <c r="B24" s="5" t="n">
+        <v>45</v>
+      </c>
+      <c r="C24" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="4" t="inlineStr">
+        <is>
+          <t>When Did You Get Hot</t>
+        </is>
+      </c>
+      <c r="B25" s="5" t="n">
+        <v>45</v>
+      </c>
+      <c r="C25" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="4" t="inlineStr">
+        <is>
+          <t>Dont Worry Ill Make</t>
+        </is>
+      </c>
+      <c r="B26" s="5" t="n">
+        <v>45</v>
+      </c>
+      <c r="C26" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="4" t="inlineStr">
+        <is>
+          <t>Goodbye</t>
+        </is>
+      </c>
+      <c r="B27" s="5" t="n">
+        <v>21</v>
+      </c>
+      <c r="C27" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="4" t="inlineStr">
+        <is>
+          <t>Mans Best Friend</t>
+        </is>
+      </c>
+      <c r="B28" s="5" t="n">
+        <v>21</v>
+      </c>
+      <c r="C28" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="4" t="inlineStr">
+        <is>
+          <t>Lavender Haze</t>
+        </is>
+      </c>
+      <c r="B29" s="5" t="n">
+        <v>21</v>
+      </c>
+      <c r="C29" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="4" t="inlineStr">
+        <is>
+          <t>Never Getting Laid</t>
+        </is>
+      </c>
+      <c r="B30" s="5" t="n">
+        <v>115</v>
+      </c>
+      <c r="C30" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="4" t="inlineStr">
+        <is>
+          <t>My Man on Willpower</t>
+        </is>
+      </c>
+      <c r="B31" s="5" t="n">
+        <v>32</v>
+      </c>
+      <c r="C31" s="5" t="inlineStr">
+        <is>
+          <t>+32</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="4" t="inlineStr">
+        <is>
+          <t>Manchild</t>
+        </is>
+      </c>
+      <c r="B32" s="5" t="n">
+        <v>45</v>
+      </c>
+      <c r="C32" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="4" t="inlineStr">
+        <is>
+          <t>Sugar Talking</t>
+        </is>
+      </c>
+      <c r="B33" s="5" t="n">
+        <v>45</v>
+      </c>
+      <c r="C33" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="4" t="inlineStr">
+        <is>
+          <t>My Man on Willpower</t>
+        </is>
+      </c>
+      <c r="B34" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C34" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="4" t="inlineStr">
+        <is>
+          <t>Midnight Rain</t>
+        </is>
+      </c>
+      <c r="B35" s="5" t="n">
+        <v>21</v>
+      </c>
+      <c r="C35" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="4" t="inlineStr">
+        <is>
+          <t>Nobodys Son</t>
+        </is>
+      </c>
+      <c r="B36" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C36" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="4" t="inlineStr">
+        <is>
+          <t>House Tour</t>
+        </is>
+      </c>
+      <c r="B37" s="5" t="n">
+        <v>45</v>
+      </c>
+      <c r="C37" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="4" t="inlineStr">
+        <is>
+          <t>Hanabi  Î±Î·Ð²Ï…</t>
+        </is>
+      </c>
+      <c r="B38" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C38" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="4" t="inlineStr">
+        <is>
+          <t>Saiyajin anbuâ„¢</t>
+        </is>
+      </c>
+      <c r="B39" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C39" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="4" t="inlineStr">
+        <is>
+          <t>Dummy</t>
+        </is>
+      </c>
+      <c r="B40" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C40" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="4" t="inlineStr">
+        <is>
+          <t>Cazador anbu â„¢</t>
+        </is>
+      </c>
+      <c r="B41" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C41" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="4" t="inlineStr">
+        <is>
+          <t>Besos Mojados</t>
+        </is>
+      </c>
+      <c r="B42" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C42" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="4" t="inlineStr">
+        <is>
+          <t>DarkFire</t>
+        </is>
+      </c>
+      <c r="B43" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C43" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="4" t="inlineStr">
+        <is>
+          <t>DarkSunny</t>
+        </is>
+      </c>
+      <c r="B44" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C44" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="4" t="inlineStr">
+        <is>
+          <t>Dairen Uchiha</t>
+        </is>
+      </c>
+      <c r="B45" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C45" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="4" t="inlineStr">
+        <is>
+          <t>LILI ZENIN®</t>
+        </is>
+      </c>
+      <c r="B46" s="5" t="n">
+        <v>64</v>
+      </c>
+      <c r="C46" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="4" t="inlineStr">
+        <is>
+          <t>ryumichel ZENIN ®</t>
+        </is>
+      </c>
+      <c r="B47" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C47" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="4" t="inlineStr">
+        <is>
+          <t>margot ZENIN ®</t>
+        </is>
+      </c>
+      <c r="B48" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C48" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="4" t="inlineStr">
+        <is>
+          <t>linda ZENIN ®</t>
+        </is>
+      </c>
+      <c r="B49" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C49" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="4" t="inlineStr">
+        <is>
+          <t>equin0x</t>
+        </is>
+      </c>
+      <c r="B50" s="5" t="n">
+        <v>30</v>
+      </c>
+      <c r="C50" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="4" t="inlineStr">
+        <is>
+          <t>Jhayco - Mokai</t>
+        </is>
+      </c>
+      <c r="B51" s="5" t="n">
+        <v>182</v>
+      </c>
+      <c r="C51" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="4" t="inlineStr">
+        <is>
+          <t>Jhayco - Joe</t>
+        </is>
+      </c>
+      <c r="B52" s="5" t="n">
+        <v>85</v>
+      </c>
+      <c r="C52" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="4" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="B53" s="5" t="n">
+        <v>45</v>
+      </c>
+      <c r="C53" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="4" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="B54" s="5" t="n">
+        <v>45</v>
+      </c>
+      <c r="C54" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="4" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="B55" s="5" t="n">
+        <v>45</v>
+      </c>
+      <c r="C55" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="4" t="inlineStr">
+        <is>
+          <t>Go Go Juice</t>
+        </is>
+      </c>
+      <c r="B56" s="5" t="n">
+        <v>45</v>
+      </c>
+      <c r="C56" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="4" t="inlineStr">
+        <is>
+          <t>Jhayco - Imaginaste</t>
+        </is>
+      </c>
+      <c r="B57" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C57" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="4" t="inlineStr">
+        <is>
+          <t>PuNch</t>
+        </is>
+      </c>
+      <c r="B58" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C58" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A2:C2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
auto: snapshot 2026-09-05 13:31:01
</commit_message>
<xml_diff>
--- a/clan_3815.xlsx
+++ b/clan_3815.xlsx
@@ -40226,7 +40226,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Timestamp: 2026-09-05 13:01:00</t>
+          <t>Timestamp: 2026-09-05 13:31:00</t>
         </is>
       </c>
     </row>
@@ -40254,11 +40254,11 @@
         </is>
       </c>
       <c r="B4" s="5" t="n">
-        <v>553</v>
+        <v>1303</v>
       </c>
       <c r="C4" s="5" t="inlineStr">
         <is>
-          <t>+553</t>
+          <t>+1303</t>
         </is>
       </c>
     </row>
@@ -40434,11 +40434,11 @@
         </is>
       </c>
       <c r="B16" s="5" t="n">
-        <v>218</v>
+        <v>968</v>
       </c>
       <c r="C16" s="5" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>+750</t>
         </is>
       </c>
     </row>
@@ -40464,11 +40464,11 @@
         </is>
       </c>
       <c r="B18" s="5" t="n">
-        <v>0</v>
+        <v>750</v>
       </c>
       <c r="C18" s="5" t="inlineStr">
         <is>
-          <t>-45</t>
+          <t>+705</t>
         </is>
       </c>
     </row>
@@ -40479,11 +40479,11 @@
         </is>
       </c>
       <c r="B19" s="5" t="n">
-        <v>25</v>
+        <v>775</v>
       </c>
       <c r="C19" s="5" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>+750</t>
         </is>
       </c>
     </row>
@@ -40494,11 +40494,11 @@
         </is>
       </c>
       <c r="B20" s="5" t="n">
-        <v>225</v>
+        <v>975</v>
       </c>
       <c r="C20" s="5" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>+750</t>
         </is>
       </c>
     </row>
@@ -40509,11 +40509,11 @@
         </is>
       </c>
       <c r="B21" s="5" t="n">
-        <v>130</v>
+        <v>880</v>
       </c>
       <c r="C21" s="5" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>+750</t>
         </is>
       </c>
     </row>
@@ -40524,11 +40524,11 @@
         </is>
       </c>
       <c r="B22" s="5" t="n">
-        <v>57</v>
+        <v>807</v>
       </c>
       <c r="C22" s="5" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>+750</t>
         </is>
       </c>
     </row>
@@ -40539,11 +40539,11 @@
         </is>
       </c>
       <c r="B23" s="5" t="n">
-        <v>45</v>
+        <v>795</v>
       </c>
       <c r="C23" s="5" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>+750</t>
         </is>
       </c>
     </row>
@@ -40599,11 +40599,11 @@
         </is>
       </c>
       <c r="B27" s="5" t="n">
-        <v>21</v>
+        <v>428</v>
       </c>
       <c r="C27" s="5" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>+407</t>
         </is>
       </c>
     </row>
@@ -40644,11 +40644,11 @@
         </is>
       </c>
       <c r="B30" s="5" t="n">
-        <v>115</v>
+        <v>865</v>
       </c>
       <c r="C30" s="5" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>+750</t>
         </is>
       </c>
     </row>
@@ -40659,11 +40659,11 @@
         </is>
       </c>
       <c r="B31" s="5" t="n">
-        <v>32</v>
+        <v>532</v>
       </c>
       <c r="C31" s="5" t="inlineStr">
         <is>
-          <t>+32</t>
+          <t>+532</t>
         </is>
       </c>
     </row>
@@ -40674,11 +40674,11 @@
         </is>
       </c>
       <c r="B32" s="5" t="n">
-        <v>45</v>
+        <v>795</v>
       </c>
       <c r="C32" s="5" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>+750</t>
         </is>
       </c>
     </row>
@@ -40959,11 +40959,11 @@
         </is>
       </c>
       <c r="B51" s="5" t="n">
-        <v>182</v>
+        <v>932</v>
       </c>
       <c r="C51" s="5" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>+750</t>
         </is>
       </c>
     </row>
@@ -40974,11 +40974,11 @@
         </is>
       </c>
       <c r="B52" s="5" t="n">
-        <v>85</v>
+        <v>835</v>
       </c>
       <c r="C52" s="5" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>+750</t>
         </is>
       </c>
     </row>
@@ -40989,11 +40989,11 @@
         </is>
       </c>
       <c r="B53" s="5" t="n">
-        <v>45</v>
+        <v>795</v>
       </c>
       <c r="C53" s="5" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>+750</t>
         </is>
       </c>
     </row>
@@ -41004,11 +41004,11 @@
         </is>
       </c>
       <c r="B54" s="5" t="n">
-        <v>45</v>
+        <v>795</v>
       </c>
       <c r="C54" s="5" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>+750</t>
         </is>
       </c>
     </row>
@@ -41019,11 +41019,11 @@
         </is>
       </c>
       <c r="B55" s="5" t="n">
-        <v>45</v>
+        <v>795</v>
       </c>
       <c r="C55" s="5" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>+750</t>
         </is>
       </c>
     </row>
@@ -41034,11 +41034,11 @@
         </is>
       </c>
       <c r="B56" s="5" t="n">
-        <v>45</v>
+        <v>795</v>
       </c>
       <c r="C56" s="5" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>+750</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: snapshot 2026-09-06 13:01:01
</commit_message>
<xml_diff>
--- a/clan_3815.xlsx
+++ b/clan_3815.xlsx
@@ -60,6 +60,7 @@
     <sheet name="2026-09-03" sheetId="51" state="visible" r:id="rId51"/>
     <sheet name="2026-09-04" sheetId="52" state="visible" r:id="rId52"/>
     <sheet name="2026-09-05" sheetId="53" state="visible" r:id="rId53"/>
+    <sheet name="2026-09-06" sheetId="54" state="visible" r:id="rId54"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -41081,6 +41082,885 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet54.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C58"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="29" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Clan: Mans Best Friend (3815)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Timestamp: 2026-09-06 13:01:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>Total Reps</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>Daily Reps (+1d)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>Nobodys Son</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="n">
+        <v>7764</v>
+      </c>
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>+7764</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>Player</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>Player</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>X y L O T A</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>AbdiHyde ID 13496</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>Create Character III</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C9" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>Create Character IV</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>Create Character V</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C11" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t>Player</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C12" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="4" t="inlineStr">
+        <is>
+          <t>Player</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C13" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="4" t="inlineStr">
+        <is>
+          <t>hunry</t>
+        </is>
+      </c>
+      <c r="B14" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C14" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="4" t="inlineStr">
+        <is>
+          <t>BlacKRin O</t>
+        </is>
+      </c>
+      <c r="B15" s="5" t="n">
+        <v>106</v>
+      </c>
+      <c r="C15" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="4" t="inlineStr">
+        <is>
+          <t>Tears</t>
+        </is>
+      </c>
+      <c r="B16" s="5" t="n">
+        <v>6810</v>
+      </c>
+      <c r="C16" s="5" t="inlineStr">
+        <is>
+          <t>+5842</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="4" t="inlineStr">
+        <is>
+          <t>NPC | SNOOPY</t>
+        </is>
+      </c>
+      <c r="B17" s="5" t="n">
+        <v>3165</v>
+      </c>
+      <c r="C17" s="5" t="inlineStr">
+        <is>
+          <t>+3120</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="4" t="inlineStr">
+        <is>
+          <t>Sugar Talking</t>
+        </is>
+      </c>
+      <c r="B18" s="5" t="n">
+        <v>1650</v>
+      </c>
+      <c r="C18" s="5" t="inlineStr">
+        <is>
+          <t>+1605</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="4" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B19" s="5" t="n">
+        <v>6644</v>
+      </c>
+      <c r="C19" s="5" t="inlineStr">
+        <is>
+          <t>+5869</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="4" t="inlineStr">
+        <is>
+          <t>Anti-Hero</t>
+        </is>
+      </c>
+      <c r="B20" s="5" t="n">
+        <v>7405</v>
+      </c>
+      <c r="C20" s="5" t="inlineStr">
+        <is>
+          <t>+6430</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="4" t="inlineStr">
+        <is>
+          <t>Vigilante Shit</t>
+        </is>
+      </c>
+      <c r="B21" s="5" t="n">
+        <v>6840</v>
+      </c>
+      <c r="C21" s="5" t="inlineStr">
+        <is>
+          <t>+5960</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="4" t="inlineStr">
+        <is>
+          <t>Sweet Nothing</t>
+        </is>
+      </c>
+      <c r="B22" s="5" t="n">
+        <v>5889</v>
+      </c>
+      <c r="C22" s="5" t="inlineStr">
+        <is>
+          <t>+5082</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="4" t="inlineStr">
+        <is>
+          <t>The Great War</t>
+        </is>
+      </c>
+      <c r="B23" s="5" t="n">
+        <v>6990</v>
+      </c>
+      <c r="C23" s="5" t="inlineStr">
+        <is>
+          <t>+6195</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">We Almost Broke Up </t>
+        </is>
+      </c>
+      <c r="B24" s="5" t="n">
+        <v>2802</v>
+      </c>
+      <c r="C24" s="5" t="inlineStr">
+        <is>
+          <t>+2757</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="4" t="inlineStr">
+        <is>
+          <t>When Did You Get Hot</t>
+        </is>
+      </c>
+      <c r="B25" s="5" t="n">
+        <v>3165</v>
+      </c>
+      <c r="C25" s="5" t="inlineStr">
+        <is>
+          <t>+3120</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="4" t="inlineStr">
+        <is>
+          <t>Dont Worry Ill Make</t>
+        </is>
+      </c>
+      <c r="B26" s="5" t="n">
+        <v>2897</v>
+      </c>
+      <c r="C26" s="5" t="inlineStr">
+        <is>
+          <t>+2852</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="4" t="inlineStr">
+        <is>
+          <t>Goodbye</t>
+        </is>
+      </c>
+      <c r="B27" s="5" t="n">
+        <v>6516</v>
+      </c>
+      <c r="C27" s="5" t="inlineStr">
+        <is>
+          <t>+6088</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="4" t="inlineStr">
+        <is>
+          <t>Mans Best Friend</t>
+        </is>
+      </c>
+      <c r="B28" s="5" t="n">
+        <v>6508</v>
+      </c>
+      <c r="C28" s="5" t="inlineStr">
+        <is>
+          <t>+6487</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="4" t="inlineStr">
+        <is>
+          <t>Lavender Haze</t>
+        </is>
+      </c>
+      <c r="B29" s="5" t="n">
+        <v>6381</v>
+      </c>
+      <c r="C29" s="5" t="inlineStr">
+        <is>
+          <t>+6360</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="4" t="inlineStr">
+        <is>
+          <t>Never Getting Laid</t>
+        </is>
+      </c>
+      <c r="B30" s="5" t="n">
+        <v>7476</v>
+      </c>
+      <c r="C30" s="5" t="inlineStr">
+        <is>
+          <t>+6611</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="4" t="inlineStr">
+        <is>
+          <t>My Man on Willpower</t>
+        </is>
+      </c>
+      <c r="B31" s="5" t="n">
+        <v>6518</v>
+      </c>
+      <c r="C31" s="5" t="inlineStr">
+        <is>
+          <t>+6518</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="4" t="inlineStr">
+        <is>
+          <t>Manchild</t>
+        </is>
+      </c>
+      <c r="B32" s="5" t="n">
+        <v>5890</v>
+      </c>
+      <c r="C32" s="5" t="inlineStr">
+        <is>
+          <t>+5095</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="4" t="inlineStr">
+        <is>
+          <t>Sugar Talking</t>
+        </is>
+      </c>
+      <c r="B33" s="5" t="n">
+        <v>3049</v>
+      </c>
+      <c r="C33" s="5" t="inlineStr">
+        <is>
+          <t>+3004</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="4" t="inlineStr">
+        <is>
+          <t>My Man on Willpower</t>
+        </is>
+      </c>
+      <c r="B34" s="5" t="n">
+        <v>1150</v>
+      </c>
+      <c r="C34" s="5" t="inlineStr">
+        <is>
+          <t>+1150</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="4" t="inlineStr">
+        <is>
+          <t>Midnight Rain</t>
+        </is>
+      </c>
+      <c r="B35" s="5" t="n">
+        <v>6356</v>
+      </c>
+      <c r="C35" s="5" t="inlineStr">
+        <is>
+          <t>+6335</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="4" t="inlineStr">
+        <is>
+          <t>Nobodys Son</t>
+        </is>
+      </c>
+      <c r="B36" s="5" t="n">
+        <v>1052</v>
+      </c>
+      <c r="C36" s="5" t="inlineStr">
+        <is>
+          <t>+1052</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="4" t="inlineStr">
+        <is>
+          <t>House Tour</t>
+        </is>
+      </c>
+      <c r="B37" s="5" t="n">
+        <v>2782</v>
+      </c>
+      <c r="C37" s="5" t="inlineStr">
+        <is>
+          <t>+2737</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="4" t="inlineStr">
+        <is>
+          <t>Hanabi  Î±Î·Ð²Ï…</t>
+        </is>
+      </c>
+      <c r="B38" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C38" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="4" t="inlineStr">
+        <is>
+          <t>Saiyajin anbuâ„¢</t>
+        </is>
+      </c>
+      <c r="B39" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C39" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="4" t="inlineStr">
+        <is>
+          <t>Dummy</t>
+        </is>
+      </c>
+      <c r="B40" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C40" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="4" t="inlineStr">
+        <is>
+          <t>Cazador anbu â„¢</t>
+        </is>
+      </c>
+      <c r="B41" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C41" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="4" t="inlineStr">
+        <is>
+          <t>Besos Mojados</t>
+        </is>
+      </c>
+      <c r="B42" s="5" t="n">
+        <v>2762</v>
+      </c>
+      <c r="C42" s="5" t="inlineStr">
+        <is>
+          <t>+2762</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="4" t="inlineStr">
+        <is>
+          <t>DarkFire</t>
+        </is>
+      </c>
+      <c r="B43" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C43" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="4" t="inlineStr">
+        <is>
+          <t>DarkSunny</t>
+        </is>
+      </c>
+      <c r="B44" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C44" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="4" t="inlineStr">
+        <is>
+          <t>Dairen Uchiha</t>
+        </is>
+      </c>
+      <c r="B45" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C45" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="4" t="inlineStr">
+        <is>
+          <t>LILI ZENIN®</t>
+        </is>
+      </c>
+      <c r="B46" s="5" t="n">
+        <v>64</v>
+      </c>
+      <c r="C46" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="4" t="inlineStr">
+        <is>
+          <t>ryumichel ZENIN ®</t>
+        </is>
+      </c>
+      <c r="B47" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C47" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="4" t="inlineStr">
+        <is>
+          <t>margot ZENIN ®</t>
+        </is>
+      </c>
+      <c r="B48" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C48" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="4" t="inlineStr">
+        <is>
+          <t>linda ZENIN ®</t>
+        </is>
+      </c>
+      <c r="B49" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C49" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="4" t="inlineStr">
+        <is>
+          <t>equin0x</t>
+        </is>
+      </c>
+      <c r="B50" s="5" t="n">
+        <v>992</v>
+      </c>
+      <c r="C50" s="5" t="inlineStr">
+        <is>
+          <t>+962</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="4" t="inlineStr">
+        <is>
+          <t>Jhayco - Mokai</t>
+        </is>
+      </c>
+      <c r="B51" s="5" t="n">
+        <v>6984</v>
+      </c>
+      <c r="C51" s="5" t="inlineStr">
+        <is>
+          <t>+6052</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="4" t="inlineStr">
+        <is>
+          <t>Jhayco - Joe</t>
+        </is>
+      </c>
+      <c r="B52" s="5" t="n">
+        <v>6918</v>
+      </c>
+      <c r="C52" s="5" t="inlineStr">
+        <is>
+          <t>+6083</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="4" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="B53" s="5" t="n">
+        <v>7045</v>
+      </c>
+      <c r="C53" s="5" t="inlineStr">
+        <is>
+          <t>+6250</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="4" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="B54" s="5" t="n">
+        <v>7002</v>
+      </c>
+      <c r="C54" s="5" t="inlineStr">
+        <is>
+          <t>+6207</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="4" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="B55" s="5" t="n">
+        <v>6856</v>
+      </c>
+      <c r="C55" s="5" t="inlineStr">
+        <is>
+          <t>+6061</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="4" t="inlineStr">
+        <is>
+          <t>Go Go Juice</t>
+        </is>
+      </c>
+      <c r="B56" s="5" t="n">
+        <v>6998</v>
+      </c>
+      <c r="C56" s="5" t="inlineStr">
+        <is>
+          <t>+6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="4" t="inlineStr">
+        <is>
+          <t>Jhayco - Imaginaste</t>
+        </is>
+      </c>
+      <c r="B57" s="5" t="n">
+        <v>2640</v>
+      </c>
+      <c r="C57" s="5" t="inlineStr">
+        <is>
+          <t>+2640</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="4" t="inlineStr">
+        <is>
+          <t>PuNch</t>
+        </is>
+      </c>
+      <c r="B58" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C58" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A2:C2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
auto: snapshot 2026-09-07 13:01:01
</commit_message>
<xml_diff>
--- a/clan_3815.xlsx
+++ b/clan_3815.xlsx
@@ -61,6 +61,7 @@
     <sheet name="2026-09-04" sheetId="52" state="visible" r:id="rId52"/>
     <sheet name="2026-09-05" sheetId="53" state="visible" r:id="rId53"/>
     <sheet name="2026-09-06" sheetId="54" state="visible" r:id="rId54"/>
+    <sheet name="2026-09-07" sheetId="55" state="visible" r:id="rId55"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -41961,6 +41962,885 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet55.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C58"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="29" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Clan: Mans Best Friend (3815)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Timestamp: 2026-09-07 13:01:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>Total Reps</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>Daily Reps (+1d)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>Nobodys Son</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="n">
+        <v>8524</v>
+      </c>
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>+7472</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>Player</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>Player</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>X y L O T A</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>AbdiHyde ID 13496</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>Create Character III</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C9" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>Create Character IV</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>Create Character V</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C11" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t>Player</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C12" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="4" t="inlineStr">
+        <is>
+          <t>Player</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C13" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="4" t="inlineStr">
+        <is>
+          <t>hunry</t>
+        </is>
+      </c>
+      <c r="B14" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C14" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="4" t="inlineStr">
+        <is>
+          <t>BlacKRin O</t>
+        </is>
+      </c>
+      <c r="B15" s="5" t="n">
+        <v>106</v>
+      </c>
+      <c r="C15" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="4" t="inlineStr">
+        <is>
+          <t>Tears</t>
+        </is>
+      </c>
+      <c r="B16" s="5" t="n">
+        <v>7483</v>
+      </c>
+      <c r="C16" s="5" t="inlineStr">
+        <is>
+          <t>+673</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="4" t="inlineStr">
+        <is>
+          <t>NPC | SNOOPY</t>
+        </is>
+      </c>
+      <c r="B17" s="5" t="n">
+        <v>3165</v>
+      </c>
+      <c r="C17" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="4" t="inlineStr">
+        <is>
+          <t>Sugar Talking</t>
+        </is>
+      </c>
+      <c r="B18" s="5" t="n">
+        <v>2410</v>
+      </c>
+      <c r="C18" s="5" t="inlineStr">
+        <is>
+          <t>-639</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="4" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B19" s="5" t="n">
+        <v>7444</v>
+      </c>
+      <c r="C19" s="5" t="inlineStr">
+        <is>
+          <t>+800</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="4" t="inlineStr">
+        <is>
+          <t>Anti-Hero</t>
+        </is>
+      </c>
+      <c r="B20" s="5" t="n">
+        <v>8116</v>
+      </c>
+      <c r="C20" s="5" t="inlineStr">
+        <is>
+          <t>+711</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="4" t="inlineStr">
+        <is>
+          <t>Vigilante Shit</t>
+        </is>
+      </c>
+      <c r="B21" s="5" t="n">
+        <v>7522</v>
+      </c>
+      <c r="C21" s="5" t="inlineStr">
+        <is>
+          <t>+682</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="4" t="inlineStr">
+        <is>
+          <t>Sweet Nothing</t>
+        </is>
+      </c>
+      <c r="B22" s="5" t="n">
+        <v>6490</v>
+      </c>
+      <c r="C22" s="5" t="inlineStr">
+        <is>
+          <t>+601</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="4" t="inlineStr">
+        <is>
+          <t>The Great War</t>
+        </is>
+      </c>
+      <c r="B23" s="5" t="n">
+        <v>7618</v>
+      </c>
+      <c r="C23" s="5" t="inlineStr">
+        <is>
+          <t>+628</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">We Almost Broke Up </t>
+        </is>
+      </c>
+      <c r="B24" s="5" t="n">
+        <v>2802</v>
+      </c>
+      <c r="C24" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="4" t="inlineStr">
+        <is>
+          <t>When Did You Get Hot</t>
+        </is>
+      </c>
+      <c r="B25" s="5" t="n">
+        <v>3165</v>
+      </c>
+      <c r="C25" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="4" t="inlineStr">
+        <is>
+          <t>Dont Worry Ill Make</t>
+        </is>
+      </c>
+      <c r="B26" s="5" t="n">
+        <v>2897</v>
+      </c>
+      <c r="C26" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="4" t="inlineStr">
+        <is>
+          <t>Goodbye</t>
+        </is>
+      </c>
+      <c r="B27" s="5" t="n">
+        <v>7276</v>
+      </c>
+      <c r="C27" s="5" t="inlineStr">
+        <is>
+          <t>+760</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="4" t="inlineStr">
+        <is>
+          <t>Mans Best Friend</t>
+        </is>
+      </c>
+      <c r="B28" s="5" t="n">
+        <v>7187</v>
+      </c>
+      <c r="C28" s="5" t="inlineStr">
+        <is>
+          <t>+679</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="4" t="inlineStr">
+        <is>
+          <t>Lavender Haze</t>
+        </is>
+      </c>
+      <c r="B29" s="5" t="n">
+        <v>7141</v>
+      </c>
+      <c r="C29" s="5" t="inlineStr">
+        <is>
+          <t>+760</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="4" t="inlineStr">
+        <is>
+          <t>Never Getting Laid</t>
+        </is>
+      </c>
+      <c r="B30" s="5" t="n">
+        <v>8176</v>
+      </c>
+      <c r="C30" s="5" t="inlineStr">
+        <is>
+          <t>+700</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="4" t="inlineStr">
+        <is>
+          <t>My Man on Willpower</t>
+        </is>
+      </c>
+      <c r="B31" s="5" t="n">
+        <v>6998</v>
+      </c>
+      <c r="C31" s="5" t="inlineStr">
+        <is>
+          <t>+5848</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="4" t="inlineStr">
+        <is>
+          <t>Manchild</t>
+        </is>
+      </c>
+      <c r="B32" s="5" t="n">
+        <v>6402</v>
+      </c>
+      <c r="C32" s="5" t="inlineStr">
+        <is>
+          <t>+512</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="4" t="inlineStr">
+        <is>
+          <t>Sugar Talking</t>
+        </is>
+      </c>
+      <c r="B33" s="5" t="n">
+        <v>3049</v>
+      </c>
+      <c r="C33" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="4" t="inlineStr">
+        <is>
+          <t>My Man on Willpower</t>
+        </is>
+      </c>
+      <c r="B34" s="5" t="n">
+        <v>1802</v>
+      </c>
+      <c r="C34" s="5" t="inlineStr">
+        <is>
+          <t>+652</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="4" t="inlineStr">
+        <is>
+          <t>Midnight Rain</t>
+        </is>
+      </c>
+      <c r="B35" s="5" t="n">
+        <v>7116</v>
+      </c>
+      <c r="C35" s="5" t="inlineStr">
+        <is>
+          <t>+760</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="4" t="inlineStr">
+        <is>
+          <t>Nobodys Son</t>
+        </is>
+      </c>
+      <c r="B36" s="5" t="n">
+        <v>1812</v>
+      </c>
+      <c r="C36" s="5" t="inlineStr">
+        <is>
+          <t>+760</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="4" t="inlineStr">
+        <is>
+          <t>House Tour</t>
+        </is>
+      </c>
+      <c r="B37" s="5" t="n">
+        <v>2782</v>
+      </c>
+      <c r="C37" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="4" t="inlineStr">
+        <is>
+          <t>Hanabi  Î±Î·Ð²Ï…</t>
+        </is>
+      </c>
+      <c r="B38" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C38" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="4" t="inlineStr">
+        <is>
+          <t>Saiyajin anbuâ„¢</t>
+        </is>
+      </c>
+      <c r="B39" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C39" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="4" t="inlineStr">
+        <is>
+          <t>Dummy</t>
+        </is>
+      </c>
+      <c r="B40" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C40" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="4" t="inlineStr">
+        <is>
+          <t>Cazador anbu â„¢</t>
+        </is>
+      </c>
+      <c r="B41" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C41" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="4" t="inlineStr">
+        <is>
+          <t>Besos Mojados</t>
+        </is>
+      </c>
+      <c r="B42" s="5" t="n">
+        <v>3182</v>
+      </c>
+      <c r="C42" s="5" t="inlineStr">
+        <is>
+          <t>+420</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="4" t="inlineStr">
+        <is>
+          <t>DarkFire</t>
+        </is>
+      </c>
+      <c r="B43" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C43" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="4" t="inlineStr">
+        <is>
+          <t>DarkSunny</t>
+        </is>
+      </c>
+      <c r="B44" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C44" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="4" t="inlineStr">
+        <is>
+          <t>Dairen Uchiha</t>
+        </is>
+      </c>
+      <c r="B45" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C45" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="4" t="inlineStr">
+        <is>
+          <t>LILI ZENIN®</t>
+        </is>
+      </c>
+      <c r="B46" s="5" t="n">
+        <v>64</v>
+      </c>
+      <c r="C46" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="4" t="inlineStr">
+        <is>
+          <t>ryumichel ZENIN ®</t>
+        </is>
+      </c>
+      <c r="B47" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C47" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="4" t="inlineStr">
+        <is>
+          <t>margot ZENIN ®</t>
+        </is>
+      </c>
+      <c r="B48" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C48" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="4" t="inlineStr">
+        <is>
+          <t>linda ZENIN ®</t>
+        </is>
+      </c>
+      <c r="B49" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C49" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="4" t="inlineStr">
+        <is>
+          <t>equin0x</t>
+        </is>
+      </c>
+      <c r="B50" s="5" t="n">
+        <v>992</v>
+      </c>
+      <c r="C50" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="4" t="inlineStr">
+        <is>
+          <t>Jhayco - Mokai</t>
+        </is>
+      </c>
+      <c r="B51" s="5" t="n">
+        <v>7784</v>
+      </c>
+      <c r="C51" s="5" t="inlineStr">
+        <is>
+          <t>+800</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="4" t="inlineStr">
+        <is>
+          <t>Jhayco - Joe</t>
+        </is>
+      </c>
+      <c r="B52" s="5" t="n">
+        <v>7610</v>
+      </c>
+      <c r="C52" s="5" t="inlineStr">
+        <is>
+          <t>+692</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="4" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="B53" s="5" t="n">
+        <v>7727</v>
+      </c>
+      <c r="C53" s="5" t="inlineStr">
+        <is>
+          <t>+682</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="4" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="B54" s="5" t="n">
+        <v>7622</v>
+      </c>
+      <c r="C54" s="5" t="inlineStr">
+        <is>
+          <t>+620</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="4" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="B55" s="5" t="n">
+        <v>7503</v>
+      </c>
+      <c r="C55" s="5" t="inlineStr">
+        <is>
+          <t>+647</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="4" t="inlineStr">
+        <is>
+          <t>Go Go Juice</t>
+        </is>
+      </c>
+      <c r="B56" s="5" t="n">
+        <v>7572</v>
+      </c>
+      <c r="C56" s="5" t="inlineStr">
+        <is>
+          <t>+574</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="4" t="inlineStr">
+        <is>
+          <t>Jhayco - Imaginaste</t>
+        </is>
+      </c>
+      <c r="B57" s="5" t="n">
+        <v>3060</v>
+      </c>
+      <c r="C57" s="5" t="inlineStr">
+        <is>
+          <t>+420</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="4" t="inlineStr">
+        <is>
+          <t>PuNch</t>
+        </is>
+      </c>
+      <c r="B58" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C58" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A2:C2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
auto: snapshot 2026-09-08 13:01:01
</commit_message>
<xml_diff>
--- a/clan_3815.xlsx
+++ b/clan_3815.xlsx
@@ -62,6 +62,7 @@
     <sheet name="2026-09-05" sheetId="53" state="visible" r:id="rId53"/>
     <sheet name="2026-09-06" sheetId="54" state="visible" r:id="rId54"/>
     <sheet name="2026-09-07" sheetId="55" state="visible" r:id="rId55"/>
+    <sheet name="2026-09-08" sheetId="56" state="visible" r:id="rId56"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -42841,6 +42842,885 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet56.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C58"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="29" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Clan: Mans Best Friend (3815)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Timestamp: 2026-09-08 13:01:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>Total Reps</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>Daily Reps (+1d)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>Nobodys Son</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="n">
+        <v>9934</v>
+      </c>
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>+8122</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>Player</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>Player</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>X y L O T A</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>AbdiHyde ID 13496</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>Create Character III</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C9" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>Create Character IV</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>Create Character V</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C11" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t>Player</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C12" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="4" t="inlineStr">
+        <is>
+          <t>Player</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C13" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="4" t="inlineStr">
+        <is>
+          <t>hunry</t>
+        </is>
+      </c>
+      <c r="B14" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C14" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="4" t="inlineStr">
+        <is>
+          <t>BlacKRin O</t>
+        </is>
+      </c>
+      <c r="B15" s="5" t="n">
+        <v>106</v>
+      </c>
+      <c r="C15" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="4" t="inlineStr">
+        <is>
+          <t>Tears</t>
+        </is>
+      </c>
+      <c r="B16" s="5" t="n">
+        <v>7483</v>
+      </c>
+      <c r="C16" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="4" t="inlineStr">
+        <is>
+          <t>NPC | SNOOPY</t>
+        </is>
+      </c>
+      <c r="B17" s="5" t="n">
+        <v>3165</v>
+      </c>
+      <c r="C17" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="4" t="inlineStr">
+        <is>
+          <t>Sugar Talking</t>
+        </is>
+      </c>
+      <c r="B18" s="5" t="n">
+        <v>3310</v>
+      </c>
+      <c r="C18" s="5" t="inlineStr">
+        <is>
+          <t>+261</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="4" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B19" s="5" t="n">
+        <v>8504</v>
+      </c>
+      <c r="C19" s="5" t="inlineStr">
+        <is>
+          <t>+1060</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="4" t="inlineStr">
+        <is>
+          <t>Anti-Hero</t>
+        </is>
+      </c>
+      <c r="B20" s="5" t="n">
+        <v>9266</v>
+      </c>
+      <c r="C20" s="5" t="inlineStr">
+        <is>
+          <t>+1150</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="4" t="inlineStr">
+        <is>
+          <t>Vigilante Shit</t>
+        </is>
+      </c>
+      <c r="B21" s="5" t="n">
+        <v>8672</v>
+      </c>
+      <c r="C21" s="5" t="inlineStr">
+        <is>
+          <t>+1150</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="4" t="inlineStr">
+        <is>
+          <t>Sweet Nothing</t>
+        </is>
+      </c>
+      <c r="B22" s="5" t="n">
+        <v>7631</v>
+      </c>
+      <c r="C22" s="5" t="inlineStr">
+        <is>
+          <t>+1141</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="4" t="inlineStr">
+        <is>
+          <t>The Great War</t>
+        </is>
+      </c>
+      <c r="B23" s="5" t="n">
+        <v>8732</v>
+      </c>
+      <c r="C23" s="5" t="inlineStr">
+        <is>
+          <t>+1114</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">We Almost Broke Up </t>
+        </is>
+      </c>
+      <c r="B24" s="5" t="n">
+        <v>2802</v>
+      </c>
+      <c r="C24" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="4" t="inlineStr">
+        <is>
+          <t>When Did You Get Hot</t>
+        </is>
+      </c>
+      <c r="B25" s="5" t="n">
+        <v>3165</v>
+      </c>
+      <c r="C25" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="4" t="inlineStr">
+        <is>
+          <t>Dont Worry Ill Make</t>
+        </is>
+      </c>
+      <c r="B26" s="5" t="n">
+        <v>2897</v>
+      </c>
+      <c r="C26" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="4" t="inlineStr">
+        <is>
+          <t>Goodbye</t>
+        </is>
+      </c>
+      <c r="B27" s="5" t="n">
+        <v>8776</v>
+      </c>
+      <c r="C27" s="5" t="inlineStr">
+        <is>
+          <t>+1500</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="4" t="inlineStr">
+        <is>
+          <t>Mans Best Friend</t>
+        </is>
+      </c>
+      <c r="B28" s="5" t="n">
+        <v>8687</v>
+      </c>
+      <c r="C28" s="5" t="inlineStr">
+        <is>
+          <t>+1500</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="4" t="inlineStr">
+        <is>
+          <t>Lavender Haze</t>
+        </is>
+      </c>
+      <c r="B29" s="5" t="n">
+        <v>8560</v>
+      </c>
+      <c r="C29" s="5" t="inlineStr">
+        <is>
+          <t>+1419</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="4" t="inlineStr">
+        <is>
+          <t>Never Getting Laid</t>
+        </is>
+      </c>
+      <c r="B30" s="5" t="n">
+        <v>8176</v>
+      </c>
+      <c r="C30" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="4" t="inlineStr">
+        <is>
+          <t>My Man on Willpower</t>
+        </is>
+      </c>
+      <c r="B31" s="5" t="n">
+        <v>6998</v>
+      </c>
+      <c r="C31" s="5" t="inlineStr">
+        <is>
+          <t>+5196</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="4" t="inlineStr">
+        <is>
+          <t>Manchild</t>
+        </is>
+      </c>
+      <c r="B32" s="5" t="n">
+        <v>6402</v>
+      </c>
+      <c r="C32" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="4" t="inlineStr">
+        <is>
+          <t>Sugar Talking</t>
+        </is>
+      </c>
+      <c r="B33" s="5" t="n">
+        <v>3049</v>
+      </c>
+      <c r="C33" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="4" t="inlineStr">
+        <is>
+          <t>My Man on Willpower</t>
+        </is>
+      </c>
+      <c r="B34" s="5" t="n">
+        <v>2702</v>
+      </c>
+      <c r="C34" s="5" t="inlineStr">
+        <is>
+          <t>+900</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="4" t="inlineStr">
+        <is>
+          <t>Midnight Rain</t>
+        </is>
+      </c>
+      <c r="B35" s="5" t="n">
+        <v>8404</v>
+      </c>
+      <c r="C35" s="5" t="inlineStr">
+        <is>
+          <t>+1288</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="4" t="inlineStr">
+        <is>
+          <t>Nobodys Son</t>
+        </is>
+      </c>
+      <c r="B36" s="5" t="n">
+        <v>2527</v>
+      </c>
+      <c r="C36" s="5" t="inlineStr">
+        <is>
+          <t>+715</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="4" t="inlineStr">
+        <is>
+          <t>House Tour</t>
+        </is>
+      </c>
+      <c r="B37" s="5" t="n">
+        <v>2782</v>
+      </c>
+      <c r="C37" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="4" t="inlineStr">
+        <is>
+          <t>Hanabi  Î±Î·Ð²Ï…</t>
+        </is>
+      </c>
+      <c r="B38" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C38" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="4" t="inlineStr">
+        <is>
+          <t>Saiyajin anbuâ„¢</t>
+        </is>
+      </c>
+      <c r="B39" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C39" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="4" t="inlineStr">
+        <is>
+          <t>Dummy</t>
+        </is>
+      </c>
+      <c r="B40" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C40" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="4" t="inlineStr">
+        <is>
+          <t>Cazador anbu â„¢</t>
+        </is>
+      </c>
+      <c r="B41" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C41" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="4" t="inlineStr">
+        <is>
+          <t>Besos Mojados</t>
+        </is>
+      </c>
+      <c r="B42" s="5" t="n">
+        <v>3732</v>
+      </c>
+      <c r="C42" s="5" t="inlineStr">
+        <is>
+          <t>+550</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="4" t="inlineStr">
+        <is>
+          <t>DarkFire</t>
+        </is>
+      </c>
+      <c r="B43" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C43" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="4" t="inlineStr">
+        <is>
+          <t>DarkSunny</t>
+        </is>
+      </c>
+      <c r="B44" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C44" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="4" t="inlineStr">
+        <is>
+          <t>Dairen Uchiha</t>
+        </is>
+      </c>
+      <c r="B45" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C45" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="4" t="inlineStr">
+        <is>
+          <t>LILI ZENIN®</t>
+        </is>
+      </c>
+      <c r="B46" s="5" t="n">
+        <v>64</v>
+      </c>
+      <c r="C46" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="4" t="inlineStr">
+        <is>
+          <t>ryumichel ZENIN ®</t>
+        </is>
+      </c>
+      <c r="B47" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C47" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="4" t="inlineStr">
+        <is>
+          <t>margot ZENIN ®</t>
+        </is>
+      </c>
+      <c r="B48" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C48" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="4" t="inlineStr">
+        <is>
+          <t>linda ZENIN ®</t>
+        </is>
+      </c>
+      <c r="B49" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C49" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="4" t="inlineStr">
+        <is>
+          <t>equin0x</t>
+        </is>
+      </c>
+      <c r="B50" s="5" t="n">
+        <v>992</v>
+      </c>
+      <c r="C50" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="4" t="inlineStr">
+        <is>
+          <t>Jhayco - Mokai</t>
+        </is>
+      </c>
+      <c r="B51" s="5" t="n">
+        <v>8484</v>
+      </c>
+      <c r="C51" s="5" t="inlineStr">
+        <is>
+          <t>+700</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="4" t="inlineStr">
+        <is>
+          <t>Jhayco - Joe</t>
+        </is>
+      </c>
+      <c r="B52" s="5" t="n">
+        <v>8310</v>
+      </c>
+      <c r="C52" s="5" t="inlineStr">
+        <is>
+          <t>+700</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="4" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="B53" s="5" t="n">
+        <v>8427</v>
+      </c>
+      <c r="C53" s="5" t="inlineStr">
+        <is>
+          <t>+700</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="4" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="B54" s="5" t="n">
+        <v>8322</v>
+      </c>
+      <c r="C54" s="5" t="inlineStr">
+        <is>
+          <t>+700</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="4" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="B55" s="5" t="n">
+        <v>8194</v>
+      </c>
+      <c r="C55" s="5" t="inlineStr">
+        <is>
+          <t>+691</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="4" t="inlineStr">
+        <is>
+          <t>Go Go Juice</t>
+        </is>
+      </c>
+      <c r="B56" s="5" t="n">
+        <v>7572</v>
+      </c>
+      <c r="C56" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="4" t="inlineStr">
+        <is>
+          <t>Jhayco - Imaginaste</t>
+        </is>
+      </c>
+      <c r="B57" s="5" t="n">
+        <v>3610</v>
+      </c>
+      <c r="C57" s="5" t="inlineStr">
+        <is>
+          <t>+550</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="4" t="inlineStr">
+        <is>
+          <t>PuNch</t>
+        </is>
+      </c>
+      <c r="B58" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C58" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A2:C2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
auto: snapshot 2026-09-09 13:01:01
</commit_message>
<xml_diff>
--- a/clan_3815.xlsx
+++ b/clan_3815.xlsx
@@ -63,6 +63,7 @@
     <sheet name="2026-09-06" sheetId="54" state="visible" r:id="rId54"/>
     <sheet name="2026-09-07" sheetId="55" state="visible" r:id="rId55"/>
     <sheet name="2026-09-08" sheetId="56" state="visible" r:id="rId56"/>
+    <sheet name="2026-09-09" sheetId="57" state="visible" r:id="rId57"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -43721,6 +43722,885 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet57.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C58"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="29" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Clan: Mans Best Friend (3815)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Timestamp: 2026-09-09 13:01:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>Total Reps</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>Daily Reps (+1d)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>Nobodys Son</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="n">
+        <v>11034</v>
+      </c>
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>+8507</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>Player</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>Player</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>X y L O T A</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>AbdiHyde ID 13496</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>Create Character III</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C9" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>Create Character IV</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>Create Character V</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C11" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t>Player</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C12" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="4" t="inlineStr">
+        <is>
+          <t>Player</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C13" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="4" t="inlineStr">
+        <is>
+          <t>hunry</t>
+        </is>
+      </c>
+      <c r="B14" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C14" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="4" t="inlineStr">
+        <is>
+          <t>BlacKRin O</t>
+        </is>
+      </c>
+      <c r="B15" s="5" t="n">
+        <v>106</v>
+      </c>
+      <c r="C15" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="4" t="inlineStr">
+        <is>
+          <t>Tears</t>
+        </is>
+      </c>
+      <c r="B16" s="5" t="n">
+        <v>7683</v>
+      </c>
+      <c r="C16" s="5" t="inlineStr">
+        <is>
+          <t>+200</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="4" t="inlineStr">
+        <is>
+          <t>NPC | SNOOPY</t>
+        </is>
+      </c>
+      <c r="B17" s="5" t="n">
+        <v>3165</v>
+      </c>
+      <c r="C17" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="4" t="inlineStr">
+        <is>
+          <t>Sugar Talking</t>
+        </is>
+      </c>
+      <c r="B18" s="5" t="n">
+        <v>4110</v>
+      </c>
+      <c r="C18" s="5" t="inlineStr">
+        <is>
+          <t>+1061</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="4" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B19" s="5" t="n">
+        <v>9754</v>
+      </c>
+      <c r="C19" s="5" t="inlineStr">
+        <is>
+          <t>+1250</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="4" t="inlineStr">
+        <is>
+          <t>Anti-Hero</t>
+        </is>
+      </c>
+      <c r="B20" s="5" t="n">
+        <v>10489</v>
+      </c>
+      <c r="C20" s="5" t="inlineStr">
+        <is>
+          <t>+1223</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="4" t="inlineStr">
+        <is>
+          <t>Vigilante Shit</t>
+        </is>
+      </c>
+      <c r="B21" s="5" t="n">
+        <v>9922</v>
+      </c>
+      <c r="C21" s="5" t="inlineStr">
+        <is>
+          <t>+1250</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="4" t="inlineStr">
+        <is>
+          <t>Sweet Nothing</t>
+        </is>
+      </c>
+      <c r="B22" s="5" t="n">
+        <v>8881</v>
+      </c>
+      <c r="C22" s="5" t="inlineStr">
+        <is>
+          <t>+1250</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="4" t="inlineStr">
+        <is>
+          <t>The Great War</t>
+        </is>
+      </c>
+      <c r="B23" s="5" t="n">
+        <v>9928</v>
+      </c>
+      <c r="C23" s="5" t="inlineStr">
+        <is>
+          <t>+1196</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">We Almost Broke Up </t>
+        </is>
+      </c>
+      <c r="B24" s="5" t="n">
+        <v>2802</v>
+      </c>
+      <c r="C24" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="4" t="inlineStr">
+        <is>
+          <t>When Did You Get Hot</t>
+        </is>
+      </c>
+      <c r="B25" s="5" t="n">
+        <v>3165</v>
+      </c>
+      <c r="C25" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="4" t="inlineStr">
+        <is>
+          <t>Dont Worry Ill Make</t>
+        </is>
+      </c>
+      <c r="B26" s="5" t="n">
+        <v>2897</v>
+      </c>
+      <c r="C26" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="4" t="inlineStr">
+        <is>
+          <t>Goodbye</t>
+        </is>
+      </c>
+      <c r="B27" s="5" t="n">
+        <v>9876</v>
+      </c>
+      <c r="C27" s="5" t="inlineStr">
+        <is>
+          <t>+1100</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="4" t="inlineStr">
+        <is>
+          <t>Mans Best Friend</t>
+        </is>
+      </c>
+      <c r="B28" s="5" t="n">
+        <v>9787</v>
+      </c>
+      <c r="C28" s="5" t="inlineStr">
+        <is>
+          <t>+1100</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="4" t="inlineStr">
+        <is>
+          <t>Lavender Haze</t>
+        </is>
+      </c>
+      <c r="B29" s="5" t="n">
+        <v>9615</v>
+      </c>
+      <c r="C29" s="5" t="inlineStr">
+        <is>
+          <t>+1055</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="4" t="inlineStr">
+        <is>
+          <t>Never Getting Laid</t>
+        </is>
+      </c>
+      <c r="B30" s="5" t="n">
+        <v>8376</v>
+      </c>
+      <c r="C30" s="5" t="inlineStr">
+        <is>
+          <t>+200</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="4" t="inlineStr">
+        <is>
+          <t>My Man on Willpower</t>
+        </is>
+      </c>
+      <c r="B31" s="5" t="n">
+        <v>7098</v>
+      </c>
+      <c r="C31" s="5" t="inlineStr">
+        <is>
+          <t>+4396</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="4" t="inlineStr">
+        <is>
+          <t>Manchild</t>
+        </is>
+      </c>
+      <c r="B32" s="5" t="n">
+        <v>6552</v>
+      </c>
+      <c r="C32" s="5" t="inlineStr">
+        <is>
+          <t>+150</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="4" t="inlineStr">
+        <is>
+          <t>Sugar Talking</t>
+        </is>
+      </c>
+      <c r="B33" s="5" t="n">
+        <v>3049</v>
+      </c>
+      <c r="C33" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="4" t="inlineStr">
+        <is>
+          <t>My Man on Willpower</t>
+        </is>
+      </c>
+      <c r="B34" s="5" t="n">
+        <v>3502</v>
+      </c>
+      <c r="C34" s="5" t="inlineStr">
+        <is>
+          <t>+800</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="4" t="inlineStr">
+        <is>
+          <t>Midnight Rain</t>
+        </is>
+      </c>
+      <c r="B35" s="5" t="n">
+        <v>9504</v>
+      </c>
+      <c r="C35" s="5" t="inlineStr">
+        <is>
+          <t>+1100</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="4" t="inlineStr">
+        <is>
+          <t>Nobodys Son</t>
+        </is>
+      </c>
+      <c r="B36" s="5" t="n">
+        <v>3277</v>
+      </c>
+      <c r="C36" s="5" t="inlineStr">
+        <is>
+          <t>+750</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="4" t="inlineStr">
+        <is>
+          <t>House Tour</t>
+        </is>
+      </c>
+      <c r="B37" s="5" t="n">
+        <v>2782</v>
+      </c>
+      <c r="C37" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="4" t="inlineStr">
+        <is>
+          <t>Hanabi  Î±Î·Ð²Ï…</t>
+        </is>
+      </c>
+      <c r="B38" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C38" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="4" t="inlineStr">
+        <is>
+          <t>Saiyajin anbuâ„¢</t>
+        </is>
+      </c>
+      <c r="B39" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C39" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="4" t="inlineStr">
+        <is>
+          <t>Dummy</t>
+        </is>
+      </c>
+      <c r="B40" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C40" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="4" t="inlineStr">
+        <is>
+          <t>Cazador anbu â„¢</t>
+        </is>
+      </c>
+      <c r="B41" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C41" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="4" t="inlineStr">
+        <is>
+          <t>Besos Mojados</t>
+        </is>
+      </c>
+      <c r="B42" s="5" t="n">
+        <v>4432</v>
+      </c>
+      <c r="C42" s="5" t="inlineStr">
+        <is>
+          <t>+700</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="4" t="inlineStr">
+        <is>
+          <t>DarkFire</t>
+        </is>
+      </c>
+      <c r="B43" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C43" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="4" t="inlineStr">
+        <is>
+          <t>DarkSunny</t>
+        </is>
+      </c>
+      <c r="B44" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C44" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="4" t="inlineStr">
+        <is>
+          <t>Dairen Uchiha</t>
+        </is>
+      </c>
+      <c r="B45" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C45" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="4" t="inlineStr">
+        <is>
+          <t>LILI ZENIN®</t>
+        </is>
+      </c>
+      <c r="B46" s="5" t="n">
+        <v>64</v>
+      </c>
+      <c r="C46" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="4" t="inlineStr">
+        <is>
+          <t>ryumichel ZENIN ®</t>
+        </is>
+      </c>
+      <c r="B47" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C47" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="4" t="inlineStr">
+        <is>
+          <t>margot ZENIN ®</t>
+        </is>
+      </c>
+      <c r="B48" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C48" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="4" t="inlineStr">
+        <is>
+          <t>linda ZENIN ®</t>
+        </is>
+      </c>
+      <c r="B49" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C49" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="4" t="inlineStr">
+        <is>
+          <t>equin0x</t>
+        </is>
+      </c>
+      <c r="B50" s="5" t="n">
+        <v>992</v>
+      </c>
+      <c r="C50" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="4" t="inlineStr">
+        <is>
+          <t>Jhayco - Mokai</t>
+        </is>
+      </c>
+      <c r="B51" s="5" t="n">
+        <v>9734</v>
+      </c>
+      <c r="C51" s="5" t="inlineStr">
+        <is>
+          <t>+1250</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="4" t="inlineStr">
+        <is>
+          <t>Jhayco - Joe</t>
+        </is>
+      </c>
+      <c r="B52" s="5" t="n">
+        <v>9560</v>
+      </c>
+      <c r="C52" s="5" t="inlineStr">
+        <is>
+          <t>+1250</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="4" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="B53" s="5" t="n">
+        <v>9659</v>
+      </c>
+      <c r="C53" s="5" t="inlineStr">
+        <is>
+          <t>+1232</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="4" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="B54" s="5" t="n">
+        <v>9536</v>
+      </c>
+      <c r="C54" s="5" t="inlineStr">
+        <is>
+          <t>+1214</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="4" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="B55" s="5" t="n">
+        <v>9444</v>
+      </c>
+      <c r="C55" s="5" t="inlineStr">
+        <is>
+          <t>+1250</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="4" t="inlineStr">
+        <is>
+          <t>Go Go Juice</t>
+        </is>
+      </c>
+      <c r="B56" s="5" t="n">
+        <v>7722</v>
+      </c>
+      <c r="C56" s="5" t="inlineStr">
+        <is>
+          <t>+150</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="4" t="inlineStr">
+        <is>
+          <t>Jhayco - Imaginaste</t>
+        </is>
+      </c>
+      <c r="B57" s="5" t="n">
+        <v>4310</v>
+      </c>
+      <c r="C57" s="5" t="inlineStr">
+        <is>
+          <t>+700</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="4" t="inlineStr">
+        <is>
+          <t>PuNch</t>
+        </is>
+      </c>
+      <c r="B58" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C58" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A2:C2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
auto: snapshot 2026-09-10 13:01:01
</commit_message>
<xml_diff>
--- a/clan_3815.xlsx
+++ b/clan_3815.xlsx
@@ -64,6 +64,7 @@
     <sheet name="2026-09-07" sheetId="55" state="visible" r:id="rId55"/>
     <sheet name="2026-09-08" sheetId="56" state="visible" r:id="rId56"/>
     <sheet name="2026-09-09" sheetId="57" state="visible" r:id="rId57"/>
+    <sheet name="2026-09-10" sheetId="58" state="visible" r:id="rId58"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -44601,6 +44602,885 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet58.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C58"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="29" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Clan: Mans Best Friend (3815)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Timestamp: 2026-09-10 13:01:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>Total Reps</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>Daily Reps (+1d)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>Nobodys Son</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="n">
+        <v>12044</v>
+      </c>
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>+8767</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>Player</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>Player</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>X y L O T A</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>AbdiHyde ID 13496</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>Create Character III</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C9" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>Create Character IV</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>Create Character V</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C11" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t>Player</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C12" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="4" t="inlineStr">
+        <is>
+          <t>Player</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C13" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="4" t="inlineStr">
+        <is>
+          <t>hunry</t>
+        </is>
+      </c>
+      <c r="B14" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C14" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="4" t="inlineStr">
+        <is>
+          <t>BlacKRin O</t>
+        </is>
+      </c>
+      <c r="B15" s="5" t="n">
+        <v>106</v>
+      </c>
+      <c r="C15" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="4" t="inlineStr">
+        <is>
+          <t>Tears</t>
+        </is>
+      </c>
+      <c r="B16" s="5" t="n">
+        <v>8383</v>
+      </c>
+      <c r="C16" s="5" t="inlineStr">
+        <is>
+          <t>+700</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="4" t="inlineStr">
+        <is>
+          <t>NPC | SNOOPY</t>
+        </is>
+      </c>
+      <c r="B17" s="5" t="n">
+        <v>3165</v>
+      </c>
+      <c r="C17" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="4" t="inlineStr">
+        <is>
+          <t>Sugar Talking</t>
+        </is>
+      </c>
+      <c r="B18" s="5" t="n">
+        <v>4510</v>
+      </c>
+      <c r="C18" s="5" t="inlineStr">
+        <is>
+          <t>+1461</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="4" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B19" s="5" t="n">
+        <v>10804</v>
+      </c>
+      <c r="C19" s="5" t="inlineStr">
+        <is>
+          <t>+1050</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="4" t="inlineStr">
+        <is>
+          <t>Anti-Hero</t>
+        </is>
+      </c>
+      <c r="B20" s="5" t="n">
+        <v>11439</v>
+      </c>
+      <c r="C20" s="5" t="inlineStr">
+        <is>
+          <t>+950</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="4" t="inlineStr">
+        <is>
+          <t>Vigilante Shit</t>
+        </is>
+      </c>
+      <c r="B21" s="5" t="n">
+        <v>10872</v>
+      </c>
+      <c r="C21" s="5" t="inlineStr">
+        <is>
+          <t>+950</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="4" t="inlineStr">
+        <is>
+          <t>Sweet Nothing</t>
+        </is>
+      </c>
+      <c r="B22" s="5" t="n">
+        <v>9673</v>
+      </c>
+      <c r="C22" s="5" t="inlineStr">
+        <is>
+          <t>+792</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="4" t="inlineStr">
+        <is>
+          <t>The Great War</t>
+        </is>
+      </c>
+      <c r="B23" s="5" t="n">
+        <v>10828</v>
+      </c>
+      <c r="C23" s="5" t="inlineStr">
+        <is>
+          <t>+900</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">We Almost Broke Up </t>
+        </is>
+      </c>
+      <c r="B24" s="5" t="n">
+        <v>2802</v>
+      </c>
+      <c r="C24" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="4" t="inlineStr">
+        <is>
+          <t>When Did You Get Hot</t>
+        </is>
+      </c>
+      <c r="B25" s="5" t="n">
+        <v>3165</v>
+      </c>
+      <c r="C25" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="4" t="inlineStr">
+        <is>
+          <t>Dont Worry Ill Make</t>
+        </is>
+      </c>
+      <c r="B26" s="5" t="n">
+        <v>2897</v>
+      </c>
+      <c r="C26" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="4" t="inlineStr">
+        <is>
+          <t>Goodbye</t>
+        </is>
+      </c>
+      <c r="B27" s="5" t="n">
+        <v>10913</v>
+      </c>
+      <c r="C27" s="5" t="inlineStr">
+        <is>
+          <t>+1037</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="4" t="inlineStr">
+        <is>
+          <t>Mans Best Friend</t>
+        </is>
+      </c>
+      <c r="B28" s="5" t="n">
+        <v>10842</v>
+      </c>
+      <c r="C28" s="5" t="inlineStr">
+        <is>
+          <t>+1055</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="4" t="inlineStr">
+        <is>
+          <t>Lavender Haze</t>
+        </is>
+      </c>
+      <c r="B29" s="5" t="n">
+        <v>10715</v>
+      </c>
+      <c r="C29" s="5" t="inlineStr">
+        <is>
+          <t>+1100</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="4" t="inlineStr">
+        <is>
+          <t>Never Getting Laid</t>
+        </is>
+      </c>
+      <c r="B30" s="5" t="n">
+        <v>8976</v>
+      </c>
+      <c r="C30" s="5" t="inlineStr">
+        <is>
+          <t>+600</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="4" t="inlineStr">
+        <is>
+          <t>My Man on Willpower</t>
+        </is>
+      </c>
+      <c r="B31" s="5" t="n">
+        <v>7648</v>
+      </c>
+      <c r="C31" s="5" t="inlineStr">
+        <is>
+          <t>+4146</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="4" t="inlineStr">
+        <is>
+          <t>Manchild</t>
+        </is>
+      </c>
+      <c r="B32" s="5" t="n">
+        <v>7152</v>
+      </c>
+      <c r="C32" s="5" t="inlineStr">
+        <is>
+          <t>+600</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="4" t="inlineStr">
+        <is>
+          <t>Sugar Talking</t>
+        </is>
+      </c>
+      <c r="B33" s="5" t="n">
+        <v>3049</v>
+      </c>
+      <c r="C33" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="4" t="inlineStr">
+        <is>
+          <t>My Man on Willpower</t>
+        </is>
+      </c>
+      <c r="B34" s="5" t="n">
+        <v>3902</v>
+      </c>
+      <c r="C34" s="5" t="inlineStr">
+        <is>
+          <t>+400</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="4" t="inlineStr">
+        <is>
+          <t>Midnight Rain</t>
+        </is>
+      </c>
+      <c r="B35" s="5" t="n">
+        <v>10568</v>
+      </c>
+      <c r="C35" s="5" t="inlineStr">
+        <is>
+          <t>+1064</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="4" t="inlineStr">
+        <is>
+          <t>Nobodys Son</t>
+        </is>
+      </c>
+      <c r="B36" s="5" t="n">
+        <v>3677</v>
+      </c>
+      <c r="C36" s="5" t="inlineStr">
+        <is>
+          <t>+400</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="4" t="inlineStr">
+        <is>
+          <t>House Tour</t>
+        </is>
+      </c>
+      <c r="B37" s="5" t="n">
+        <v>2782</v>
+      </c>
+      <c r="C37" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="4" t="inlineStr">
+        <is>
+          <t>Hanabi  Î±Î·Ð²Ï…</t>
+        </is>
+      </c>
+      <c r="B38" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C38" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="4" t="inlineStr">
+        <is>
+          <t>Saiyajin anbuâ„¢</t>
+        </is>
+      </c>
+      <c r="B39" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C39" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="4" t="inlineStr">
+        <is>
+          <t>Dummy</t>
+        </is>
+      </c>
+      <c r="B40" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C40" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="4" t="inlineStr">
+        <is>
+          <t>Cazador anbu â„¢</t>
+        </is>
+      </c>
+      <c r="B41" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C41" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="4" t="inlineStr">
+        <is>
+          <t>Besos Mojados</t>
+        </is>
+      </c>
+      <c r="B42" s="5" t="n">
+        <v>4682</v>
+      </c>
+      <c r="C42" s="5" t="inlineStr">
+        <is>
+          <t>+250</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="4" t="inlineStr">
+        <is>
+          <t>DarkFire</t>
+        </is>
+      </c>
+      <c r="B43" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C43" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="4" t="inlineStr">
+        <is>
+          <t>DarkSunny</t>
+        </is>
+      </c>
+      <c r="B44" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C44" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="4" t="inlineStr">
+        <is>
+          <t>Dairen Uchiha</t>
+        </is>
+      </c>
+      <c r="B45" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C45" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="4" t="inlineStr">
+        <is>
+          <t>LILI ZENIN®</t>
+        </is>
+      </c>
+      <c r="B46" s="5" t="n">
+        <v>64</v>
+      </c>
+      <c r="C46" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="4" t="inlineStr">
+        <is>
+          <t>ryumichel ZENIN ®</t>
+        </is>
+      </c>
+      <c r="B47" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C47" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="4" t="inlineStr">
+        <is>
+          <t>margot ZENIN ®</t>
+        </is>
+      </c>
+      <c r="B48" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C48" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="4" t="inlineStr">
+        <is>
+          <t>linda ZENIN ®</t>
+        </is>
+      </c>
+      <c r="B49" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C49" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="4" t="inlineStr">
+        <is>
+          <t>equin0x</t>
+        </is>
+      </c>
+      <c r="B50" s="5" t="n">
+        <v>992</v>
+      </c>
+      <c r="C50" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="4" t="inlineStr">
+        <is>
+          <t>Jhayco - Mokai</t>
+        </is>
+      </c>
+      <c r="B51" s="5" t="n">
+        <v>10771</v>
+      </c>
+      <c r="C51" s="5" t="inlineStr">
+        <is>
+          <t>+1037</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="4" t="inlineStr">
+        <is>
+          <t>Jhayco - Joe</t>
+        </is>
+      </c>
+      <c r="B52" s="5" t="n">
+        <v>10624</v>
+      </c>
+      <c r="C52" s="5" t="inlineStr">
+        <is>
+          <t>+1064</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="4" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="B53" s="5" t="n">
+        <v>10759</v>
+      </c>
+      <c r="C53" s="5" t="inlineStr">
+        <is>
+          <t>+1100</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="4" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="B54" s="5" t="n">
+        <v>10429</v>
+      </c>
+      <c r="C54" s="5" t="inlineStr">
+        <is>
+          <t>+893</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="4" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="B55" s="5" t="n">
+        <v>10444</v>
+      </c>
+      <c r="C55" s="5" t="inlineStr">
+        <is>
+          <t>+1000</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="4" t="inlineStr">
+        <is>
+          <t>Go Go Juice</t>
+        </is>
+      </c>
+      <c r="B56" s="5" t="n">
+        <v>8322</v>
+      </c>
+      <c r="C56" s="5" t="inlineStr">
+        <is>
+          <t>+600</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="4" t="inlineStr">
+        <is>
+          <t>Jhayco - Imaginaste</t>
+        </is>
+      </c>
+      <c r="B57" s="5" t="n">
+        <v>4560</v>
+      </c>
+      <c r="C57" s="5" t="inlineStr">
+        <is>
+          <t>+250</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="4" t="inlineStr">
+        <is>
+          <t>PuNch</t>
+        </is>
+      </c>
+      <c r="B58" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C58" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A2:C2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
auto: snapshot 2026-09-11 13:01:01
</commit_message>
<xml_diff>
--- a/clan_3815.xlsx
+++ b/clan_3815.xlsx
@@ -65,6 +65,7 @@
     <sheet name="2026-09-08" sheetId="56" state="visible" r:id="rId56"/>
     <sheet name="2026-09-09" sheetId="57" state="visible" r:id="rId57"/>
     <sheet name="2026-09-10" sheetId="58" state="visible" r:id="rId58"/>
+    <sheet name="2026-09-11" sheetId="59" state="visible" r:id="rId59"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -45481,6 +45482,885 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet59.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C58"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="29" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Clan: Mans Best Friend (3815)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Timestamp: 2026-09-11 13:01:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>Total Reps</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>Daily Reps (+1d)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>Nobodys Son</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="n">
+        <v>12044</v>
+      </c>
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>+8367</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>Player</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>Player</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>X y L O T A</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>AbdiHyde ID 13496</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>Create Character III</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C9" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>Create Character IV</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>Create Character V</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C11" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t>Player</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C12" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="4" t="inlineStr">
+        <is>
+          <t>Player</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C13" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="4" t="inlineStr">
+        <is>
+          <t>hunry</t>
+        </is>
+      </c>
+      <c r="B14" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C14" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="4" t="inlineStr">
+        <is>
+          <t>BlacKRin O</t>
+        </is>
+      </c>
+      <c r="B15" s="5" t="n">
+        <v>106</v>
+      </c>
+      <c r="C15" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="4" t="inlineStr">
+        <is>
+          <t>Tears</t>
+        </is>
+      </c>
+      <c r="B16" s="5" t="n">
+        <v>8383</v>
+      </c>
+      <c r="C16" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="4" t="inlineStr">
+        <is>
+          <t>NPC | SNOOPY</t>
+        </is>
+      </c>
+      <c r="B17" s="5" t="n">
+        <v>3165</v>
+      </c>
+      <c r="C17" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="4" t="inlineStr">
+        <is>
+          <t>Sugar Talking</t>
+        </is>
+      </c>
+      <c r="B18" s="5" t="n">
+        <v>4510</v>
+      </c>
+      <c r="C18" s="5" t="inlineStr">
+        <is>
+          <t>+1461</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="4" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B19" s="5" t="n">
+        <v>10804</v>
+      </c>
+      <c r="C19" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="4" t="inlineStr">
+        <is>
+          <t>Anti-Hero</t>
+        </is>
+      </c>
+      <c r="B20" s="5" t="n">
+        <v>11439</v>
+      </c>
+      <c r="C20" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="4" t="inlineStr">
+        <is>
+          <t>Vigilante Shit</t>
+        </is>
+      </c>
+      <c r="B21" s="5" t="n">
+        <v>10872</v>
+      </c>
+      <c r="C21" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="4" t="inlineStr">
+        <is>
+          <t>Sweet Nothing</t>
+        </is>
+      </c>
+      <c r="B22" s="5" t="n">
+        <v>9673</v>
+      </c>
+      <c r="C22" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="4" t="inlineStr">
+        <is>
+          <t>The Great War</t>
+        </is>
+      </c>
+      <c r="B23" s="5" t="n">
+        <v>10828</v>
+      </c>
+      <c r="C23" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">We Almost Broke Up </t>
+        </is>
+      </c>
+      <c r="B24" s="5" t="n">
+        <v>2802</v>
+      </c>
+      <c r="C24" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="4" t="inlineStr">
+        <is>
+          <t>When Did You Get Hot</t>
+        </is>
+      </c>
+      <c r="B25" s="5" t="n">
+        <v>3165</v>
+      </c>
+      <c r="C25" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="4" t="inlineStr">
+        <is>
+          <t>Dont Worry Ill Make</t>
+        </is>
+      </c>
+      <c r="B26" s="5" t="n">
+        <v>2897</v>
+      </c>
+      <c r="C26" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="4" t="inlineStr">
+        <is>
+          <t>Goodbye</t>
+        </is>
+      </c>
+      <c r="B27" s="5" t="n">
+        <v>10913</v>
+      </c>
+      <c r="C27" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="4" t="inlineStr">
+        <is>
+          <t>Mans Best Friend</t>
+        </is>
+      </c>
+      <c r="B28" s="5" t="n">
+        <v>10842</v>
+      </c>
+      <c r="C28" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="4" t="inlineStr">
+        <is>
+          <t>Lavender Haze</t>
+        </is>
+      </c>
+      <c r="B29" s="5" t="n">
+        <v>10715</v>
+      </c>
+      <c r="C29" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="4" t="inlineStr">
+        <is>
+          <t>Never Getting Laid</t>
+        </is>
+      </c>
+      <c r="B30" s="5" t="n">
+        <v>8976</v>
+      </c>
+      <c r="C30" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="4" t="inlineStr">
+        <is>
+          <t>My Man on Willpower</t>
+        </is>
+      </c>
+      <c r="B31" s="5" t="n">
+        <v>7648</v>
+      </c>
+      <c r="C31" s="5" t="inlineStr">
+        <is>
+          <t>+3746</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="4" t="inlineStr">
+        <is>
+          <t>Manchild</t>
+        </is>
+      </c>
+      <c r="B32" s="5" t="n">
+        <v>7152</v>
+      </c>
+      <c r="C32" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="4" t="inlineStr">
+        <is>
+          <t>Sugar Talking</t>
+        </is>
+      </c>
+      <c r="B33" s="5" t="n">
+        <v>3049</v>
+      </c>
+      <c r="C33" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="4" t="inlineStr">
+        <is>
+          <t>My Man on Willpower</t>
+        </is>
+      </c>
+      <c r="B34" s="5" t="n">
+        <v>3902</v>
+      </c>
+      <c r="C34" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="4" t="inlineStr">
+        <is>
+          <t>Midnight Rain</t>
+        </is>
+      </c>
+      <c r="B35" s="5" t="n">
+        <v>10568</v>
+      </c>
+      <c r="C35" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="4" t="inlineStr">
+        <is>
+          <t>Nobodys Son</t>
+        </is>
+      </c>
+      <c r="B36" s="5" t="n">
+        <v>3677</v>
+      </c>
+      <c r="C36" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="4" t="inlineStr">
+        <is>
+          <t>House Tour</t>
+        </is>
+      </c>
+      <c r="B37" s="5" t="n">
+        <v>2782</v>
+      </c>
+      <c r="C37" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="4" t="inlineStr">
+        <is>
+          <t>Hanabi  Î±Î·Ð²Ï…</t>
+        </is>
+      </c>
+      <c r="B38" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C38" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="4" t="inlineStr">
+        <is>
+          <t>Saiyajin anbuâ„¢</t>
+        </is>
+      </c>
+      <c r="B39" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C39" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="4" t="inlineStr">
+        <is>
+          <t>Dummy</t>
+        </is>
+      </c>
+      <c r="B40" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C40" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="4" t="inlineStr">
+        <is>
+          <t>Cazador anbu â„¢</t>
+        </is>
+      </c>
+      <c r="B41" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C41" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="4" t="inlineStr">
+        <is>
+          <t>Besos Mojados</t>
+        </is>
+      </c>
+      <c r="B42" s="5" t="n">
+        <v>4682</v>
+      </c>
+      <c r="C42" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="4" t="inlineStr">
+        <is>
+          <t>DarkFire</t>
+        </is>
+      </c>
+      <c r="B43" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C43" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="4" t="inlineStr">
+        <is>
+          <t>DarkSunny</t>
+        </is>
+      </c>
+      <c r="B44" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C44" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="4" t="inlineStr">
+        <is>
+          <t>Dairen Uchiha</t>
+        </is>
+      </c>
+      <c r="B45" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C45" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="4" t="inlineStr">
+        <is>
+          <t>LILI ZENIN®</t>
+        </is>
+      </c>
+      <c r="B46" s="5" t="n">
+        <v>64</v>
+      </c>
+      <c r="C46" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="4" t="inlineStr">
+        <is>
+          <t>ryumichel ZENIN ®</t>
+        </is>
+      </c>
+      <c r="B47" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C47" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="4" t="inlineStr">
+        <is>
+          <t>margot ZENIN ®</t>
+        </is>
+      </c>
+      <c r="B48" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C48" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="4" t="inlineStr">
+        <is>
+          <t>linda ZENIN ®</t>
+        </is>
+      </c>
+      <c r="B49" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C49" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="4" t="inlineStr">
+        <is>
+          <t>equin0x</t>
+        </is>
+      </c>
+      <c r="B50" s="5" t="n">
+        <v>992</v>
+      </c>
+      <c r="C50" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="4" t="inlineStr">
+        <is>
+          <t>Jhayco - Mokai</t>
+        </is>
+      </c>
+      <c r="B51" s="5" t="n">
+        <v>10771</v>
+      </c>
+      <c r="C51" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="4" t="inlineStr">
+        <is>
+          <t>Jhayco - Joe</t>
+        </is>
+      </c>
+      <c r="B52" s="5" t="n">
+        <v>10624</v>
+      </c>
+      <c r="C52" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="4" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="B53" s="5" t="n">
+        <v>10759</v>
+      </c>
+      <c r="C53" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="4" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="B54" s="5" t="n">
+        <v>10429</v>
+      </c>
+      <c r="C54" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="4" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="B55" s="5" t="n">
+        <v>10444</v>
+      </c>
+      <c r="C55" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="4" t="inlineStr">
+        <is>
+          <t>Go Go Juice</t>
+        </is>
+      </c>
+      <c r="B56" s="5" t="n">
+        <v>8322</v>
+      </c>
+      <c r="C56" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="4" t="inlineStr">
+        <is>
+          <t>Jhayco - Imaginaste</t>
+        </is>
+      </c>
+      <c r="B57" s="5" t="n">
+        <v>4560</v>
+      </c>
+      <c r="C57" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="4" t="inlineStr">
+        <is>
+          <t>PuNch</t>
+        </is>
+      </c>
+      <c r="B58" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C58" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A2:C2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
auto: snapshot 2026-09-12 13:01:01
</commit_message>
<xml_diff>
--- a/clan_3815.xlsx
+++ b/clan_3815.xlsx
@@ -66,6 +66,7 @@
     <sheet name="2026-09-09" sheetId="57" state="visible" r:id="rId57"/>
     <sheet name="2026-09-10" sheetId="58" state="visible" r:id="rId58"/>
     <sheet name="2026-09-11" sheetId="59" state="visible" r:id="rId59"/>
+    <sheet name="2026-09-12" sheetId="60" state="visible" r:id="rId60"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -47045,6 +47046,885 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet60.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C58"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="29" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Clan: Mans Best Friend (3815)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Timestamp: 2026-09-12 13:01:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>Total Reps</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>Daily Reps (+1d)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>Nobodys Son</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="n">
+        <v>12044</v>
+      </c>
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>+8367</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>Player</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>Player</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>X y L O T A</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>AbdiHyde ID 13496</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>Create Character III</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C9" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>Create Character IV</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>Create Character V</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C11" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t>Player</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C12" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="4" t="inlineStr">
+        <is>
+          <t>Player</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C13" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="4" t="inlineStr">
+        <is>
+          <t>hunry</t>
+        </is>
+      </c>
+      <c r="B14" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C14" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="4" t="inlineStr">
+        <is>
+          <t>BlacKRin O</t>
+        </is>
+      </c>
+      <c r="B15" s="5" t="n">
+        <v>106</v>
+      </c>
+      <c r="C15" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="4" t="inlineStr">
+        <is>
+          <t>Tears</t>
+        </is>
+      </c>
+      <c r="B16" s="5" t="n">
+        <v>8383</v>
+      </c>
+      <c r="C16" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="4" t="inlineStr">
+        <is>
+          <t>NPC | SNOOPY</t>
+        </is>
+      </c>
+      <c r="B17" s="5" t="n">
+        <v>3165</v>
+      </c>
+      <c r="C17" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="4" t="inlineStr">
+        <is>
+          <t>Sugar Talking</t>
+        </is>
+      </c>
+      <c r="B18" s="5" t="n">
+        <v>4510</v>
+      </c>
+      <c r="C18" s="5" t="inlineStr">
+        <is>
+          <t>+1461</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="4" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B19" s="5" t="n">
+        <v>10804</v>
+      </c>
+      <c r="C19" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="4" t="inlineStr">
+        <is>
+          <t>Anti-Hero</t>
+        </is>
+      </c>
+      <c r="B20" s="5" t="n">
+        <v>11439</v>
+      </c>
+      <c r="C20" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="4" t="inlineStr">
+        <is>
+          <t>Vigilante Shit</t>
+        </is>
+      </c>
+      <c r="B21" s="5" t="n">
+        <v>10872</v>
+      </c>
+      <c r="C21" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="4" t="inlineStr">
+        <is>
+          <t>Sweet Nothing</t>
+        </is>
+      </c>
+      <c r="B22" s="5" t="n">
+        <v>9673</v>
+      </c>
+      <c r="C22" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="4" t="inlineStr">
+        <is>
+          <t>The Great War</t>
+        </is>
+      </c>
+      <c r="B23" s="5" t="n">
+        <v>10828</v>
+      </c>
+      <c r="C23" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">We Almost Broke Up </t>
+        </is>
+      </c>
+      <c r="B24" s="5" t="n">
+        <v>2802</v>
+      </c>
+      <c r="C24" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="4" t="inlineStr">
+        <is>
+          <t>When Did You Get Hot</t>
+        </is>
+      </c>
+      <c r="B25" s="5" t="n">
+        <v>3165</v>
+      </c>
+      <c r="C25" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="4" t="inlineStr">
+        <is>
+          <t>Dont Worry Ill Make</t>
+        </is>
+      </c>
+      <c r="B26" s="5" t="n">
+        <v>2897</v>
+      </c>
+      <c r="C26" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="4" t="inlineStr">
+        <is>
+          <t>Goodbye</t>
+        </is>
+      </c>
+      <c r="B27" s="5" t="n">
+        <v>10913</v>
+      </c>
+      <c r="C27" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="4" t="inlineStr">
+        <is>
+          <t>Mans Best Friend</t>
+        </is>
+      </c>
+      <c r="B28" s="5" t="n">
+        <v>10842</v>
+      </c>
+      <c r="C28" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="4" t="inlineStr">
+        <is>
+          <t>Lavender Haze</t>
+        </is>
+      </c>
+      <c r="B29" s="5" t="n">
+        <v>10715</v>
+      </c>
+      <c r="C29" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="4" t="inlineStr">
+        <is>
+          <t>Never Getting Laid</t>
+        </is>
+      </c>
+      <c r="B30" s="5" t="n">
+        <v>8976</v>
+      </c>
+      <c r="C30" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="4" t="inlineStr">
+        <is>
+          <t>My Man on Willpower</t>
+        </is>
+      </c>
+      <c r="B31" s="5" t="n">
+        <v>7648</v>
+      </c>
+      <c r="C31" s="5" t="inlineStr">
+        <is>
+          <t>+3746</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="4" t="inlineStr">
+        <is>
+          <t>Manchild</t>
+        </is>
+      </c>
+      <c r="B32" s="5" t="n">
+        <v>7152</v>
+      </c>
+      <c r="C32" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="4" t="inlineStr">
+        <is>
+          <t>Sugar Talking</t>
+        </is>
+      </c>
+      <c r="B33" s="5" t="n">
+        <v>3049</v>
+      </c>
+      <c r="C33" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="4" t="inlineStr">
+        <is>
+          <t>My Man on Willpower</t>
+        </is>
+      </c>
+      <c r="B34" s="5" t="n">
+        <v>3902</v>
+      </c>
+      <c r="C34" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="4" t="inlineStr">
+        <is>
+          <t>Midnight Rain</t>
+        </is>
+      </c>
+      <c r="B35" s="5" t="n">
+        <v>10568</v>
+      </c>
+      <c r="C35" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="4" t="inlineStr">
+        <is>
+          <t>Nobodys Son</t>
+        </is>
+      </c>
+      <c r="B36" s="5" t="n">
+        <v>3677</v>
+      </c>
+      <c r="C36" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="4" t="inlineStr">
+        <is>
+          <t>House Tour</t>
+        </is>
+      </c>
+      <c r="B37" s="5" t="n">
+        <v>2782</v>
+      </c>
+      <c r="C37" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="4" t="inlineStr">
+        <is>
+          <t>Hanabi  Î±Î·Ð²Ï…</t>
+        </is>
+      </c>
+      <c r="B38" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C38" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="4" t="inlineStr">
+        <is>
+          <t>Saiyajin anbuâ„¢</t>
+        </is>
+      </c>
+      <c r="B39" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C39" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="4" t="inlineStr">
+        <is>
+          <t>Dummy</t>
+        </is>
+      </c>
+      <c r="B40" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C40" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="4" t="inlineStr">
+        <is>
+          <t>Cazador anbu â„¢</t>
+        </is>
+      </c>
+      <c r="B41" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C41" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="4" t="inlineStr">
+        <is>
+          <t>Besos Mojados</t>
+        </is>
+      </c>
+      <c r="B42" s="5" t="n">
+        <v>4682</v>
+      </c>
+      <c r="C42" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="4" t="inlineStr">
+        <is>
+          <t>DarkFire</t>
+        </is>
+      </c>
+      <c r="B43" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C43" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="4" t="inlineStr">
+        <is>
+          <t>DarkSunny</t>
+        </is>
+      </c>
+      <c r="B44" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C44" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="4" t="inlineStr">
+        <is>
+          <t>Dairen Uchiha</t>
+        </is>
+      </c>
+      <c r="B45" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C45" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="4" t="inlineStr">
+        <is>
+          <t>LILI ZENIN®</t>
+        </is>
+      </c>
+      <c r="B46" s="5" t="n">
+        <v>64</v>
+      </c>
+      <c r="C46" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="4" t="inlineStr">
+        <is>
+          <t>ryumichel ZENIN ®</t>
+        </is>
+      </c>
+      <c r="B47" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C47" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="4" t="inlineStr">
+        <is>
+          <t>margot ZENIN ®</t>
+        </is>
+      </c>
+      <c r="B48" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C48" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="4" t="inlineStr">
+        <is>
+          <t>linda ZENIN ®</t>
+        </is>
+      </c>
+      <c r="B49" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C49" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="4" t="inlineStr">
+        <is>
+          <t>equin0x</t>
+        </is>
+      </c>
+      <c r="B50" s="5" t="n">
+        <v>992</v>
+      </c>
+      <c r="C50" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="4" t="inlineStr">
+        <is>
+          <t>Jhayco - Mokai</t>
+        </is>
+      </c>
+      <c r="B51" s="5" t="n">
+        <v>10771</v>
+      </c>
+      <c r="C51" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="4" t="inlineStr">
+        <is>
+          <t>Jhayco - Joe</t>
+        </is>
+      </c>
+      <c r="B52" s="5" t="n">
+        <v>10624</v>
+      </c>
+      <c r="C52" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="4" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="B53" s="5" t="n">
+        <v>10759</v>
+      </c>
+      <c r="C53" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="4" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="B54" s="5" t="n">
+        <v>10429</v>
+      </c>
+      <c r="C54" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="4" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="B55" s="5" t="n">
+        <v>10444</v>
+      </c>
+      <c r="C55" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="4" t="inlineStr">
+        <is>
+          <t>Go Go Juice</t>
+        </is>
+      </c>
+      <c r="B56" s="5" t="n">
+        <v>8322</v>
+      </c>
+      <c r="C56" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="4" t="inlineStr">
+        <is>
+          <t>Jhayco - Imaginaste</t>
+        </is>
+      </c>
+      <c r="B57" s="5" t="n">
+        <v>4560</v>
+      </c>
+      <c r="C57" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="4" t="inlineStr">
+        <is>
+          <t>PuNch</t>
+        </is>
+      </c>
+      <c r="B58" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C58" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A2:C2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>